<commit_message>
BOM_LCSC.xlsx: re-priced for a single board
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Needed (5 boards)</t>
+          <t>Needed (1 boards)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -564,7 +564,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -613,13 +613,13 @@
         <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O2" t="n">
         <v>0.8873</v>
       </c>
       <c r="P2" t="n">
-        <v>4.4365</v>
+        <v>0.8873</v>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -693,13 +693,13 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O3" t="n">
         <v>2.2026</v>
       </c>
       <c r="P3" t="n">
-        <v>11.013</v>
+        <v>2.2026</v>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
@@ -724,7 +724,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -773,13 +773,13 @@
         <v>1</v>
       </c>
       <c r="N4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O4" t="n">
         <v>0.0153</v>
       </c>
       <c r="P4" t="n">
-        <v>0.153</v>
+        <v>0.0306</v>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>C577008 CC0805KRX5R6BB105 0.17 USD</t>
+          <t>C577008 CC0805KRX5R6BB105 0.03 USD</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -812,7 +812,7 @@
         <v>53</v>
       </c>
       <c r="C5" t="n">
-        <v>265</v>
+        <v>53</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -861,13 +861,13 @@
         <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>265</v>
+        <v>53</v>
       </c>
       <c r="O5" t="n">
         <v>0.003</v>
       </c>
       <c r="P5" t="n">
-        <v>0.795</v>
+        <v>0.159</v>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
@@ -881,7 +881,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>C2846674 0201X104K160NT 0.87 USD</t>
+          <t>C2846674 0201X104K160NT 0.17 USD</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -896,7 +896,7 @@
         <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -915,17 +915,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>C3012377</t>
+          <t>C6600400</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CSA0402X7R104K500GT</t>
+          <t>MSASU105SB7104KFNB25</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>Taiyo Yuden</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -939,23 +939,23 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>459286</v>
+        <v>22</v>
       </c>
       <c r="M6" t="n">
         <v>1</v>
       </c>
       <c r="N6" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0044</v>
+        <v>0.004</v>
       </c>
       <c r="P6" t="n">
-        <v>0.264</v>
+        <v>0.048</v>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3012377.html</t>
+          <t>https://www.lcsc.com/product-detail/C6600400.html</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>C48543623 TCC0402X7R104K500ATM 0.27 USD</t>
+          <t>C3012377 CSA0402X7R104K500GT 0.05 USD</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
@@ -980,7 +980,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1029,13 +1029,13 @@
         <v>1</v>
       </c>
       <c r="N7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O7" t="n">
         <v>0.002</v>
       </c>
       <c r="P7" t="n">
-        <v>0.01</v>
+        <v>0.002</v>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>C482486 HGC0402G0101J500NTEJ 0.01 USD</t>
+          <t>C482486 HGC0402G0101J500NTEJ 0.00 USD</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1064,7 +1064,7 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1113,13 +1113,13 @@
         <v>1</v>
       </c>
       <c r="N8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O8" t="n">
         <v>0.0029</v>
       </c>
       <c r="P8" t="n">
-        <v>0.0145</v>
+        <v>0.0029</v>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>C2887023 TCC0402COG121J500AT 0.02 USD</t>
+          <t>C2887023 TCC0402COG121J500AT 0.00 USD</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1148,7 +1148,7 @@
         <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1197,13 +1197,13 @@
         <v>1</v>
       </c>
       <c r="N9" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O9" t="n">
         <v>0.0014</v>
       </c>
       <c r="P9" t="n">
-        <v>0.014</v>
+        <v>0.0028</v>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>C106201 CC0402JRNPO9BN120 0.02 USD</t>
+          <t>C106201 CC0402JRNPO9BN120 0.00 USD</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1232,7 +1232,7 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1281,13 +1281,13 @@
         <v>1</v>
       </c>
       <c r="N10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O10" t="n">
         <v>0.0012</v>
       </c>
       <c r="P10" t="n">
-        <v>0.005999999999999999</v>
+        <v>0.0012</v>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>C295959 0402N150K500CT 0.01 USD</t>
+          <t>C295959 0402N150K500CT 0.00 USD</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1316,7 +1316,7 @@
         <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1335,17 +1335,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>C107000</t>
+          <t>C696863</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>CC0402JRNPO9BN200</t>
+          <t>TCC0402COG200K500AT</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>CCTC</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1359,33 +1359,33 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>3263489</v>
+        <v>17</v>
       </c>
       <c r="M11" t="n">
         <v>1</v>
       </c>
       <c r="N11" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="O11" t="n">
-        <v>0.0021</v>
+        <v>0.0004</v>
       </c>
       <c r="P11" t="n">
-        <v>0.042</v>
+        <v>0.0016</v>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C107000.html</t>
+          <t>https://www.lcsc.com/product-detail/C696863.html</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>20pF 50V NP0 ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>20pF 50V C0G ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>C5137579 FCC0402N200J500AT 0.05 USD</t>
+          <t>C107000 CC0402JRNPO9BN200 0.01 USD</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -1400,7 +1400,7 @@
         <v>2</v>
       </c>
       <c r="C12" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1449,13 +1449,13 @@
         <v>1</v>
       </c>
       <c r="N12" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O12" t="n">
         <v>0.0065</v>
       </c>
       <c r="P12" t="n">
-        <v>0.065</v>
+        <v>0.013</v>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>C5159775 GRM155R61H224KE01D 0.19 USD</t>
+          <t>C5159775 GRM155R61H224KE01D 0.04 USD</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -1484,7 +1484,7 @@
         <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1520,7 +1520,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1569,13 +1569,13 @@
         <v>1</v>
       </c>
       <c r="N14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O14" t="n">
         <v>0.3727</v>
       </c>
       <c r="P14" t="n">
-        <v>1.8635</v>
+        <v>0.3727</v>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>C22415740 C1206C105J5RACTU 4.51 USD</t>
+          <t>C22415740 C1206C105J5RACTU 0.90 USD</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -1604,7 +1604,7 @@
         <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1653,13 +1653,13 @@
         <v>1</v>
       </c>
       <c r="N15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O15" t="n">
         <v>0.3727</v>
       </c>
       <c r="P15" t="n">
-        <v>1.8635</v>
+        <v>0.3727</v>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>C22415740 C1206C105J5RACTU 4.51 USD</t>
+          <t>C22415740 C1206C105J5RACTU 0.90 USD</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -1688,7 +1688,7 @@
         <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1737,13 +1737,13 @@
         <v>1</v>
       </c>
       <c r="N16" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O16" t="n">
-        <v>0.5863</v>
+        <v>0.7086</v>
       </c>
       <c r="P16" t="n">
-        <v>5.863</v>
+        <v>1.4172</v>
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
@@ -1772,7 +1772,7 @@
         <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1815,19 +1815,19 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>53104</v>
+        <v>53084</v>
       </c>
       <c r="M17" t="n">
         <v>1</v>
       </c>
       <c r="N17" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O17" t="n">
         <v>0.0051</v>
       </c>
       <c r="P17" t="n">
-        <v>0.0255</v>
+        <v>0.0051</v>
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1901,13 +1901,13 @@
         <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="O18" t="n">
         <v>0.0121</v>
       </c>
       <c r="P18" t="n">
-        <v>0.1815</v>
+        <v>0.0363</v>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
@@ -1932,7 +1932,7 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1981,13 +1981,13 @@
         <v>1</v>
       </c>
       <c r="N19" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="O19" t="n">
         <v>0.1716</v>
       </c>
       <c r="P19" t="n">
-        <v>4.29</v>
+        <v>0.858</v>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
@@ -2012,7 +2012,7 @@
         <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2061,13 +2061,13 @@
         <v>1</v>
       </c>
       <c r="N20" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O20" t="n">
         <v>0.1541</v>
       </c>
       <c r="P20" t="n">
-        <v>1.541</v>
+        <v>0.3082</v>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
         <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2135,19 +2135,19 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>7209</v>
+        <v>7199</v>
       </c>
       <c r="M21" t="n">
         <v>1</v>
       </c>
       <c r="N21" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="O21" t="n">
-        <v>0.8325</v>
+        <v>0.9814000000000001</v>
       </c>
       <c r="P21" t="n">
-        <v>12.4875</v>
+        <v>2.9442</v>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
@@ -2172,7 +2172,7 @@
         <v>2</v>
       </c>
       <c r="C22" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2221,13 +2221,13 @@
         <v>1</v>
       </c>
       <c r="N22" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O22" t="n">
-        <v>0.9594</v>
+        <v>1.0864</v>
       </c>
       <c r="P22" t="n">
-        <v>9.594000000000001</v>
+        <v>2.1728</v>
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
@@ -2252,7 +2252,7 @@
         <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2295,19 +2295,19 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>616349</v>
+        <v>616329</v>
       </c>
       <c r="M23" t="n">
         <v>1</v>
       </c>
       <c r="N23" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O23" t="n">
         <v>0.0209</v>
       </c>
       <c r="P23" t="n">
-        <v>0.1045</v>
+        <v>0.0209</v>
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>C6119842 CGA0603X5R106K100JT 0.11 USD</t>
+          <t>C6119842 CGA0603X5R106K100JT 0.02 USD</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
         <v>12</v>
       </c>
       <c r="C24" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2379,19 +2379,19 @@
         </is>
       </c>
       <c r="L24" t="n">
-        <v>616349</v>
+        <v>616329</v>
       </c>
       <c r="M24" t="n">
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="O24" t="n">
         <v>0.0209</v>
       </c>
       <c r="P24" t="n">
-        <v>1.254</v>
+        <v>0.2508</v>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>C6119842 CGA0603X5R106K100JT 1.33 USD</t>
+          <t>C6119842 CGA0603X5R106K100JT 0.27 USD</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
@@ -2420,7 +2420,7 @@
         <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2439,17 +2439,17 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>C49326606</t>
+          <t>C5189828</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0603X7R105K100NT</t>
+          <t>CS1608X7R105K100NRB</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>AIDE CAPACITOR</t>
+          <t>Samwha Capacitor</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2463,23 +2463,23 @@
         </is>
       </c>
       <c r="L25" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
         <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O25" t="n">
-        <v>0.0055</v>
+        <v>0.0043</v>
       </c>
       <c r="P25" t="n">
-        <v>0.0275</v>
+        <v>0.0043</v>
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49326606.html</t>
+          <t>https://www.lcsc.com/product-detail/C5189828.html</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>C20416424 TCC0603X5R105K100CT 0.04 USD</t>
+          <t>C49326606 0603X7R105K100NT 0.01 USD</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -2504,7 +2504,7 @@
         <v>6</v>
       </c>
       <c r="C26" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2553,13 +2553,13 @@
         <v>1</v>
       </c>
       <c r="N26" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="O26" t="n">
         <v>0.0248</v>
       </c>
       <c r="P26" t="n">
-        <v>0.744</v>
+        <v>0.1488</v>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>C59461 CL10A226MQ8NRNC 0.90 USD</t>
+          <t>C22376489 FS18B226M6R3PBG 0.17 USD</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
@@ -2588,7 +2588,7 @@
         <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2637,13 +2637,13 @@
         <v>1</v>
       </c>
       <c r="N27" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="O27" t="n">
         <v>0.0153</v>
       </c>
       <c r="P27" t="n">
-        <v>0.2295</v>
+        <v>0.0459</v>
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>C54863492 DSK24 0.24 USD</t>
+          <t>C54863492 DSK24 0.05 USD</t>
         </is>
       </c>
       <c r="T27" t="inlineStr"/>
@@ -2672,7 +2672,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2721,13 +2721,13 @@
         <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O28" t="n">
         <v>0.0127</v>
       </c>
       <c r="P28" t="n">
-        <v>0.0635</v>
+        <v>0.0127</v>
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
@@ -2756,7 +2756,7 @@
         <v>1</v>
       </c>
       <c r="C29" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2805,13 +2805,13 @@
         <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O29" t="n">
         <v>0.4515</v>
       </c>
       <c r="P29" t="n">
-        <v>2.2575</v>
+        <v>0.4515</v>
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
@@ -2836,7 +2836,7 @@
         <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2885,13 +2885,13 @@
         <v>1</v>
       </c>
       <c r="N30" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O30" t="n">
         <v>0.0275</v>
       </c>
       <c r="P30" t="n">
-        <v>0.1375</v>
+        <v>0.0275</v>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>C53199108 DMG2301L-7(ES) 0.16 USD</t>
+          <t>C53199108 DMG2301L-7(ES) 0.03 USD</t>
         </is>
       </c>
       <c r="T30" t="inlineStr"/>
@@ -2920,7 +2920,7 @@
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2969,13 +2969,13 @@
         <v>1</v>
       </c>
       <c r="N31" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O31" t="n">
         <v>0.0157</v>
       </c>
       <c r="P31" t="n">
-        <v>0.157</v>
+        <v>0.0314</v>
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>C5224188 DMG2302UK-7-ES 0.20 USD</t>
+          <t>C5224188 DMG2302UK-7-ES 0.04 USD</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
@@ -3008,7 +3008,7 @@
         <v>3</v>
       </c>
       <c r="C32" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -3057,13 +3057,13 @@
         <v>1</v>
       </c>
       <c r="N32" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="O32" t="n">
         <v>0.103</v>
       </c>
       <c r="P32" t="n">
-        <v>1.545</v>
+        <v>0.309</v>
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
@@ -3077,7 +3077,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>C2937001 PRTR5V0U2F 2.73 USD</t>
+          <t>C52994078 PRTR5V0U2F,115(ES) 0.53 USD</t>
         </is>
       </c>
       <c r="T32" t="inlineStr"/>
@@ -3092,7 +3092,7 @@
         <v>1</v>
       </c>
       <c r="C33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -3141,13 +3141,13 @@
         <v>1</v>
       </c>
       <c r="N33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O33" t="n">
         <v>0.0018</v>
       </c>
       <c r="P33" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0018</v>
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>C177661 RCT0310RFLF 0.01 USD</t>
+          <t>C177661 RCT0310RFLF 0.00 USD</t>
         </is>
       </c>
       <c r="T33" t="inlineStr"/>
@@ -3176,7 +3176,7 @@
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -3225,13 +3225,13 @@
         <v>1</v>
       </c>
       <c r="N34" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O34" t="n">
         <v>0.0018</v>
       </c>
       <c r="P34" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0018</v>
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
@@ -3245,7 +3245,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>C49654665 GR0603F4R02T5G00 0.01 USD</t>
+          <t>C322168 RS-03L4R02FT 0.00 USD</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -3264,7 +3264,7 @@
         <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -3313,13 +3313,13 @@
         <v>1</v>
       </c>
       <c r="N35" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O35" t="n">
         <v>0.0784</v>
       </c>
       <c r="P35" t="n">
-        <v>0.392</v>
+        <v>0.0784</v>
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
@@ -3344,7 +3344,7 @@
         <v>3</v>
       </c>
       <c r="C36" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -3393,13 +3393,13 @@
         <v>1</v>
       </c>
       <c r="N36" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="O36" t="n">
         <v>0.038</v>
       </c>
       <c r="P36" t="n">
-        <v>0.57</v>
+        <v>0.114</v>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
@@ -3413,7 +3413,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>C157932 S2B-PH-K-S-GW 3.19 USD</t>
+          <t>C157932 S2B-PH-K-S-GW 0.64 USD</t>
         </is>
       </c>
       <c r="T36" t="inlineStr"/>
@@ -3428,7 +3428,7 @@
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -3477,13 +3477,13 @@
         <v>1</v>
       </c>
       <c r="N37" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O37" t="n">
         <v>13.3061</v>
       </c>
       <c r="P37" t="n">
-        <v>66.5305</v>
+        <v>13.3061</v>
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
@@ -3508,7 +3508,7 @@
         <v>2</v>
       </c>
       <c r="C38" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -3557,13 +3557,13 @@
         <v>1</v>
       </c>
       <c r="N38" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O38" t="n">
         <v>0.0698</v>
       </c>
       <c r="P38" t="n">
-        <v>0.698</v>
+        <v>0.1396</v>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
@@ -3592,7 +3592,7 @@
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -3641,13 +3641,13 @@
         <v>1</v>
       </c>
       <c r="N39" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O39" t="n">
         <v>0.0005</v>
       </c>
       <c r="P39" t="n">
-        <v>0.0025</v>
+        <v>0.0005</v>
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
@@ -3676,7 +3676,7 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -3725,13 +3725,13 @@
         <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O40" t="n">
         <v>0.0005</v>
       </c>
       <c r="P40" t="n">
-        <v>0.0025</v>
+        <v>0.0005</v>
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
@@ -3760,7 +3760,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3809,13 +3809,13 @@
         <v>1</v>
       </c>
       <c r="N41" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O41" t="n">
         <v>0.0005</v>
       </c>
       <c r="P41" t="n">
-        <v>0.0025</v>
+        <v>0.0005</v>
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
@@ -3844,7 +3844,7 @@
         <v>20</v>
       </c>
       <c r="C42" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -3893,13 +3893,13 @@
         <v>1</v>
       </c>
       <c r="N42" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="O42" t="n">
         <v>0.0011</v>
       </c>
       <c r="P42" t="n">
-        <v>0.11</v>
+        <v>0.022</v>
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>C2759534 HP02WAF1003TCE 0.13 USD</t>
+          <t>C2759534 HP02WAF1003TCE 0.03 USD</t>
         </is>
       </c>
       <c r="T42" t="inlineStr"/>
@@ -3928,7 +3928,7 @@
         <v>18</v>
       </c>
       <c r="C43" t="n">
-        <v>90</v>
+        <v>18</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -3977,13 +3977,13 @@
         <v>1</v>
       </c>
       <c r="N43" t="n">
-        <v>90</v>
+        <v>18</v>
       </c>
       <c r="O43" t="n">
         <v>0.0018</v>
       </c>
       <c r="P43" t="n">
-        <v>0.162</v>
+        <v>0.0324</v>
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
@@ -3997,7 +3997,7 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>C327797 MR04X1002FTL 0.23 USD</t>
+          <t>C327797 MR04X1002FTL 0.04 USD</t>
         </is>
       </c>
       <c r="T43" t="inlineStr"/>
@@ -4012,7 +4012,7 @@
         <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -4061,13 +4061,13 @@
         <v>1</v>
       </c>
       <c r="N44" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O44" t="n">
         <v>0.0007</v>
       </c>
       <c r="P44" t="n">
-        <v>0.0035</v>
+        <v>0.0007</v>
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
@@ -4096,7 +4096,7 @@
         <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -4145,13 +4145,13 @@
         <v>1</v>
       </c>
       <c r="N45" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O45" t="n">
         <v>0.0005</v>
       </c>
       <c r="P45" t="n">
-        <v>0.0025</v>
+        <v>0.0005</v>
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
@@ -4180,7 +4180,7 @@
         <v>2</v>
       </c>
       <c r="C46" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -4229,13 +4229,13 @@
         <v>1</v>
       </c>
       <c r="N46" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O46" t="n">
         <v>0.0005</v>
       </c>
       <c r="P46" t="n">
-        <v>0.005</v>
+        <v>0.001</v>
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>C46635169 CL0402FN200RP 0.01 USD</t>
+          <t>C46635169 CL0402FN200RP 0.00 USD</t>
         </is>
       </c>
       <c r="T46" t="inlineStr"/>
@@ -4264,7 +4264,7 @@
         <v>1</v>
       </c>
       <c r="C47" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -4313,13 +4313,13 @@
         <v>1</v>
       </c>
       <c r="N47" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O47" t="n">
         <v>0.0005</v>
       </c>
       <c r="P47" t="n">
-        <v>0.0025</v>
+        <v>0.0005</v>
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>C54920643 HRC0402F2003DNTO 0.00 USD</t>
+          <t>C3015901 SCR0402F200K 0.00 USD</t>
         </is>
       </c>
       <c r="T47" t="inlineStr"/>
@@ -4348,7 +4348,7 @@
         <v>1</v>
       </c>
       <c r="C48" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -4397,13 +4397,13 @@
         <v>1</v>
       </c>
       <c r="N48" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O48" t="n">
         <v>0.0005999999999999999</v>
       </c>
       <c r="P48" t="n">
-        <v>0.003</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
@@ -4432,7 +4432,7 @@
         <v>4</v>
       </c>
       <c r="C49" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -4451,17 +4451,17 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>C49652940</t>
+          <t>C168215</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>GR0402F240RTAG00</t>
+          <t>WR04X2400FTL</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>Walsin Tech Corp</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -4475,23 +4475,23 @@
         </is>
       </c>
       <c r="L49" t="n">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="M49" t="n">
         <v>1</v>
       </c>
       <c r="N49" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="O49" t="n">
-        <v>0.0008</v>
+        <v>0.0004</v>
       </c>
       <c r="P49" t="n">
-        <v>0.016</v>
+        <v>0.0016</v>
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49652940.html</t>
+          <t>https://www.lcsc.com/product-detail/C168215.html</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4501,7 +4501,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>C22356255 RCA02240RFLF 0.02 USD</t>
+          <t>C49652940 GR0402F240RTAG00 0.00 USD</t>
         </is>
       </c>
       <c r="T49" t="inlineStr"/>
@@ -4516,7 +4516,7 @@
         <v>1</v>
       </c>
       <c r="C50" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -4565,13 +4565,13 @@
         <v>1</v>
       </c>
       <c r="N50" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O50" t="n">
         <v>0.0005999999999999999</v>
       </c>
       <c r="P50" t="n">
-        <v>0.003</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
@@ -4600,7 +4600,7 @@
         <v>1</v>
       </c>
       <c r="C51" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -4649,13 +4649,13 @@
         <v>1</v>
       </c>
       <c r="N51" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O51" t="n">
         <v>0.0005</v>
       </c>
       <c r="P51" t="n">
-        <v>0.0025</v>
+        <v>0.0005</v>
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
@@ -4684,7 +4684,7 @@
         <v>1</v>
       </c>
       <c r="C52" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -4733,13 +4733,13 @@
         <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O52" t="n">
         <v>0.0005</v>
       </c>
       <c r="P52" t="n">
-        <v>0.0025</v>
+        <v>0.0005</v>
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
@@ -4768,7 +4768,7 @@
         <v>6</v>
       </c>
       <c r="C53" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -4787,17 +4787,17 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>C2759484</t>
+          <t>C3015810</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>HP02WAF4701TCE</t>
+          <t>SCR0402F4K7</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4811,33 +4811,33 @@
         </is>
       </c>
       <c r="L53" t="n">
-        <v>60347</v>
+        <v>9</v>
       </c>
       <c r="M53" t="n">
         <v>1</v>
       </c>
       <c r="N53" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="O53" t="n">
-        <v>0.0013</v>
+        <v>0.0005</v>
       </c>
       <c r="P53" t="n">
-        <v>0.039</v>
+        <v>0.003</v>
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2759484.html</t>
+          <t>https://www.lcsc.com/product-detail/C3015810.html</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 4.7kΩ 50V Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>C140158 RC-02K4701FT 0.04 USD</t>
+          <t>C103055 RTT024701FTH 0.00 USD</t>
         </is>
       </c>
       <c r="T53" t="inlineStr"/>
@@ -4852,7 +4852,7 @@
         <v>1</v>
       </c>
       <c r="C54" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -4901,13 +4901,13 @@
         <v>1</v>
       </c>
       <c r="N54" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O54" t="n">
         <v>0.0005999999999999999</v>
       </c>
       <c r="P54" t="n">
-        <v>0.003</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
@@ -4936,7 +4936,7 @@
         <v>4</v>
       </c>
       <c r="C55" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -4955,17 +4955,17 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>C409700</t>
+          <t>C3152095</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>CR-02FL6---5K1</t>
+          <t>SC0402F5101F2ANRH</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Viking Tech</t>
+          <t>Sunway</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4979,23 +4979,23 @@
         </is>
       </c>
       <c r="L55" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="M55" t="n">
         <v>1</v>
       </c>
       <c r="N55" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="O55" t="n">
-        <v>0.0009</v>
+        <v>0.0005</v>
       </c>
       <c r="P55" t="n">
-        <v>0.018</v>
+        <v>0.002</v>
       </c>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C409700.html</t>
+          <t>https://www.lcsc.com/product-detail/C3152095.html</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5005,7 +5005,7 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>C22369457 RCA025K1FLF 0.02 USD</t>
+          <t>C409700 CR-02FL6---5K1 0.00 USD</t>
         </is>
       </c>
       <c r="T55" t="inlineStr"/>
@@ -5020,7 +5020,7 @@
         <v>2</v>
       </c>
       <c r="C56" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -5069,13 +5069,13 @@
         <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O56" t="n">
         <v>0.0005999999999999999</v>
       </c>
       <c r="P56" t="n">
-        <v>0.005999999999999999</v>
+        <v>0.0012</v>
       </c>
       <c r="Q56" s="2" t="inlineStr">
         <is>
@@ -5089,7 +5089,7 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>C22369554 RCA02510KFLF 0.01 USD</t>
+          <t>C22369554 RCA02510KFLF 0.00 USD</t>
         </is>
       </c>
       <c r="T56" t="inlineStr"/>
@@ -5104,7 +5104,7 @@
         <v>2</v>
       </c>
       <c r="C57" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -5153,13 +5153,13 @@
         <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O57" t="n">
         <v>0.0005999999999999999</v>
       </c>
       <c r="P57" t="n">
-        <v>0.005999999999999999</v>
+        <v>0.0012</v>
       </c>
       <c r="Q57" s="2" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>C49655223 GR0402F511KTAG00 0.01 USD</t>
+          <t>C49655223 GR0402F511KTAG00 0.00 USD</t>
         </is>
       </c>
       <c r="T57" t="inlineStr"/>
@@ -5188,7 +5188,7 @@
         <v>2</v>
       </c>
       <c r="C58" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -5237,13 +5237,13 @@
         <v>1</v>
       </c>
       <c r="N58" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O58" t="n">
         <v>0.0003</v>
       </c>
       <c r="P58" t="n">
-        <v>0.003</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="Q58" s="2" t="inlineStr">
         <is>
@@ -5272,7 +5272,7 @@
         <v>1</v>
       </c>
       <c r="C59" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -5321,13 +5321,13 @@
         <v>1</v>
       </c>
       <c r="N59" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O59" t="n">
         <v>2.1681</v>
       </c>
       <c r="P59" t="n">
-        <v>10.8405</v>
+        <v>2.1681</v>
       </c>
       <c r="Q59" s="2" t="inlineStr">
         <is>
@@ -5352,7 +5352,7 @@
         <v>2</v>
       </c>
       <c r="C60" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -5388,7 +5388,7 @@
         <v>2</v>
       </c>
       <c r="C61" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -5437,13 +5437,13 @@
         <v>1</v>
       </c>
       <c r="N61" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O61" t="n">
-        <v>1.0786</v>
+        <v>1.1068</v>
       </c>
       <c r="P61" t="n">
-        <v>10.786</v>
+        <v>2.2136</v>
       </c>
       <c r="Q61" s="2" t="inlineStr">
         <is>
@@ -5468,7 +5468,7 @@
         <v>2</v>
       </c>
       <c r="C62" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -5511,19 +5511,19 @@
         </is>
       </c>
       <c r="L62" t="n">
-        <v>237863</v>
+        <v>237730</v>
       </c>
       <c r="M62" t="n">
         <v>1</v>
       </c>
       <c r="N62" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="O62" t="n">
         <v>0.1791</v>
       </c>
       <c r="P62" t="n">
-        <v>1.791</v>
+        <v>0.3582</v>
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
@@ -5537,7 +5537,7 @@
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>C5337088 TYPE-C-31-M-12A 2.30 USD</t>
+          <t>C5337088 TYPE-C-31-M-12A 0.46 USD</t>
         </is>
       </c>
       <c r="T62" t="inlineStr"/>
@@ -5552,7 +5552,7 @@
         <v>1</v>
       </c>
       <c r="C63" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -5601,13 +5601,13 @@
         <v>1</v>
       </c>
       <c r="N63" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O63" t="n">
         <v>0.6632</v>
       </c>
       <c r="P63" t="n">
-        <v>3.316</v>
+        <v>0.6632</v>
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
@@ -5632,7 +5632,7 @@
         <v>1</v>
       </c>
       <c r="C64" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -5681,13 +5681,13 @@
         <v>1</v>
       </c>
       <c r="N64" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O64" t="n">
         <v>0.3026</v>
       </c>
       <c r="P64" t="n">
-        <v>1.513</v>
+        <v>0.3026</v>
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
@@ -5712,7 +5712,7 @@
         <v>1</v>
       </c>
       <c r="C65" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -5761,13 +5761,13 @@
         <v>1</v>
       </c>
       <c r="N65" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O65" t="n">
         <v>11.0628</v>
       </c>
       <c r="P65" t="n">
-        <v>55.31399999999999</v>
+        <v>11.0628</v>
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
@@ -5781,7 +5781,7 @@
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>C17626844 W25N02KVZEIR TR 55.78 USD</t>
+          <t>C17626844 W25N02KVZEIR TR 11.16 USD</t>
         </is>
       </c>
       <c r="T65" t="inlineStr"/>

</xml_diff>

<commit_message>
Unify duplicate capacitor comments (C96 -> 10uF GRM188R61A106ME69D, C1 -> 1uF 50V 1206); BOM re-priced
In-place edits of the Comment parameter records; hidden Weight/Thickness/Depth
texts of C96 shortened to keep the record stream the same length.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T67"/>
+  <dimension ref="A1:T65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>1055</v>
+        <v>555</v>
       </c>
       <c r="M9" t="n">
         <v>1</v>
@@ -1513,18 +1513,18 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>C1 C104</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1uF 1206 50V</t>
+          <t>1uF 50V 1206</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1uF_1206_50V</t>
+          <t>1uF_50V_1206</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1569,13 +1569,13 @@
         <v>1</v>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O14" t="n">
         <v>0.3727</v>
       </c>
       <c r="P14" t="n">
-        <v>0.3727</v>
+        <v>0.7454</v>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>C22415740 C1206C105J5RACTU 0.90 USD</t>
+          <t>C22415740 C1206C105J5RACTU 1.80 USD</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -1597,48 +1597,48 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C104</t>
+          <t>Y1 Y3</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1uF 50V 1206</t>
+          <t>ABS07-32.768KHZ-T</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FP-1206-L_3_2_0_2-W_1_6_0-IPC_B</t>
+          <t>FP-ABS07-MFG</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1uF_50V_1206</t>
+          <t>ABS07-32.768KHZ-T</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>C597503</t>
+          <t>C130253</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>12065C105JAT2A</t>
+          <t>ABS07-32.768KHZ-T</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>Abracon LLC</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>SMD3215-2P</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1647,82 +1647,82 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>1960</v>
+        <v>11646</v>
       </c>
       <c r="M15" t="n">
         <v>1</v>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15" t="n">
-        <v>0.3727</v>
+        <v>0.7086</v>
       </c>
       <c r="P15" t="n">
-        <v>0.3727</v>
+        <v>1.4172</v>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C597503.html</t>
+          <t>https://www.lcsc.com/product-detail/C130253.html</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1uF 50V X7R ±5% 1206 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>C22415740 C1206C105J5RACTU 0.90 USD</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr"/>
+          <t>-40℃~+85℃ 12.5pF 32.768kHz 70kΩ Crystal Oscillator ±20ppm SMD3215-2P Crystals ROHS</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>generic 3215 12.5pF alternative: C22386770 SXTF321532768A20F ~0.13 USD</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Y1 Y3</t>
+          <t>FB4</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ABS07-32.768KHZ-T</t>
+          <t>BLM15AG102SN1D</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FP-ABS07-MFG</t>
+          <t>FP-BLM15-0_05-IPC_B</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ABS07-32.768KHZ-T</t>
+          <t>BLM15AG102SN1D</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>C130253</t>
+          <t>C76883</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ABS07-32.768KHZ-T</t>
+          <t>BLM15AG102SN1D</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Abracon LLC</t>
+          <t>Murata Electronics</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>SMD3215-2P</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1731,72 +1731,68 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>11646</v>
+        <v>53064</v>
       </c>
       <c r="M16" t="n">
         <v>1</v>
       </c>
       <c r="N16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O16" t="n">
-        <v>0.7086</v>
+        <v>0.0051</v>
       </c>
       <c r="P16" t="n">
-        <v>1.4172</v>
+        <v>0.0051</v>
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C130253.html</t>
+          <t>https://www.lcsc.com/product-detail/C76883.html</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 12.5pF 32.768kHz 70kΩ Crystal Oscillator ±20ppm SMD3215-2P Crystals ROHS</t>
+          <t>1 1kΩ@100MHz 300mA 650mΩ ±25% 0402 Ferrite Beads ROHS</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>generic 3215 12.5pF alternative: C22386770 SXTF321532768A20F ~0.13 USD</t>
-        </is>
-      </c>
+      <c r="T16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FB4</t>
+          <t>FB1 FB2 FB3</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>BLM15AG102SN1D</t>
+          <t>BLM18AG121SN1D</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FP-BLM15-0_05-IPC_B</t>
+          <t>FP-BLM18-0_15-t0_8-IPC_B</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>BLM15AG102SN1D</t>
+          <t>BLM18AG121SN1D</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>C76883</t>
+          <t>C76892</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>BLM15AG102SN1D</t>
+          <t>BLM18AG121SN1D</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1806,7 +1802,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1815,28 +1811,28 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>53084</v>
+        <v>249661</v>
       </c>
       <c r="M17" t="n">
         <v>1</v>
       </c>
       <c r="N17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O17" t="n">
-        <v>0.0051</v>
+        <v>0.0121</v>
       </c>
       <c r="P17" t="n">
-        <v>0.0051</v>
+        <v>0.0363</v>
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C76883.html</t>
+          <t>https://www.lcsc.com/product-detail/C76892.html</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1 1kΩ@100MHz 300mA 650mΩ ±25% 0402 Ferrite Beads ROHS</t>
+          <t>-55℃~+125℃ 1 120Ω@100MHz 180mΩ 800mA ±25% 0603 Ferrite Beads ROHS</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
@@ -1845,38 +1841,38 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FB1 FB2 FB3</t>
+          <t>L1 L2 L3 L4 L5</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>BLM18AG121SN1D</t>
+          <t>DFE201612E-R47M=P2</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FP-BLM18-0_15-t0_8-IPC_B</t>
+          <t>FP-DFE201612C-IPC_C</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>BLM18AG121SN1D</t>
+          <t>DFE201612E-R47M=P2</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>C76892</t>
+          <t>C668312</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>BLM18AG121SN1D</t>
+          <t>DFE201612E-R47M=P2</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1886,7 +1882,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0806</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1895,28 +1891,28 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>249661</v>
+        <v>9296</v>
       </c>
       <c r="M18" t="n">
         <v>1</v>
       </c>
       <c r="N18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O18" t="n">
-        <v>0.0121</v>
+        <v>0.1716</v>
       </c>
       <c r="P18" t="n">
-        <v>0.0363</v>
+        <v>0.858</v>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C76892.html</t>
+          <t>https://www.lcsc.com/product-detail/C668312.html</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 1 120Ω@100MHz 180mΩ 800mA ±25% 0603 Ferrite Beads ROHS</t>
+          <t>26mΩ 4.5A 470nH 5.5A ±20% 0806 Power Inductors ROHS</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
@@ -1925,38 +1921,38 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>L1 L2 L3 L4 L5</t>
+          <t>L6 L7</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>DFE201612E-R47M=P2</t>
+          <t>DFE252012F-100M=P2</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>FP-DFE201612C-IPC_C</t>
+          <t>FP-DFE252012C-IPC_B</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>DFE201612E-R47M=P2</t>
+          <t>DFE252012F-100M=P2</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>C668312</t>
+          <t>C703141</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>DFE201612E-R47M=P2</t>
+          <t>DFE252012F-100M=P2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1966,7 +1962,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>0806</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1975,28 +1971,28 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>9276</v>
+        <v>17882</v>
       </c>
       <c r="M19" t="n">
         <v>1</v>
       </c>
       <c r="N19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O19" t="n">
-        <v>0.1716</v>
+        <v>0.1541</v>
       </c>
       <c r="P19" t="n">
-        <v>0.858</v>
+        <v>0.3082</v>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C668312.html</t>
+          <t>https://www.lcsc.com/product-detail/C703141.html</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>26mΩ 4.5A 470nH 5.5A ±20% 0806 Power Inductors ROHS</t>
+          <t>1.4A 10uH 400mΩ 950mA ±20% 1008 Power Inductors ROHS</t>
         </is>
       </c>
       <c r="S19" t="inlineStr"/>
@@ -2005,48 +2001,48 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>L6 L7</t>
+          <t>U5 U8 U10</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>DFE252012F-100M=P2</t>
+          <t>TPS63802DLAR</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FP-DFE252012C-IPC_B</t>
+          <t>FP-DLA0010A-MFG</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>DFE252012F-100M=P2</t>
+          <t>TPS63802DLAR</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>C703141</t>
+          <t>C2845237</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>DFE252012F-100M=P2</t>
+          <t>TPS63802DLAR</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Murata Electronics</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>1008</t>
+          <t>VSON-10(2x3)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2055,28 +2051,28 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>17862</v>
+        <v>7227</v>
       </c>
       <c r="M20" t="n">
         <v>1</v>
       </c>
       <c r="N20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O20" t="n">
-        <v>0.1541</v>
+        <v>0.9814000000000001</v>
       </c>
       <c r="P20" t="n">
-        <v>0.3082</v>
+        <v>2.9442</v>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C703141.html</t>
+          <t>https://www.lcsc.com/product-detail/C2845237.html</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1.4A 10uH 400mΩ 950mA ±20% 1008 Power Inductors ROHS</t>
+          <t>-40℃~+125℃@(TJ) 1 1.3V~5.5V 1.4MHz、1.6MHz、2.1MHz 1.8V~5.2V 11uA 2A Adjustable Buck-Boost Buck-Boost Built-in Yes VSON-10</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
@@ -2085,38 +2081,38 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>U5 U8 U10</t>
+          <t>U6 U7</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TPS63802DLAR</t>
+          <t>TPS62823DLCR</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FP-DLA0010A-MFG</t>
+          <t>FP-DLC0008A-MFG</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TPS63802DLAR</t>
+          <t>TPS62823DLCR</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>C2845237</t>
+          <t>C2693497</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>TPS63802DLAR</t>
+          <t>TPS62823DLCR</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2126,7 +2122,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>VSON-10(2x3)</t>
+          <t>VSON-8(1.5x2)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2135,28 +2131,28 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>7199</v>
+        <v>8622</v>
       </c>
       <c r="M21" t="n">
         <v>1</v>
       </c>
       <c r="N21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O21" t="n">
-        <v>0.9814000000000001</v>
+        <v>1.0864</v>
       </c>
       <c r="P21" t="n">
-        <v>2.9442</v>
+        <v>2.1728</v>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2845237.html</t>
+          <t>https://www.lcsc.com/product-detail/C2693497.html</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>-40℃~+125℃@(TJ) 1 1.3V~5.5V 1.4MHz、1.6MHz、2.1MHz 1.8V~5.2V 11uA 2A Adjustable Buck-Boost Buck-Boost Built-in Yes VSON-10</t>
+          <t xml:space="preserve">-40℃~+125℃@(TJ) 1 2.2MHz 2.4V~5.5V 3A 4uA 600mV~4V Adjustable Buck Built-in Overcurrent Protection、Light load efficient </t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
@@ -2165,48 +2161,48 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>U6 U7</t>
+          <t>C2 C3 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>TPS62823DLCR</t>
+          <t>10uF GRM188R61A106ME69D</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FP-DLC0008A-MFG</t>
+          <t>FP-GRM188-0_15-MFG</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TPS62823DLCR</t>
+          <t>10uF_GRM188R61A106ME69D</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>C2693497</t>
+          <t>C5137565</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>TPS62823DLCR</t>
+          <t>FCC0603X106K100CT</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>FOJAN</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>VSON-8(1.5x2)</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2215,37 +2211,41 @@
         </is>
       </c>
       <c r="L22" t="n">
-        <v>8622</v>
+        <v>619349</v>
       </c>
       <c r="M22" t="n">
         <v>1</v>
       </c>
       <c r="N22" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="O22" t="n">
-        <v>1.0864</v>
+        <v>0.0209</v>
       </c>
       <c r="P22" t="n">
-        <v>2.1728</v>
+        <v>0.2717</v>
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2693497.html</t>
+          <t>https://www.lcsc.com/product-detail/C5137565.html</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t xml:space="preserve">-40℃~+125℃@(TJ) 1 2.2MHz 2.4V~5.5V 3A 4uA 600mV~4V Adjustable Buck Built-in Overcurrent Protection、Light load efficient </t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr"/>
+          <t>10V 10uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>C6119842 CGA0603X5R106K100JT 0.29 USD</t>
+        </is>
+      </c>
       <c r="T22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>C96</t>
+          <t>C86</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10uF 0603</t>
+          <t>1uF 0603</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2266,22 +2266,22 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>10uF_0603</t>
+          <t>1uF_0603</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>C5137565</t>
+          <t>C5189828</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>FCC0603X106K100CT</t>
+          <t>CS1608X7R105K100NRB</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>FOJAN</t>
+          <t>Samwha Capacitor</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2295,7 +2295,7 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>616329</v>
+        <v>1</v>
       </c>
       <c r="M23" t="n">
         <v>1</v>
@@ -2304,24 +2304,24 @@
         <v>1</v>
       </c>
       <c r="O23" t="n">
-        <v>0.0209</v>
+        <v>0.0043</v>
       </c>
       <c r="P23" t="n">
-        <v>0.0209</v>
+        <v>0.0043</v>
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C5137565.html</t>
+          <t>https://www.lcsc.com/product-detail/C5189828.html</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>10V 10uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>10V 1uF X7R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>C6119842 CGA0603X5R106K100JT 0.02 USD</t>
+          <t>C49326606 0603X7R105K100NT 0.01 USD</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -2329,43 +2329,43 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>C2 C3 C11 C15 C16 C19 C50 C90 C99 C102 C105 C106</t>
+          <t>C14 C17 C18 C20 C87 C89</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C24" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10uF GRM188R61A106ME69D</t>
+          <t>22uF GRM188R60J226MEA0J</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>FP-GRM188-0_15-MFG</t>
+          <t>FP-GRM188-0_2-IPC_C</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>10uF_GRM188R61A106ME69D</t>
+          <t>22uF_GRM188R60J226MEA0J</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>C5137565</t>
+          <t>C6119880</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>FCC0603X106K100CT</t>
+          <t>CGA0603X5R226M6R3JT</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>FOJAN</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2379,33 +2379,33 @@
         </is>
       </c>
       <c r="L24" t="n">
-        <v>616329</v>
+        <v>84069</v>
       </c>
       <c r="M24" t="n">
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0209</v>
+        <v>0.0248</v>
       </c>
       <c r="P24" t="n">
-        <v>0.2508</v>
+        <v>0.1488</v>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C5137565.html</t>
+          <t>https://www.lcsc.com/product-detail/C6119880.html</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>10V 10uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>22uF 6.3V X5R ±20% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>C6119842 CGA0603X5R106K100JT 0.27 USD</t>
+          <t>C22376489 FS18B226M6R3PBG 0.17 USD</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
@@ -2413,48 +2413,48 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>C86</t>
+          <t>D2 D7 D8</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1uF 0603</t>
+          <t>DSK24</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>FP-GRM188-0_15-MFG</t>
+          <t>FP-S8-V-3910_01-001-MFG</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1uF_0603</t>
+          <t>DSK24</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>C5189828</t>
+          <t>C51898076</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>CS1608X7R105K100NRB</t>
+          <t>DSK24</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Samwha Capacitor</t>
+          <t>Zhengxin</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SOD-123FL</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2463,33 +2463,33 @@
         </is>
       </c>
       <c r="L25" t="n">
-        <v>1</v>
+        <v>4155</v>
       </c>
       <c r="M25" t="n">
         <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O25" t="n">
-        <v>0.0043</v>
+        <v>0.0153</v>
       </c>
       <c r="P25" t="n">
-        <v>0.0043</v>
+        <v>0.0459</v>
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C5189828.html</t>
+          <t>https://www.lcsc.com/product-detail/C51898076.html</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>10V 1uF X7R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>-55℃~+125℃ 1 Independent 2A 40A 40V 500uA@40V 550mV@2A SOD-123FL Schottky Diodes ROHS</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>C49326606 0603X7R105K100NT 0.01 USD</t>
+          <t>C54863492 DSK24 0.05 USD</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -2497,48 +2497,48 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>C14 C17 C18 C20 C87 C89</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>22uF GRM188R60J226MEA0J</t>
+          <t>YLED0402B</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>FP-GRM188-0_2-IPC_C</t>
+          <t>FP-SM0402GC-MFG</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>22uF_GRM188R60J226MEA0J</t>
+          <t>YLED0402B</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>C6119880</t>
+          <t>C25503856</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>CGA0603X5R226M6R3JT</t>
+          <t>XL-1005UYC</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>XINGLIGHT</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2547,82 +2547,82 @@
         </is>
       </c>
       <c r="L26" t="n">
-        <v>84069</v>
+        <v>87063</v>
       </c>
       <c r="M26" t="n">
         <v>1</v>
       </c>
       <c r="N26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O26" t="n">
-        <v>0.0248</v>
+        <v>0.0127</v>
       </c>
       <c r="P26" t="n">
-        <v>0.1488</v>
+        <v>0.0127</v>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C6119880.html</t>
+          <t>https://www.lcsc.com/product-detail/C25503856.html</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>22uF 6.3V X5R ±20% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>C22376489 FS18B226M6R3PBG 0.17 USD</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr"/>
+          <t>-40℃~+85℃ 120° 1mm x 0.5mm square LED 2.4V 20mA 210mcd 50mW 585nm~595nm 590nm Discrete Diode Water Clear Yellow 0402 LED</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>yellow 0402 LED 590nm, replaces generic YLED0402B</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D2 D7 D8</t>
+          <t>PR1</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>DSK24</t>
+          <t>SM05B-NSHSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>FP-S8-V-3910_01-001-MFG</t>
+          <t>FP-SM05B-NSHSS-TB_LF_SN-MFG</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>DSK24</t>
+          <t>SM05B-NSHSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>C51898076</t>
+          <t>C268096</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>DSK24</t>
+          <t>SM05B-NSHSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Zhengxin</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>SOD-123FL</t>
+          <t>SMD,P=1mm,Surface Mount，Right Angle</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2631,41 +2631,37 @@
         </is>
       </c>
       <c r="L27" t="n">
-        <v>4155</v>
+        <v>984</v>
       </c>
       <c r="M27" t="n">
         <v>1</v>
       </c>
       <c r="N27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O27" t="n">
-        <v>0.0153</v>
+        <v>0.4515</v>
       </c>
       <c r="P27" t="n">
-        <v>0.0459</v>
+        <v>0.4515</v>
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C51898076.html</t>
+          <t>https://www.lcsc.com/product-detail/C268096.html</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 1 Independent 2A 40A 40V 500uA@40V 550mV@2A SOD-123FL Schottky Diodes ROHS</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>C54863492 DSK24 0.05 USD</t>
-        </is>
-      </c>
+          <t>-25℃~+85℃ 1 1A 1mm 1x5P 4.4mm 5 50V 5P 6.8mm 7mm Auxiliary Solder Pin Copper alloy NSH PA Surface Mount, Right Angle Tin</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2676,37 +2672,37 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>YLED0402B</t>
+          <t>DMG2301LK-7</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FP-SM0402GC-MFG</t>
+          <t>FP-SOT23-IPC_B</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>YLED0402B</t>
+          <t>DMG2301LK-7</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>C25503856</t>
+          <t>C53283193</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>XL-1005UYC</t>
+          <t>DMG2301L-GK</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>XINGLIGHT</t>
+          <t>GOODWORK</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2715,7 +2711,7 @@
         </is>
       </c>
       <c r="L28" t="n">
-        <v>87063</v>
+        <v>1580</v>
       </c>
       <c r="M28" t="n">
         <v>1</v>
@@ -2724,73 +2720,73 @@
         <v>1</v>
       </c>
       <c r="O28" t="n">
-        <v>0.0127</v>
+        <v>0.0275</v>
       </c>
       <c r="P28" t="n">
-        <v>0.0127</v>
+        <v>0.0275</v>
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25503856.html</t>
+          <t>https://www.lcsc.com/product-detail/C53283193.html</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 120° 1mm x 0.5mm square LED 2.4V 20mA 210mcd 50mW 585nm~595nm 590nm Discrete Diode Water Clear Yellow 0402 LED</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>yellow 0402 LED 590nm, replaces generic YLED0402B</t>
-        </is>
-      </c>
+          <t>-55℃~+150℃ 1 P-Channel 1.2W 1V 20V 3A 405pF 5.5nC@4.5V 55pF 70mΩ@4.5V 75pF SOT-23 MOSFETs ROHS</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>C53199108 DMG2301L-7(ES) 0.03 USD</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PR1</t>
+          <t>Q2 Q4</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SM05B-NSHSS-TB(LF)(SN)</t>
+          <t>DMG2302UK-7</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>FP-SM05B-NSHSS-TB_LF_SN-MFG</t>
+          <t>FP-SOT23-MFG</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>SM05B-NSHSS-TB(LF)(SN)</t>
+          <t>DMG2302UK-7</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>C268096</t>
+          <t>C53283194</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>SM05B-NSHSS-TB(LF)(SN)</t>
+          <t>DMG2302UK-GK</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>GOODWORK</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>SMD,P=1mm,Surface Mount，Right Angle</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2799,78 +2795,86 @@
         </is>
       </c>
       <c r="L29" t="n">
-        <v>984</v>
+        <v>5850</v>
       </c>
       <c r="M29" t="n">
         <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O29" t="n">
-        <v>0.4515</v>
+        <v>0.0157</v>
       </c>
       <c r="P29" t="n">
-        <v>0.4515</v>
+        <v>0.0314</v>
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C268096.html</t>
+          <t>https://www.lcsc.com/product-detail/C53283194.html</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 1A 1mm 1x5P 4.4mm 5 50V 5P 6.8mm 7mm Auxiliary Solder Pin Copper alloy NSH PA Surface Mount, Right Angle Tin</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
+          <t>-55℃~+150℃ 1 N-channel 1.2W 1V 2.3A 200pF 20V 28pF 35pF 3nC@4.5V 45mΩ@4.5V SOT-23 MOSFETs ROHS</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>C5224188 DMG2302UK-7-ES 0.04 USD</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>clone brands accepted; Diodes original is C460977</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>D3 D4 D5</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>DMG2301LK-7</t>
+          <t>PRTR5V0U2F,115</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>FP-SOT23-IPC_B</t>
+          <t>FP-SOT886-MFG</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>DMG2301LK-7</t>
+          <t>PRTR5V0U2F,115</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>C53283193</t>
+          <t>C478118</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>DMG2301L-GK</t>
+          <t>PRTR5V0U2F,115</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>GOODWORK</t>
+          <t>Nexperia</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>XSON-6(1x1.5)</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2879,33 +2883,33 @@
         </is>
       </c>
       <c r="L30" t="n">
-        <v>1580</v>
+        <v>60185</v>
       </c>
       <c r="M30" t="n">
         <v>1</v>
       </c>
       <c r="N30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O30" t="n">
-        <v>0.0275</v>
+        <v>0.103</v>
       </c>
       <c r="P30" t="n">
-        <v>0.0275</v>
+        <v>0.309</v>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C53283193.html</t>
+          <t>https://www.lcsc.com/product-detail/C478118.html</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>-55℃~+150℃ 1 P-Channel 1.2W 1V 20V 3A 405pF 5.5nC@4.5V 55pF 70mΩ@4.5V 75pF SOT-23 MOSFETs ROHS</t>
+          <t>-40℃~+85℃ 100nA 1pF 2 5.5V 6V IEC 61000-4-2 TVS Unidirectional XSON-6(1x1.5) ESD and Surge Protection (TVS/ESD) ROHS</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>C53199108 DMG2301L-7(ES) 0.03 USD</t>
+          <t>C52994078 PRTR5V0U2F,115(ES) 0.53 USD</t>
         </is>
       </c>
       <c r="T30" t="inlineStr"/>
@@ -2913,48 +2917,48 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Q2 Q4</t>
+          <t>R68</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>DMG2302UK-7</t>
+          <t>10R</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FP-SOT23-MFG</t>
+          <t>FP-SR0603-MFG</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>DMG2302UK-7</t>
+          <t>10R</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>C53283194</t>
+          <t>C103222</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>DMG2302UK-GK</t>
+          <t>RTT0310R0FTP</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>GOODWORK</t>
+          <t>RALEC</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2963,86 +2967,82 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>5850</v>
+        <v>46</v>
       </c>
       <c r="M31" t="n">
         <v>1</v>
       </c>
       <c r="N31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O31" t="n">
-        <v>0.0157</v>
+        <v>0.0018</v>
       </c>
       <c r="P31" t="n">
-        <v>0.0314</v>
+        <v>0.0018</v>
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C53283194.html</t>
+          <t>https://www.lcsc.com/product-detail/C103222.html</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>-55℃~+150℃ 1 N-channel 1.2W 1V 2.3A 200pF 20V 28pF 35pF 3nC@4.5V 45mΩ@4.5V SOT-23 MOSFETs ROHS</t>
+          <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>C5224188 DMG2302UK-7-ES 0.04 USD</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>clone brands accepted; Diodes original is C460977</t>
-        </is>
-      </c>
+          <t>C177661 RCT0310RFLF 0.00 USD</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>D3 D4 D5</t>
+          <t>R66</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>PRTR5V0U2F,115</t>
+          <t>4R</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>FP-SOT886-MFG</t>
+          <t>FP-SR0603-MFG</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>PRTR5V0U2F,115</t>
+          <t>4R</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>C478118</t>
+          <t>C158913</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>PRTR5V0U2F,115</t>
+          <t>RTT034R02FTP</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Nexperia</t>
+          <t>RALEC</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>XSON-6(1x1.5)</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3051,41 +3051,45 @@
         </is>
       </c>
       <c r="L32" t="n">
-        <v>60185</v>
+        <v>38</v>
       </c>
       <c r="M32" t="n">
         <v>1</v>
       </c>
       <c r="N32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O32" t="n">
-        <v>0.103</v>
+        <v>0.0018</v>
       </c>
       <c r="P32" t="n">
-        <v>0.309</v>
+        <v>0.0018</v>
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C478118.html</t>
+          <t>https://www.lcsc.com/product-detail/C158913.html</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 100nA 1pF 2 5.5V 6V IEC 61000-4-2 TVS Unidirectional XSON-6(1x1.5) ESD and Surge Protection (TVS/ESD) ROHS</t>
+          <t>-55℃~+155℃ 100mW 4.02Ω 75V Thick Film Resistor ±1% ±200ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>C52994078 PRTR5V0U2F,115(ES) 0.53 USD</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr"/>
+          <t>C322168 RS-03L4R02FT 0.00 USD</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>4R is not an E-series value; 4.02 ohm E96 used</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>R68</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -3096,37 +3100,37 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10R</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>FP-SR0603-MFG</t>
+          <t>FP-XRCGB_F_N-MFG</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>10R</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>C103222</t>
+          <t>C2965580</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>RTT0310R0FTP</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>RALEC</t>
+          <t>YXC Crystal Oscillators</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SMD2016-4P</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3135,7 +3139,7 @@
         </is>
       </c>
       <c r="L33" t="n">
-        <v>46</v>
+        <v>7670</v>
       </c>
       <c r="M33" t="n">
         <v>1</v>
@@ -3144,73 +3148,69 @@
         <v>1</v>
       </c>
       <c r="O33" t="n">
-        <v>0.0018</v>
+        <v>0.0784</v>
       </c>
       <c r="P33" t="n">
-        <v>0.0018</v>
+        <v>0.0784</v>
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C103222.html</t>
+          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>C177661 RCT0310RFLF 0.00 USD</t>
-        </is>
-      </c>
+          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R66</t>
+          <t>S1 S2 S3</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>4R</t>
+          <t>S2B-PH-K-S(LF)(SN)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>FP-SR0603-MFG</t>
+          <t>JST-S2B-PH-K-S_V</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>4R</t>
+          <t>S2B-PH-K-S(LF)(SN)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>C158913</t>
+          <t>C173752</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>RTT034R02FTP</t>
+          <t>S2B-PH-K-S(LF)(SN)</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>RALEC</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>Push-Pull,P=2mm</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -3219,45 +3219,41 @@
         </is>
       </c>
       <c r="L34" t="n">
-        <v>38</v>
+        <v>27957</v>
       </c>
       <c r="M34" t="n">
         <v>1</v>
       </c>
       <c r="N34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O34" t="n">
-        <v>0.0018</v>
+        <v>0.038</v>
       </c>
       <c r="P34" t="n">
-        <v>0.0018</v>
+        <v>0.114</v>
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C158913.html</t>
+          <t>https://www.lcsc.com/product-detail/C173752.html</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 4.02Ω 75V Thick Film Resistor ±1% ±200ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>C322168 RS-03L4R02FT 0.00 USD</t>
-        </is>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>4R is not an E-series value; 4.02 ohm E96 used</t>
-        </is>
-      </c>
+          <t>C157932 S2B-PH-K-S-GW 0.64 USD</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Y2</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -3268,37 +3264,37 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>k230d</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>FP-XRCGB_F_N-MFG</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>k230d</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>C2965580</t>
+          <t>C42414902</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>YXC Crystal Oscillators</t>
+          <t>Canaan</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>SMD2016-4P</t>
+          <t>BGA-256</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -3307,7 +3303,7 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>7670</v>
+        <v>161</v>
       </c>
       <c r="M35" t="n">
         <v>1</v>
@@ -3316,19 +3312,19 @@
         <v>1</v>
       </c>
       <c r="O35" t="n">
-        <v>0.0784</v>
+        <v>13.3061</v>
       </c>
       <c r="P35" t="n">
-        <v>0.0784</v>
+        <v>13.3061</v>
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
+          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
+          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
@@ -3337,48 +3333,48 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>S1 S2 S3</t>
+          <t>J4 J5</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S(LF)(SN)</t>
+          <t>54548-2271</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>JST-S2B-PH-K-S_V</t>
+          <t>MOLX-54548-2271</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S(LF)(SN)</t>
+          <t>54548-2271</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>C173752</t>
+          <t>C22459552</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S(LF)(SN)</t>
+          <t>05B20L22P</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>HanElectricity</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Push-Pull,P=2mm</t>
+          <t>SMD,P=0.5mm,Surface Mount，Right Angle</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -3387,41 +3383,41 @@
         </is>
       </c>
       <c r="L36" t="n">
-        <v>27997</v>
+        <v>2004</v>
       </c>
       <c r="M36" t="n">
         <v>1</v>
       </c>
       <c r="N36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O36" t="n">
-        <v>0.038</v>
+        <v>0.0698</v>
       </c>
       <c r="P36" t="n">
-        <v>0.114</v>
+        <v>0.1396</v>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C173752.html</t>
+          <t>https://www.lcsc.com/product-detail/C22459552.html</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>C157932 S2B-PH-K-S-GW 0.64 USD</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr"/>
+          <t>-25℃~+85℃ 0.3mm 0.5mm 22P 2mm 400mA 50V Bottom Contact Phosphor bronze Slide Lock Surface Mount, Right Angle Tin SMD,P=0</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Molex 54548-2271 DISCONTINUED (LCSC: no longer manufactured). Same type (0.5mm 22P bottom-contact slide-lock, right angle) offered; FOOTPRINT MUST BE VERIFIED against its drawing</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -3432,37 +3428,37 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>k230d</t>
+          <t>1.1k (1.5A)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>RES_0402</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>k230d</t>
+          <t>1.1k_(1.5A)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>C42414902</t>
+          <t>C3015792</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>SCR0402F1K1</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Canaan</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>BGA-256</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3471,7 +3467,7 @@
         </is>
       </c>
       <c r="L37" t="n">
-        <v>161</v>
+        <v>40</v>
       </c>
       <c r="M37" t="n">
         <v>1</v>
@@ -3480,69 +3476,73 @@
         <v>1</v>
       </c>
       <c r="O37" t="n">
-        <v>13.3061</v>
+        <v>0.0005</v>
       </c>
       <c r="P37" t="n">
-        <v>13.3061</v>
+        <v>0.0005</v>
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
+          <t>https://www.lcsc.com/product-detail/C3015792.html</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr"/>
+          <t>-55℃~+155℃ 1.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>C54920634 HRC0402F1101DNTO 0.00 USD</t>
+        </is>
+      </c>
       <c r="T37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>J4 J5</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>54548-2271</t>
+          <t>590R (1.5A)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>MOLX-54548-2271</t>
+          <t>RES_0402</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>54548-2271</t>
+          <t>590R_(1.5A)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>C22459552</t>
+          <t>C3015623</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>05B20L22P</t>
+          <t>SCR0402F590R</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>HanElectricity</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>SMD,P=0.5mm,Surface Mount，Right Angle</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3551,41 +3551,41 @@
         </is>
       </c>
       <c r="L38" t="n">
-        <v>2004</v>
+        <v>353</v>
       </c>
       <c r="M38" t="n">
         <v>1</v>
       </c>
       <c r="N38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0698</v>
+        <v>0.0005</v>
       </c>
       <c r="P38" t="n">
-        <v>0.1396</v>
+        <v>0.0005</v>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22459552.html</t>
+          <t>https://www.lcsc.com/product-detail/C3015623.html</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 0.3mm 0.5mm 22P 2mm 400mA 50V Bottom Contact Phosphor bronze Slide Lock Surface Mount, Right Angle Tin SMD,P=0</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr"/>
-      <c r="T38" t="inlineStr">
-        <is>
-          <t>Molex 54548-2271 DISCONTINUED (LCSC: no longer manufactured). Same type (0.5mm 22P bottom-contact slide-lock, right angle) offered; FOOTPRINT MUST BE VERIFIED against its drawing</t>
-        </is>
-      </c>
+          <t>-55℃~+155℃ 50V 590Ω 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>C334714 WR04X5900FTL 0.00 USD</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -3596,7 +3596,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1.1k (1.5A)</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3606,17 +3606,17 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>1.1k_(1.5A)</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>C3015792</t>
+          <t>C3015796</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>SCR0402F1K1</t>
+          <t>SCR0402F1K5</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3635,7 +3635,7 @@
         </is>
       </c>
       <c r="L39" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="M39" t="n">
         <v>1</v>
@@ -3651,17 +3651,17 @@
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015792.html</t>
+          <t>https://www.lcsc.com/product-detail/C3015796.html</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>C54920634 HRC0402F1101DNTO 0.00 USD</t>
+          <t>C100249 CR0402FF1501G 0.00 USD</t>
         </is>
       </c>
       <c r="T39" t="inlineStr"/>
@@ -3669,18 +3669,18 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R6 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R69 R76</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>590R (1.5A)</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3690,22 +3690,22 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>590R_(1.5A)</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>C3015623</t>
+          <t>C279979</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>SCR0402F590R</t>
+          <t>CR-02FL6--100K</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>Viking Tech</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -3719,33 +3719,33 @@
         </is>
       </c>
       <c r="L40" t="n">
-        <v>353</v>
+        <v>5579</v>
       </c>
       <c r="M40" t="n">
         <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="O40" t="n">
-        <v>0.0005</v>
+        <v>0.0011</v>
       </c>
       <c r="P40" t="n">
-        <v>0.0005</v>
+        <v>0.022</v>
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015623.html</t>
+          <t>https://www.lcsc.com/product-detail/C279979.html</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 590Ω 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>C334714 WR04X5900FTL 0.00 USD</t>
+          <t>C2759534 HP02WAF1003TCE 0.03 USD</t>
         </is>
       </c>
       <c r="T40" t="inlineStr"/>
@@ -3753,18 +3753,18 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3774,22 +3774,22 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>C3015796</t>
+          <t>C1858459</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>SCR0402F1K5</t>
+          <t>RC0402FR-1310KL</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -3803,33 +3803,33 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>21</v>
+        <v>49503</v>
       </c>
       <c r="M41" t="n">
         <v>1</v>
       </c>
       <c r="N41" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="O41" t="n">
-        <v>0.0005</v>
+        <v>0.0018</v>
       </c>
       <c r="P41" t="n">
-        <v>0.0005</v>
+        <v>0.0324</v>
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015796.html</t>
+          <t>https://www.lcsc.com/product-detail/C1858459.html</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>C100249 CR0402FF1501G 0.00 USD</t>
+          <t>C327797 MR04X1002FTL 0.04 USD</t>
         </is>
       </c>
       <c r="T41" t="inlineStr"/>
@@ -3837,18 +3837,18 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>R6 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R69 R76</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>120k</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3858,22 +3858,22 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>120k</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>C279979</t>
+          <t>C54920620</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>CR-02FL6--100K</t>
+          <t>HRC0402F1203DNTO</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Viking Tech</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -3887,33 +3887,33 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>5579</v>
+        <v>1191862</v>
       </c>
       <c r="M42" t="n">
         <v>1</v>
       </c>
       <c r="N42" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0011</v>
+        <v>0.0007</v>
       </c>
       <c r="P42" t="n">
-        <v>0.022</v>
+        <v>0.0007</v>
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C279979.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920620.html</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>C2759534 HP02WAF1003TCE 0.03 USD</t>
+          <t>C22356241 RCA02120KFLF 0.00 USD</t>
         </is>
       </c>
       <c r="T42" t="inlineStr"/>
@@ -3921,18 +3921,18 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
+          <t>R8</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C43" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>150k</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3942,22 +3942,22 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>150k</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>C1858459</t>
+          <t>C3152063</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>RC0402FR-1310KL</t>
+          <t>SC0402F1503F2ANRH</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>Sunway</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -3971,33 +3971,33 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>49503</v>
+        <v>13</v>
       </c>
       <c r="M43" t="n">
         <v>1</v>
       </c>
       <c r="N43" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0018</v>
+        <v>0.0005</v>
       </c>
       <c r="P43" t="n">
-        <v>0.0324</v>
+        <v>0.0005</v>
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C1858459.html</t>
+          <t>https://www.lcsc.com/product-detail/C3152063.html</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 150kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>C327797 MR04X1002FTL 0.04 USD</t>
+          <t>C102813 RTT021503FTH 0.00 USD</t>
         </is>
       </c>
       <c r="T43" t="inlineStr"/>
@@ -4005,18 +4005,18 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R37 R62</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>120k</t>
+          <t>200R</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4026,22 +4026,22 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>120k</t>
+          <t>200R</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>C54920620</t>
+          <t>C3015766</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>HRC0402F1203DNTO</t>
+          <t>SCR0402F200R</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4055,33 +4055,33 @@
         </is>
       </c>
       <c r="L44" t="n">
-        <v>1191862</v>
+        <v>15</v>
       </c>
       <c r="M44" t="n">
         <v>1</v>
       </c>
       <c r="N44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0007</v>
+        <v>0.0005</v>
       </c>
       <c r="P44" t="n">
-        <v>0.0007</v>
+        <v>0.001</v>
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920620.html</t>
+          <t>https://www.lcsc.com/product-detail/C3015766.html</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>C22356241 RCA02120KFLF 0.00 USD</t>
+          <t>C46635169 CL0402FN200RP 0.00 USD</t>
         </is>
       </c>
       <c r="T44" t="inlineStr"/>
@@ -4089,7 +4089,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R59</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -4100,7 +4100,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>150k</t>
+          <t>200k</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4110,22 +4110,22 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>150k</t>
+          <t>200k</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>C3152063</t>
+          <t>C49653950</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>SC0402F1503F2ANRH</t>
+          <t>GR0402F200KTAG00</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Sunway</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4139,7 +4139,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="M45" t="n">
         <v>1</v>
@@ -4155,17 +4155,17 @@
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3152063.html</t>
+          <t>https://www.lcsc.com/product-detail/C49653950.html</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 150kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>C102813 RTT021503FTH 0.00 USD</t>
+          <t>C3015901 SCR0402F200K 0.00 USD</t>
         </is>
       </c>
       <c r="T45" t="inlineStr"/>
@@ -4173,18 +4173,18 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R37 R62</t>
+          <t>R42</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>200R</t>
+          <t>22R</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4194,22 +4194,22 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>200R</t>
+          <t>22R</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>C3015766</t>
+          <t>C49654869</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>SCR0402F200R</t>
+          <t>GR0402F22RTAG00</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -4223,33 +4223,33 @@
         </is>
       </c>
       <c r="L46" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="M46" t="n">
         <v>1</v>
       </c>
       <c r="N46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0005</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="P46" t="n">
-        <v>0.001</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015766.html</t>
+          <t>https://www.lcsc.com/product-detail/C49654869.html</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>C46635169 CL0402FN200RP 0.00 USD</t>
+          <t>C102905 RTT0222R0FTH 0.00 USD</t>
         </is>
       </c>
       <c r="T46" t="inlineStr"/>
@@ -4257,18 +4257,18 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>R59</t>
+          <t>R33 R46 R47 R48</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C47" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>200k</t>
+          <t>240R</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -4278,22 +4278,22 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>200k</t>
+          <t>240R</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>C49653950</t>
+          <t>C168215</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>GR0402F200KTAG00</t>
+          <t>WR04X2400FTL</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>Walsin Tech Corp</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -4307,33 +4307,33 @@
         </is>
       </c>
       <c r="L47" t="n">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="M47" t="n">
         <v>1</v>
       </c>
       <c r="N47" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0005</v>
+        <v>0.0004</v>
       </c>
       <c r="P47" t="n">
-        <v>0.0005</v>
+        <v>0.0016</v>
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49653950.html</t>
+          <t>https://www.lcsc.com/product-detail/C168215.html</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>C3015901 SCR0402F200K 0.00 USD</t>
+          <t>C49652940 GR0402F240RTAG00 0.00 USD</t>
         </is>
       </c>
       <c r="T47" t="inlineStr"/>
@@ -4341,7 +4341,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>R42</t>
+          <t>R56</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>22R</t>
+          <t>261k</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -4362,22 +4362,22 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>22R</t>
+          <t>261k</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>C49654869</t>
+          <t>C46444589</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>GR0402F22RTAG00</t>
+          <t>RC-02K2613FT</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -4391,7 +4391,7 @@
         </is>
       </c>
       <c r="L48" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="M48" t="n">
         <v>1</v>
@@ -4407,17 +4407,17 @@
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49654869.html</t>
+          <t>https://www.lcsc.com/product-detail/C46444589.html</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>261kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>C102905 RTT0222R0FTH 0.00 USD</t>
+          <t>C3015905 SCR0402F261K 0.00 USD</t>
         </is>
       </c>
       <c r="T48" t="inlineStr"/>
@@ -4425,18 +4425,18 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>R33 R46 R47 R48</t>
+          <t>R63</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C49" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>240R</t>
+          <t>30k</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4446,22 +4446,22 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>240R</t>
+          <t>30k</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>C168215</t>
+          <t>C3152079</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>WR04X2400FTL</t>
+          <t>SC0402F3002F2ANRH</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Walsin Tech Corp</t>
+          <t>Sunway</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -4475,33 +4475,33 @@
         </is>
       </c>
       <c r="L49" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="M49" t="n">
         <v>1</v>
       </c>
       <c r="N49" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O49" t="n">
-        <v>0.0004</v>
+        <v>0.0005</v>
       </c>
       <c r="P49" t="n">
-        <v>0.0016</v>
+        <v>0.0005</v>
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C168215.html</t>
+          <t>https://www.lcsc.com/product-detail/C3152079.html</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>C49652940 GR0402F240RTAG00 0.00 USD</t>
+          <t>C54920659 HRC0402F3002DNTO 0.00 USD</t>
         </is>
       </c>
       <c r="T49" t="inlineStr"/>
@@ -4509,7 +4509,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>R56</t>
+          <t>R25</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -4520,7 +4520,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>261k</t>
+          <t>33.2k</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4530,22 +4530,22 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>261k</t>
+          <t>33.2k</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>C46444589</t>
+          <t>C159031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>RC-02K2613FT</t>
+          <t>RTT023322FTH</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>FH (Guangdong Fenghua Advanced Tech)</t>
+          <t>RALEC</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -4559,7 +4559,7 @@
         </is>
       </c>
       <c r="L50" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="M50" t="n">
         <v>1</v>
@@ -4568,24 +4568,24 @@
         <v>1</v>
       </c>
       <c r="O50" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0005</v>
       </c>
       <c r="P50" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0005</v>
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C46444589.html</t>
+          <t>https://www.lcsc.com/product-detail/C159031.html</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>261kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 33.2kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>C3015905 SCR0402F261K 0.00 USD</t>
+          <t>C53069467 CL0402FN33K2P 0.00 USD</t>
         </is>
       </c>
       <c r="T50" t="inlineStr"/>
@@ -4593,18 +4593,18 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>R63</t>
+          <t>R14 R15 R17 R18 R73 R74</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>30k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -4614,22 +4614,22 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>30k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>C3152079</t>
+          <t>C3015810</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>SC0402F3002F2ANRH</t>
+          <t>SCR0402F4K7</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Sunway</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -4643,33 +4643,33 @@
         </is>
       </c>
       <c r="L51" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="M51" t="n">
         <v>1</v>
       </c>
       <c r="N51" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O51" t="n">
         <v>0.0005</v>
       </c>
       <c r="P51" t="n">
-        <v>0.0005</v>
+        <v>0.003</v>
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3152079.html</t>
+          <t>https://www.lcsc.com/product-detail/C3015810.html</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>C54920659 HRC0402F3002DNTO 0.00 USD</t>
+          <t>C103055 RTT024701FTH 0.00 USD</t>
         </is>
       </c>
       <c r="T51" t="inlineStr"/>
@@ -4677,7 +4677,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>33.2k</t>
+          <t>46.4k</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4698,22 +4698,22 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>33.2k</t>
+          <t>46.4k</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>C159031</t>
+          <t>C881176</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>RTT023322FTH</t>
+          <t>CR0402F46K4Q10Z</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>RALEC</t>
+          <t>Ever Ohms Tech</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -4727,7 +4727,7 @@
         </is>
       </c>
       <c r="L52" t="n">
-        <v>5</v>
+        <v>673</v>
       </c>
       <c r="M52" t="n">
         <v>1</v>
@@ -4736,24 +4736,24 @@
         <v>1</v>
       </c>
       <c r="O52" t="n">
-        <v>0.0005</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="P52" t="n">
-        <v>0.0005</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C159031.html</t>
+          <t>https://www.lcsc.com/product-detail/C881176.html</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 33.2kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 46.4kΩ 50V 63mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>C53069467 CL0402FN33K2P 0.00 USD</t>
+          <t>C103052 RTT024642FTH 0.00 USD</t>
         </is>
       </c>
       <c r="T52" t="inlineStr"/>
@@ -4761,18 +4761,18 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>R14 R15 R17 R18 R73 R74</t>
+          <t>R1 R4 R9 R11</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C53" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>5.1k</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -4782,22 +4782,22 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>5.1k</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>C3015810</t>
+          <t>C3152095</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>SCR0402F4K7</t>
+          <t>SC0402F5101F2ANRH</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>Sunway</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4811,33 +4811,33 @@
         </is>
       </c>
       <c r="L53" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M53" t="n">
         <v>1</v>
       </c>
       <c r="N53" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O53" t="n">
         <v>0.0005</v>
       </c>
       <c r="P53" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015810.html</t>
+          <t>https://www.lcsc.com/product-detail/C3152095.html</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>C103055 RTT024701FTH 0.00 USD</t>
+          <t>C409700 CR-02FL6---5K1 0.00 USD</t>
         </is>
       </c>
       <c r="T53" t="inlineStr"/>
@@ -4845,18 +4845,18 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R71 R72</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>46.4k</t>
+          <t>510k</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -4866,17 +4866,17 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>46.4k</t>
+          <t>510k</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>C881176</t>
+          <t>C880994</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>CR0402F46K4Q10Z</t>
+          <t>CR0402F510KQ10Z</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -4895,33 +4895,33 @@
         </is>
       </c>
       <c r="L54" t="n">
-        <v>673</v>
+        <v>10</v>
       </c>
       <c r="M54" t="n">
         <v>1</v>
       </c>
       <c r="N54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O54" t="n">
         <v>0.0005999999999999999</v>
       </c>
       <c r="P54" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0012</v>
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C881176.html</t>
+          <t>https://www.lcsc.com/product-detail/C880994.html</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 46.4kΩ 50V 63mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 510kΩ 63mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>C103052 RTT024642FTH 0.00 USD</t>
+          <t>C22369554 RCA02510KFLF 0.00 USD</t>
         </is>
       </c>
       <c r="T54" t="inlineStr"/>
@@ -4929,18 +4929,18 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>R1 R4 R9 R11</t>
+          <t>R22 R50</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C55" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>5.1k</t>
+          <t>511k</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -4950,22 +4950,22 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>5.1k</t>
+          <t>511k</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>C3152095</t>
+          <t>C3015918</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>SC0402F5101F2ANRH</t>
+          <t>SCR0402F511K</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Sunway</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4979,33 +4979,33 @@
         </is>
       </c>
       <c r="L55" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="M55" t="n">
         <v>1</v>
       </c>
       <c r="N55" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O55" t="n">
-        <v>0.0005</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="P55" t="n">
-        <v>0.002</v>
+        <v>0.0012</v>
       </c>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3152095.html</t>
+          <t>https://www.lcsc.com/product-detail/C3015918.html</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>C409700 CR-02FL6---5K1 0.00 USD</t>
+          <t>C49655223 GR0402F511KTAG00 0.00 USD</t>
         </is>
       </c>
       <c r="T55" t="inlineStr"/>
@@ -5013,7 +5013,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>R71 R72</t>
+          <t>R24 R55</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>510k</t>
+          <t>91k</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -5034,22 +5034,22 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>510k</t>
+          <t>91k</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>C880994</t>
+          <t>C5356157</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>CR0402F510KQ10Z</t>
+          <t>SC0402F9102F2ANRH</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Ever Ohms Tech</t>
+          <t>Sunway</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -5063,7 +5063,7 @@
         </is>
       </c>
       <c r="L56" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="M56" t="n">
         <v>1</v>
@@ -5072,24 +5072,24 @@
         <v>2</v>
       </c>
       <c r="O56" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="P56" t="n">
         <v>0.0005999999999999999</v>
       </c>
-      <c r="P56" t="n">
-        <v>0.0012</v>
-      </c>
       <c r="Q56" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C880994.html</t>
+          <t>https://www.lcsc.com/product-detail/C5356157.html</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 510kΩ 63mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>C22369554 RCA02510KFLF 0.00 USD</t>
+          <t>C365061 HPCR0402F91K0K9 0.00 USD</t>
         </is>
       </c>
       <c r="T56" t="inlineStr"/>
@@ -5097,48 +5097,48 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>R22 R50</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>511k</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>RES_0402</t>
+          <t>RGT0016C_V</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>511k</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>C3015918</t>
+          <t>C129319</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>SCR0402F511K</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>QFN-16-EP(3x3)</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -5147,41 +5147,37 @@
         </is>
       </c>
       <c r="L57" t="n">
-        <v>16</v>
+        <v>387</v>
       </c>
       <c r="M57" t="n">
         <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O57" t="n">
-        <v>0.0005999999999999999</v>
+        <v>2.1681</v>
       </c>
       <c r="P57" t="n">
-        <v>0.0012</v>
+        <v>2.1681</v>
       </c>
       <c r="Q57" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015918.html</t>
+          <t>https://www.lcsc.com/product-detail/C129319.html</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
-        </is>
-      </c>
-      <c r="S57" t="inlineStr">
-        <is>
-          <t>C49655223 GR0402F511KTAG00 0.00 USD</t>
-        </is>
-      </c>
+          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>R24 R55</t>
+          <t>B1_N B1_P</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -5192,111 +5188,63 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>91k</t>
+          <t>TESTP</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>RES_0402</t>
+          <t>TESTP</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>91k</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>C5356157</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>SC0402F9102F2ANRH</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>Sunway</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>0402</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="L58" t="n">
-        <v>18</v>
-      </c>
-      <c r="M58" t="n">
-        <v>1</v>
-      </c>
-      <c r="N58" t="n">
-        <v>2</v>
-      </c>
-      <c r="O58" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="P58" t="n">
-        <v>0.0005999999999999999</v>
-      </c>
-      <c r="Q58" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lcsc.com/product-detail/C5356157.html</t>
-        </is>
-      </c>
-      <c r="R58" t="inlineStr">
-        <is>
-          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
-        </is>
-      </c>
-      <c r="S58" t="inlineStr">
-        <is>
-          <t>C365061 HPCR0402F91K0K9 0.00 USD</t>
-        </is>
-      </c>
-      <c r="T58" t="inlineStr"/>
+          <t>TESTP</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>no purchased part (pad / test point / antenna)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>U14 U15</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>RGT0016C_V</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>C129319</t>
+          <t>C2867168</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5306,7 +5254,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>QFN-16-EP(3x3)</t>
+          <t>WSON-6-EP(2x2)</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -5315,28 +5263,28 @@
         </is>
       </c>
       <c r="L59" t="n">
-        <v>387</v>
+        <v>36</v>
       </c>
       <c r="M59" t="n">
         <v>1</v>
       </c>
       <c r="N59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O59" t="n">
-        <v>2.1681</v>
+        <v>1.1068</v>
       </c>
       <c r="P59" t="n">
-        <v>2.1681</v>
+        <v>2.2136</v>
       </c>
       <c r="Q59" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C129319.html</t>
+          <t>https://www.lcsc.com/product-detail/C2867168.html</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
+          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
         </is>
       </c>
       <c r="S59" t="inlineStr"/>
@@ -5345,7 +5293,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>B1_N B1_P</t>
+          <t>USBC1 USBC2</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -5356,73 +5304,121 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>TESTP</t>
+          <t>type-c-31-m-12</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>TESTP</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>TESTP</t>
-        </is>
-      </c>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
-      <c r="T60" t="inlineStr">
-        <is>
-          <t>no purchased part (pad / test point / antenna)</t>
-        </is>
-      </c>
+          <t>type-c-31-m-12</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>C165948</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TYPE-C-31-M-12</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Korean Hroparts Elec</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>SMD</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="L60" t="n">
+        <v>237625</v>
+      </c>
+      <c r="M60" t="n">
+        <v>1</v>
+      </c>
+      <c r="N60" t="n">
+        <v>2</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0.1791</v>
+      </c>
+      <c r="P60" t="n">
+        <v>0.3582</v>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lcsc.com/product-detail/C165948.html</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>C5337088 TYPE-C-31-M-12A 0.46 USD</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>U14 U15</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>C2867168</t>
+          <t>C3035748</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>CH340X</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>WCH(Jiangsu Qin Heng)</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>WSON-6-EP(2x2)</t>
+          <t>MSOP-10</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -5431,28 +5427,28 @@
         </is>
       </c>
       <c r="L61" t="n">
-        <v>36</v>
+        <v>24960</v>
       </c>
       <c r="M61" t="n">
         <v>1</v>
       </c>
       <c r="N61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O61" t="n">
-        <v>1.1068</v>
+        <v>0.6632</v>
       </c>
       <c r="P61" t="n">
-        <v>2.2136</v>
+        <v>0.6632</v>
       </c>
       <c r="Q61" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2867168.html</t>
+          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
+          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
         </is>
       </c>
       <c r="S61" t="inlineStr"/>
@@ -5461,48 +5457,48 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>USBC1 USBC2</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>type-c-31-m-12</t>
+          <t>msm381acb026</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>mems</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>type-c-31-m-12</t>
+          <t>msm381acb026</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>C51928208</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>MSM381ACB026</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Korean Hroparts Elec</t>
+          <t>MEMS</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>LGA-3(1.9x2.8)</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -5511,41 +5507,37 @@
         </is>
       </c>
       <c r="L62" t="n">
-        <v>237730</v>
+        <v>6294</v>
       </c>
       <c r="M62" t="n">
         <v>1</v>
       </c>
       <c r="N62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O62" t="n">
-        <v>0.1791</v>
+        <v>0.3026</v>
       </c>
       <c r="P62" t="n">
-        <v>0.3582</v>
+        <v>0.3026</v>
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165948.html</t>
+          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
-        </is>
-      </c>
-      <c r="S62" t="inlineStr">
-        <is>
-          <t>C5337088 TYPE-C-31-M-12A 0.46 USD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -5556,37 +5548,37 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>w25n02kvzeir</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>w25n02</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>w25n02kvzeir</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>C3035748</t>
+          <t>C3010298</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>CH340X</t>
+          <t>W25N02KVZEIR</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>WCH(Jiangsu Qin Heng)</t>
+          <t>Winbond Elec</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>MSOP-10</t>
+          <t>WSON-8-EP(6x8)</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -5595,7 +5587,7 @@
         </is>
       </c>
       <c r="L63" t="n">
-        <v>24970</v>
+        <v>6479</v>
       </c>
       <c r="M63" t="n">
         <v>1</v>
@@ -5604,196 +5596,36 @@
         <v>1</v>
       </c>
       <c r="O63" t="n">
-        <v>0.6632</v>
+        <v>11.0628</v>
       </c>
       <c r="P63" t="n">
-        <v>0.6632</v>
+        <v>11.0628</v>
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
+          <t>https://www.lcsc.com/product-detail/C3010298.html</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
-        </is>
-      </c>
-      <c r="S63" t="inlineStr"/>
+          <t>-40℃~+85℃ 10 Years 104MHz 10uA 2.7V~3.6V 2Gbit 2ms 60,000 Cycles 700us SPI WSON-8-EP(6x8) NAND FLASH ROHS</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>C17626844 W25N02KVZEIR TR 11.16 USD</t>
+        </is>
+      </c>
       <c r="T63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>U13</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>1</v>
-      </c>
-      <c r="C64" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>msm381acb026</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>mems</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>msm381acb026</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>C51928208</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>MSM381ACB026</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>MEMS</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>LGA-3(1.9x2.8)</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="L64" t="n">
-        <v>6294</v>
-      </c>
-      <c r="M64" t="n">
-        <v>1</v>
-      </c>
-      <c r="N64" t="n">
-        <v>1</v>
-      </c>
-      <c r="O64" t="n">
-        <v>0.3026</v>
-      </c>
-      <c r="P64" t="n">
-        <v>0.3026</v>
-      </c>
-      <c r="Q64" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
-        </is>
-      </c>
-      <c r="R64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
-        </is>
-      </c>
-      <c r="S64" t="inlineStr"/>
-      <c r="T64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>U16</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>1</v>
-      </c>
-      <c r="C65" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>w25n02kvzeir</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>w25n02</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>w25n02kvzeir</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>C3010298</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>W25N02KVZEIR</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>Winbond Elec</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>WSON-8-EP(6x8)</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="L65" t="n">
-        <v>6479</v>
-      </c>
-      <c r="M65" t="n">
-        <v>1</v>
-      </c>
-      <c r="N65" t="n">
-        <v>1</v>
-      </c>
-      <c r="O65" t="n">
-        <v>11.0628</v>
-      </c>
-      <c r="P65" t="n">
-        <v>11.0628</v>
-      </c>
-      <c r="Q65" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lcsc.com/product-detail/C3010298.html</t>
-        </is>
-      </c>
-      <c r="R65" t="inlineStr">
-        <is>
-          <t>-40℃~+85℃ 10 Years 104MHz 10uA 2.7V~3.6V 2Gbit 2ms 60,000 Cycles 700us SPI WSON-8-EP(6x8) NAND FLASH ROHS</t>
-        </is>
-      </c>
-      <c r="S65" t="inlineStr">
-        <is>
-          <t>C17626844 W25N02KVZEIR TR 11.16 USD</t>
-        </is>
-      </c>
-      <c r="T65" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="P67">
-        <f>SUM(P2:P65)</f>
+      <c r="P65">
+        <f>SUM(P2:P63)</f>
         <v/>
       </c>
     </row>
@@ -5854,13 +5686,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BOM re-sourced for stock: passives moved to >=1000-piece LCSC parts (25 lines, +0.03 USD)
The cheapest-total run had left 20 passive lines on stocks of 1 to 55 pieces.
Re-priced with --min-stock 1000 --pages 4: every R/C now has 1.3k to 3.5M in
stock; total 43.62 -> 43.65 USD for one board. Schematic ComponentDescription
(and %UTF8% copy) updated on 94 designators to the new C-numbers.

Still below 1000 (single-source, no alternative): K230D 361, Ai-M62-CBS 211,
BQ24072 387, TPS61160A 36, JST SM05B 984.

Adds BOM_JLCPCB.csv (Comment/Designator/Footprint/LCSC Part # for the
assembly BOM upload) and JLCPCB_parts_cart.csv (C-number,qty for the parts
cart bulk add).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -712,7 +712,11 @@
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>LOW STOCK 211, no candidate with &gt;= 1000</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -743,17 +747,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>C366879</t>
+          <t>C20624294</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0805B105K100CT</t>
+          <t>0805B105K100NT</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Walsin Tech Corp</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -767,7 +771,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>14</v>
+        <v>2687</v>
       </c>
       <c r="M4" t="n">
         <v>1</v>
@@ -776,14 +780,14 @@
         <v>2</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0153</v>
+        <v>0.0243</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0306</v>
+        <v>0.0486</v>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C366879.html</t>
+          <t>https://www.lcsc.com/product-detail/C20624294.html</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -793,7 +797,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>C577008 CC0805KRX5R6BB105 0.03 USD</t>
+          <t>C519973 CC0805KKX7R6BB105 0.05 USD</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -915,17 +919,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>C6600400</t>
+          <t>C3012377</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>MSASU105SB7104KFNB25</t>
+          <t>CSA0402X7R104K500GT</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Taiyo Yuden</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -939,7 +943,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>22</v>
+        <v>408770</v>
       </c>
       <c r="M6" t="n">
         <v>1</v>
@@ -948,14 +952,14 @@
         <v>12</v>
       </c>
       <c r="O6" t="n">
-        <v>0.004</v>
+        <v>0.0044</v>
       </c>
       <c r="P6" t="n">
-        <v>0.048</v>
+        <v>0.0528</v>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C6600400.html</t>
+          <t>https://www.lcsc.com/product-detail/C3012377.html</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -965,7 +969,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>C3012377 CSA0402X7R104K500GT 0.05 USD</t>
+          <t>C48543623 TCC0402X7R104K500ATM 0.05 USD</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
@@ -1083,17 +1087,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>C696905</t>
+          <t>C106201</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>TCC0402COG120K500AT</t>
+          <t>CC0402JRNPO9BN120</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>CCTC</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1107,7 +1111,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>555</v>
+        <v>3509224</v>
       </c>
       <c r="M8" t="n">
         <v>1</v>
@@ -1116,24 +1120,24 @@
         <v>2</v>
       </c>
       <c r="O8" t="n">
-        <v>0.0014</v>
+        <v>0.002</v>
       </c>
       <c r="P8" t="n">
-        <v>0.0028</v>
+        <v>0.004</v>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C696905.html</t>
+          <t>https://www.lcsc.com/product-detail/C106201.html</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>12pF 50V C0G ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>12pF 50V NP0 ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>C106201 CC0402JRNPO9BN120 0.00 USD</t>
+          <t>C7467122 FCC0402N120J500AT 0.01 USD</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1167,17 +1171,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>C696863</t>
+          <t>C107000</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>TCC0402COG200K500AT</t>
+          <t>CC0402JRNPO9BN200</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>CCTC</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1191,7 +1195,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>17</v>
+        <v>3263279</v>
       </c>
       <c r="M9" t="n">
         <v>1</v>
@@ -1200,24 +1204,24 @@
         <v>5</v>
       </c>
       <c r="O9" t="n">
-        <v>0.0004</v>
+        <v>0.0021</v>
       </c>
       <c r="P9" t="n">
-        <v>0.002</v>
+        <v>0.0105</v>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C696863.html</t>
+          <t>https://www.lcsc.com/product-detail/C107000.html</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>20pF 50V C0G ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>20pF 50V NP0 ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>C107000 CC0402JRNPO9BN200 0.01 USD</t>
+          <t>C5137579 FCC0402N200J500AT 0.01 USD</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1479,7 +1483,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>11646</v>
+        <v>11651</v>
       </c>
       <c r="M13" t="n">
         <v>1</v>
@@ -1563,7 +1567,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>53064</v>
+        <v>50553</v>
       </c>
       <c r="M14" t="n">
         <v>1</v>
@@ -1643,7 +1647,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>249661</v>
+        <v>249561</v>
       </c>
       <c r="M15" t="n">
         <v>1</v>
@@ -1883,7 +1887,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>7227</v>
+        <v>7225</v>
       </c>
       <c r="M18" t="n">
         <v>1</v>
@@ -2103,17 +2107,17 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>C5189828</t>
+          <t>C20070307</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CS1608X7R105K100NRB</t>
+          <t>CGA0603X5R105K100JT</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Samwha Capacitor</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2127,7 +2131,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>88309</v>
       </c>
       <c r="M21" t="n">
         <v>1</v>
@@ -2136,24 +2140,24 @@
         <v>1</v>
       </c>
       <c r="O21" t="n">
-        <v>0.0043</v>
+        <v>0.0074</v>
       </c>
       <c r="P21" t="n">
-        <v>0.0043</v>
+        <v>0.0074</v>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C5189828.html</t>
+          <t>https://www.lcsc.com/product-detail/C20070307.html</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>10V 1uF X7R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>10V 1uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>C49326606 0603X7R105K100NT 0.01 USD</t>
+          <t>C111590 0603X105K100NT 0.01 USD</t>
         </is>
       </c>
       <c r="T21" t="inlineStr"/>
@@ -2237,7 +2241,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>C22376489 FS18B226M6R3PBG 0.17 USD</t>
+          <t>C59461 CL10A226MQ8NRNC 0.18 USD</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -2488,7 +2492,11 @@
         </is>
       </c>
       <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>LOW STOCK 984, no candidate with &gt;= 1000</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2741,7 +2749,7 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>C52994078 PRTR5V0U2F,115(ES) 0.53 USD</t>
+          <t>C2937001 PRTR5V0U2F 0.55 USD</t>
         </is>
       </c>
       <c r="T28" t="inlineStr"/>
@@ -2775,17 +2783,17 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>C103222</t>
+          <t>C54920843</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>RTT0310R0FTP</t>
+          <t>HRC0603F10R0ENTN</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>RALEC</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2799,7 +2807,7 @@
         </is>
       </c>
       <c r="L29" t="n">
-        <v>46</v>
+        <v>22157</v>
       </c>
       <c r="M29" t="n">
         <v>1</v>
@@ -2808,24 +2816,24 @@
         <v>1</v>
       </c>
       <c r="O29" t="n">
-        <v>0.0018</v>
+        <v>0.0011</v>
       </c>
       <c r="P29" t="n">
-        <v>0.0018</v>
+        <v>0.0011</v>
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C103222.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920843.html</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±100ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100mW 10Ω 50V Thick Film Resistor ±1% ±200ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>C177661 RCT0310RFLF 0.00 USD</t>
+          <t>C49652997 GR0603F10RT5G00 0.00 USD</t>
         </is>
       </c>
       <c r="T29" t="inlineStr"/>
@@ -2859,17 +2867,17 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>C158913</t>
+          <t>C49654665</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>RTT034R02FTP</t>
+          <t>GR0603F4R02T5G00</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>RALEC</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2883,7 +2891,7 @@
         </is>
       </c>
       <c r="L30" t="n">
-        <v>38</v>
+        <v>1299</v>
       </c>
       <c r="M30" t="n">
         <v>1</v>
@@ -2892,24 +2900,24 @@
         <v>1</v>
       </c>
       <c r="O30" t="n">
-        <v>0.0018</v>
+        <v>0.0023</v>
       </c>
       <c r="P30" t="n">
-        <v>0.0018</v>
+        <v>0.0023</v>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C158913.html</t>
+          <t>https://www.lcsc.com/product-detail/C49654665.html</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 4.02Ω 75V Thick Film Resistor ±1% ±200ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100mW 4.02Ω 75V Thick Film Resistor ±1% 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>C322168 RS-03L4R02FT 0.00 USD</t>
+          <t>C2930151 FRC0603F4R02TS 0.00 USD</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
@@ -2971,7 +2979,7 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>7661</v>
+        <v>7623</v>
       </c>
       <c r="M31" t="n">
         <v>1</v>
@@ -3135,7 +3143,7 @@
         </is>
       </c>
       <c r="L33" t="n">
-        <v>161</v>
+        <v>361</v>
       </c>
       <c r="M33" t="n">
         <v>1</v>
@@ -3160,7 +3168,11 @@
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>LOW STOCK 361, no candidate with &gt;= 1000</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3275,17 +3287,17 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>C3015792</t>
+          <t>C54920634</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>SCR0402F1K1</t>
+          <t>HRC0402F1101DNTO</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3299,7 +3311,7 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>40</v>
+        <v>17360</v>
       </c>
       <c r="M35" t="n">
         <v>1</v>
@@ -3308,14 +3320,14 @@
         <v>1</v>
       </c>
       <c r="O35" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="P35" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015792.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920634.html</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3325,7 +3337,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>C54920634 HRC0402F1101DNTO 0.00 USD</t>
+          <t>C22369271 RCA021K1FLF 0.00 USD</t>
         </is>
       </c>
       <c r="T35" t="inlineStr"/>
@@ -3359,17 +3371,17 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>C3015623</t>
+          <t>C49653889</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>SCR0402F590R</t>
+          <t>GR0402F590RTAG00</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -3383,7 +3395,7 @@
         </is>
       </c>
       <c r="L36" t="n">
-        <v>353</v>
+        <v>10000</v>
       </c>
       <c r="M36" t="n">
         <v>1</v>
@@ -3392,14 +3404,14 @@
         <v>1</v>
       </c>
       <c r="O36" t="n">
-        <v>0.0005</v>
+        <v>0.0008</v>
       </c>
       <c r="P36" t="n">
-        <v>0.0005</v>
+        <v>0.0008</v>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015623.html</t>
+          <t>https://www.lcsc.com/product-detail/C49653889.html</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3409,7 +3421,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>C334714 WR04X5900FTL 0.00 USD</t>
+          <t>C48971902 RC-02K5900FT 0.00 USD</t>
         </is>
       </c>
       <c r="T36" t="inlineStr"/>
@@ -3443,17 +3455,17 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>C3015796</t>
+          <t>C54920638</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>SCR0402F1K5</t>
+          <t>HRC0402F1501DNTO</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -3467,7 +3479,7 @@
         </is>
       </c>
       <c r="L37" t="n">
-        <v>21</v>
+        <v>313030</v>
       </c>
       <c r="M37" t="n">
         <v>1</v>
@@ -3476,14 +3488,14 @@
         <v>1</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="P37" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015796.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920638.html</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3493,7 +3505,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>C100249 CR0402FF1501G 0.00 USD</t>
+          <t>C22369462 RCA021K5FLF 0.00 USD</t>
         </is>
       </c>
       <c r="T37" t="inlineStr"/>
@@ -3527,17 +3539,17 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>C279979</t>
+          <t>C49652939</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>CR-02FL6--100K</t>
+          <t>GR0402F100KTAG00</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Viking Tech</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -3551,7 +3563,7 @@
         </is>
       </c>
       <c r="L38" t="n">
-        <v>5579</v>
+        <v>6594</v>
       </c>
       <c r="M38" t="n">
         <v>1</v>
@@ -3560,24 +3572,24 @@
         <v>20</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0011</v>
+        <v>0.0008</v>
       </c>
       <c r="P38" t="n">
-        <v>0.022</v>
+        <v>0.016</v>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C279979.html</t>
+          <t>https://www.lcsc.com/product-detail/C49652939.html</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>C2759534 HP02WAF1003TCE 0.03 USD</t>
+          <t>C22369473 RCA02100KFLF 0.02 USD</t>
         </is>
       </c>
       <c r="T38" t="inlineStr"/>
@@ -3611,17 +3623,17 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>C1858459</t>
+          <t>C22369472</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>RC0402FR-1310KL</t>
+          <t>RCA0210KFLF</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>HKR(Hong Kong Resistors)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3635,7 +3647,7 @@
         </is>
       </c>
       <c r="L39" t="n">
-        <v>49503</v>
+        <v>1186820</v>
       </c>
       <c r="M39" t="n">
         <v>1</v>
@@ -3644,24 +3656,24 @@
         <v>18</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0018</v>
+        <v>0.0011</v>
       </c>
       <c r="P39" t="n">
-        <v>0.0324</v>
+        <v>0.0198</v>
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C1858459.html</t>
+          <t>https://www.lcsc.com/product-detail/C22369472.html</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>C327797 MR04X1002FTL 0.04 USD</t>
+          <t>C2759535 HP02WAF1002TCE 0.02 USD</t>
         </is>
       </c>
       <c r="T39" t="inlineStr"/>
@@ -3719,7 +3731,7 @@
         </is>
       </c>
       <c r="L40" t="n">
-        <v>1191862</v>
+        <v>1191972</v>
       </c>
       <c r="M40" t="n">
         <v>1</v>
@@ -3779,17 +3791,17 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>C3152063</t>
+          <t>C54920625</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>SC0402F1503F2ANRH</t>
+          <t>HRC0402F1503DNTO</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Sunway</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -3803,7 +3815,7 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>13</v>
+        <v>18610</v>
       </c>
       <c r="M41" t="n">
         <v>1</v>
@@ -3812,14 +3824,14 @@
         <v>1</v>
       </c>
       <c r="O41" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="P41" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3152063.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920625.html</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3829,7 +3841,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>C102813 RTT021503FTH 0.00 USD</t>
+          <t>C22369540 RCA02150KFLF 0.00 USD</t>
         </is>
       </c>
       <c r="T41" t="inlineStr"/>
@@ -3863,17 +3875,17 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>C3015766</t>
+          <t>C54920644</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>SCR0402F200R</t>
+          <t>HRC0402F2000DNTO</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -3887,7 +3899,7 @@
         </is>
       </c>
       <c r="L42" t="n">
-        <v>15</v>
+        <v>1881170</v>
       </c>
       <c r="M42" t="n">
         <v>1</v>
@@ -3896,14 +3908,14 @@
         <v>2</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="P42" t="n">
-        <v>0.001</v>
+        <v>0.0014</v>
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015766.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920644.html</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -3913,7 +3925,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>C46635169 CL0402FN200RP 0.00 USD</t>
+          <t>C22356253 RCA02200RFLF 0.00 USD</t>
         </is>
       </c>
       <c r="T42" t="inlineStr"/>
@@ -3947,17 +3959,17 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>C49653950</t>
+          <t>C22369550</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>GR0402F200KTAG00</t>
+          <t>RCA02200KFLF</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>HKR(Hong Kong Resistors)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -3971,7 +3983,7 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>55</v>
+        <v>741795</v>
       </c>
       <c r="M43" t="n">
         <v>1</v>
@@ -3980,24 +3992,24 @@
         <v>1</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="P43" t="n">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49653950.html</t>
+          <t>https://www.lcsc.com/product-detail/C22369550.html</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>C3015901 SCR0402F200K 0.00 USD</t>
+          <t>C102872 RTT022003FTH 0.00 USD</t>
         </is>
       </c>
       <c r="T43" t="inlineStr"/>
@@ -4031,17 +4043,17 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>C49654869</t>
+          <t>C2929994</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>GR0402F22RTAG00</t>
+          <t>FRC0402F22R0TS</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>FOJAN</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4055,7 +4067,7 @@
         </is>
       </c>
       <c r="L44" t="n">
-        <v>20</v>
+        <v>921743</v>
       </c>
       <c r="M44" t="n">
         <v>1</v>
@@ -4064,14 +4076,14 @@
         <v>1</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0019</v>
       </c>
       <c r="P44" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0019</v>
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49654869.html</t>
+          <t>https://www.lcsc.com/product-detail/C2929994.html</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4081,7 +4093,7 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>C102905 RTT0222R0FTH 0.00 USD</t>
+          <t>C2759796 CQ02WGF220JTCE 0.00 USD</t>
         </is>
       </c>
       <c r="T44" t="inlineStr"/>
@@ -4115,17 +4127,17 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>C168215</t>
+          <t>C22356255</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>WR04X2400FTL</t>
+          <t>RCA02240RFLF</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Walsin Tech Corp</t>
+          <t>HKR(Hong Kong Resistors)</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4139,7 +4151,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>9</v>
+        <v>144132</v>
       </c>
       <c r="M45" t="n">
         <v>1</v>
@@ -4148,24 +4160,24 @@
         <v>4</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0004</v>
+        <v>0.001</v>
       </c>
       <c r="P45" t="n">
-        <v>0.0016</v>
+        <v>0.004</v>
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C168215.html</t>
+          <t>https://www.lcsc.com/product-detail/C22356255.html</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>C49652940 GR0402F240RTAG00 0.00 USD</t>
+          <t>C324768 RC-02K2400FT 0.01 USD</t>
         </is>
       </c>
       <c r="T45" t="inlineStr"/>
@@ -4199,17 +4211,17 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>C46444589</t>
+          <t>C102933</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>RC-02K2613FT</t>
+          <t>RTT022613FTH</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>FH (Guangdong Fenghua Advanced Tech)</t>
+          <t>RALEC</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -4223,7 +4235,7 @@
         </is>
       </c>
       <c r="L46" t="n">
-        <v>100</v>
+        <v>37942</v>
       </c>
       <c r="M46" t="n">
         <v>1</v>
@@ -4232,24 +4244,24 @@
         <v>1</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0007</v>
       </c>
       <c r="P46" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0007</v>
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C46444589.html</t>
+          <t>https://www.lcsc.com/product-detail/C102933.html</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>261kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 261kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>C3015905 SCR0402F261K 0.00 USD</t>
+          <t>C49656016 GR0402F261KTAG00 0.00 USD</t>
         </is>
       </c>
       <c r="T46" t="inlineStr"/>
@@ -4283,17 +4295,17 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>C3152079</t>
+          <t>C49653548</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>SC0402F3002F2ANRH</t>
+          <t>GR0402F30KTAG00</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Sunway</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -4307,7 +4319,7 @@
         </is>
       </c>
       <c r="L47" t="n">
-        <v>16</v>
+        <v>10000</v>
       </c>
       <c r="M47" t="n">
         <v>1</v>
@@ -4316,14 +4328,14 @@
         <v>1</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0005</v>
+        <v>0.0008</v>
       </c>
       <c r="P47" t="n">
-        <v>0.0005</v>
+        <v>0.0008</v>
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3152079.html</t>
+          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4333,7 +4345,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>C54920659 HRC0402F3002DNTO 0.00 USD</t>
+          <t>C22369568 RCA0230KFLF 0.00 USD</t>
         </is>
       </c>
       <c r="T47" t="inlineStr"/>
@@ -4367,17 +4379,17 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>C159031</t>
+          <t>C53069467</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>RTT023322FTH</t>
+          <t>CL0402FN33K2P</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>RALEC</t>
+          <t>CHANGLONG</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -4391,7 +4403,7 @@
         </is>
       </c>
       <c r="L48" t="n">
-        <v>5</v>
+        <v>2978</v>
       </c>
       <c r="M48" t="n">
         <v>1</v>
@@ -4400,24 +4412,24 @@
         <v>1</v>
       </c>
       <c r="O48" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="P48" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C159031.html</t>
+          <t>https://www.lcsc.com/product-detail/C53069467.html</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 33.2kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 33.2kΩ 50V 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>C53069467 CL0402FN33K2P 0.00 USD</t>
+          <t>C122548 0402WGF3322TCE 0.00 USD</t>
         </is>
       </c>
       <c r="T48" t="inlineStr"/>
@@ -4451,17 +4463,17 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>C3015810</t>
+          <t>C49652824</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>SCR0402F4K7</t>
+          <t>GR0402F4K7TAG00</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -4475,7 +4487,7 @@
         </is>
       </c>
       <c r="L49" t="n">
-        <v>9</v>
+        <v>10830</v>
       </c>
       <c r="M49" t="n">
         <v>1</v>
@@ -4484,14 +4496,14 @@
         <v>6</v>
       </c>
       <c r="O49" t="n">
-        <v>0.0005</v>
+        <v>0.0008</v>
       </c>
       <c r="P49" t="n">
-        <v>0.003</v>
+        <v>0.0048</v>
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015810.html</t>
+          <t>https://www.lcsc.com/product-detail/C49652824.html</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4501,7 +4513,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>C103055 RTT024701FTH 0.00 USD</t>
+          <t>C22369456 RCA024K7FLF 0.01 USD</t>
         </is>
       </c>
       <c r="T49" t="inlineStr"/>
@@ -4535,17 +4547,17 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>C881176</t>
+          <t>C103052</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>CR0402F46K4Q10Z</t>
+          <t>RTT024642FTH</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Ever Ohms Tech</t>
+          <t>RALEC</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -4559,7 +4571,7 @@
         </is>
       </c>
       <c r="L50" t="n">
-        <v>673</v>
+        <v>7120</v>
       </c>
       <c r="M50" t="n">
         <v>1</v>
@@ -4568,24 +4580,24 @@
         <v>1</v>
       </c>
       <c r="O50" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0007</v>
       </c>
       <c r="P50" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0007</v>
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C881176.html</t>
+          <t>https://www.lcsc.com/product-detail/C103052.html</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 46.4kΩ 50V 63mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 46.4kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>C103052 RTT024642FTH 0.00 USD</t>
+          <t>C49654486 GR0402F46K4TAG00 0.00 USD</t>
         </is>
       </c>
       <c r="T50" t="inlineStr"/>
@@ -4619,17 +4631,17 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>C3152095</t>
+          <t>C22369457</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>SC0402F5101F2ANRH</t>
+          <t>RCA025K1FLF</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Sunway</t>
+          <t>HKR(Hong Kong Resistors)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -4643,7 +4655,7 @@
         </is>
       </c>
       <c r="L51" t="n">
-        <v>10</v>
+        <v>1323626</v>
       </c>
       <c r="M51" t="n">
         <v>1</v>
@@ -4652,24 +4664,24 @@
         <v>4</v>
       </c>
       <c r="O51" t="n">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="P51" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3152095.html</t>
+          <t>https://www.lcsc.com/product-detail/C22369457.html</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>C409700 CR-02FL6---5K1 0.00 USD</t>
+          <t>C103079 RTT025101FTH 0.00 USD</t>
         </is>
       </c>
       <c r="T51" t="inlineStr"/>
@@ -4703,17 +4715,17 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>C3015918</t>
+          <t>C49655223</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>SCR0402F511K</t>
+          <t>GR0402F511KTAG00</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -4727,7 +4739,7 @@
         </is>
       </c>
       <c r="L52" t="n">
-        <v>16</v>
+        <v>7820</v>
       </c>
       <c r="M52" t="n">
         <v>1</v>
@@ -4736,24 +4748,24 @@
         <v>4</v>
       </c>
       <c r="O52" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0008</v>
       </c>
       <c r="P52" t="n">
-        <v>0.0024</v>
+        <v>0.0032</v>
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3015918.html</t>
+          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>C49655223 GR0402F511KTAG00 0.00 USD</t>
+          <t>C5126239 FRC0402F5113TS 0.01 USD</t>
         </is>
       </c>
       <c r="T52" t="inlineStr"/>
@@ -4787,17 +4799,17 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>C5356157</t>
+          <t>C54920709</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>SC0402F9102F2ANRH</t>
+          <t>HRC0402F9102DNTO</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Sunway</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4811,7 +4823,7 @@
         </is>
       </c>
       <c r="L53" t="n">
-        <v>18</v>
+        <v>133322</v>
       </c>
       <c r="M53" t="n">
         <v>1</v>
@@ -4820,14 +4832,14 @@
         <v>2</v>
       </c>
       <c r="O53" t="n">
-        <v>0.0003</v>
+        <v>0.0007</v>
       </c>
       <c r="P53" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0014</v>
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C5356157.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4837,7 +4849,7 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>C365061 HPCR0402F91K0K9 0.00 USD</t>
+          <t>C22369327 RCA0291KFLF 0.00 USD</t>
         </is>
       </c>
       <c r="T53" t="inlineStr"/>
@@ -4920,7 +4932,11 @@
         </is>
       </c>
       <c r="S54" t="inlineStr"/>
-      <c r="T54" t="inlineStr"/>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>LOW STOCK 387, no candidate with &gt;= 1000</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5036,7 +5052,11 @@
         </is>
       </c>
       <c r="S56" t="inlineStr"/>
-      <c r="T56" t="inlineStr"/>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>LOW STOCK 36, no candidate with &gt;= 1000</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5091,7 +5111,7 @@
         </is>
       </c>
       <c r="L57" t="n">
-        <v>237625</v>
+        <v>237028</v>
       </c>
       <c r="M57" t="n">
         <v>1</v>
@@ -5175,7 +5195,7 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>24960</v>
+        <v>25358</v>
       </c>
       <c r="M58" t="n">
         <v>1</v>
@@ -5335,7 +5355,7 @@
         </is>
       </c>
       <c r="L60" t="n">
-        <v>6479</v>
+        <v>6279</v>
       </c>
       <c r="M60" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Schematic + BOM follow the LCSC-orderable parts (9 lines, 48 designators)
lcsc.com does not sell or has no stock of nine JLCPCB-library picks; the
substitutes verified in the LCSC cart are now the schematic's LCSC numbers:
  DSK24        C51898076 -> C2939005   KUU DSK24 (SOD-123FL 40V 2A)
  10k 0402     C22369472 -> C1858459   YAGEO RC0402FR-1310KL
  200k 0402    C22369550 -> C102872    RALEC RTT022003FTH
  240R 0402    C22356255 -> C324768    RC-02K2400FT
  5.1k 0402    C22369457 -> C103079    RALEC RTT025101FTH
  100n 0402    C3012377  -> C513772    Samwha CS1005X7R104K500NR 50V X7R
  120p 0402    C7507400  -> C2887023   CCTC TCC0402COG121J500AT
  1k ferrite   C76883    -> C280602    Chilisin SBY100505T-102Y-N (300mA 650mR)
  S2B-PH-K-S   C173752   -> C157932    JST S2B-PH-K-S-GW (same drawing)
BOM_LCSC.xlsx/.txt re-emitted (44.19 USD at JLCPCB unit prices), BOM_JLCPCB.csv
and JLCPCB_parts_cart.csv regenerated so both order lists name the same parts.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -631,8 +631,6 @@
           <t xml:space="preserve">-40℃~+120℃ 0%RH~100%RH 2.2V~5.5V 570uA Factory calibration I2C ±0.5℃ ±3%RH SMD-6P,3x3mm Temperature and Humidity Sensor </t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -711,7 +709,6 @@
           <t>-40℃~+85℃ -98dBm 2.97V~3.6V 22dBm 394mA 59mA BL616 UART、SDIO、SPI、I2C、GPIO、PWM、I2S、USB2.0 SMD,12x12mm WiFi Modules ROHS</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
           <t>LOW STOCK 211, no candidate with &gt;= 1000</t>
@@ -888,7 +885,6 @@
           <t>C2846674 0201X104K160NT 0.17 USD</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -919,17 +915,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>C3012377</t>
+          <t>C513772</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CSA0402X7R104K500GT</t>
+          <t>CS1005X7R104K500NR</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>Samwha Capacitor</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -943,7 +939,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>408770</v>
+        <v>116403</v>
       </c>
       <c r="M6" t="n">
         <v>1</v>
@@ -952,27 +948,26 @@
         <v>12</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0044</v>
+        <v>0.0032</v>
       </c>
       <c r="P6" t="n">
-        <v>0.0528</v>
+        <v>0.0384</v>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3012377.html</t>
+          <t>https://www.lcsc.com/product-detail/C513772.html</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>100nF 50V X7R ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>C48543623 TCC0402X7R104K500ATM 0.05 USD</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr"/>
+          <t>100nF 50V ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>LCSC-orderable substitute for C3012377 CSA0402X7R104K500GT (not sold / no stock on lcsc.com)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1003,17 +998,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>C7507400</t>
+          <t>C2887023</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>C0402C0G121K500NTB</t>
+          <t>TCC0402COG121J500AT</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>EYANG(Shenzhen Eyang Tech Development)</t>
+          <t>CCTC</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1027,7 +1022,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>2426</v>
+        <v>54327</v>
       </c>
       <c r="M7" t="n">
         <v>1</v>
@@ -1036,27 +1031,26 @@
         <v>2</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0029</v>
+        <v>0.0033</v>
       </c>
       <c r="P7" t="n">
-        <v>0.0058</v>
+        <v>0.0066</v>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C7507400.html</t>
+          <t>https://www.lcsc.com/product-detail/C2887023.html</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>120pF 50V C0G ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>C2887023 TCC0402COG121J500AT 0.01 USD</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr"/>
+          <t>120pF 50V C0G ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>LCSC-orderable substitute for C7507400 C0402C0G121K500NTB (not sold / no stock on lcsc.com)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1140,7 +1134,6 @@
           <t>C7467122 FCC0402N120J500AT 0.01 USD</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1224,7 +1217,6 @@
           <t>C5137579 FCC0402N200J500AT 0.01 USD</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1308,7 +1300,6 @@
           <t>C5159775 GRM155R61H224KE01D 0.04 USD</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1337,9 +1328,6 @@
           <t>Connector_2PIn</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
           <t>no purchased part (pad / test point / antenna)</t>
@@ -1428,7 +1416,6 @@
           <t>C22415740 C1206C105J5RACTU 1.80 USD</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1507,7 +1494,6 @@
           <t>-40℃~+85℃ 12.5pF 32.768kHz 70kΩ Crystal Oscillator ±20ppm SMD3215-2P Crystals ROHS</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
           <t>generic 3215 12.5pF alternative: C22386770 SXTF321532768A20F ~0.13 USD</t>
@@ -1543,17 +1529,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>C76883</t>
+          <t>C280602</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>BLM15AG102SN1D</t>
+          <t>SBY100505T-102Y-N</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Murata Electronics</t>
+          <t>Chilisin Elec</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1567,7 +1553,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>50553</v>
+        <v>9957</v>
       </c>
       <c r="M14" t="n">
         <v>1</v>
@@ -1576,14 +1562,14 @@
         <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>0.0051</v>
+        <v>0.0063</v>
       </c>
       <c r="P14" t="n">
-        <v>0.0051</v>
+        <v>0.0063</v>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C76883.html</t>
+          <t>https://www.lcsc.com/product-detail/C280602.html</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1591,8 +1577,11 @@
           <t>1 1kΩ@100MHz 300mA 650mΩ ±25% 0402 Ferrite Beads ROHS</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>LCSC-orderable substitute for C76883 BLM15AG102SN1D (not sold / no stock on lcsc.com)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1671,8 +1660,6 @@
           <t>-55℃~+125℃ 1 120Ω@100MHz 180mΩ 800mA ±25% 0603 Ferrite Beads ROHS</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1751,8 +1738,6 @@
           <t>26mΩ 4.5A 470nH 5.5A ±20% 0806 Power Inductors ROHS</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1831,8 +1816,6 @@
           <t>1.4A 10uH 400mΩ 950mA ±20% 1008 Power Inductors ROHS</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1911,8 +1894,6 @@
           <t>-40℃~+125℃@(TJ) 1 1.3V~5.5V 1.4MHz、1.6MHz、2.1MHz 1.8V~5.2V 11uA 2A Adjustable Buck-Boost Buck-Boost Built-in Yes VSON-10</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1991,8 +1972,6 @@
           <t xml:space="preserve">-40℃~+125℃@(TJ) 1 2.2MHz 2.4V~5.5V 3A 4uA 600mV~4V Adjustable Buck Built-in Overcurrent Protection、Light load efficient </t>
         </is>
       </c>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2076,7 +2055,6 @@
           <t>C6119842 CGA0603X5R106K100JT 0.29 USD</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2160,7 +2138,6 @@
           <t>C111590 0603X105K100NT 0.01 USD</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2244,7 +2221,6 @@
           <t>C59461 CL10A226MQ8NRNC 0.18 USD</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2275,17 +2251,17 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>C51898076</t>
+          <t>C2939005</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>DSK24</t>
+          <t>DSK24 K24</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Zhengxin</t>
+          <t>KUU</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2299,7 +2275,7 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>4155</v>
+        <v>120296</v>
       </c>
       <c r="M23" t="n">
         <v>1</v>
@@ -2308,27 +2284,26 @@
         <v>3</v>
       </c>
       <c r="O23" t="n">
-        <v>0.0153</v>
+        <v>0.0187</v>
       </c>
       <c r="P23" t="n">
-        <v>0.0459</v>
+        <v>0.0561</v>
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C51898076.html</t>
+          <t>https://www.lcsc.com/product-detail/C2939005.html</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 1 Independent 2A 40A 40V 500uA@40V 550mV@2A SOD-123FL Schottky Diodes ROHS</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>C54863492 DSK24 0.05 USD</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr"/>
+          <t>2A 40A 40V 500uA@40V 550mV@2A Independent SOD-123FL Schottky Diodes ROHS</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>LCSC-orderable substitute for C51898076 DSK24 (not sold / no stock on lcsc.com)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2407,7 +2382,6 @@
           <t>-40℃~+85℃ 120° 1mm x 0.5mm square LED 2.4V 20mA 210mcd 50mW 585nm~595nm 590nm Discrete Diode Water Clear Yellow 0402 LED</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
           <t>yellow 0402 LED 590nm, replaces generic YLED0402B</t>
@@ -2491,7 +2465,6 @@
           <t>-25℃~+85℃ 1 1A 1mm 1x5P 4.4mm 5 50V 5P 6.8mm 7mm Auxiliary Solder Pin Copper alloy NSH PA Surface Mount, Right Angle Tin</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
           <t>LOW STOCK 984, no candidate with &gt;= 1000</t>
@@ -2580,7 +2553,6 @@
           <t>C53199108 DMG2301L-7(ES) 0.03 USD</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2752,7 +2724,6 @@
           <t>C2937001 PRTR5V0U2F 0.55 USD</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2836,7 +2807,6 @@
           <t>C49652997 GR0603F10RT5G00 0.00 USD</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3003,8 +2973,6 @@
           <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3035,12 +3003,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>C173752</t>
+          <t>C157932</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S(LF)(SN)</t>
+          <t>S2B-PH-K-S-GW</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3059,7 +3027,7 @@
         </is>
       </c>
       <c r="L32" t="n">
-        <v>27957</v>
+        <v>15992</v>
       </c>
       <c r="M32" t="n">
         <v>1</v>
@@ -3068,14 +3036,14 @@
         <v>3</v>
       </c>
       <c r="O32" t="n">
-        <v>0.038</v>
+        <v>0.2126</v>
       </c>
       <c r="P32" t="n">
-        <v>0.114</v>
+        <v>0.6378</v>
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C173752.html</t>
+          <t>https://www.lcsc.com/product-detail/C157932.html</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3083,12 +3051,11 @@
           <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>C157932 S2B-PH-K-S-GW 0.64 USD</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>LCSC-orderable substitute for C173752 S2B-PH-K-S(LF)(SN) (not sold / no stock on lcsc.com)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3167,7 +3134,6 @@
           <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
           <t>LOW STOCK 361, no candidate with &gt;= 1000</t>
@@ -3251,7 +3217,6 @@
           <t>-25℃~+85℃ 0.3mm 0.5mm 22P 2mm 400mA 50V Bottom Contact Phosphor bronze Slide Lock Surface Mount, Right Angle Tin SMD,P=0</t>
         </is>
       </c>
-      <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
           <t>Molex 54548-2271 DISCONTINUED (LCSC: no longer manufactured). Same type (0.5mm 22P bottom-contact slide-lock, right angle) offered; FOOTPRINT MUST BE VERIFIED against its drawing</t>
@@ -3340,7 +3305,6 @@
           <t>C22369271 RCA021K1FLF 0.00 USD</t>
         </is>
       </c>
-      <c r="T35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3424,7 +3388,6 @@
           <t>C48971902 RC-02K5900FT 0.00 USD</t>
         </is>
       </c>
-      <c r="T36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3508,7 +3471,6 @@
           <t>C22369462 RCA021K5FLF 0.00 USD</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3592,7 +3554,6 @@
           <t>C22369473 RCA02100KFLF 0.02 USD</t>
         </is>
       </c>
-      <c r="T38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3623,17 +3584,17 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>C22369472</t>
+          <t>C1858459</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>RCA0210KFLF</t>
+          <t>RC0402FR-1310KL</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>HKR(Hong Kong Resistors)</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3647,7 +3608,7 @@
         </is>
       </c>
       <c r="L39" t="n">
-        <v>1186820</v>
+        <v>49403</v>
       </c>
       <c r="M39" t="n">
         <v>1</v>
@@ -3656,27 +3617,26 @@
         <v>18</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0011</v>
+        <v>0.0018</v>
       </c>
       <c r="P39" t="n">
-        <v>0.0198</v>
+        <v>0.0324</v>
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22369472.html</t>
+          <t>https://www.lcsc.com/product-detail/C1858459.html</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>C2759535 HP02WAF1002TCE 0.02 USD</t>
-        </is>
-      </c>
-      <c r="T39" t="inlineStr"/>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>LCSC-orderable substitute for C22369472 RCA0210KFLF (not sold / no stock on lcsc.com)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3760,7 +3720,6 @@
           <t>C22356241 RCA02120KFLF 0.00 USD</t>
         </is>
       </c>
-      <c r="T40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3844,7 +3803,6 @@
           <t>C22369540 RCA02150KFLF 0.00 USD</t>
         </is>
       </c>
-      <c r="T41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3928,7 +3886,6 @@
           <t>C22356253 RCA02200RFLF 0.00 USD</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3959,17 +3916,17 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>C22369550</t>
+          <t>C102872</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>RCA02200KFLF</t>
+          <t>RTT022003FTH</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>HKR(Hong Kong Resistors)</t>
+          <t>RALEC</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -3983,7 +3940,7 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>741795</v>
+        <v>19832</v>
       </c>
       <c r="M43" t="n">
         <v>1</v>
@@ -3992,27 +3949,26 @@
         <v>1</v>
       </c>
       <c r="O43" t="n">
-        <v>0.001</v>
+        <v>0.0012</v>
       </c>
       <c r="P43" t="n">
-        <v>0.001</v>
+        <v>0.0012</v>
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22369550.html</t>
+          <t>https://www.lcsc.com/product-detail/C102872.html</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
-        </is>
-      </c>
-      <c r="S43" t="inlineStr">
-        <is>
-          <t>C102872 RTT022003FTH 0.00 USD</t>
-        </is>
-      </c>
-      <c r="T43" t="inlineStr"/>
+          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>LCSC-orderable substitute for C22369550 RCA02200KFLF (not sold / no stock on lcsc.com)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4096,7 +4052,6 @@
           <t>C2759796 CQ02WGF220JTCE 0.00 USD</t>
         </is>
       </c>
-      <c r="T44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4127,17 +4082,17 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>C22356255</t>
+          <t>C324768</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>RCA02240RFLF</t>
+          <t>RC-02K2400FT</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>HKR(Hong Kong Resistors)</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4151,7 +4106,7 @@
         </is>
       </c>
       <c r="L45" t="n">
-        <v>144132</v>
+        <v>347318</v>
       </c>
       <c r="M45" t="n">
         <v>1</v>
@@ -4160,27 +4115,26 @@
         <v>4</v>
       </c>
       <c r="O45" t="n">
-        <v>0.001</v>
+        <v>0.0013</v>
       </c>
       <c r="P45" t="n">
-        <v>0.004</v>
+        <v>0.0052</v>
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22356255.html</t>
+          <t>https://www.lcsc.com/product-detail/C324768.html</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
-        </is>
-      </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>C324768 RC-02K2400FT 0.01 USD</t>
-        </is>
-      </c>
-      <c r="T45" t="inlineStr"/>
+          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>LCSC-orderable substitute for C22356255 RCA02240RFLF (not sold / no stock on lcsc.com)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4264,7 +4218,6 @@
           <t>C49656016 GR0402F261KTAG00 0.00 USD</t>
         </is>
       </c>
-      <c r="T46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4348,7 +4301,6 @@
           <t>C22369568 RCA0230KFLF 0.00 USD</t>
         </is>
       </c>
-      <c r="T47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4432,7 +4384,6 @@
           <t>C122548 0402WGF3322TCE 0.00 USD</t>
         </is>
       </c>
-      <c r="T48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4516,7 +4467,6 @@
           <t>C22369456 RCA024K7FLF 0.01 USD</t>
         </is>
       </c>
-      <c r="T49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4600,7 +4550,6 @@
           <t>C49654486 GR0402F46K4TAG00 0.00 USD</t>
         </is>
       </c>
-      <c r="T50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4631,17 +4580,17 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>C22369457</t>
+          <t>C103079</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>RCA025K1FLF</t>
+          <t>RTT025101FTH</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>HKR(Hong Kong Resistors)</t>
+          <t>RALEC</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -4655,7 +4604,7 @@
         </is>
       </c>
       <c r="L51" t="n">
-        <v>1323626</v>
+        <v>19468</v>
       </c>
       <c r="M51" t="n">
         <v>1</v>
@@ -4664,27 +4613,26 @@
         <v>4</v>
       </c>
       <c r="O51" t="n">
-        <v>0.001</v>
+        <v>0.0012</v>
       </c>
       <c r="P51" t="n">
-        <v>0.004</v>
+        <v>0.0048</v>
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22369457.html</t>
+          <t>https://www.lcsc.com/product-detail/C103079.html</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
-        </is>
-      </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t>C103079 RTT025101FTH 0.00 USD</t>
-        </is>
-      </c>
-      <c r="T51" t="inlineStr"/>
+          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>LCSC-orderable substitute for C22369457 RCA025K1FLF (not sold / no stock on lcsc.com)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4768,7 +4716,6 @@
           <t>C5126239 FRC0402F5113TS 0.01 USD</t>
         </is>
       </c>
-      <c r="T52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4852,7 +4799,6 @@
           <t>C22369327 RCA0291KFLF 0.00 USD</t>
         </is>
       </c>
-      <c r="T53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4931,7 +4877,6 @@
           <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
         </is>
       </c>
-      <c r="S54" t="inlineStr"/>
       <c r="T54" t="inlineStr">
         <is>
           <t>LOW STOCK 387, no candidate with &gt;= 1000</t>
@@ -4965,9 +4910,6 @@
           <t>TESTP</t>
         </is>
       </c>
-      <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr">
         <is>
           <t>no purchased part (pad / test point / antenna)</t>
@@ -5051,7 +4993,6 @@
           <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
         </is>
       </c>
-      <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr">
         <is>
           <t>LOW STOCK 36, no candidate with &gt;= 1000</t>
@@ -5140,7 +5081,6 @@
           <t>C5337088 TYPE-C-31-M-12A 0.46 USD</t>
         </is>
       </c>
-      <c r="T57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5219,8 +5159,6 @@
           <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
         </is>
       </c>
-      <c r="S58" t="inlineStr"/>
-      <c r="T58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5299,8 +5237,6 @@
           <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
         </is>
       </c>
-      <c r="S59" t="inlineStr"/>
-      <c r="T59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5384,7 +5320,6 @@
           <t>C17626844 W25N02KVZEIR TR 11.16 USD</t>
         </is>
       </c>
-      <c r="T60" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">

</xml_diff>

<commit_message>
Use JLCPCB Basic parts where they meet the spec (26 lines); full Basic parts list added
JLCPCB_BASIC_PARTS.txt: all 351 Basic parts from the parts API (no loading fee).
Switched: 18 passive lines (exact value/package/voltage/tolerance match),
FB1-3 -> BLM18PG121SN1D, Q1 -> AO3401A, Q2/Q4 -> AO3400A, Y1/Y3 -> Q13FC13500004.
Value changes: R25 33.2k -> 33k (0V8 rail -1 mV), R21 46.4k -> 47k (charge
timer 6.2 -> 6.3 h). Schematic Description = new C-number, Comment updated
where the MPN or value changed; all order lists follow.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -744,17 +744,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>C20624294</t>
+          <t>C28323</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0805B105K100NT</t>
+          <t>CL21B105KBFNNNE</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>FH (Guangdong Fenghua Advanced Tech)</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -764,11 +764,11 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>2687</v>
+        <v>3278922</v>
       </c>
       <c r="M4" t="n">
         <v>1</v>
@@ -777,19 +777,19 @@
         <v>2</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0243</v>
+        <v>0.0384</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0486</v>
+        <v>0.07679999999999999</v>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C20624294.html</t>
+          <t>https://www.lcsc.com/product-detail/C28323.html</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>10V 1uF X7R ±10% 0805 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>1uF 50V X7R ±10% 0805 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>no voltage rating in schematic, assumed 10V</t>
+          <t>Basic part; no voltage rating in schematic, assumed 10V</t>
         </is>
       </c>
     </row>
@@ -915,17 +915,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>C513772</t>
+          <t>C307331</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CS1005X7R104K500NR</t>
+          <t>CL05B104KB54PNC</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Samwha Capacitor</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -935,11 +935,11 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>116403</v>
+        <v>17690101</v>
       </c>
       <c r="M6" t="n">
         <v>1</v>
@@ -948,24 +948,24 @@
         <v>12</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0032</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="P6" t="n">
-        <v>0.0384</v>
+        <v>0.102</v>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C513772.html</t>
+          <t>https://www.lcsc.com/product-detail/C307331.html</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>100nF 50V ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>100nF 50V X7R ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>LCSC-orderable substitute for C3012377 CSA0402X7R104K500GT (not sold / no stock on lcsc.com)</t>
+          <t>Basic part; LCSC-orderable substitute for C3012377 CSA0402X7R104K500GT (not sold / no stock on lcsc.com)</t>
         </is>
       </c>
     </row>
@@ -1081,17 +1081,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>C106201</t>
+          <t>C1547</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>CC0402JRNPO9BN120</t>
+          <t>0402CG120J500NT</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1101,11 +1101,11 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>3509224</v>
+        <v>1591176</v>
       </c>
       <c r="M8" t="n">
         <v>1</v>
@@ -1114,24 +1114,29 @@
         <v>2</v>
       </c>
       <c r="O8" t="n">
-        <v>0.002</v>
+        <v>0.0055</v>
       </c>
       <c r="P8" t="n">
-        <v>0.004</v>
+        <v>0.011</v>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C106201.html</t>
+          <t>https://www.lcsc.com/product-detail/C1547.html</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>12pF 50V NP0 ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>12pF 50V C0G ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
           <t>C7467122 FCC0402N120J500AT 0.01 USD</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -1164,17 +1169,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>C107000</t>
+          <t>C1554</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>CC0402JRNPO9BN200</t>
+          <t>0402CG200J500NT</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1184,11 +1189,11 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L9" t="n">
-        <v>3263279</v>
+        <v>868282</v>
       </c>
       <c r="M9" t="n">
         <v>1</v>
@@ -1197,24 +1202,29 @@
         <v>5</v>
       </c>
       <c r="O9" t="n">
-        <v>0.0021</v>
+        <v>0.007</v>
       </c>
       <c r="P9" t="n">
-        <v>0.0105</v>
+        <v>0.035</v>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C107000.html</t>
+          <t>https://www.lcsc.com/product-detail/C1554.html</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>20pF 50V NP0 ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>20pF 50V C0G ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
           <t>C5137579 FCC0402N200J500AT 0.01 USD</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -1431,32 +1441,32 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>Q13FC13500004</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>FP-ABS07-MFG</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>ABS07-32.768KHZ-T</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>FP-ABS07-MFG</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>ABS07-32.768KHZ-T</t>
-        </is>
-      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>C130253</t>
+          <t>C32346</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>ABS07-32.768KHZ-T</t>
+          <t>Q13FC13500004</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Abracon LLC</t>
+          <t>Seiko Epson</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1466,11 +1476,11 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L13" t="n">
-        <v>11651</v>
+        <v>627364</v>
       </c>
       <c r="M13" t="n">
         <v>1</v>
@@ -1479,14 +1489,14 @@
         <v>2</v>
       </c>
       <c r="O13" t="n">
-        <v>0.7086</v>
+        <v>0.1655</v>
       </c>
       <c r="P13" t="n">
-        <v>1.4172</v>
+        <v>0.331</v>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C130253.html</t>
+          <t>https://www.lcsc.com/product-detail/C32346.html</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1496,7 +1506,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>generic 3215 12.5pF alternative: C22386770 SXTF321532768A20F ~0.13 USD</t>
+          <t>Basic part; generic 3215 12.5pF alternative: C22386770 SXTF321532768A20F ~0.13 USD</t>
         </is>
       </c>
     </row>
@@ -1597,27 +1607,27 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>BLM18PG121SN1D</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>FP-BLM18-0_15-t0_8-IPC_B</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>BLM18AG121SN1D</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>FP-BLM18-0_15-t0_8-IPC_B</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>BLM18AG121SN1D</t>
-        </is>
-      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>C76892</t>
+          <t>C14709</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>BLM18AG121SN1D</t>
+          <t>BLM18PG121SN1D</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1632,11 +1642,11 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L15" t="n">
-        <v>249561</v>
+        <v>2646830</v>
       </c>
       <c r="M15" t="n">
         <v>1</v>
@@ -1645,19 +1655,24 @@
         <v>3</v>
       </c>
       <c r="O15" t="n">
-        <v>0.0121</v>
+        <v>0.0151</v>
       </c>
       <c r="P15" t="n">
-        <v>0.0363</v>
+        <v>0.0453</v>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C76892.html</t>
+          <t>https://www.lcsc.com/product-detail/C14709.html</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 1 120Ω@100MHz 180mΩ 800mA ±25% 0603 Ferrite Beads ROHS</t>
+          <t>-55℃~+125℃ 1 120Ω@100MHz 2A 50mΩ ±25% 0603 Ferrite Beads ROHS</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -2002,17 +2017,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>C5137565</t>
+          <t>C19702</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>FCC0603X106K100CT</t>
+          <t>CL10A106KP8NNNC</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>FOJAN</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -2022,11 +2037,11 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L20" t="n">
-        <v>619349</v>
+        <v>13165696</v>
       </c>
       <c r="M20" t="n">
         <v>1</v>
@@ -2035,14 +2050,14 @@
         <v>13</v>
       </c>
       <c r="O20" t="n">
-        <v>0.0209</v>
+        <v>0.0308</v>
       </c>
       <c r="P20" t="n">
-        <v>0.2717</v>
+        <v>0.4004</v>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C5137565.html</t>
+          <t>https://www.lcsc.com/product-detail/C19702.html</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2053,6 +2068,11 @@
       <c r="S20" t="inlineStr">
         <is>
           <t>C6119842 CGA0603X5R106K100JT 0.29 USD</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -2085,17 +2105,17 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>C20070307</t>
+          <t>C15849</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CGA0603X5R105K100JT</t>
+          <t>CL10A105KB8NNNC</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2105,11 +2125,11 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>88309</v>
+        <v>7674757</v>
       </c>
       <c r="M21" t="n">
         <v>1</v>
@@ -2118,24 +2138,29 @@
         <v>1</v>
       </c>
       <c r="O21" t="n">
-        <v>0.0074</v>
+        <v>0.0165</v>
       </c>
       <c r="P21" t="n">
-        <v>0.0074</v>
+        <v>0.0165</v>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C20070307.html</t>
+          <t>https://www.lcsc.com/product-detail/C15849.html</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>10V 1uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>1uF 50V X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
           <t>C111590 0603X105K100NT 0.01 USD</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -2168,17 +2193,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>C6119880</t>
+          <t>C59461</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>CGA0603X5R226M6R3JT</t>
+          <t>CL10A226MQ8NRNC</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2188,11 +2213,11 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L22" t="n">
-        <v>84069</v>
+        <v>9805302</v>
       </c>
       <c r="M22" t="n">
         <v>1</v>
@@ -2201,14 +2226,14 @@
         <v>6</v>
       </c>
       <c r="O22" t="n">
-        <v>0.0248</v>
+        <v>0.03</v>
       </c>
       <c r="P22" t="n">
-        <v>0.1488</v>
+        <v>0.18</v>
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C6119880.html</t>
+          <t>https://www.lcsc.com/product-detail/C59461.html</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2219,6 +2244,11 @@
       <c r="S22" t="inlineStr">
         <is>
           <t>C59461 CL10A226MQ8NRNC 0.18 USD</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -2485,32 +2515,32 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
+          <t>AO3401A</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>FP-SOT23-IPC_B</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>DMG2301LK-7</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>FP-SOT23-IPC_B</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>DMG2301LK-7</t>
-        </is>
-      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>C53283193</t>
+          <t>C15127</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>DMG2301L-GK</t>
+          <t>AO3401A</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>GOODWORK</t>
+          <t>Alpha &amp; Omega Semicon</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2520,11 +2550,11 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L26" t="n">
-        <v>1580</v>
+        <v>495550</v>
       </c>
       <c r="M26" t="n">
         <v>1</v>
@@ -2533,24 +2563,29 @@
         <v>1</v>
       </c>
       <c r="O26" t="n">
-        <v>0.0275</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="P26" t="n">
-        <v>0.0275</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C53283193.html</t>
+          <t>https://www.lcsc.com/product-detail/C15127.html</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>-55℃~+150℃ 1 P-Channel 1.2W 1V 20V 3A 405pF 5.5nC@4.5V 55pF 70mΩ@4.5V 75pF SOT-23 MOSFETs ROHS</t>
+          <t>1 P-Channel 14nC@10V 30V 47mΩ@10V、60mΩ@4.5V、85mΩ@2.5V 4A 55pF 645pF 80pF 900mV SOT-23 MOSFETs ROHS</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
           <t>C53199108 DMG2301L-7(ES) 0.03 USD</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -2568,32 +2603,32 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
+          <t>AO3400A</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>FP-SOT23-MFG</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>DMG2302UK-7</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>FP-SOT23-MFG</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>DMG2302UK-7</t>
-        </is>
-      </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>C53283194</t>
+          <t>C20917</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>DMG2302UK-GK</t>
+          <t>AO3400A</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>GOODWORK</t>
+          <t>Alpha &amp; Omega Semicon</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2603,11 +2638,11 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L27" t="n">
-        <v>5850</v>
+        <v>821792</v>
       </c>
       <c r="M27" t="n">
         <v>1</v>
@@ -2616,19 +2651,19 @@
         <v>2</v>
       </c>
       <c r="O27" t="n">
-        <v>0.0157</v>
+        <v>0.0815</v>
       </c>
       <c r="P27" t="n">
-        <v>0.0314</v>
+        <v>0.163</v>
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C53283194.html</t>
+          <t>https://www.lcsc.com/product-detail/C20917.html</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>-55℃~+150℃ 1 N-channel 1.2W 1V 2.3A 200pF 20V 28pF 35pF 3nC@4.5V 45mΩ@4.5V SOT-23 MOSFETs ROHS</t>
+          <t>-55℃~+150℃ 1 N-channel 1.45V 1.4W 30V 48mΩ@2.5V 5.7A 50pF 630pF 75pF 7nC@10V N-Channel SOT-23 MOSFETs ROHS</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -2638,7 +2673,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>clone brands accepted; Diodes original is C460977</t>
+          <t>Basic part; clone brands accepted; Diodes original is C460977</t>
         </is>
       </c>
     </row>
@@ -2754,17 +2789,17 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>C54920843</t>
+          <t>C22859</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>HRC0603F10R0ENTN</t>
+          <t>0603WAF100JT5E</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2774,11 +2809,11 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L29" t="n">
-        <v>22157</v>
+        <v>8772359</v>
       </c>
       <c r="M29" t="n">
         <v>1</v>
@@ -2787,24 +2822,29 @@
         <v>1</v>
       </c>
       <c r="O29" t="n">
-        <v>0.0011</v>
+        <v>0.0036</v>
       </c>
       <c r="P29" t="n">
-        <v>0.0011</v>
+        <v>0.0036</v>
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920843.html</t>
+          <t>https://www.lcsc.com/product-detail/C22859.html</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 10Ω 50V Thick Film Resistor ±1% ±200ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
           <t>C49652997 GR0603F10RT5G00 0.00 USD</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -3418,17 +3458,17 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>C54920638</t>
+          <t>C25867</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>HRC0402F1501DNTO</t>
+          <t>0402WGF1501TCE</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -3438,11 +3478,11 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L37" t="n">
-        <v>313030</v>
+        <v>2485240</v>
       </c>
       <c r="M37" t="n">
         <v>1</v>
@@ -3451,14 +3491,14 @@
         <v>1</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0007</v>
+        <v>0.0028</v>
       </c>
       <c r="P37" t="n">
-        <v>0.0007</v>
+        <v>0.0028</v>
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920638.html</t>
+          <t>https://www.lcsc.com/product-detail/C25867.html</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3469,6 +3509,11 @@
       <c r="S37" t="inlineStr">
         <is>
           <t>C22369462 RCA021K5FLF 0.00 USD</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -3501,17 +3546,17 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>C49652939</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>GR0402F100KTAG00</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -3521,11 +3566,11 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L38" t="n">
-        <v>6594</v>
+        <v>11296591</v>
       </c>
       <c r="M38" t="n">
         <v>1</v>
@@ -3534,14 +3579,14 @@
         <v>20</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0008</v>
+        <v>0.0024</v>
       </c>
       <c r="P38" t="n">
-        <v>0.016</v>
+        <v>0.048</v>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49652939.html</t>
+          <t>https://www.lcsc.com/product-detail/C25741.html</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3552,6 +3597,11 @@
       <c r="S38" t="inlineStr">
         <is>
           <t>C22369473 RCA02100KFLF 0.02 USD</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -3584,17 +3634,17 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>C1858459</t>
+          <t>C25744</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>RC0402FR-1310KL</t>
+          <t>0402WGF1002TCE</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3604,11 +3654,11 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L39" t="n">
-        <v>49403</v>
+        <v>27833513</v>
       </c>
       <c r="M39" t="n">
         <v>1</v>
@@ -3617,14 +3667,14 @@
         <v>18</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0018</v>
+        <v>0.003</v>
       </c>
       <c r="P39" t="n">
-        <v>0.0324</v>
+        <v>0.054</v>
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C1858459.html</t>
+          <t>https://www.lcsc.com/product-detail/C25744.html</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3634,7 +3684,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>LCSC-orderable substitute for C22369472 RCA0210KFLF (not sold / no stock on lcsc.com)</t>
+          <t>Basic part; LCSC-orderable substitute for C22369472 RCA0210KFLF (not sold / no stock on lcsc.com)</t>
         </is>
       </c>
     </row>
@@ -3833,17 +3883,17 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>C54920644</t>
+          <t>C25087</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>HRC0402F2000DNTO</t>
+          <t>0402WGF2000TCE</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -3853,11 +3903,11 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L42" t="n">
-        <v>1881170</v>
+        <v>2969246</v>
       </c>
       <c r="M42" t="n">
         <v>1</v>
@@ -3866,14 +3916,14 @@
         <v>2</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0007</v>
+        <v>0.0028</v>
       </c>
       <c r="P42" t="n">
-        <v>0.0014</v>
+        <v>0.0056</v>
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920644.html</t>
+          <t>https://www.lcsc.com/product-detail/C25087.html</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -3884,6 +3934,11 @@
       <c r="S42" t="inlineStr">
         <is>
           <t>C22356253 RCA02200RFLF 0.00 USD</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -3916,17 +3971,17 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>C102872</t>
+          <t>C25764</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>RTT022003FTH</t>
+          <t>0402WGF2003TCE</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>RALEC</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -3936,11 +3991,11 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L43" t="n">
-        <v>19832</v>
+        <v>2016817</v>
       </c>
       <c r="M43" t="n">
         <v>1</v>
@@ -3949,14 +4004,14 @@
         <v>1</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0012</v>
+        <v>0.0019</v>
       </c>
       <c r="P43" t="n">
-        <v>0.0012</v>
+        <v>0.0019</v>
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C102872.html</t>
+          <t>https://www.lcsc.com/product-detail/C25764.html</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -3966,7 +4021,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>LCSC-orderable substitute for C22369550 RCA02200KFLF (not sold / no stock on lcsc.com)</t>
+          <t>Basic part; LCSC-orderable substitute for C22369550 RCA02200KFLF (not sold / no stock on lcsc.com)</t>
         </is>
       </c>
     </row>
@@ -3999,17 +4054,17 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>C2929994</t>
+          <t>C25092</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>FRC0402F22R0TS</t>
+          <t>0402WGF220JTCE</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>FOJAN</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -4019,11 +4074,11 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L44" t="n">
-        <v>921743</v>
+        <v>6486917</v>
       </c>
       <c r="M44" t="n">
         <v>1</v>
@@ -4032,14 +4087,14 @@
         <v>1</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0019</v>
+        <v>0.0028</v>
       </c>
       <c r="P44" t="n">
-        <v>0.0019</v>
+        <v>0.0028</v>
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2929994.html</t>
+          <t>https://www.lcsc.com/product-detail/C25092.html</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4050,6 +4105,11 @@
       <c r="S44" t="inlineStr">
         <is>
           <t>C2759796 CQ02WGF220JTCE 0.00 USD</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -4316,32 +4376,32 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
+          <t>33k</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>RES_0402</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
           <t>33.2k</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>RES_0402</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>33.2k</t>
-        </is>
-      </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>C53069467</t>
+          <t>C25779</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>CL0402FN33K2P</t>
+          <t>0402WGF3302TCE</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>CHANGLONG</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -4351,11 +4411,11 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L48" t="n">
-        <v>2978</v>
+        <v>1404931</v>
       </c>
       <c r="M48" t="n">
         <v>1</v>
@@ -4364,24 +4424,29 @@
         <v>1</v>
       </c>
       <c r="O48" t="n">
-        <v>0.0007</v>
+        <v>0.0089</v>
       </c>
       <c r="P48" t="n">
-        <v>0.0007</v>
+        <v>0.0089</v>
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C53069467.html</t>
+          <t>https://www.lcsc.com/product-detail/C25779.html</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 33.2kΩ 50V 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
           <t>C122548 0402WGF3322TCE 0.00 USD</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -4414,17 +4479,17 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>C49652824</t>
+          <t>C25900</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>GR0402F4K7TAG00</t>
+          <t>0402WGF4701TCE</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -4434,11 +4499,11 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L49" t="n">
-        <v>10830</v>
+        <v>17899557</v>
       </c>
       <c r="M49" t="n">
         <v>1</v>
@@ -4447,14 +4512,14 @@
         <v>6</v>
       </c>
       <c r="O49" t="n">
-        <v>0.0008</v>
+        <v>0.0028</v>
       </c>
       <c r="P49" t="n">
-        <v>0.0048</v>
+        <v>0.0168</v>
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49652824.html</t>
+          <t>https://www.lcsc.com/product-detail/C25900.html</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4465,6 +4530,11 @@
       <c r="S49" t="inlineStr">
         <is>
           <t>C22369456 RCA024K7FLF 0.01 USD</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -4482,32 +4552,32 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
+          <t>47k</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>RES_0402</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
           <t>46.4k</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>RES_0402</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>46.4k</t>
-        </is>
-      </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>C103052</t>
+          <t>C25792</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>RTT024642FTH</t>
+          <t>0402WGF4702TCE</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>RALEC</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -4517,11 +4587,11 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L50" t="n">
-        <v>7120</v>
+        <v>6019599</v>
       </c>
       <c r="M50" t="n">
         <v>1</v>
@@ -4530,24 +4600,29 @@
         <v>1</v>
       </c>
       <c r="O50" t="n">
-        <v>0.0007</v>
+        <v>0.0026</v>
       </c>
       <c r="P50" t="n">
-        <v>0.0007</v>
+        <v>0.0026</v>
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C103052.html</t>
+          <t>https://www.lcsc.com/product-detail/C25792.html</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 46.4kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
           <t>C49654486 GR0402F46K4TAG00 0.00 USD</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Basic part; </t>
         </is>
       </c>
     </row>
@@ -4580,17 +4655,17 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>C103079</t>
+          <t>C25905</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>RTT025101FTH</t>
+          <t>0402WGF5101TCE</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>RALEC</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -4600,11 +4675,11 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L51" t="n">
-        <v>19468</v>
+        <v>7309528</v>
       </c>
       <c r="M51" t="n">
         <v>1</v>
@@ -4613,14 +4688,14 @@
         <v>4</v>
       </c>
       <c r="O51" t="n">
-        <v>0.0012</v>
+        <v>0.0024</v>
       </c>
       <c r="P51" t="n">
-        <v>0.0048</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C103079.html</t>
+          <t>https://www.lcsc.com/product-detail/C25905.html</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4630,7 +4705,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>LCSC-orderable substitute for C22369457 RCA025K1FLF (not sold / no stock on lcsc.com)</t>
+          <t>Basic part; LCSC-orderable substitute for C22369457 RCA025K1FLF (not sold / no stock on lcsc.com)</t>
         </is>
       </c>
     </row>
@@ -5321,6 +5396,7 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
220n COMP caps and Cff caps to Basic parts (C16772 16V X7R, C1546 100pF C0G)
TPS61160A datasheet: COMP = 220nF, pin below 3V so 16V is fine.
TPS62823 Cff = 12ms/R2 -> 120pF (0V8, R2=100k) and 100pF (1V1, R2=120k);
both now 100pF, within loop tolerance.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -983,32 +983,32 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>100pf</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>CAP_0402</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>120pf</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>CAP_0402</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>120pf</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>C2887023</t>
+          <t>C1546</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>TCC0402COG121J500AT</t>
+          <t>0402CG101J500NT</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>CCTC</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1018,11 +1018,11 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L7" t="n">
-        <v>54327</v>
+        <v>3959584</v>
       </c>
       <c r="M7" t="n">
         <v>1</v>
@@ -1031,24 +1031,24 @@
         <v>2</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0033</v>
+        <v>0.004</v>
       </c>
       <c r="P7" t="n">
-        <v>0.0066</v>
+        <v>0.008</v>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2887023.html</t>
+          <t>https://www.lcsc.com/product-detail/C1546.html</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>120pF 50V C0G ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>100pF 50V C0G ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>LCSC-orderable substitute for C7507400 C0402C0G121K500NTB (not sold / no stock on lcsc.com)</t>
+          <t>Basic part; Cff for TPS62823: 12ms/R2 gives 120pF (0V8) and 100pF (1V1); 100pF within loop tolerance</t>
         </is>
       </c>
     </row>
@@ -1257,17 +1257,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>C36911358</t>
+          <t>C16772</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>CGA0402X5R224K500GT</t>
+          <t>CL05B224KO5NNNC</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1277,11 +1277,11 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>69931</v>
+        <v>2986441</v>
       </c>
       <c r="M10" t="n">
         <v>1</v>
@@ -1290,24 +1290,29 @@
         <v>2</v>
       </c>
       <c r="O10" t="n">
-        <v>0.0065</v>
+        <v>0.0049</v>
       </c>
       <c r="P10" t="n">
-        <v>0.013</v>
+        <v>0.0098</v>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C36911358.html</t>
+          <t>https://www.lcsc.com/product-detail/C16772.html</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>220nF 50V X5R ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>16V 220nF X7R ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
           <t>C5159775 GRM155R61H224KE01D 0.04 USD</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Basic part; 16V part; COMP pin of TPS61160A sits below 3V</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
D1 charge LED -> Basic red 0603 KT-0603R (C2286); footprint 0402 -> 0603 to be changed in the library
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -2354,46 +2354,46 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
+          <t>KT-0603R</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>FP-SM0402GC-MFG</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>YLED0402B</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>FP-SM0402GC-MFG</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>YLED0402B</t>
-        </is>
-      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>C25503856</t>
+          <t>C2286</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>XL-1005UYC</t>
+          <t>KT-0603R</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>XINGLIGHT</t>
+          <t>Hubei KENTO Elec</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="L24" t="n">
-        <v>87063</v>
+        <v>3623693</v>
       </c>
       <c r="M24" t="n">
         <v>1</v>
@@ -2402,24 +2402,24 @@
         <v>1</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0127</v>
+        <v>0.0072</v>
       </c>
       <c r="P24" t="n">
-        <v>0.0127</v>
+        <v>0.0072</v>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25503856.html</t>
+          <t>https://www.lcsc.com/product-detail/C2286.html</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 120° 1mm x 0.5mm square LED 2.4V 20mA 210mcd 50mW 585nm~595nm 590nm Discrete Diode Water Clear Yellow 0402 LED</t>
+          <t>-40℃~+85℃ 1.6mm x 0.8mm square LED 1.8V~2.4V 120° 20mA 300mcd 40mW 615nm~630nm 645nm Discrete Diode Red Water Clear 0603</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>yellow 0402 LED 590nm, replaces generic YLED0402B</t>
+          <t>Basic part; red 0603 LED, footprint change 0402 -&gt; 0603 needed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "D1 charge LED -> Basic red 0603 KT-0603R (C2286); footprint 0402 -> 0603 to be changed in the library"
This reverts commit ce13db8fbb8fb8dcc5b02b97936a9742eb360d52.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -2354,7 +2354,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>KT-0603R</t>
+          <t>YLED0402B</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2369,31 +2369,31 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>C2286</t>
+          <t>C25503856</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>KT-0603R</t>
+          <t>XL-1005UYC</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Hubei KENTO Elec</t>
+          <t>XINGLIGHT</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="L24" t="n">
-        <v>3623693</v>
+        <v>87063</v>
       </c>
       <c r="M24" t="n">
         <v>1</v>
@@ -2402,24 +2402,24 @@
         <v>1</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0072</v>
+        <v>0.0127</v>
       </c>
       <c r="P24" t="n">
-        <v>0.0072</v>
+        <v>0.0127</v>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2286.html</t>
+          <t>https://www.lcsc.com/product-detail/C25503856.html</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1.6mm x 0.8mm square LED 1.8V~2.4V 120° 20mA 300mcd 40mW 615nm~630nm 645nm Discrete Diode Red Water Clear 0603</t>
+          <t>-40℃~+85℃ 120° 1mm x 0.5mm square LED 2.4V 20mA 210mcd 50mW 585nm~595nm 590nm Discrete Diode Water Clear Yellow 0402 LED</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Basic part; red 0603 LED, footprint change 0402 -&gt; 0603 needed</t>
+          <t>yellow 0402 LED 590nm, replaces generic YLED0402B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply the resistor/Basic changes announced in 6e6a6a1 (map generation had failed); 120k has no Basic part and stays Extended
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3274287</v>
+        <v>3274112</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>17662265</v>
+        <v>17663114</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3956541</v>
+        <v>3956681</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1578926</v>
+        <v>1578706</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>858315</v>
+        <v>858285</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>627112</v>
+        <v>627252</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2638307</v>
+        <v>2637817</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>13150509</v>
+        <v>13129771</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>7676092</v>
+        <v>7677530</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>9809696</v>
+        <v>9809655</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -1999,116 +1999,116 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>D2 D7 D8</t>
+          <t>FB4</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DSK24</t>
+          <t>GZ1608D601TF</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FP-S8-V-3910_01-001-MFG</t>
+          <t>FP-MMZ0603-MFG</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>C2939005</t>
+          <t>C1002</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>DSK24 K24</t>
+          <t>GZ1608D601TF</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>KUU</t>
+          <t>Sunlord</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>SOD-123FL</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K22" t="n">
-        <v>120296</v>
+        <v>978645</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N22" t="n">
-        <v>0.0187</v>
+        <v>0.019</v>
       </c>
       <c r="O22" t="n">
-        <v>0.0561</v>
+        <v>0.019</v>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2939005.html</t>
+          <t>https://www.lcsc.com/product-detail/C1002.html</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>2A 40A 40V 500uA@40V 550mV@2A Independent SOD-123FL Schottky Diodes ROHS</t>
+          <t>-55℃~+125℃ 1 200mA 450mΩ 600Ω@100MHz ±25% 0603 Ferrite Beads ROHS</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PR1</t>
+          <t>D2 D7 D8</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SM05B-NSHSS-TB(LF)(SN)</t>
+          <t>DSK24</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FP-SM05B-NSHSS-TB_LF_SN-MFG</t>
+          <t>FP-S8-V-3910_01-001-MFG</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>C268096</t>
+          <t>C2939005</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SM05B-NSHSS-TB(LF)(SN)</t>
+          <t>DSK24 K24</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>KUU</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>SMD,P=1mm,Surface Mount，Right Angle</t>
+          <t>SOD-123FL</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2117,35 +2117,35 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>1984</v>
+        <v>120296</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N23" t="n">
-        <v>0.4749</v>
+        <v>0.0187</v>
       </c>
       <c r="O23" t="n">
-        <v>0.4749</v>
+        <v>0.0561</v>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C268096.html</t>
+          <t>https://www.lcsc.com/product-detail/C2939005.html</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 1A 1mm 1x5P 4.4mm 5 50V 5P 6.8mm 7mm Auxiliary Solder Pin Copper alloy NSH PA Surface Mount, Right Angle Tin</t>
+          <t>2A 40A 40V 500uA@40V 550mV@2A Independent SOD-123FL Schottky Diodes ROHS</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>PR1</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2156,41 +2156,41 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AO3401A</t>
+          <t>SM05B-NSHSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>FP-SOT23-IPC_B</t>
+          <t>FP-SM05B-NSHSS-TB_LF_SN-MFG</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>C15127</t>
+          <t>C268096</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>AO3401A</t>
+          <t>SM05B-NSHSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Alpha &amp; Omega Semicon</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>SMD,P=1mm,Surface Mount，Right Angle</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K24" t="n">
-        <v>493960</v>
+        <v>1984</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2199,62 +2199,62 @@
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.4749</v>
       </c>
       <c r="O24" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.4749</v>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C15127.html</t>
+          <t>https://www.lcsc.com/product-detail/C268096.html</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>1 P-Channel 14nC@10V 30V 47mΩ@10V、60mΩ@4.5V、85mΩ@2.5V 4A 55pF 645pF 80pF 900mV SOT-23 MOSFETs ROHS</t>
+          <t>-25℃~+85℃ 1 1A 1mm 1x5P 4.4mm 5 50V 5P 6.8mm 7mm Auxiliary Solder Pin Copper alloy NSH PA Surface Mount, Right Angle Tin</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Q2 Q4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AO3400A</t>
+          <t>KT-0603R</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>FP-SOT23-MFG</t>
+          <t>FP-SML-LX0603IW-TR-MFG</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>C20917</t>
+          <t>C2286</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>AO3400A</t>
+          <t>KT-0603R</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Alpha &amp; Omega Semicon</t>
+          <t>Hubei KENTO Elec</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2263,144 +2263,144 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>816975</v>
+        <v>3620363</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>0.0815</v>
+        <v>0.0072</v>
       </c>
       <c r="O25" t="n">
-        <v>0.163</v>
+        <v>0.0072</v>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C20917.html</t>
+          <t>https://www.lcsc.com/product-detail/C2286.html</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>-55℃~+150℃ 1 N-channel 1.45V 1.4W 30V 48mΩ@2.5V 5.7A 50pF 630pF 75pF 7nC@10V N-Channel SOT-23 MOSFETs ROHS</t>
+          <t>-40℃~+85℃ 1.6mm x 0.8mm square LED 1.8V~2.4V 120° 20mA 300mcd 40mW 615nm~630nm 645nm Discrete Diode Red Water Clear 0603</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>D3 D4 D5</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>PRTR5V0U2F,115</t>
+          <t>AO3401A</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>FP-SOT886-MFG</t>
+          <t>FP-SOT23-IPC_B</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>C478118</t>
+          <t>C15127</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>PRTR5V0U2F,115</t>
+          <t>AO3401A</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Nexperia</t>
+          <t>Alpha &amp; Omega Semicon</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>XSON-6(1x1.5)</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K26" t="n">
-        <v>60131</v>
+        <v>494064</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N26" t="n">
-        <v>0.103</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="O26" t="n">
-        <v>0.309</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C478118.html</t>
+          <t>https://www.lcsc.com/product-detail/C15127.html</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 100nA 1pF 2 5.5V 6V IEC 61000-4-2 TVS Unidirectional XSON-6(1x1.5) ESD and Surge Protection (TVS/ESD) ROHS</t>
+          <t>1 P-Channel 14nC@10V 30V 47mΩ@10V、60mΩ@4.5V、85mΩ@2.5V 4A 55pF 645pF 80pF 900mV SOT-23 MOSFETs ROHS</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>R68</t>
+          <t>Q2 Q4</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10R</t>
+          <t>AO3400A</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>FP-SR0603-MFG</t>
+          <t>FP-SOT23-MFG</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C22859</t>
+          <t>C20917</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0603WAF100JT5E</t>
+          <t>AO3400A</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>Alpha &amp; Omega Semicon</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2409,71 +2409,71 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>8743606</v>
+        <v>816954</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N27" t="n">
-        <v>0.0036</v>
+        <v>0.0815</v>
       </c>
       <c r="O27" t="n">
-        <v>0.0036</v>
+        <v>0.163</v>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22859.html</t>
+          <t>https://www.lcsc.com/product-detail/C20917.html</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+150℃ 1 N-channel 1.45V 1.4W 30V 48mΩ@2.5V 5.7A 50pF 630pF 75pF 7nC@10V N-Channel SOT-23 MOSFETs ROHS</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>R66</t>
+          <t>D3 D4 D5</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>4R</t>
+          <t>PRTR5V0U2F,115</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FP-SR0603-MFG</t>
+          <t>FP-SOT886-MFG</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C49654665</t>
+          <t>C478118</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>GR0603F4R02T5G00</t>
+          <t>PRTR5V0U2F,115</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>Nexperia</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>XSON-6(1x1.5)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2482,35 +2482,35 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>1299</v>
+        <v>60131</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N28" t="n">
-        <v>0.0023</v>
+        <v>0.103</v>
       </c>
       <c r="O28" t="n">
-        <v>0.0023</v>
+        <v>0.309</v>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49654665.html</t>
+          <t>https://www.lcsc.com/product-detail/C478118.html</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 4.02Ω 75V Thick Film Resistor ±1% 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-40℃~+85℃ 100nA 1pF 2 5.5V 6V IEC 61000-4-2 TVS Unidirectional XSON-6(1x1.5) ESD and Surge Protection (TVS/ESD) ROHS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Y2</t>
+          <t>R68</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2521,41 +2521,41 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>10R</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>FP-XRCGB_F_N-MFG</t>
+          <t>FP-SR0603-MFG</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C2965580</t>
+          <t>C22859</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>0603WAF100JT5E</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>YXC Crystal Oscillators</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>SMD2016-4P</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K29" t="n">
-        <v>4425</v>
+        <v>8743973</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2564,99 +2564,99 @@
         <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>0.0784</v>
+        <v>0.0036</v>
       </c>
       <c r="O29" t="n">
-        <v>0.0784</v>
+        <v>0.0036</v>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
+          <t>https://www.lcsc.com/product-detail/C22859.html</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
+          <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>S1 S2 S3</t>
+          <t>R66</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S(LF)(SN)</t>
+          <t>4.7R</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>JST-S2B-PH-K-S_V</t>
+          <t>FP-SR0603-MFG</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C157932</t>
+          <t>C23164</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S-GW</t>
+          <t>0603WAF470KT5E</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Push-Pull,P=2mm</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K30" t="n">
-        <v>15851</v>
+        <v>855576</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N30" t="n">
-        <v>0.2125</v>
+        <v>0.0027</v>
       </c>
       <c r="O30" t="n">
-        <v>0.6375</v>
+        <v>0.0027</v>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C157932.html</t>
+          <t>https://www.lcsc.com/product-detail/C23164.html</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
+          <t>-55℃~+155℃ 100mW 4.7Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -2667,32 +2667,32 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>k230d</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>FP-XRCGB_F_N-MFG</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C42414902</t>
+          <t>C2965580</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Canaan</t>
+          <t>YXC Crystal Oscillators</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BGA-256</t>
+          <t>SMD2016-4P</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>361</v>
+        <v>4425</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
@@ -2710,62 +2710,62 @@
         <v>1</v>
       </c>
       <c r="N31" t="n">
-        <v>13.3007</v>
+        <v>0.0784</v>
       </c>
       <c r="O31" t="n">
-        <v>13.3007</v>
+        <v>0.0784</v>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
+          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
+          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>S1 S2 S3</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1.1k (1.5A)</t>
+          <t>S2B-PH-K-S(LF)(SN)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>RES_0402</t>
+          <t>JST-S2B-PH-K-S_V</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C54920634</t>
+          <t>C157932</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>HRC0402F1101DNTO</t>
+          <t>S2B-PH-K-S-GW</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>Push-Pull,P=2mm</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2774,35 +2774,35 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>16860</v>
+        <v>15851</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N32" t="n">
-        <v>0.0007</v>
+        <v>0.2125</v>
       </c>
       <c r="O32" t="n">
-        <v>0.0007</v>
+        <v>0.6375</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920634.html</t>
+          <t>https://www.lcsc.com/product-detail/C157932.html</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -2813,41 +2813,41 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>k230d</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>RES_0402</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C25867</t>
+          <t>C42414902</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0402WGF1501TCE</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>Canaan</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>BGA-256</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2483159</v>
+        <v>361</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2856,37 +2856,37 @@
         <v>1</v>
       </c>
       <c r="N33" t="n">
-        <v>0.0028</v>
+        <v>13.3007</v>
       </c>
       <c r="O33" t="n">
-        <v>0.0028</v>
+        <v>13.3007</v>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25867.html</t>
+          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R6 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R69 R76</t>
+          <t>R5 R12</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2896,12 +2896,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C25867</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>0402WGF1003TCE</t>
+          <t>0402WGF1501TCE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2920,46 +2920,46 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>11303132</v>
+        <v>2483299</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="N34" t="n">
-        <v>0.0024</v>
+        <v>0.0028</v>
       </c>
       <c r="O34" t="n">
-        <v>0.048</v>
+        <v>0.0056</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25741.html</t>
+          <t>https://www.lcsc.com/product-detail/C25867.html</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
+          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C35" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2969,12 +2969,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C25744</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0402WGF1002TCE</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2993,46 +2993,46 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>27813160</v>
+        <v>11302366</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="N35" t="n">
-        <v>0.003</v>
+        <v>0.0024</v>
       </c>
       <c r="O35" t="n">
-        <v>0.054</v>
+        <v>0.048</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25744.html</t>
+          <t>https://www.lcsc.com/product-detail/C25741.html</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>120k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3042,17 +3042,17 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C54920620</t>
+          <t>C25744</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>HRC0402F1203DNTO</t>
+          <t>0402WGF1002TCE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3062,39 +3062,39 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K36" t="n">
-        <v>1181872</v>
+        <v>27810802</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="N36" t="n">
-        <v>0.0007</v>
+        <v>0.003</v>
       </c>
       <c r="O36" t="n">
-        <v>0.0007</v>
+        <v>0.054</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920620.html</t>
+          <t>https://www.lcsc.com/product-detail/C25744.html</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>150k</t>
+          <t>120k</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3115,12 +3115,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C54920625</t>
+          <t>C54920620</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>HRC0402F1503DNTO</t>
+          <t>HRC0402F1203DNTO</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>18510</v>
+        <v>1181872</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3155,19 +3155,19 @@
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920625.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920620.html</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 150kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R37 R62</t>
+          <t>R71 R72</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>200R</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3188,12 +3188,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C25087</t>
+          <t>C26083</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0402WGF2000TCE</t>
+          <t>0402WGF1004TCE</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2967919</v>
+        <v>2698020</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3221,26 +3221,26 @@
         <v>2</v>
       </c>
       <c r="N38" t="n">
-        <v>0.0028</v>
+        <v>0.0023</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0056</v>
+        <v>0.0046</v>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25087.html</t>
+          <t>https://www.lcsc.com/product-detail/C26083.html</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R59</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>200k</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C25764</t>
+          <t>C11702</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0402WGF2003TCE</t>
+          <t>0402WGF1001TCE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2025935</v>
+        <v>11756377</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3294,37 +3294,37 @@
         <v>1</v>
       </c>
       <c r="N39" t="n">
-        <v>0.0019</v>
+        <v>0.0021</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0019</v>
+        <v>0.0021</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25764.html</t>
+          <t>https://www.lcsc.com/product-detail/C11702.html</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>R42</t>
+          <t>R37 R62</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>22R</t>
+          <t>200R</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3334,12 +3334,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>C25092</t>
+          <t>C25087</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>0402WGF220JTCE</t>
+          <t>0402WGF2000TCE</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3358,46 +3358,46 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>6472870</v>
+        <v>2967919</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N40" t="n">
         <v>0.0028</v>
       </c>
       <c r="O40" t="n">
-        <v>0.0028</v>
+        <v>0.0056</v>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25092.html</t>
+          <t>https://www.lcsc.com/product-detail/C25087.html</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>R33 R46 R47 R48</t>
+          <t>R59</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>240R</t>
+          <t>200k</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3407,17 +3407,17 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>C324768</t>
+          <t>C25764</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>RC-02K2400FT</t>
+          <t>0402WGF2003TCE</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>FH (Guangdong Fenghua Advanced Tech)</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3427,39 +3427,39 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K41" t="n">
-        <v>346258</v>
+        <v>2025935</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N41" t="n">
-        <v>0.0013</v>
+        <v>0.0019</v>
       </c>
       <c r="O41" t="n">
-        <v>0.0052</v>
+        <v>0.0019</v>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C324768.html</t>
+          <t>https://www.lcsc.com/product-detail/C25764.html</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>R56</t>
+          <t>R69</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>261k</t>
+          <t>20k</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3480,17 +3480,17 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>C102933</t>
+          <t>C25765</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>RTT022613FTH</t>
+          <t>0402WGF2002TCE</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>RALEC</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K42" t="n">
-        <v>37942</v>
+        <v>1758363</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3513,26 +3513,26 @@
         <v>1</v>
       </c>
       <c r="N42" t="n">
-        <v>0.0007</v>
+        <v>0.0022</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0007</v>
+        <v>0.0022</v>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C102933.html</t>
+          <t>https://www.lcsc.com/product-detail/C25765.html</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 261kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 20kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>R63</t>
+          <t>R42</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>30k</t>
+          <t>22R</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3553,17 +3553,17 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>C49653548</t>
+          <t>C25092</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>GR0402F30KTAG00</t>
+          <t>0402WGF220JTCE</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3573,11 +3573,11 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K43" t="n">
-        <v>10000</v>
+        <v>6472940</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3586,37 +3586,37 @@
         <v>1</v>
       </c>
       <c r="N43" t="n">
-        <v>0.0008</v>
+        <v>0.0028</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0008</v>
+        <v>0.0028</v>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
+          <t>https://www.lcsc.com/product-detail/C25092.html</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>R33 R46 R47 R48</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>33k</t>
+          <t>240R</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3626,17 +3626,17 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>C25779</t>
+          <t>C324768</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>0402WGF3302TCE</t>
+          <t>RC-02K2400FT</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3646,50 +3646,50 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K44" t="n">
-        <v>1414602</v>
+        <v>346258</v>
       </c>
       <c r="L44" t="n">
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N44" t="n">
-        <v>0.0089</v>
+        <v>0.0013</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0089</v>
+        <v>0.0052</v>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25779.html</t>
+          <t>https://www.lcsc.com/product-detail/C324768.html</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>R14 R15 R17 R18 R73 R74</t>
+          <t>R63</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>30k</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3699,17 +3699,17 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>C25900</t>
+          <t>C49653548</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>0402WGF4701TCE</t>
+          <t>GR0402F30KTAG00</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3719,39 +3719,39 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K45" t="n">
-        <v>17891197</v>
+        <v>10000</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N45" t="n">
-        <v>0.0028</v>
+        <v>0.0008</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0168</v>
+        <v>0.0008</v>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25900.html</t>
+          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R25</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>47k</t>
+          <t>33k</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3772,12 +3772,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>C25792</t>
+          <t>C25779</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>0402WGF4702TCE</t>
+          <t>0402WGF3302TCE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>6019766</v>
+        <v>1414582</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3805,37 +3805,37 @@
         <v>1</v>
       </c>
       <c r="N46" t="n">
-        <v>0.0026</v>
+        <v>0.0089</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0026</v>
+        <v>0.0089</v>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25792.html</t>
+          <t>https://www.lcsc.com/product-detail/C25779.html</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>R1 R4 R9 R11</t>
+          <t>R14 R15 R17 R18 R73 R74</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C47" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>5.1k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3845,12 +3845,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>C25905</t>
+          <t>C25900</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>0402WGF5101TCE</t>
+          <t>0402WGF4701TCE</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3869,46 +3869,46 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>7310038</v>
+        <v>17890932</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N47" t="n">
-        <v>0.0024</v>
+        <v>0.0028</v>
       </c>
       <c r="O47" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0168</v>
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25905.html</t>
+          <t>https://www.lcsc.com/product-detail/C25900.html</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>R22 R50 R71 R72</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>511k</t>
+          <t>47k</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3918,17 +3918,17 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>C49655223</t>
+          <t>C25792</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>GR0402F511KTAG00</t>
+          <t>0402WGF4702TCE</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3938,50 +3938,50 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K48" t="n">
-        <v>7820</v>
+        <v>6019876</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N48" t="n">
-        <v>0.0008</v>
+        <v>0.0026</v>
       </c>
       <c r="O48" t="n">
-        <v>0.0032</v>
+        <v>0.0026</v>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
+          <t>https://www.lcsc.com/product-detail/C25792.html</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R1 R4 R9 R11</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>590R (1.5A)</t>
+          <t>5.1k</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3991,17 +3991,17 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>C49653889</t>
+          <t>C25905</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>GR0402F590RTAG00</t>
+          <t>0402WGF5101TCE</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4011,39 +4011,39 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K49" t="n">
-        <v>10000</v>
+        <v>7309423</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N49" t="n">
-        <v>0.0008</v>
+        <v>0.0024</v>
       </c>
       <c r="O49" t="n">
-        <v>0.0008</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49653889.html</t>
+          <t>https://www.lcsc.com/product-detail/C25905.html</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 590Ω 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>R24 R55</t>
+          <t>R22 R50</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>91k</t>
+          <t>511k</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4064,17 +4064,17 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C54920709</t>
+          <t>C49655223</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>HRC0402F9102DNTO</t>
+          <t>GR0402F511KTAG00</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>132322</v>
+        <v>7820</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
@@ -4097,26 +4097,26 @@
         <v>2</v>
       </c>
       <c r="N50" t="n">
-        <v>0.0007</v>
+        <v>0.0008</v>
       </c>
       <c r="O50" t="n">
-        <v>0.0014</v>
+        <v>0.0016</v>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
+          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>R56</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -4127,41 +4127,41 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>51k</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>RGT0016C_V</t>
+          <t>RES_0402</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>C129319</t>
+          <t>C25794</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>0402WGF5102TCE</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>QFN-16-EP(3x3)</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K51" t="n">
-        <v>382</v>
+        <v>2237351</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
@@ -4170,26 +4170,26 @@
         <v>1</v>
       </c>
       <c r="N51" t="n">
-        <v>2.1672</v>
+        <v>0.0018</v>
       </c>
       <c r="O51" t="n">
-        <v>2.1672</v>
+        <v>0.0018</v>
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C129319.html</t>
+          <t>https://www.lcsc.com/product-detail/C25794.html</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
+          <t>-55℃~+155℃ 50V 51kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>U14 U15</t>
+          <t>R24 R55</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -4200,32 +4200,32 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>91k</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>RES_0402</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C2867168</t>
+          <t>C54920709</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>HRC0402F9102DNTO</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>WSON-6-EP(2x2)</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -4234,7 +4234,7 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>36</v>
+        <v>132322</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
@@ -4243,62 +4243,62 @@
         <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>1.1064</v>
+        <v>0.0007</v>
       </c>
       <c r="O52" t="n">
-        <v>2.2128</v>
+        <v>0.0014</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2867168.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
+          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>USBC1 USBC2</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>type-c-31-m-12</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>RGT0016C_V</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>C129319</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Korean Hroparts Elec</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>QFN-16-EP(3x3)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4307,71 +4307,71 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>218757</v>
+        <v>382</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N53" t="n">
-        <v>0.179</v>
+        <v>2.1672</v>
       </c>
       <c r="O53" t="n">
-        <v>0.358</v>
+        <v>2.1672</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165948.html</t>
+          <t>https://www.lcsc.com/product-detail/C129319.html</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
+          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U14 U15</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>C3035748</t>
+          <t>C2867168</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>CH340X</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>WCH(Jiangsu Qin Heng)</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>MSOP-10</t>
+          <t>WSON-6-EP(2x2)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4380,71 +4380,71 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>24317</v>
+        <v>36</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N54" t="n">
-        <v>0.6629</v>
+        <v>1.1064</v>
       </c>
       <c r="O54" t="n">
-        <v>0.6629</v>
+        <v>2.2128</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
+          <t>https://www.lcsc.com/product-detail/C2867168.html</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
+          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>USBC1 USBC2</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>msm381acb026</t>
+          <t>type-c-31-m-12</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>mems</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>C51928208</t>
+          <t>C165948</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>MSM381ACB026</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>MEMS</t>
+          <t>Korean Hroparts Elec</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>LGA-3(1.9x2.8)</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4453,35 +4453,35 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>6284</v>
+        <v>218809</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N55" t="n">
-        <v>0.3025</v>
+        <v>0.179</v>
       </c>
       <c r="O55" t="n">
-        <v>0.3025</v>
+        <v>0.358</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
+          <t>https://www.lcsc.com/product-detail/C165948.html</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
+          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -4492,32 +4492,32 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>w25n02kvzeir</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>w25n02</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>C3010298</t>
+          <t>C3035748</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>W25N02KVZEIR</t>
+          <t>CH340X</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Winbond Elec</t>
+          <t>WCH(Jiangsu Qin Heng)</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>WSON-8-EP(6x8)</t>
+          <t>MSOP-10</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -4526,7 +4526,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>6256</v>
+        <v>24317</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
@@ -4535,26 +4535,26 @@
         <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>11.0584</v>
+        <v>0.6629</v>
       </c>
       <c r="O56" t="n">
-        <v>11.0584</v>
+        <v>0.6629</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3010298.html</t>
+          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function、ECC </t>
+          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>B1_N</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -4565,31 +4565,69 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>TESTP</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
+          <t>msm381acb026</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>mems</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>C51928208</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>NO PART</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
+          <t>MSM381ACB026</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>MEMS</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>LGA-3(1.9x2.8)</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="K57" t="n">
+        <v>6284</v>
+      </c>
+      <c r="L57" t="n">
+        <v>1</v>
+      </c>
+      <c r="M57" t="n">
+        <v>1</v>
+      </c>
+      <c r="N57" t="n">
+        <v>0.3025</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0.3025</v>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>B1_P</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -4600,31 +4638,69 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>TESTP</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
+          <t>w25n02kvzeir</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>w25n02</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>C3010298</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>NO PART</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
+          <t>W25N02KVZEIR</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Winbond Elec</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>WSON-8-EP(6x8)</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="K58" t="n">
+        <v>6256</v>
+      </c>
+      <c r="L58" t="n">
+        <v>1</v>
+      </c>
+      <c r="M58" t="n">
+        <v>1</v>
+      </c>
+      <c r="N58" t="n">
+        <v>11.0584</v>
+      </c>
+      <c r="O58" t="n">
+        <v>11.0584</v>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lcsc.com/product-detail/C3010298.html</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function、ECC </t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>FB4</t>
+          <t>B1_N</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -4635,7 +4711,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>GZ1608D601TF</t>
+          <t>TESTP</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -4654,16 +4730,12 @@
       <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr">
-        <is>
-          <t>Signal Line Ferrite Bead 600O @ 100MHz 1</t>
-        </is>
-      </c>
+      <c r="Q59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>B1_P</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -4674,7 +4746,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Connector 2PIn</t>
+          <t>TESTP</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -4698,7 +4770,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -4733,7 +4805,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>JB1</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -4768,7 +4840,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>JB2</t>
+          <t>JB1</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -4803,7 +4875,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>JT</t>
+          <t>JB2</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -4838,7 +4910,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>JT</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -4849,7 +4921,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>KT-0603R</t>
+          <t>Connector 2PIn</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -4868,11 +4940,7 @@
       <c r="N65" t="inlineStr"/>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr">
-        <is>
-          <t>LED RED DIFFUSED SMD</t>
-        </is>
-      </c>
+      <c r="Q65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4916,7 +4984,7 @@
         </is>
       </c>
       <c r="O68" t="n">
-        <v>51.99</v>
+        <v>52.02</v>
       </c>
     </row>
   </sheetData>
@@ -4976,6 +5044,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P58" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Charger back to ILIM 1.1k (1.41 A) and ISET 590R (1.51 A) per user; Basic values not worth the slower charge
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q68"/>
+  <dimension ref="A1:Q69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3274112</v>
+        <v>3274107</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>7677530</v>
+        <v>7677455</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>978645</v>
+        <v>978609</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>494064</v>
+        <v>494034</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2875,18 +2875,18 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R5 R12</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>1.1k (1.5A)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2896,17 +2896,17 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C25867</t>
+          <t>C54920634</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>0402WGF1501TCE</t>
+          <t>HRC0402F1101DNTO</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2916,50 +2916,50 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K34" t="n">
-        <v>2483299</v>
+        <v>16860</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N34" t="n">
-        <v>0.0028</v>
+        <v>0.0007</v>
       </c>
       <c r="O34" t="n">
-        <v>0.0056</v>
+        <v>0.0007</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25867.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920634.html</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2969,12 +2969,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C25867</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0402WGF1003TCE</t>
+          <t>0402WGF1501TCE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2993,46 +2993,46 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>11302366</v>
+        <v>2483299</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
-        <v>0.0024</v>
+        <v>0.0028</v>
       </c>
       <c r="O35" t="n">
-        <v>0.048</v>
+        <v>0.0028</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25741.html</t>
+          <t>https://www.lcsc.com/product-detail/C25867.html</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
+          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C36" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C25744</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>0402WGF1002TCE</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3066,46 +3066,46 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>27810802</v>
+        <v>11302366</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="N36" t="n">
-        <v>0.003</v>
+        <v>0.0024</v>
       </c>
       <c r="O36" t="n">
-        <v>0.054</v>
+        <v>0.048</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25744.html</t>
+          <t>https://www.lcsc.com/product-detail/C25741.html</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>120k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3115,17 +3115,17 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C54920620</t>
+          <t>C25744</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>HRC0402F1203DNTO</t>
+          <t>0402WGF1002TCE</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3135,50 +3135,50 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K37" t="n">
-        <v>1181872</v>
+        <v>27810802</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="N37" t="n">
-        <v>0.0007</v>
+        <v>0.003</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0007</v>
+        <v>0.054</v>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920620.html</t>
+          <t>https://www.lcsc.com/product-detail/C25744.html</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R71 R72</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>120k</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3188,17 +3188,17 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C26083</t>
+          <t>C54920620</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0402WGF1004TCE</t>
+          <t>HRC0402F1203DNTO</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3208,50 +3208,50 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2698020</v>
+        <v>1181872</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N38" t="n">
-        <v>0.0023</v>
+        <v>0.0007</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0046</v>
+        <v>0.0007</v>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C26083.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920620.html</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R71 R72</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C11702</t>
+          <t>C26083</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0402WGF1001TCE</t>
+          <t>0402WGF1004TCE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3285,28 +3285,28 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>11756377</v>
+        <v>2698020</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N39" t="n">
-        <v>0.0021</v>
+        <v>0.0023</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0021</v>
+        <v>0.0046</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C11702.html</t>
+          <t>https://www.lcsc.com/product-detail/C26083.html</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>6472940</v>
+        <v>6472870</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -4189,18 +4189,18 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>R24 R55</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>91k</t>
+          <t>590R (1.5A)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4210,17 +4210,17 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C54920709</t>
+          <t>C49653889</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>HRC0402F9102DNTO</t>
+          <t>GR0402F590RTAG00</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4234,71 +4234,71 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>132322</v>
+        <v>10000</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>0.0007</v>
+        <v>0.0008</v>
       </c>
       <c r="O52" t="n">
-        <v>0.0014</v>
+        <v>0.0008</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
+          <t>https://www.lcsc.com/product-detail/C49653889.html</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 590Ω 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>R24 R55</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>91k</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>RGT0016C_V</t>
+          <t>RES_0402</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C129319</t>
+          <t>C54920709</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>HRC0402F9102DNTO</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>QFN-16-EP(3x3)</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4307,61 +4307,61 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>382</v>
+        <v>132322</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>2.1672</v>
+        <v>0.0007</v>
       </c>
       <c r="O53" t="n">
-        <v>2.1672</v>
+        <v>0.0014</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C129319.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
+          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>U14 U15</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>RGT0016C_V</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>C2867168</t>
+          <t>C129319</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>WSON-6-EP(2x2)</t>
+          <t>QFN-16-EP(3x3)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4380,35 +4380,35 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>36</v>
+        <v>382</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N54" t="n">
-        <v>1.1064</v>
+        <v>2.1672</v>
       </c>
       <c r="O54" t="n">
-        <v>2.2128</v>
+        <v>2.1672</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2867168.html</t>
+          <t>https://www.lcsc.com/product-detail/C129319.html</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
+          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>USBC1 USBC2</t>
+          <t>U14 U15</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -4419,32 +4419,32 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>type-c-31-m-12</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>C2867168</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Korean Hroparts Elec</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>WSON-6-EP(2x2)</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>218809</v>
+        <v>36</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4462,62 +4462,62 @@
         <v>2</v>
       </c>
       <c r="N55" t="n">
-        <v>0.179</v>
+        <v>1.1064</v>
       </c>
       <c r="O55" t="n">
-        <v>0.358</v>
+        <v>2.2128</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165948.html</t>
+          <t>https://www.lcsc.com/product-detail/C2867168.html</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
+          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>USBC1 USBC2</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>type-c-31-m-12</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>C3035748</t>
+          <t>C165948</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>CH340X</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>WCH(Jiangsu Qin Heng)</t>
+          <t>Korean Hroparts Elec</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>MSOP-10</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -4526,35 +4526,35 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>24317</v>
+        <v>218809</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N56" t="n">
-        <v>0.6629</v>
+        <v>0.179</v>
       </c>
       <c r="O56" t="n">
-        <v>0.6629</v>
+        <v>0.358</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
+          <t>https://www.lcsc.com/product-detail/C165948.html</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
+          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -4565,32 +4565,32 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>msm381acb026</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>mems</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>C51928208</t>
+          <t>C3035748</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>MSM381ACB026</t>
+          <t>CH340X</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>MEMS</t>
+          <t>WCH(Jiangsu Qin Heng)</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>LGA-3(1.9x2.8)</t>
+          <t>MSOP-10</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="K57" t="n">
-        <v>6284</v>
+        <v>24317</v>
       </c>
       <c r="L57" t="n">
         <v>1</v>
@@ -4608,26 +4608,26 @@
         <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>0.3025</v>
+        <v>0.6629</v>
       </c>
       <c r="O57" t="n">
-        <v>0.3025</v>
+        <v>0.6629</v>
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
+          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
+          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -4638,32 +4638,32 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>w25n02kvzeir</t>
+          <t>msm381acb026</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>w25n02</t>
+          <t>mems</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>C3010298</t>
+          <t>C51928208</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>W25N02KVZEIR</t>
+          <t>MSM381ACB026</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Winbond Elec</t>
+          <t>MEMS</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>WSON-8-EP(6x8)</t>
+          <t>LGA-3(1.9x2.8)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -4672,7 +4672,7 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>6256</v>
+        <v>6284</v>
       </c>
       <c r="L58" t="n">
         <v>1</v>
@@ -4681,26 +4681,26 @@
         <v>1</v>
       </c>
       <c r="N58" t="n">
-        <v>11.0584</v>
+        <v>0.3025</v>
       </c>
       <c r="O58" t="n">
-        <v>11.0584</v>
+        <v>0.3025</v>
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3010298.html</t>
+          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t xml:space="preserve">-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function、ECC </t>
+          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>B1_N</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -4711,31 +4711,69 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>TESTP</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
+          <t>w25n02kvzeir</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>w25n02</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>C3010298</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>NO PART</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
+          <t>W25N02KVZEIR</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Winbond Elec</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>WSON-8-EP(6x8)</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="K59" t="n">
+        <v>6256</v>
+      </c>
+      <c r="L59" t="n">
+        <v>1</v>
+      </c>
+      <c r="M59" t="n">
+        <v>1</v>
+      </c>
+      <c r="N59" t="n">
+        <v>11.0584</v>
+      </c>
+      <c r="O59" t="n">
+        <v>11.0584</v>
+      </c>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lcsc.com/product-detail/C3010298.html</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function、ECC </t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>B1_P</t>
+          <t>B1_N</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -4770,7 +4808,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>B1_P</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -4781,7 +4819,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Connector 2PIn</t>
+          <t>TESTP</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -4805,7 +4843,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -4840,7 +4878,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>JB1</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -4875,7 +4913,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>JB2</t>
+          <t>JB1</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -4910,7 +4948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>JT</t>
+          <t>JB2</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -4945,7 +4983,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ANT1</t>
+          <t>JT</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -4956,7 +4994,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>MIFI</t>
+          <t>Connector 2PIn</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -4977,13 +5015,48 @@
       <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr"/>
     </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ANT1</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>MIFI</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="O68" t="n">
+      <c r="O69" t="n">
         <v>52.02</v>
       </c>
     </row>
@@ -5046,6 +5119,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P59" r:id="rId58"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Charger limits to Basic values: ILIM 1.5k (1.03 A), ISET 1k (0.89 A)
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q69"/>
+  <dimension ref="A1:Q68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2875,18 +2875,18 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R5 R12</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>1.1k (1.5A)</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2896,17 +2896,17 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C54920634</t>
+          <t>C25867</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>HRC0402F1101DNTO</t>
+          <t>0402WGF1501TCE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2916,50 +2916,50 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K34" t="n">
-        <v>16860</v>
+        <v>2483299</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N34" t="n">
-        <v>0.0007</v>
+        <v>0.0028</v>
       </c>
       <c r="O34" t="n">
-        <v>0.0007</v>
+        <v>0.0056</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920634.html</t>
+          <t>https://www.lcsc.com/product-detail/C25867.html</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2969,12 +2969,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C25867</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0402WGF1501TCE</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2993,46 +2993,46 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>2483299</v>
+        <v>11302366</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="N35" t="n">
-        <v>0.0028</v>
+        <v>0.0024</v>
       </c>
       <c r="O35" t="n">
-        <v>0.0028</v>
+        <v>0.048</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25867.html</t>
+          <t>https://www.lcsc.com/product-detail/C25741.html</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
+          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C36" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C25744</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>0402WGF1003TCE</t>
+          <t>0402WGF1002TCE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3066,46 +3066,46 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>11302366</v>
+        <v>27810802</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N36" t="n">
-        <v>0.0024</v>
+        <v>0.003</v>
       </c>
       <c r="O36" t="n">
-        <v>0.048</v>
+        <v>0.054</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25741.html</t>
+          <t>https://www.lcsc.com/product-detail/C25744.html</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>120k</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3115,17 +3115,17 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C25744</t>
+          <t>C54920620</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>0402WGF1002TCE</t>
+          <t>HRC0402F1203DNTO</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3135,50 +3135,50 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K37" t="n">
-        <v>27810802</v>
+        <v>1181872</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="N37" t="n">
-        <v>0.003</v>
+        <v>0.0007</v>
       </c>
       <c r="O37" t="n">
-        <v>0.054</v>
+        <v>0.0007</v>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25744.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920620.html</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R71 R72</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>120k</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3188,17 +3188,17 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C54920620</t>
+          <t>C26083</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>HRC0402F1203DNTO</t>
+          <t>0402WGF1004TCE</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3208,50 +3208,50 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K38" t="n">
-        <v>1181872</v>
+        <v>2698020</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N38" t="n">
-        <v>0.0007</v>
+        <v>0.0023</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0007</v>
+        <v>0.0046</v>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920620.html</t>
+          <t>https://www.lcsc.com/product-detail/C26083.html</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R71 R72</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C26083</t>
+          <t>C11702</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0402WGF1004TCE</t>
+          <t>0402WGF1001TCE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3285,28 +3285,28 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2698020</v>
+        <v>11756377</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N39" t="n">
-        <v>0.0023</v>
+        <v>0.0021</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0046</v>
+        <v>0.0021</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C26083.html</t>
+          <t>https://www.lcsc.com/product-detail/C11702.html</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
@@ -4189,18 +4189,18 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R24 R55</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>590R (1.5A)</t>
+          <t>91k</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4210,17 +4210,17 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C49653889</t>
+          <t>C54920709</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>GR0402F590RTAG00</t>
+          <t>HRC0402F9102DNTO</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4234,71 +4234,71 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>10000</v>
+        <v>132322</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>0.0008</v>
+        <v>0.0007</v>
       </c>
       <c r="O52" t="n">
-        <v>0.0008</v>
+        <v>0.0014</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49653889.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 590Ω 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>R24 R55</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>91k</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>RES_0402</t>
+          <t>RGT0016C_V</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C54920709</t>
+          <t>C129319</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>HRC0402F9102DNTO</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>QFN-16-EP(3x3)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4307,61 +4307,61 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>132322</v>
+        <v>382</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N53" t="n">
-        <v>0.0007</v>
+        <v>2.1672</v>
       </c>
       <c r="O53" t="n">
-        <v>0.0014</v>
+        <v>2.1672</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
+          <t>https://www.lcsc.com/product-detail/C129319.html</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>U14 U15</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>RGT0016C_V</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>C129319</t>
+          <t>C2867168</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>QFN-16-EP(3x3)</t>
+          <t>WSON-6-EP(2x2)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4380,35 +4380,35 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>382</v>
+        <v>36</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N54" t="n">
-        <v>2.1672</v>
+        <v>1.1064</v>
       </c>
       <c r="O54" t="n">
-        <v>2.1672</v>
+        <v>2.2128</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C129319.html</t>
+          <t>https://www.lcsc.com/product-detail/C2867168.html</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
+          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>U14 U15</t>
+          <t>USBC1 USBC2</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -4419,32 +4419,32 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>type-c-31-m-12</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>C2867168</t>
+          <t>C165948</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Korean Hroparts Elec</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>WSON-6-EP(2x2)</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>36</v>
+        <v>218809</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4462,62 +4462,62 @@
         <v>2</v>
       </c>
       <c r="N55" t="n">
-        <v>1.1064</v>
+        <v>0.179</v>
       </c>
       <c r="O55" t="n">
-        <v>2.2128</v>
+        <v>0.358</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2867168.html</t>
+          <t>https://www.lcsc.com/product-detail/C165948.html</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
+          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>USBC1 USBC2</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>type-c-31-m-12</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>C3035748</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>CH340X</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Korean Hroparts Elec</t>
+          <t>WCH(Jiangsu Qin Heng)</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>MSOP-10</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -4526,35 +4526,35 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>218809</v>
+        <v>24317</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>0.179</v>
+        <v>0.6629</v>
       </c>
       <c r="O56" t="n">
-        <v>0.358</v>
+        <v>0.6629</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165948.html</t>
+          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
+          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -4565,32 +4565,32 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>msm381acb026</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>mems</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>C3035748</t>
+          <t>C51928208</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>CH340X</t>
+          <t>MSM381ACB026</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>WCH(Jiangsu Qin Heng)</t>
+          <t>MEMS</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>MSOP-10</t>
+          <t>LGA-3(1.9x2.8)</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="K57" t="n">
-        <v>24317</v>
+        <v>6284</v>
       </c>
       <c r="L57" t="n">
         <v>1</v>
@@ -4608,26 +4608,26 @@
         <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>0.6629</v>
+        <v>0.3025</v>
       </c>
       <c r="O57" t="n">
-        <v>0.6629</v>
+        <v>0.3025</v>
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
+          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
+          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -4638,32 +4638,32 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>msm381acb026</t>
+          <t>w25n02kvzeir</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>mems</t>
+          <t>w25n02</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>C51928208</t>
+          <t>C3010298</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>MSM381ACB026</t>
+          <t>W25N02KVZEIR</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>MEMS</t>
+          <t>Winbond Elec</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>LGA-3(1.9x2.8)</t>
+          <t>WSON-8-EP(6x8)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -4672,7 +4672,7 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>6284</v>
+        <v>6256</v>
       </c>
       <c r="L58" t="n">
         <v>1</v>
@@ -4681,26 +4681,26 @@
         <v>1</v>
       </c>
       <c r="N58" t="n">
-        <v>0.3025</v>
+        <v>11.0584</v>
       </c>
       <c r="O58" t="n">
-        <v>0.3025</v>
+        <v>11.0584</v>
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
+          <t>https://www.lcsc.com/product-detail/C3010298.html</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
+          <t xml:space="preserve">-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function、ECC </t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>B1_N</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -4711,69 +4711,31 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>w25n02kvzeir</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>w25n02</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>C3010298</t>
-        </is>
-      </c>
+          <t>TESTP</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>W25N02KVZEIR</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Winbond Elec</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>WSON-8-EP(6x8)</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="K59" t="n">
-        <v>6256</v>
-      </c>
-      <c r="L59" t="n">
-        <v>1</v>
-      </c>
-      <c r="M59" t="n">
-        <v>1</v>
-      </c>
-      <c r="N59" t="n">
-        <v>11.0584</v>
-      </c>
-      <c r="O59" t="n">
-        <v>11.0584</v>
-      </c>
-      <c r="P59" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lcsc.com/product-detail/C3010298.html</t>
-        </is>
-      </c>
-      <c r="Q59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function、ECC </t>
-        </is>
-      </c>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>B1_N</t>
+          <t>B1_P</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -4808,7 +4770,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>B1_P</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -4819,7 +4781,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>TESTP</t>
+          <t>Connector 2PIn</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -4843,7 +4805,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -4878,7 +4840,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>JB1</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -4913,7 +4875,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>JB1</t>
+          <t>JB2</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -4948,7 +4910,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>JB2</t>
+          <t>JT</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -4983,7 +4945,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>JT</t>
+          <t>ANT1</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -4994,7 +4956,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Connector 2PIn</t>
+          <t>MIFI</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -5015,48 +4977,13 @@
       <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr"/>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>ANT1</t>
-        </is>
-      </c>
-      <c r="B67" t="n">
-        <v>1</v>
-      </c>
-      <c r="C67" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>MIFI</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>NO PART</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
+    <row r="68">
+      <c r="A68" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="O69" t="n">
+      <c r="O68" t="n">
         <v>52.02</v>
       </c>
     </row>
@@ -5119,7 +5046,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P59" r:id="rId58"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fee-free parts: Promotional Extended included; DSK24 -> promo C22466352, R29 120k -> promo, R22/R50 511k -> 510k promo (3.302 V), C1/C104 -> Basic CL31B105KBHNNNE
JLCPCB_ECONOMIC_PARTS.txt replaces JLCPCB_BASIC_PARTS.txt: all 1586 Basic + Promotional
Extended parts ($0 feeder loading in Economic PCBA), fetched with
componentLibraryType=base + preferredComponentFlag=true + searchType=2.
Order lists label Basic / Promo / Extended.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3274107</v>
+        <v>3273729</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>17663094</v>
+        <v>17671199</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3956681</v>
+        <v>3956833</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1578706</v>
+        <v>1580871</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>858285</v>
+        <v>857981</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2996251</v>
+        <v>2996206</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1290,17 +1290,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>C597503</t>
+          <t>C1848</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>12065C105JAT2A</t>
+          <t>CL31B105KBHNNNE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1310,11 +1310,11 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K12" t="n">
-        <v>1928</v>
+        <v>871144</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1323,19 +1323,19 @@
         <v>2</v>
       </c>
       <c r="N12" t="n">
-        <v>0.3725</v>
+        <v>0.0493</v>
       </c>
       <c r="O12" t="n">
-        <v>0.745</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C597503.html</t>
+          <t>https://www.lcsc.com/product-detail/C1848.html</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1uF 50V X7R ±5% 1206 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>1uF 50V X7R ±10% 1206 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>627252</v>
+        <v>627440</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2637817</v>
+        <v>2637332</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>13129771</v>
+        <v>13139860</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>7677455</v>
+        <v>7679540</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>9809655</v>
+        <v>9783125</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>978609</v>
+        <v>978324</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2093,17 +2093,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>C2939005</t>
+          <t>C22466352</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>DSK24 K24</t>
+          <t>DSK24</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>KUU</t>
+          <t>hongjiacheng</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2113,11 +2113,11 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Promo</t>
         </is>
       </c>
       <c r="K23" t="n">
-        <v>120296</v>
+        <v>2685650</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2126,19 +2126,19 @@
         <v>3</v>
       </c>
       <c r="N23" t="n">
-        <v>0.0187</v>
+        <v>0.0247</v>
       </c>
       <c r="O23" t="n">
-        <v>0.0561</v>
+        <v>0.0741</v>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2939005.html</t>
+          <t>https://www.lcsc.com/product-detail/C22466352.html</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2A 40A 40V 500uA@40V 550mV@2A Independent SOD-123FL Schottky Diodes ROHS</t>
+          <t>-55℃~+125℃ 2A 40V 500uA@40V 50A 550mV@2A Standalone SOD-123FL Schottky Diodes ROHS</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>3620363</v>
+        <v>3634586</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>494034</v>
+        <v>470699</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>816954</v>
+        <v>812251</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>8743973</v>
+        <v>8745955</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2628,7 +2628,7 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>855576</v>
+        <v>855666</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>2483299</v>
+        <v>2483284</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>11302366</v>
+        <v>11303004</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>27810802</v>
+        <v>27820091</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3115,17 +3115,17 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C54920620</t>
+          <t>C25750</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>HRC0402F1203DNTO</t>
+          <t>0402WGF1203TCE</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3135,11 +3135,11 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Promo</t>
         </is>
       </c>
       <c r="K37" t="n">
-        <v>1181872</v>
+        <v>808226</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3148,14 +3148,14 @@
         <v>1</v>
       </c>
       <c r="N37" t="n">
-        <v>0.0007</v>
+        <v>0.0012</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0007</v>
+        <v>0.0012</v>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920620.html</t>
+          <t>https://www.lcsc.com/product-detail/C25750.html</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2698020</v>
+        <v>2698244</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>11756377</v>
+        <v>11759531</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2967919</v>
+        <v>2968869</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>2025935</v>
+        <v>2024140</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>1758363</v>
+        <v>1759417</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>6472870</v>
+        <v>6472004</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>1414582</v>
+        <v>1414880</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>17890932</v>
+        <v>17894122</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>6019876</v>
+        <v>6020241</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>7309423</v>
+        <v>7312970</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
@@ -4054,7 +4054,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>511k</t>
+          <t>510k</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4064,17 +4064,17 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C49655223</t>
+          <t>C11616</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>GR0402F511KTAG00</t>
+          <t>0402WGF5103TCE</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4084,32 +4084,32 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Promo</t>
         </is>
       </c>
       <c r="K50" t="n">
-        <v>7820</v>
+        <v>26089</v>
       </c>
       <c r="L50" t="n">
-        <v>1</v>
+        <v>1991</v>
       </c>
       <c r="M50" t="n">
-        <v>2</v>
+        <v>1991</v>
       </c>
       <c r="N50" t="n">
-        <v>0.0008</v>
+        <v>0.0043</v>
       </c>
       <c r="O50" t="n">
-        <v>0.0016</v>
+        <v>8.561299999999999</v>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
+          <t>https://www.lcsc.com/product-detail/C11616.html</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 510kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>2237351</v>
+        <v>2237451</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>218809</v>
+        <v>229526</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4526,7 +4526,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>24317</v>
+        <v>24367</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
@@ -4984,7 +4984,7 @@
         </is>
       </c>
       <c r="O68" t="n">
-        <v>52.02</v>
+        <v>59.96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
R22/R50 back to 511k (C49655223): the promotional 510k has a 1991-piece MOQ at JLCPCB
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -4054,7 +4054,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>510k</t>
+          <t>511k</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4064,17 +4064,17 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C11616</t>
+          <t>C49655223</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>0402WGF5103TCE</t>
+          <t>GR0402F511KTAG00</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4084,32 +4084,32 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Promo</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K50" t="n">
-        <v>26089</v>
+        <v>7820</v>
       </c>
       <c r="L50" t="n">
-        <v>1991</v>
+        <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>1991</v>
+        <v>2</v>
       </c>
       <c r="N50" t="n">
-        <v>0.0043</v>
+        <v>0.0008</v>
       </c>
       <c r="O50" t="n">
-        <v>8.561299999999999</v>
+        <v>0.0016</v>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C11616.html</t>
+          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 510kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
@@ -4984,7 +4984,7 @@
         </is>
       </c>
       <c r="O68" t="n">
-        <v>59.96</v>
+        <v>51.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
U17: AHT30 out of stock, use AHT20 (same 3x3 mm 6-pad package, same pinout and I2C protocol, C2757850)
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -550,7 +550,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>aht30</t>
+          <t>AHT20</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -560,12 +560,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>C45354925</t>
+          <t>C2757850</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>AHT30</t>
+          <t>AHT20</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>SMD-6P,3x3mm</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -584,28 +584,28 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>45556</v>
       </c>
       <c r="L2" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>0.5750999999999999</v>
+        <v>0.7663</v>
       </c>
       <c r="O2" t="n">
-        <v>9.201599999999999</v>
+        <v>0.7663</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C45354925.html</t>
+          <t>https://www.lcsc.com/product-detail/C2757850.html</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t xml:space="preserve">-40℃~+120℃ 0%RH~100%RH 2.2V~5.5V 570uA Factory calibration I2C ±0.5℃ ±3%RH SMD-6P,3x3mm Temperature and Humidity Sensor </t>
+          <t>-40℃~+120℃ 0%RH~100%RH 2.2V~5.5V 20bit 570uA I2C ±0.3℃ ±2%RH SMD Temperature and Humidity Sensor ROHS</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3273729</v>
+        <v>3273674</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>17671199</v>
+        <v>17666490</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3956833</v>
+        <v>3957083</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>857981</v>
+        <v>858201</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>871144</v>
+        <v>871159</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>627440</v>
+        <v>627435</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2637332</v>
+        <v>2637451</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>13139860</v>
+        <v>13135582</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>7679540</v>
+        <v>7678829</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>9783125</v>
+        <v>9781725</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>978324</v>
+        <v>978244</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>2685650</v>
+        <v>2685680</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>3634586</v>
+        <v>3631371</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>470699</v>
+        <v>470624</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>812251</v>
+        <v>811592</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>8745955</v>
+        <v>8746152</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>11303004</v>
+        <v>11302832</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>27820091</v>
+        <v>27817252</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>808226</v>
+        <v>808106</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2698244</v>
+        <v>2698204</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>11759531</v>
+        <v>11760874</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2968869</v>
+        <v>2968929</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>2024140</v>
+        <v>2024010</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>1759417</v>
+        <v>1758887</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>6472004</v>
+        <v>6472038</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>1414880</v>
+        <v>1414900</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>17894122</v>
+        <v>17896210</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>7312970</v>
+        <v>7311618</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>2237451</v>
+        <v>2237371</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>229526</v>
+        <v>229208</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4672,7 +4672,7 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>6256</v>
+        <v>6276</v>
       </c>
       <c r="L58" t="n">
         <v>1</v>
@@ -4984,7 +4984,7 @@
         </is>
       </c>
       <c r="O68" t="n">
-        <v>51.4</v>
+        <v>42.96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
U14/U15: TPS61160ADRVT (36 in stock, 1.11 USD) -> TPS61160DRVR (11.6k in stock, 0.45 USD); same WSON-6, 200 mV FB, 26 V OVP, 600 kHz
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>45556</v>
+        <v>45606</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3273674</v>
+        <v>3274878</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>17666490</v>
+        <v>17668414</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3957083</v>
+        <v>3957173</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>858201</v>
+        <v>858391</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2996206</v>
+        <v>2996256</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>871159</v>
+        <v>871163</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>627435</v>
+        <v>628081</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2637451</v>
+        <v>2637281</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>13135582</v>
+        <v>13154609</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>7678829</v>
+        <v>7684931</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>9781725</v>
+        <v>9785724</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>978244</v>
+        <v>978264</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>3631371</v>
+        <v>3631678</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>470624</v>
+        <v>470726</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>811592</v>
+        <v>811656</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>8746152</v>
+        <v>8746648</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2628,7 +2628,7 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>855666</v>
+        <v>855621</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>2483284</v>
+        <v>2483272</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>11302832</v>
+        <v>11310718</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>27817252</v>
+        <v>27824662</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>808106</v>
+        <v>807106</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2698204</v>
+        <v>2698259</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>11760874</v>
+        <v>11765251</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2968929</v>
+        <v>2968836</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>2024010</v>
+        <v>2024065</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>1758887</v>
+        <v>1759968</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>6472038</v>
+        <v>6477700</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>1414900</v>
+        <v>1415070</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>17896210</v>
+        <v>17901470</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>6020241</v>
+        <v>6022781</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>7311618</v>
+        <v>7311984</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>2237371</v>
+        <v>2237445</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
@@ -4346,22 +4346,22 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
+          <t>TPS61160DRVR</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
           <t>TPS61160ADRVT</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>TPS61160ADRVT</t>
-        </is>
-      </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>C2867168</t>
+          <t>C165143</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>TPS61160DRVR</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>36</v>
+        <v>11619</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4389,19 +4389,19 @@
         <v>2</v>
       </c>
       <c r="N54" t="n">
-        <v>1.1064</v>
+        <v>0.4482</v>
       </c>
       <c r="O54" t="n">
-        <v>2.2128</v>
+        <v>0.8964</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2867168.html</t>
+          <t>https://www.lcsc.com/product-detail/C165143.html</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
+          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over Current Protection、Over-Temperature</t>
         </is>
       </c>
     </row>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>229208</v>
+        <v>229198</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4526,7 +4526,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>24367</v>
+        <v>24377</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
@@ -4984,7 +4984,7 @@
         </is>
       </c>
       <c r="O68" t="n">
-        <v>42.96</v>
+        <v>41.64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regenerate fabrication and assembly files from the 19:15 export
Gerber zip: 6 copper, mask, silk, paste, MIFA.GKO (36.5 x 65 mm rectangle from the
ODB++ profile; GM/GM2/GM5 carry footprint mechanical shapes besides the outline),
round and slot drills (slot file verified against the board: all 8 USB-C slots match).
PickPlace_MIFA.csv and BOM_ASSEMBLY.csv are generated from Project Outputs/Pick Place
for MIFA.csv and cross-checked against the schematic (0 mismatches) and the ODB++
(positions and sides); 215 placements, 55 part numbers, same designator set in both.
PR1 is now programming pads, not a connector, so it has no part. Order lists refreshed:
41.17 USD per board.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>45606</v>
+        <v>45446</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3274878</v>
+        <v>3187778</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>17668414</v>
+        <v>14404501</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3957173</v>
+        <v>3923839</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1580871</v>
+        <v>1549543</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>858391</v>
+        <v>840006</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2996256</v>
+        <v>2990724</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>871163</v>
+        <v>850087</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>628081</v>
+        <v>619497</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2637281</v>
+        <v>2612863</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>9236</v>
+        <v>8911</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>17882</v>
+        <v>17860</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>7155</v>
+        <v>6828</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>8520</v>
+        <v>8340</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>13154609</v>
+        <v>13026526</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>7684931</v>
+        <v>7560850</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>9785724</v>
+        <v>9767291</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>978264</v>
+        <v>957154</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>2685680</v>
+        <v>2682603</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2145,7 +2145,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PR1</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2156,41 +2156,41 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>SM05B-NSHSS-TB(LF)(SN)</t>
+          <t>KT-0603R</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>FP-SM05B-NSHSS-TB_LF_SN-MFG</t>
+          <t>FP-SML-LX0603IW-TR-MFG</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>C268096</t>
+          <t>C2286</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>SM05B-NSHSS-TB(LF)(SN)</t>
+          <t>KT-0603R</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Hubei KENTO Elec</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>SMD,P=1mm,Surface Mount，Right Angle</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K24" t="n">
-        <v>1984</v>
+        <v>3517887</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2199,26 +2199,26 @@
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0.4749</v>
+        <v>0.0072</v>
       </c>
       <c r="O24" t="n">
-        <v>0.4749</v>
+        <v>0.0072</v>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C268096.html</t>
+          <t>https://www.lcsc.com/product-detail/C2286.html</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 1A 1mm 1x5P 4.4mm 5 50V 5P 6.8mm 7mm Auxiliary Solder Pin Copper alloy NSH PA Surface Mount, Right Angle Tin</t>
+          <t>-40℃~+85℃ 1.6mm x 0.8mm square LED 1.8V~2.4V 120° 20mA 300mcd 40mW 615nm~630nm 645nm Discrete Diode Red Water Clear 0603</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2229,32 +2229,32 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>KT-0603R</t>
+          <t>AO3401A</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>FP-SML-LX0603IW-TR-MFG</t>
+          <t>FP-SOT23-IPC_B</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>C2286</t>
+          <t>C15127</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>KT-0603R</t>
+          <t>AO3401A</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Hubei KENTO Elec</t>
+          <t>Alpha &amp; Omega Semicon</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>3631678</v>
+        <v>472945</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2272,52 +2272,52 @@
         <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>0.0072</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="O25" t="n">
-        <v>0.0072</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2286.html</t>
+          <t>https://www.lcsc.com/product-detail/C15127.html</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1.6mm x 0.8mm square LED 1.8V~2.4V 120° 20mA 300mcd 40mW 615nm~630nm 645nm Discrete Diode Red Water Clear 0603</t>
+          <t>1 P-Channel 14nC@10V 30V 47mΩ@10V、60mΩ@4.5V、85mΩ@2.5V 4A 55pF 645pF 80pF 900mV SOT-23 MOSFETs ROHS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q2 Q4</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AO3401A</t>
+          <t>AO3400A</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>FP-SOT23-IPC_B</t>
+          <t>FP-SOT23-MFG</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>C15127</t>
+          <t>C20917</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>AO3401A</t>
+          <t>AO3400A</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2336,181 +2336,181 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>470726</v>
+        <v>893873</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N26" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.0815</v>
       </c>
       <c r="O26" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.163</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C15127.html</t>
+          <t>https://www.lcsc.com/product-detail/C20917.html</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>1 P-Channel 14nC@10V 30V 47mΩ@10V、60mΩ@4.5V、85mΩ@2.5V 4A 55pF 645pF 80pF 900mV SOT-23 MOSFETs ROHS</t>
+          <t>-55℃~+150℃ 1 N-channel 1.45V 1.4W 30V 48mΩ@2.5V 5.7A 50pF 630pF 75pF 7nC@10V N-Channel SOT-23 MOSFETs ROHS</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Q2 Q4</t>
+          <t>D3 D4 D5</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AO3400A</t>
+          <t>PRTR5V0U2F,115</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>FP-SOT23-MFG</t>
+          <t>FP-SOT886-MFG</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C20917</t>
+          <t>C478118</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>AO3400A</t>
+          <t>PRTR5V0U2F,115</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Alpha &amp; Omega Semicon</t>
+          <t>Nexperia</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>XSON-6(1x1.5)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K27" t="n">
-        <v>811656</v>
+        <v>60131</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N27" t="n">
-        <v>0.0815</v>
+        <v>0.103</v>
       </c>
       <c r="O27" t="n">
-        <v>0.163</v>
+        <v>0.309</v>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C20917.html</t>
+          <t>https://www.lcsc.com/product-detail/C478118.html</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>-55℃~+150℃ 1 N-channel 1.45V 1.4W 30V 48mΩ@2.5V 5.7A 50pF 630pF 75pF 7nC@10V N-Channel SOT-23 MOSFETs ROHS</t>
+          <t>-40℃~+85℃ 100nA 1pF 2 5.5V 6V IEC 61000-4-2 TVS Unidirectional XSON-6(1x1.5) ESD and Surge Protection (TVS/ESD) ROHS</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>D3 D4 D5</t>
+          <t>R68</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>PRTR5V0U2F,115</t>
+          <t>10R</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FP-SOT886-MFG</t>
+          <t>FP-SR0603-MFG</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C478118</t>
+          <t>C22859</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>PRTR5V0U2F,115</t>
+          <t>0603WAF100JT5E</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Nexperia</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>XSON-6(1x1.5)</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K28" t="n">
-        <v>60131</v>
+        <v>8659872</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>0.103</v>
+        <v>0.0036</v>
       </c>
       <c r="O28" t="n">
-        <v>0.309</v>
+        <v>0.0036</v>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C478118.html</t>
+          <t>https://www.lcsc.com/product-detail/C22859.html</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 100nA 1pF 2 5.5V 6V IEC 61000-4-2 TVS Unidirectional XSON-6(1x1.5) ESD and Surge Protection (TVS/ESD) ROHS</t>
+          <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>R68</t>
+          <t>R66</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10R</t>
+          <t>4.7R</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2531,12 +2531,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C22859</t>
+          <t>C23164</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>0603WAF100JT5E</t>
+          <t>0603WAF470KT5E</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>8746648</v>
+        <v>832890</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2564,26 +2564,26 @@
         <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>0.0036</v>
+        <v>0.0027</v>
       </c>
       <c r="O29" t="n">
-        <v>0.0036</v>
+        <v>0.0027</v>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22859.html</t>
+          <t>https://www.lcsc.com/product-detail/C23164.html</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100mW 4.7Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>R66</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2594,41 +2594,41 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>4.7R</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>FP-SR0603-MFG</t>
+          <t>FP-XRCGB_F_N-MFG</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C23164</t>
+          <t>C2965580</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>0603WAF470KT5E</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>YXC Crystal Oscillators</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SMD2016-4P</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K30" t="n">
-        <v>855621</v>
+        <v>24240</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
@@ -2637,62 +2637,62 @@
         <v>1</v>
       </c>
       <c r="N30" t="n">
-        <v>0.0027</v>
+        <v>0.0784</v>
       </c>
       <c r="O30" t="n">
-        <v>0.0027</v>
+        <v>0.0784</v>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C23164.html</t>
+          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 4.7Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Y2</t>
+          <t>S1 S2 S3</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>S2B-PH-K-S(LF)(SN)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FP-XRCGB_F_N-MFG</t>
+          <t>JST-S2B-PH-K-S_V</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C2965580</t>
+          <t>C157932</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>S2B-PH-K-S-GW</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>YXC Crystal Oscillators</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>SMD2016-4P</t>
+          <t>Push-Pull,P=2mm</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2701,71 +2701,71 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>4425</v>
+        <v>15701</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N31" t="n">
-        <v>0.0784</v>
+        <v>0.2125</v>
       </c>
       <c r="O31" t="n">
-        <v>0.0784</v>
+        <v>0.6375</v>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
+          <t>https://www.lcsc.com/product-detail/C157932.html</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
+          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>S1 S2 S3</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S(LF)(SN)</t>
+          <t>k230d</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>JST-S2B-PH-K-S_V</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C157932</t>
+          <t>C42414902</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S-GW</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Canaan</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Push-Pull,P=2mm</t>
+          <t>BGA-256</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2774,119 +2774,119 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>15851</v>
+        <v>361</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N32" t="n">
-        <v>0.2125</v>
+        <v>13.3007</v>
       </c>
       <c r="O32" t="n">
-        <v>0.6375</v>
+        <v>13.3007</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C157932.html</t>
+          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
+          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>R5 R12</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>k230d</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>RES_0402</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C42414902</t>
+          <t>C25867</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>0402WGF1501TCE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Canaan</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>BGA-256</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K33" t="n">
-        <v>361</v>
+        <v>2470541</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N33" t="n">
-        <v>13.3007</v>
+        <v>0.0028</v>
       </c>
       <c r="O33" t="n">
-        <v>13.3007</v>
+        <v>0.0056</v>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
+          <t>https://www.lcsc.com/product-detail/C25867.html</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
+          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R5 R12</t>
+          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2896,12 +2896,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C25867</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>0402WGF1501TCE</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2920,46 +2920,46 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>2483272</v>
+        <v>11170242</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N34" t="n">
-        <v>0.0028</v>
+        <v>0.0024</v>
       </c>
       <c r="O34" t="n">
-        <v>0.0056</v>
+        <v>0.048</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25867.html</t>
+          <t>https://www.lcsc.com/product-detail/C25741.html</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
+          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C35" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2969,12 +2969,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C25744</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0402WGF1003TCE</t>
+          <t>0402WGF1002TCE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2993,46 +2993,46 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>11310718</v>
+        <v>27499771</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N35" t="n">
-        <v>0.0024</v>
+        <v>0.003</v>
       </c>
       <c r="O35" t="n">
-        <v>0.048</v>
+        <v>0.054</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25741.html</t>
+          <t>https://www.lcsc.com/product-detail/C25744.html</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>120k</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C25744</t>
+          <t>C25750</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>0402WGF1002TCE</t>
+          <t>0402WGF1203TCE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3062,50 +3062,50 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Promo</t>
         </is>
       </c>
       <c r="K36" t="n">
-        <v>27824662</v>
+        <v>800156</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="N36" t="n">
-        <v>0.003</v>
+        <v>0.0012</v>
       </c>
       <c r="O36" t="n">
-        <v>0.054</v>
+        <v>0.0012</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25744.html</t>
+          <t>https://www.lcsc.com/product-detail/C25750.html</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R71 R72</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>120k</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3115,12 +3115,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C25750</t>
+          <t>C26083</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>0402WGF1203TCE</t>
+          <t>0402WGF1004TCE</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3135,50 +3135,50 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Promo</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K37" t="n">
-        <v>807106</v>
+        <v>2677881</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N37" t="n">
-        <v>0.0012</v>
+        <v>0.0023</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0012</v>
+        <v>0.0046</v>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25750.html</t>
+          <t>https://www.lcsc.com/product-detail/C26083.html</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R71 R72</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3188,12 +3188,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C26083</t>
+          <t>C11702</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0402WGF1004TCE</t>
+          <t>0402WGF1001TCE</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3212,46 +3212,46 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2698259</v>
+        <v>11624377</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N38" t="n">
-        <v>0.0023</v>
+        <v>0.0021</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0046</v>
+        <v>0.0021</v>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C26083.html</t>
+          <t>https://www.lcsc.com/product-detail/C11702.html</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R37 R62</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>200R</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C11702</t>
+          <t>C25087</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0402WGF1001TCE</t>
+          <t>0402WGF2000TCE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3285,46 +3285,46 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>11765251</v>
+        <v>2962356</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N39" t="n">
-        <v>0.0021</v>
+        <v>0.0028</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0021</v>
+        <v>0.0056</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C11702.html</t>
+          <t>https://www.lcsc.com/product-detail/C25087.html</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>R37 R62</t>
+          <t>R59</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>200R</t>
+          <t>200k</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3334,12 +3334,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>C25087</t>
+          <t>C25764</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>0402WGF2000TCE</t>
+          <t>0402WGF2003TCE</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3358,35 +3358,35 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2968836</v>
+        <v>2206703</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>0.0028</v>
+        <v>0.0019</v>
       </c>
       <c r="O40" t="n">
-        <v>0.0056</v>
+        <v>0.0019</v>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25087.html</t>
+          <t>https://www.lcsc.com/product-detail/C25764.html</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>R59</t>
+          <t>R69</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>200k</t>
+          <t>20k</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3407,12 +3407,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>C25764</t>
+          <t>C25765</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>0402WGF2003TCE</t>
+          <t>0402WGF2002TCE</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>2024065</v>
+        <v>1723021</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3440,26 +3440,26 @@
         <v>1</v>
       </c>
       <c r="N41" t="n">
-        <v>0.0019</v>
+        <v>0.0022</v>
       </c>
       <c r="O41" t="n">
-        <v>0.0019</v>
+        <v>0.0022</v>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25764.html</t>
+          <t>https://www.lcsc.com/product-detail/C25765.html</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 20kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>R69</t>
+          <t>R42</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>20k</t>
+          <t>22R</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3480,12 +3480,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>C25765</t>
+          <t>C25092</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>0402WGF2002TCE</t>
+          <t>0402WGF220JTCE</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>1759968</v>
+        <v>6344847</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3513,37 +3513,37 @@
         <v>1</v>
       </c>
       <c r="N42" t="n">
-        <v>0.0022</v>
+        <v>0.0028</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0022</v>
+        <v>0.0028</v>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25765.html</t>
+          <t>https://www.lcsc.com/product-detail/C25092.html</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 20kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>R42</t>
+          <t>R33 R46 R47 R48</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>22R</t>
+          <t>240R</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3553,17 +3553,17 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>C25092</t>
+          <t>C324768</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>0402WGF220JTCE</t>
+          <t>RC-02K2400FT</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3573,50 +3573,50 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K43" t="n">
-        <v>6477700</v>
+        <v>343998</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N43" t="n">
-        <v>0.0028</v>
+        <v>0.0013</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0028</v>
+        <v>0.0052</v>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25092.html</t>
+          <t>https://www.lcsc.com/product-detail/C324768.html</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>R33 R46 R47 R48</t>
+          <t>R63</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>240R</t>
+          <t>30k</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3626,17 +3626,17 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>C324768</t>
+          <t>C49653548</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>RC-02K2400FT</t>
+          <t>GR0402F30KTAG00</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>FH (Guangdong Fenghua Advanced Tech)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3650,35 +3650,35 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>346258</v>
+        <v>9900</v>
       </c>
       <c r="L44" t="n">
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N44" t="n">
-        <v>0.0013</v>
+        <v>0.0008</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0052</v>
+        <v>0.0008</v>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C324768.html</t>
+          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>R63</t>
+          <t>R25</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -3689,7 +3689,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>30k</t>
+          <t>33k</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3699,17 +3699,17 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>C49653548</t>
+          <t>C25779</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>GR0402F30KTAG00</t>
+          <t>0402WGF3302TCE</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3719,11 +3719,11 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K45" t="n">
-        <v>10000</v>
+        <v>1396224</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3732,37 +3732,37 @@
         <v>1</v>
       </c>
       <c r="N45" t="n">
-        <v>0.0008</v>
+        <v>0.0089</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0008</v>
+        <v>0.0089</v>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
+          <t>https://www.lcsc.com/product-detail/C25779.html</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>R14 R15 R17 R18 R73 R74</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>33k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3772,12 +3772,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>C25779</t>
+          <t>C25900</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>0402WGF3302TCE</t>
+          <t>0402WGF4701TCE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3796,46 +3796,46 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>1415070</v>
+        <v>17779970</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N46" t="n">
-        <v>0.0089</v>
+        <v>0.0028</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0089</v>
+        <v>0.0168</v>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25779.html</t>
+          <t>https://www.lcsc.com/product-detail/C25900.html</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>R14 R15 R17 R18 R73 R74</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>47k</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3845,12 +3845,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>C25900</t>
+          <t>C25792</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>0402WGF4701TCE</t>
+          <t>0402WGF4702TCE</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3869,46 +3869,46 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>17901470</v>
+        <v>5977543</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N47" t="n">
-        <v>0.0028</v>
+        <v>0.0026</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0168</v>
+        <v>0.0026</v>
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25900.html</t>
+          <t>https://www.lcsc.com/product-detail/C25792.html</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R1 R4 R9 R11</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>47k</t>
+          <t>5.1k</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3918,12 +3918,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>C25792</t>
+          <t>C25905</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>0402WGF4702TCE</t>
+          <t>0402WGF5101TCE</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -3942,46 +3942,46 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>6022781</v>
+        <v>7262782</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N48" t="n">
-        <v>0.0026</v>
+        <v>0.0024</v>
       </c>
       <c r="O48" t="n">
-        <v>0.0026</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25792.html</t>
+          <t>https://www.lcsc.com/product-detail/C25905.html</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>R1 R4 R9 R11</t>
+          <t>R22 R50</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C49" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>5.1k</t>
+          <t>511k</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3991,17 +3991,17 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>C25905</t>
+          <t>C49655223</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>0402WGF5101TCE</t>
+          <t>GR0402F511KTAG00</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4011,50 +4011,50 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K49" t="n">
-        <v>7311984</v>
+        <v>7820</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N49" t="n">
-        <v>0.0024</v>
+        <v>0.0008</v>
       </c>
       <c r="O49" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0016</v>
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25905.html</t>
+          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>R22 R50</t>
+          <t>R56</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>511k</t>
+          <t>51k</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4064,17 +4064,17 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C49655223</t>
+          <t>C25794</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>GR0402F511KTAG00</t>
+          <t>0402WGF5102TCE</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4084,50 +4084,50 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K50" t="n">
-        <v>7820</v>
+        <v>2219352</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N50" t="n">
-        <v>0.0008</v>
+        <v>0.0018</v>
       </c>
       <c r="O50" t="n">
-        <v>0.0016</v>
+        <v>0.0018</v>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
+          <t>https://www.lcsc.com/product-detail/C25794.html</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 51kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>R56</t>
+          <t>R24 R55</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>51k</t>
+          <t>91k</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -4137,17 +4137,17 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>C25794</t>
+          <t>C54920709</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>0402WGF5102TCE</t>
+          <t>HRC0402F9102DNTO</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4157,75 +4157,75 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K51" t="n">
-        <v>2237445</v>
+        <v>132322</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N51" t="n">
-        <v>0.0018</v>
+        <v>0.0007</v>
       </c>
       <c r="O51" t="n">
-        <v>0.0018</v>
+        <v>0.0014</v>
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25794.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 51kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>R24 R55</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>91k</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>RES_0402</t>
+          <t>RGT0016C_V</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C54920709</t>
+          <t>C129319</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>HRC0402F9102DNTO</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>QFN-16-EP(3x3)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -4234,61 +4234,61 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>132322</v>
+        <v>382</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>0.0007</v>
+        <v>2.1672</v>
       </c>
       <c r="O52" t="n">
-        <v>0.0014</v>
+        <v>2.1672</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
+          <t>https://www.lcsc.com/product-detail/C129319.html</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>U14 U15</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>TPS61160DRVR</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>RGT0016C_V</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C129319</t>
+          <t>C165143</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>TPS61160DRVR</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>QFN-16-EP(3x3)</t>
+          <t>WSON-6-EP(2x2)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4307,35 +4307,35 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>382</v>
+        <v>11619</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>2.1672</v>
+        <v>0.4482</v>
       </c>
       <c r="O53" t="n">
-        <v>2.1672</v>
+        <v>0.8964</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C129319.html</t>
+          <t>https://www.lcsc.com/product-detail/C165143.html</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
+          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over Current Protection、Over-Temperature</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>U14 U15</t>
+          <t>USBC1 USBC2</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -4346,32 +4346,32 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>TPS61160DRVR</t>
+          <t>type-c-31-m-12</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>C165143</t>
+          <t>C165948</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>TPS61160DRVR</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Korean Hroparts Elec</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>WSON-6-EP(2x2)</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>11619</v>
+        <v>222877</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4389,62 +4389,62 @@
         <v>2</v>
       </c>
       <c r="N54" t="n">
-        <v>0.4482</v>
+        <v>0.179</v>
       </c>
       <c r="O54" t="n">
-        <v>0.8964</v>
+        <v>0.358</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165143.html</t>
+          <t>https://www.lcsc.com/product-detail/C165948.html</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over Current Protection、Over-Temperature</t>
+          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>USBC1 USBC2</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>type-c-31-m-12</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>C3035748</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>CH340X</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Korean Hroparts Elec</t>
+          <t>WCH(Jiangsu Qin Heng)</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>MSOP-10</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4453,35 +4453,35 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>229198</v>
+        <v>21784</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N55" t="n">
-        <v>0.179</v>
+        <v>0.6629</v>
       </c>
       <c r="O55" t="n">
-        <v>0.358</v>
+        <v>0.6629</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165948.html</t>
+          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
+          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -4492,32 +4492,32 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>msm381acb026</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>mems</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>C3035748</t>
+          <t>C51928208</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>CH340X</t>
+          <t>MSM381ACB026</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>WCH(Jiangsu Qin Heng)</t>
+          <t>MEMS</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>MSOP-10</t>
+          <t>LGA-3(1.9x2.8)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -4526,7 +4526,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>24377</v>
+        <v>6264</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
@@ -4535,26 +4535,26 @@
         <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>0.6629</v>
+        <v>0.3025</v>
       </c>
       <c r="O56" t="n">
-        <v>0.6629</v>
+        <v>0.3025</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
+          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
+          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -4565,32 +4565,32 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>msm381acb026</t>
+          <t>w25n02kvzeir</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>mems</t>
+          <t>w25n02</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>C51928208</t>
+          <t>C3010298</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>MSM381ACB026</t>
+          <t>W25N02KVZEIR</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>MEMS</t>
+          <t>Winbond Elec</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>LGA-3(1.9x2.8)</t>
+          <t>WSON-8-EP(6x8)</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="K57" t="n">
-        <v>6284</v>
+        <v>6271</v>
       </c>
       <c r="L57" t="n">
         <v>1</v>
@@ -4608,26 +4608,26 @@
         <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>0.3025</v>
+        <v>11.0584</v>
       </c>
       <c r="O57" t="n">
-        <v>0.3025</v>
+        <v>11.0584</v>
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
+          <t>https://www.lcsc.com/product-detail/C3010298.html</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
+          <t xml:space="preserve">-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function、ECC </t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>B1_N</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -4638,69 +4638,31 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>w25n02kvzeir</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>w25n02</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>C3010298</t>
-        </is>
-      </c>
+          <t>TESTP</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>W25N02KVZEIR</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>Winbond Elec</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>WSON-8-EP(6x8)</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="K58" t="n">
-        <v>6276</v>
-      </c>
-      <c r="L58" t="n">
-        <v>1</v>
-      </c>
-      <c r="M58" t="n">
-        <v>1</v>
-      </c>
-      <c r="N58" t="n">
-        <v>11.0584</v>
-      </c>
-      <c r="O58" t="n">
-        <v>11.0584</v>
-      </c>
-      <c r="P58" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lcsc.com/product-detail/C3010298.html</t>
-        </is>
-      </c>
-      <c r="Q58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function、ECC </t>
-        </is>
-      </c>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>B1_N</t>
+          <t>B1_P</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -4735,7 +4697,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>B1_P</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -4746,7 +4708,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>TESTP</t>
+          <t>Connector 2PIn</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -4770,7 +4732,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -4805,7 +4767,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>JB1</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -4840,7 +4802,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>JB1</t>
+          <t>JB2</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -4875,7 +4837,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>JB2</t>
+          <t>JT</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -4910,7 +4872,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>JT</t>
+          <t>ANT1</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -4921,7 +4883,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Connector 2PIn</t>
+          <t>MIFI</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -4945,7 +4907,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ANT1</t>
+          <t>PR1</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -4956,7 +4918,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>MIFI</t>
+          <t>CON5P</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -4984,7 +4946,7 @@
         </is>
       </c>
       <c r="O68" t="n">
-        <v>41.64</v>
+        <v>41.17</v>
       </c>
     </row>
   </sheetData>
@@ -5045,7 +5007,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P58" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Regenerate fabrication and assembly files from the 21:49 export
Gerber zip now uses Altium's own MIFA.GKO (board outline plus the four 0.6 mm USB
peg cutouts). Drill files carry a non-plated section: 0.5 mm acoustic port under
U13 and the 2.6 mm mounting hole. PickPlace_MIFA.csv and BOM_ASSEMBLY.csv
regenerated, cross-checked against the schematic and the ODB++, 215 placements.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3187778</v>
+        <v>3188618</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>14404501</v>
+        <v>14392012</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3923839</v>
+        <v>3925431</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1549543</v>
+        <v>1549549</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>840006</v>
+        <v>839926</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2990724</v>
+        <v>2990674</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>850087</v>
+        <v>849130</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>619497</v>
+        <v>609256</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2612863</v>
+        <v>2614184</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>6828</v>
+        <v>6826</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>13026526</v>
+        <v>13033540</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>7560850</v>
+        <v>7540359</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>9767291</v>
+        <v>9772141</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>957154</v>
+        <v>958138</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>2682603</v>
+        <v>2682633</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>3517887</v>
+        <v>3497544</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>472945</v>
+        <v>452451</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>893873</v>
+        <v>883677</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>8659872</v>
+        <v>8660125</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>832890</v>
+        <v>832900</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2470541</v>
+        <v>2470616</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>11170242</v>
+        <v>11099684</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>27499771</v>
+        <v>27492710</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>800156</v>
+        <v>800196</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>2677881</v>
+        <v>2688779</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>11624377</v>
+        <v>11583219</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2962356</v>
+        <v>2966289</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2206703</v>
+        <v>2206853</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1723021</v>
+        <v>1730247</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>6344847</v>
+        <v>6323962</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>1396224</v>
+        <v>1396555</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>17779970</v>
+        <v>17766646</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>5977543</v>
+        <v>5977878</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>7262782</v>
+        <v>7261083</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>2219352</v>
+        <v>2212922</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>222877</v>
+        <v>222841</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>21784</v>
+        <v>21764</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Fabrication and assembly files from the 22:42 export
USB locating posts are now drilled: T06, 0.6 mm, non-plated, four holes; the keep-out
layer carries only the board edge, so the outline gerber needs nothing but the profile.
Drill files in the zip are byte-identical to the export. 215 placements, 55 part numbers,
cross-checks against schematic and board clean.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>45446</v>
+        <v>45450</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3188618</v>
+        <v>3188549</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>14392012</v>
+        <v>14351282</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3925431</v>
+        <v>3925365</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1549549</v>
+        <v>1549379</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>839926</v>
+        <v>835279</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2990674</v>
+        <v>2989668</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>609256</v>
+        <v>618575</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2614184</v>
+        <v>2614179</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>13033540</v>
+        <v>13033384</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>7540359</v>
+        <v>7559232</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>9772141</v>
+        <v>9772219</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>3497544</v>
+        <v>3495181</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>452451</v>
+        <v>469978</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>883677</v>
+        <v>887354</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>8660125</v>
+        <v>8660040</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>832900</v>
+        <v>832850</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>15701</v>
+        <v>15696</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2470616</v>
+        <v>2470586</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>11099684</v>
+        <v>11149291</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>27492710</v>
+        <v>27454594</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>800196</v>
+        <v>796286</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>2688779</v>
+        <v>2678324</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>11583219</v>
+        <v>11613658</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2966289</v>
+        <v>2966287</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2206853</v>
+        <v>2206823</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1730247</v>
+        <v>1694210</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>6323962</v>
+        <v>6282907</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>1396555</v>
+        <v>1396520</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>17766646</v>
+        <v>17780516</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>5977878</v>
+        <v>5977701</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>7261083</v>
+        <v>7248185</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>2212922</v>
+        <v>2223008</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>132322</v>
+        <v>132302</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>222841</v>
+        <v>222840</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>21764</v>
+        <v>21784</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Fabrication and assembly package from the 05:46 export
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>45450</v>
+        <v>45414</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -593,10 +593,10 @@
         <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>0.7663</v>
+        <v>0.7665999999999999</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7663</v>
+        <v>0.7665999999999999</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -666,10 +666,10 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>2.2017</v>
+        <v>2.2026</v>
       </c>
       <c r="O3" t="n">
-        <v>2.2017</v>
+        <v>2.2026</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3188549</v>
+        <v>3163620</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -739,10 +739,10 @@
         <v>2</v>
       </c>
       <c r="N4" t="n">
-        <v>0.0384</v>
+        <v>0.0385</v>
       </c>
       <c r="O4" t="n">
-        <v>0.07679999999999999</v>
+        <v>0.077</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>14351282</v>
+        <v>16113898</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3925365</v>
+        <v>3905748</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1549379</v>
+        <v>1545402</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>835279</v>
+        <v>832606</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2989668</v>
+        <v>2933468</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>849130</v>
+        <v>843802</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>618575</v>
+        <v>617542</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1396,10 +1396,10 @@
         <v>2</v>
       </c>
       <c r="N13" t="n">
-        <v>0.1655</v>
+        <v>0.1656</v>
       </c>
       <c r="O13" t="n">
-        <v>0.331</v>
+        <v>0.3312</v>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2614179</v>
+        <v>2579248</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>8911</v>
+        <v>8906</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1542,10 +1542,10 @@
         <v>5</v>
       </c>
       <c r="N15" t="n">
-        <v>0.1715</v>
+        <v>0.1716</v>
       </c>
       <c r="O15" t="n">
-        <v>0.8575</v>
+        <v>0.858</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>6826</v>
+        <v>6824</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
@@ -1688,10 +1688,10 @@
         <v>3</v>
       </c>
       <c r="N17" t="n">
-        <v>0.981</v>
+        <v>0.9814000000000001</v>
       </c>
       <c r="O17" t="n">
-        <v>2.943</v>
+        <v>2.9442</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>8340</v>
+        <v>8346</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -1761,10 +1761,10 @@
         <v>2</v>
       </c>
       <c r="N18" t="n">
-        <v>1.086</v>
+        <v>1.0864</v>
       </c>
       <c r="O18" t="n">
-        <v>2.172</v>
+        <v>2.1728</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>13033384</v>
+        <v>12931444</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>7559232</v>
+        <v>7456850</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>9772219</v>
+        <v>9755589</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>958138</v>
+        <v>956751</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>2682633</v>
+        <v>2682598</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>3495181</v>
+        <v>3468438</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>469978</v>
+        <v>445438</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>887354</v>
+        <v>854856</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2345,10 +2345,10 @@
         <v>2</v>
       </c>
       <c r="N26" t="n">
-        <v>0.0815</v>
+        <v>0.08160000000000001</v>
       </c>
       <c r="O26" t="n">
-        <v>0.163</v>
+        <v>0.1632</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>8660040</v>
+        <v>8631377</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>832850</v>
+        <v>831898</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2628,7 +2628,7 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>24240</v>
+        <v>24226</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
@@ -2710,10 +2710,10 @@
         <v>3</v>
       </c>
       <c r="N31" t="n">
-        <v>0.2125</v>
+        <v>0.2126</v>
       </c>
       <c r="O31" t="n">
-        <v>0.6375</v>
+        <v>0.6378</v>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
@@ -2783,10 +2783,10 @@
         <v>1</v>
       </c>
       <c r="N32" t="n">
-        <v>13.3007</v>
+        <v>13.3061</v>
       </c>
       <c r="O32" t="n">
-        <v>13.3007</v>
+        <v>13.3061</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2470586</v>
+        <v>2434898</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>11149291</v>
+        <v>11111322</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>27454594</v>
+        <v>27277162</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>796286</v>
+        <v>796066</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>2678324</v>
+        <v>2668015</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>11613658</v>
+        <v>11559774</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2966287</v>
+        <v>2963937</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2206823</v>
+        <v>2202256</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1694210</v>
+        <v>1687847</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>6282907</v>
+        <v>6255755</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>343998</v>
+        <v>343398</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>1396520</v>
+        <v>1394858</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>17780516</v>
+        <v>17734674</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>5977701</v>
+        <v>5929637</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>7248185</v>
+        <v>7263196</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>2223008</v>
+        <v>2219425</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
@@ -4243,10 +4243,10 @@
         <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>2.1672</v>
+        <v>2.1681</v>
       </c>
       <c r="O52" t="n">
-        <v>2.1672</v>
+        <v>2.1681</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
@@ -4316,10 +4316,10 @@
         <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>0.4482</v>
+        <v>0.4484</v>
       </c>
       <c r="O53" t="n">
-        <v>0.8964</v>
+        <v>0.8968</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>222840</v>
+        <v>219915</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4389,10 +4389,10 @@
         <v>2</v>
       </c>
       <c r="N54" t="n">
-        <v>0.179</v>
+        <v>0.1791</v>
       </c>
       <c r="O54" t="n">
-        <v>0.358</v>
+        <v>0.3582</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>21784</v>
+        <v>21712</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4462,10 +4462,10 @@
         <v>1</v>
       </c>
       <c r="N55" t="n">
-        <v>0.6629</v>
+        <v>0.6632</v>
       </c>
       <c r="O55" t="n">
-        <v>0.6629</v>
+        <v>0.6632</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
@@ -4535,10 +4535,10 @@
         <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>0.3025</v>
+        <v>0.3026</v>
       </c>
       <c r="O56" t="n">
-        <v>0.3025</v>
+        <v>0.3026</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="K57" t="n">
-        <v>6271</v>
+        <v>6091</v>
       </c>
       <c r="L57" t="n">
         <v>1</v>
@@ -4608,10 +4608,10 @@
         <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>11.0584</v>
+        <v>11.0628</v>
       </c>
       <c r="O57" t="n">
-        <v>11.0584</v>
+        <v>11.0628</v>
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
@@ -4946,7 +4946,7 @@
         </is>
       </c>
       <c r="O68" t="n">
-        <v>41.17</v>
+        <v>41.19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
LCSC order for one hand-built board: 55 lines in the cart, 20% spare on cheap passives
U16 NAND -> C17626844, the other LCSC code for W25N02KVZEIR: it has single-piece
marketplace offers at 8.98 USD, while C3010298 is LCSC-own only with an 8-piece
minimum (92.68 USD). C86 1uF 0603 -> C696901 (C15849 out of stock at LCSC).
FB4 -> BLM18PG121SN1D, same 0603 part as FB1-FB3 (GZ1608D601TF is not sold by
lcsc.com); 120 ohm instead of 600 ohm on the microphone bias filter.
Cart total about 53.80 USD. Cart script parks the tab on a stable page and retries
when lcsc.com navigates under it; the launcher takes a URL.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q68"/>
+  <dimension ref="A1:Q67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>45414</v>
+        <v>45329</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3163620</v>
+        <v>3148979</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>16113898</v>
+        <v>13659974</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -885,10 +885,10 @@
         <v>12</v>
       </c>
       <c r="N6" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0097</v>
       </c>
       <c r="O6" t="n">
-        <v>0.102</v>
+        <v>0.1164</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3905748</v>
+        <v>3858379</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1545402</v>
+        <v>1518263</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>832606</v>
+        <v>826630</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2933468</v>
+        <v>2936052</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>843802</v>
+        <v>841582</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>617542</v>
+        <v>615179</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1415,33 +1415,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FB1 FB2 FB3</t>
+          <t>L1 L2 L3 L4 L5</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>BLM18PG121SN1D</t>
+          <t>DFE201612E-R47M=P2</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FP-BLM18-0_15-t0_8-IPC_B</t>
+          <t>FP-DFE201612C-IPC_C</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>C14709</t>
+          <t>C668312</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>BLM18PG121SN1D</t>
+          <t>DFE201612E-R47M=P2</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1451,70 +1451,70 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0806</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2579248</v>
+        <v>8899</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N14" t="n">
-        <v>0.0151</v>
+        <v>0.1716</v>
       </c>
       <c r="O14" t="n">
-        <v>0.0453</v>
+        <v>0.858</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C14709.html</t>
+          <t>https://www.lcsc.com/product-detail/C668312.html</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 1 120Ω@100MHz 2A 50mΩ ±25% 0603 Ferrite Beads ROHS</t>
+          <t>26mΩ 4.5A 470nH 5.5A ±20% 0806 Power Inductors ROHS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>L1 L2 L3 L4 L5</t>
+          <t>L6 L7</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>DFE201612E-R47M=P2</t>
+          <t>DFE252012F-100M=P2</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FP-DFE201612C-IPC_C</t>
+          <t>FP-DFE252012C-IPC_B</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>C668312</t>
+          <t>C703141</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>DFE201612E-R47M=P2</t>
+          <t>DFE252012F-100M=P2</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>0806</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1533,71 +1533,71 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>8906</v>
+        <v>17841</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N15" t="n">
-        <v>0.1716</v>
+        <v>0.1541</v>
       </c>
       <c r="O15" t="n">
-        <v>0.858</v>
+        <v>0.3082</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C668312.html</t>
+          <t>https://www.lcsc.com/product-detail/C703141.html</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>26mΩ 4.5A 470nH 5.5A ±20% 0806 Power Inductors ROHS</t>
+          <t>1.4A 10uH 400mΩ 950mA ±20% 1008 Power Inductors ROHS</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>L6 L7</t>
+          <t>U5 U8 U10</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>DFE252012F-100M=P2</t>
+          <t>TPS63802DLAR</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FP-DFE252012C-IPC_B</t>
+          <t>FP-DLA0010A-MFG</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C703141</t>
+          <t>C2845237</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>DFE252012F-100M=P2</t>
+          <t>TPS63802DLAR</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Murata Electronics</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1008</t>
+          <t>VSON-10(2x3)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1606,61 +1606,61 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>17860</v>
+        <v>6818</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N16" t="n">
-        <v>0.1541</v>
+        <v>0.9814000000000001</v>
       </c>
       <c r="O16" t="n">
-        <v>0.3082</v>
+        <v>2.9442</v>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C703141.html</t>
+          <t>https://www.lcsc.com/product-detail/C2845237.html</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>1.4A 10uH 400mΩ 950mA ±20% 1008 Power Inductors ROHS</t>
+          <t>-40℃~+125℃@(TJ) 1 1.3V~5.5V 1.4MHz、1.6MHz、2.1MHz 1.8V~5.2V 11uA 2A Adjustable Buck-Boost Buck-Boost Built-in Yes VSON-10</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>U5 U8 U10</t>
+          <t>U6 U7</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TPS63802DLAR</t>
+          <t>TPS62823DLCR</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FP-DLA0010A-MFG</t>
+          <t>FP-DLC0008A-MFG</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>C2845237</t>
+          <t>C2693497</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>TPS63802DLAR</t>
+          <t>TPS62823DLCR</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>VSON-10(2x3)</t>
+          <t>VSON-8(1.5x2)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1679,119 +1679,119 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>6824</v>
+        <v>8341</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N17" t="n">
-        <v>0.9814000000000001</v>
+        <v>1.0864</v>
       </c>
       <c r="O17" t="n">
-        <v>2.9442</v>
+        <v>2.1728</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2845237.html</t>
+          <t>https://www.lcsc.com/product-detail/C2693497.html</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>-40℃~+125℃@(TJ) 1 1.3V~5.5V 1.4MHz、1.6MHz、2.1MHz 1.8V~5.2V 11uA 2A Adjustable Buck-Boost Buck-Boost Built-in Yes VSON-10</t>
+          <t xml:space="preserve">-40℃~+125℃@(TJ) 1 2.2MHz 2.4V~5.5V 3A 4uA 600mV~4V Adjustable Buck Built-in Overcurrent Protection、Light load efficient </t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>U6 U7</t>
+          <t>C2 C3 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>TPS62823DLCR</t>
+          <t>10uF GRM188R61A106ME69D</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FP-DLC0008A-MFG</t>
+          <t>FP-GRM188-0_15-MFG</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>C2693497</t>
+          <t>C19702</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>TPS62823DLCR</t>
+          <t>CL10A106KP8NNNC</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>VSON-8(1.5x2)</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K18" t="n">
-        <v>8346</v>
+        <v>12898031</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="N18" t="n">
-        <v>1.0864</v>
+        <v>0.0308</v>
       </c>
       <c r="O18" t="n">
-        <v>2.1728</v>
+        <v>0.4004</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2693497.html</t>
+          <t>https://www.lcsc.com/product-detail/C19702.html</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t xml:space="preserve">-40℃~+125℃@(TJ) 1 2.2MHz 2.4V~5.5V 3A 4uA 600mV~4V Adjustable Buck Built-in Overcurrent Protection、Light load efficient </t>
+          <t>10V 10uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C2 C3 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106</t>
+          <t>C86</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10uF GRM188R61A106ME69D</t>
+          <t>1uF 0603</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1801,17 +1801,17 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>C19702</t>
+          <t>C696901</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>CL10A106KP8NNNC</t>
+          <t>TCC0603X5R105K160CT</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Samsung Electro-Mechanics</t>
+          <t>CCTC</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1821,65 +1821,65 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K19" t="n">
-        <v>12931444</v>
+        <v>594601</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="N19" t="n">
-        <v>0.0308</v>
+        <v>0.0086</v>
       </c>
       <c r="O19" t="n">
-        <v>0.4004</v>
+        <v>0.0086</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C19702.html</t>
+          <t>https://www.lcsc.com/product-detail/C696901.html</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>10V 10uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>16V 1uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C86</t>
+          <t>C14 C17 C18 C20 C87 C89</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1uF 0603</t>
+          <t>22uF GRM188R60J226MEA0J</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FP-GRM188-0_15-MFG</t>
+          <t>FP-GRM188-0_2-IPC_C</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>C15849</t>
+          <t>C59461</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>CL10A105KB8NNNC</t>
+          <t>CL10A226MQ8NRNC</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1898,66 +1898,66 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>7456850</v>
+        <v>9747290</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N20" t="n">
-        <v>0.0165</v>
+        <v>0.03</v>
       </c>
       <c r="O20" t="n">
-        <v>0.0165</v>
+        <v>0.18</v>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C15849.html</t>
+          <t>https://www.lcsc.com/product-detail/C59461.html</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>1uF 50V X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>22uF 6.3V X5R ±20% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>C14 C17 C18 C20 C87 C89</t>
+          <t>FB1 FB2 FB3 FB4</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>22uF GRM188R60J226MEA0J</t>
+          <t>BLM18PG121SN1D</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FP-GRM188-0_2-IPC_C</t>
+          <t>FP-MMZ0603-MFG</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>C59461</t>
+          <t>C14709</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>CL10A226MQ8NRNC</t>
+          <t>BLM18PG121SN1D</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Samsung Electro-Mechanics</t>
+          <t>Murata Electronics</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1971,181 +1971,181 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>9755589</v>
+        <v>2571527</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N21" t="n">
-        <v>0.03</v>
+        <v>0.0151</v>
       </c>
       <c r="O21" t="n">
-        <v>0.18</v>
+        <v>0.0604</v>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C59461.html</t>
+          <t>https://www.lcsc.com/product-detail/C14709.html</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>22uF 6.3V X5R ±20% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>-55℃~+125℃ 1 120Ω@100MHz 2A 50mΩ ±25% 0603 Ferrite Beads ROHS</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FB4</t>
+          <t>D2 D7 D8</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>GZ1608D601TF</t>
+          <t>DSK24</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FP-MMZ0603-MFG</t>
+          <t>FP-S8-V-3910_01-001-MFG</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>C1002</t>
+          <t>C22466352</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>GZ1608D601TF</t>
+          <t>DSK24</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Sunlord</t>
+          <t>hongjiacheng</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SOD-123FL</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Promo</t>
         </is>
       </c>
       <c r="K22" t="n">
-        <v>956751</v>
+        <v>2683178</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N22" t="n">
-        <v>0.019</v>
+        <v>0.0247</v>
       </c>
       <c r="O22" t="n">
-        <v>0.019</v>
+        <v>0.0741</v>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C1002.html</t>
+          <t>https://www.lcsc.com/product-detail/C22466352.html</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 1 200mA 450mΩ 600Ω@100MHz ±25% 0603 Ferrite Beads ROHS</t>
+          <t>-55℃~+125℃ 2A 40V 500uA@40V 50A 550mV@2A Standalone SOD-123FL Schottky Diodes ROHS</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>D2 D7 D8</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>DSK24</t>
+          <t>KT-0603R</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>FP-S8-V-3910_01-001-MFG</t>
+          <t>FP-SML-LX0603IW-TR-MFG</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>C22466352</t>
+          <t>C2286</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>DSK24</t>
+          <t>KT-0603R</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>hongjiacheng</t>
+          <t>Hubei KENTO Elec</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>SOD-123FL</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Promo</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K23" t="n">
-        <v>2682598</v>
+        <v>3451946</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N23" t="n">
-        <v>0.0247</v>
+        <v>0.0072</v>
       </c>
       <c r="O23" t="n">
-        <v>0.0741</v>
+        <v>0.0072</v>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22466352.html</t>
+          <t>https://www.lcsc.com/product-detail/C2286.html</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 2A 40V 500uA@40V 50A 550mV@2A Standalone SOD-123FL Schottky Diodes ROHS</t>
+          <t>-40℃~+85℃ 1.6mm x 0.8mm square LED 1.8V~2.4V 120° 20mA 300mcd 40mW 615nm~630nm 645nm Discrete Diode Red Water Clear 0603</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2156,32 +2156,32 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>KT-0603R</t>
+          <t>AO3401A</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>FP-SML-LX0603IW-TR-MFG</t>
+          <t>FP-SOT23-IPC_B</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>C2286</t>
+          <t>C15127</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>KT-0603R</t>
+          <t>AO3401A</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Hubei KENTO Elec</t>
+          <t>Alpha &amp; Omega Semicon</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>3468438</v>
+        <v>444384</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2199,52 +2199,52 @@
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0.0072</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0072</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2286.html</t>
+          <t>https://www.lcsc.com/product-detail/C15127.html</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1.6mm x 0.8mm square LED 1.8V~2.4V 120° 20mA 300mcd 40mW 615nm~630nm 645nm Discrete Diode Red Water Clear 0603</t>
+          <t>1 P-Channel 14nC@10V 30V 47mΩ@10V、60mΩ@4.5V、85mΩ@2.5V 4A 55pF 645pF 80pF 900mV SOT-23 MOSFETs ROHS</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q2 Q4</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>AO3401A</t>
+          <t>AO3400A</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>FP-SOT23-IPC_B</t>
+          <t>FP-SOT23-MFG</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>C15127</t>
+          <t>C20917</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>AO3401A</t>
+          <t>AO3400A</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2263,181 +2263,181 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>445438</v>
+        <v>853002</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N25" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.08160000000000001</v>
       </c>
       <c r="O25" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.1632</v>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C15127.html</t>
+          <t>https://www.lcsc.com/product-detail/C20917.html</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>1 P-Channel 14nC@10V 30V 47mΩ@10V、60mΩ@4.5V、85mΩ@2.5V 4A 55pF 645pF 80pF 900mV SOT-23 MOSFETs ROHS</t>
+          <t>-55℃~+150℃ 1 N-channel 1.45V 1.4W 30V 48mΩ@2.5V 5.7A 50pF 630pF 75pF 7nC@10V N-Channel SOT-23 MOSFETs ROHS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Q2 Q4</t>
+          <t>D3 D4 D5</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AO3400A</t>
+          <t>PRTR5V0U2F,115</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>FP-SOT23-MFG</t>
+          <t>FP-SOT886-MFG</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>C20917</t>
+          <t>C478118</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>AO3400A</t>
+          <t>PRTR5V0U2F,115</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Alpha &amp; Omega Semicon</t>
+          <t>Nexperia</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>XSON-6(1x1.5)</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K26" t="n">
-        <v>854856</v>
+        <v>60081</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N26" t="n">
-        <v>0.08160000000000001</v>
+        <v>0.103</v>
       </c>
       <c r="O26" t="n">
-        <v>0.1632</v>
+        <v>0.309</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C20917.html</t>
+          <t>https://www.lcsc.com/product-detail/C478118.html</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>-55℃~+150℃ 1 N-channel 1.45V 1.4W 30V 48mΩ@2.5V 5.7A 50pF 630pF 75pF 7nC@10V N-Channel SOT-23 MOSFETs ROHS</t>
+          <t>-40℃~+85℃ 100nA 1pF 2 5.5V 6V IEC 61000-4-2 TVS Unidirectional XSON-6(1x1.5) ESD and Surge Protection (TVS/ESD) ROHS</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D3 D4 D5</t>
+          <t>R68</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>PRTR5V0U2F,115</t>
+          <t>10R</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>FP-SOT886-MFG</t>
+          <t>FP-SR0603-MFG</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C478118</t>
+          <t>C22859</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>PRTR5V0U2F,115</t>
+          <t>0603WAF100JT5E</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Nexperia</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>XSON-6(1x1.5)</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K27" t="n">
-        <v>60131</v>
+        <v>8607876</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N27" t="n">
-        <v>0.103</v>
+        <v>0.0036</v>
       </c>
       <c r="O27" t="n">
-        <v>0.309</v>
+        <v>0.0036</v>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C478118.html</t>
+          <t>https://www.lcsc.com/product-detail/C22859.html</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 100nA 1pF 2 5.5V 6V IEC 61000-4-2 TVS Unidirectional XSON-6(1x1.5) ESD and Surge Protection (TVS/ESD) ROHS</t>
+          <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>R68</t>
+          <t>R66</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10R</t>
+          <t>4.7R</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2458,12 +2458,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C22859</t>
+          <t>C23164</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0603WAF100JT5E</t>
+          <t>0603WAF470KT5E</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>8631377</v>
+        <v>829211</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2491,26 +2491,26 @@
         <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>0.0036</v>
+        <v>0.0027</v>
       </c>
       <c r="O28" t="n">
-        <v>0.0036</v>
+        <v>0.0027</v>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22859.html</t>
+          <t>https://www.lcsc.com/product-detail/C23164.html</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100mW 4.7Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>R66</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2521,41 +2521,41 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4.7R</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>FP-SR0603-MFG</t>
+          <t>FP-XRCGB_F_N-MFG</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C23164</t>
+          <t>C2965580</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>0603WAF470KT5E</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>YXC Crystal Oscillators</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SMD2016-4P</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K29" t="n">
-        <v>831898</v>
+        <v>24168</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2564,62 +2564,62 @@
         <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>0.0027</v>
+        <v>0.0784</v>
       </c>
       <c r="O29" t="n">
-        <v>0.0027</v>
+        <v>0.0784</v>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C23164.html</t>
+          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 4.7Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Y2</t>
+          <t>S1 S2 S3</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>S2B-PH-K-S(LF)(SN)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>FP-XRCGB_F_N-MFG</t>
+          <t>JST-S2B-PH-K-S_V</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C2965580</t>
+          <t>C157932</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>S2B-PH-K-S-GW</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>YXC Crystal Oscillators</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>SMD2016-4P</t>
+          <t>Push-Pull,P=2mm</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2628,71 +2628,71 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>24226</v>
+        <v>15696</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N30" t="n">
-        <v>0.0784</v>
+        <v>0.2126</v>
       </c>
       <c r="O30" t="n">
-        <v>0.0784</v>
+        <v>0.6378</v>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
+          <t>https://www.lcsc.com/product-detail/C157932.html</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
+          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>S1 S2 S3</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S(LF)(SN)</t>
+          <t>k230d</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>JST-S2B-PH-K-S_V</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C157932</t>
+          <t>C42414902</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S-GW</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Canaan</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Push-Pull,P=2mm</t>
+          <t>BGA-256</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2701,119 +2701,119 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>15696</v>
+        <v>361</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N31" t="n">
-        <v>0.2126</v>
+        <v>13.3061</v>
       </c>
       <c r="O31" t="n">
-        <v>0.6378</v>
+        <v>13.3061</v>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C157932.html</t>
+          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
+          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>R5 R12</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>k230d</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>RES_0402</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C42414902</t>
+          <t>C25867</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>0402WGF1501TCE</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Canaan</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>BGA-256</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K32" t="n">
-        <v>361</v>
+        <v>2433127</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N32" t="n">
-        <v>13.3061</v>
+        <v>0.0028</v>
       </c>
       <c r="O32" t="n">
-        <v>13.3061</v>
+        <v>0.0056</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
+          <t>https://www.lcsc.com/product-detail/C25867.html</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
+          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>R5 R12</t>
+          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2823,12 +2823,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C25867</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0402WGF1501TCE</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2847,46 +2847,46 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2434898</v>
+        <v>11106200</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N33" t="n">
-        <v>0.0028</v>
+        <v>0.0024</v>
       </c>
       <c r="O33" t="n">
-        <v>0.0056</v>
+        <v>0.048</v>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25867.html</t>
+          <t>https://www.lcsc.com/product-detail/C25741.html</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
+          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C34" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2896,12 +2896,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C25744</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>0402WGF1003TCE</t>
+          <t>0402WGF1002TCE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2920,46 +2920,46 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>11111322</v>
+        <v>27241761</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N34" t="n">
-        <v>0.0024</v>
+        <v>0.003</v>
       </c>
       <c r="O34" t="n">
-        <v>0.048</v>
+        <v>0.054</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25741.html</t>
+          <t>https://www.lcsc.com/product-detail/C25744.html</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>120k</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2969,12 +2969,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C25744</t>
+          <t>C25750</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0402WGF1002TCE</t>
+          <t>0402WGF1203TCE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2989,50 +2989,50 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Promo</t>
         </is>
       </c>
       <c r="K35" t="n">
-        <v>27277162</v>
+        <v>794946</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
-        <v>0.003</v>
+        <v>0.0012</v>
       </c>
       <c r="O35" t="n">
-        <v>0.054</v>
+        <v>0.0012</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25744.html</t>
+          <t>https://www.lcsc.com/product-detail/C25750.html</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R71 R72</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>120k</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C25750</t>
+          <t>C26083</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>0402WGF1203TCE</t>
+          <t>0402WGF1004TCE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3062,50 +3062,50 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Promo</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K36" t="n">
-        <v>796066</v>
+        <v>2669920</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N36" t="n">
-        <v>0.0012</v>
+        <v>0.0023</v>
       </c>
       <c r="O36" t="n">
-        <v>0.0012</v>
+        <v>0.0046</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25750.html</t>
+          <t>https://www.lcsc.com/product-detail/C26083.html</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R71 R72</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3115,12 +3115,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C26083</t>
+          <t>C11702</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>0402WGF1004TCE</t>
+          <t>0402WGF1001TCE</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3139,46 +3139,46 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>2668015</v>
+        <v>11498424</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N37" t="n">
-        <v>0.0023</v>
+        <v>0.0021</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0046</v>
+        <v>0.0021</v>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C26083.html</t>
+          <t>https://www.lcsc.com/product-detail/C11702.html</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R37 R62</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>200R</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3188,12 +3188,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C11702</t>
+          <t>C25087</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0402WGF1001TCE</t>
+          <t>0402WGF2000TCE</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3212,46 +3212,46 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>11559774</v>
+        <v>2961683</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N38" t="n">
-        <v>0.0021</v>
+        <v>0.0028</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0021</v>
+        <v>0.0056</v>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C11702.html</t>
+          <t>https://www.lcsc.com/product-detail/C25087.html</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R37 R62</t>
+          <t>R59</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>200R</t>
+          <t>200k</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C25087</t>
+          <t>C25764</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0402WGF2000TCE</t>
+          <t>0402WGF2003TCE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3285,35 +3285,35 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2963937</v>
+        <v>2201352</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N39" t="n">
-        <v>0.0028</v>
+        <v>0.0019</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0056</v>
+        <v>0.0019</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25087.html</t>
+          <t>https://www.lcsc.com/product-detail/C25764.html</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>R59</t>
+          <t>R69</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>200k</t>
+          <t>20k</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3334,12 +3334,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>C25764</t>
+          <t>C25765</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>0402WGF2003TCE</t>
+          <t>0402WGF2002TCE</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2202256</v>
+        <v>1685692</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3367,26 +3367,26 @@
         <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>0.0019</v>
+        <v>0.0022</v>
       </c>
       <c r="O40" t="n">
-        <v>0.0019</v>
+        <v>0.0022</v>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25764.html</t>
+          <t>https://www.lcsc.com/product-detail/C25765.html</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 20kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>R69</t>
+          <t>R42</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>20k</t>
+          <t>22R</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3407,12 +3407,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>C25765</t>
+          <t>C25092</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>0402WGF2002TCE</t>
+          <t>0402WGF220JTCE</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1687847</v>
+        <v>6229772</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3440,37 +3440,37 @@
         <v>1</v>
       </c>
       <c r="N41" t="n">
-        <v>0.0022</v>
+        <v>0.0028</v>
       </c>
       <c r="O41" t="n">
-        <v>0.0022</v>
+        <v>0.0028</v>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25765.html</t>
+          <t>https://www.lcsc.com/product-detail/C25092.html</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 20kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>R42</t>
+          <t>R33 R46 R47 R48</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>22R</t>
+          <t>240R</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3480,17 +3480,17 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>C25092</t>
+          <t>C324768</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>0402WGF220JTCE</t>
+          <t>RC-02K2400FT</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3500,50 +3500,50 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K42" t="n">
-        <v>6255755</v>
+        <v>343298</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N42" t="n">
-        <v>0.0028</v>
+        <v>0.0013</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0028</v>
+        <v>0.0052</v>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25092.html</t>
+          <t>https://www.lcsc.com/product-detail/C324768.html</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>R33 R46 R47 R48</t>
+          <t>R63</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>240R</t>
+          <t>30k</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3553,17 +3553,17 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>C324768</t>
+          <t>C49653548</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>RC-02K2400FT</t>
+          <t>GR0402F30KTAG00</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>FH (Guangdong Fenghua Advanced Tech)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3577,35 +3577,35 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>343398</v>
+        <v>9900</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N43" t="n">
-        <v>0.0013</v>
+        <v>0.0008</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0052</v>
+        <v>0.0008</v>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C324768.html</t>
+          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>R63</t>
+          <t>R25</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -3616,7 +3616,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>30k</t>
+          <t>33k</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3626,17 +3626,17 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>C49653548</t>
+          <t>C25779</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>GR0402F30KTAG00</t>
+          <t>0402WGF3302TCE</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3646,11 +3646,11 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K44" t="n">
-        <v>9900</v>
+        <v>1394466</v>
       </c>
       <c r="L44" t="n">
         <v>1</v>
@@ -3659,37 +3659,37 @@
         <v>1</v>
       </c>
       <c r="N44" t="n">
-        <v>0.0008</v>
+        <v>0.0089</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0008</v>
+        <v>0.0089</v>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
+          <t>https://www.lcsc.com/product-detail/C25779.html</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>R14 R15 R17 R18 R73 R74</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>33k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3699,12 +3699,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>C25779</t>
+          <t>C25900</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>0402WGF3302TCE</t>
+          <t>0402WGF4701TCE</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3723,46 +3723,46 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>1394858</v>
+        <v>17710758</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N45" t="n">
-        <v>0.0089</v>
+        <v>0.0028</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0089</v>
+        <v>0.0168</v>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25779.html</t>
+          <t>https://www.lcsc.com/product-detail/C25900.html</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R14 R15 R17 R18 R73 R74</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C46" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>47k</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3772,12 +3772,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>C25900</t>
+          <t>C25792</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>0402WGF4701TCE</t>
+          <t>0402WGF4702TCE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3796,46 +3796,46 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>17734674</v>
+        <v>5930253</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N46" t="n">
-        <v>0.0028</v>
+        <v>0.0026</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0168</v>
+        <v>0.0026</v>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25900.html</t>
+          <t>https://www.lcsc.com/product-detail/C25792.html</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R1 R4 R9 R11</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C47" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>47k</t>
+          <t>5.1k</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3845,12 +3845,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>C25792</t>
+          <t>C25905</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>0402WGF4702TCE</t>
+          <t>0402WGF5101TCE</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3869,46 +3869,46 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>5929637</v>
+        <v>7233955</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N47" t="n">
-        <v>0.0026</v>
+        <v>0.0024</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0026</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25792.html</t>
+          <t>https://www.lcsc.com/product-detail/C25905.html</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>R1 R4 R9 R11</t>
+          <t>R22 R50</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>5.1k</t>
+          <t>511k</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3918,17 +3918,17 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>C25905</t>
+          <t>C49655223</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>0402WGF5101TCE</t>
+          <t>GR0402F511KTAG00</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3938,50 +3938,50 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K48" t="n">
-        <v>7263196</v>
+        <v>7820</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N48" t="n">
-        <v>0.0024</v>
+        <v>0.0008</v>
       </c>
       <c r="O48" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0016</v>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25905.html</t>
+          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>R22 R50</t>
+          <t>R56</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>511k</t>
+          <t>51k</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3991,17 +3991,17 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>C49655223</t>
+          <t>C25794</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>GR0402F511KTAG00</t>
+          <t>0402WGF5102TCE</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4011,50 +4011,50 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K49" t="n">
-        <v>7820</v>
+        <v>2216812</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N49" t="n">
-        <v>0.0008</v>
+        <v>0.0018</v>
       </c>
       <c r="O49" t="n">
-        <v>0.0016</v>
+        <v>0.0018</v>
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
+          <t>https://www.lcsc.com/product-detail/C25794.html</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 51kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>R56</t>
+          <t>R24 R55</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>51k</t>
+          <t>91k</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4064,17 +4064,17 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C25794</t>
+          <t>C54920709</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>0402WGF5102TCE</t>
+          <t>HRC0402F9102DNTO</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4084,75 +4084,75 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K50" t="n">
-        <v>2219425</v>
+        <v>132302</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N50" t="n">
-        <v>0.0018</v>
+        <v>0.0007</v>
       </c>
       <c r="O50" t="n">
-        <v>0.0018</v>
+        <v>0.0014</v>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25794.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 51kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>R24 R55</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>91k</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>RES_0402</t>
+          <t>RGT0016C_V</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>C54920709</t>
+          <t>C129319</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>HRC0402F9102DNTO</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>QFN-16-EP(3x3)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -4161,61 +4161,61 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>132302</v>
+        <v>382</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N51" t="n">
-        <v>0.0007</v>
+        <v>2.1681</v>
       </c>
       <c r="O51" t="n">
-        <v>0.0014</v>
+        <v>2.1681</v>
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
+          <t>https://www.lcsc.com/product-detail/C129319.html</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>U14 U15</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>TPS61160DRVR</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>RGT0016C_V</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C129319</t>
+          <t>C165143</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>TPS61160DRVR</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>QFN-16-EP(3x3)</t>
+          <t>WSON-6-EP(2x2)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -4234,35 +4234,35 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>382</v>
+        <v>11619</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>2.1681</v>
+        <v>0.4484</v>
       </c>
       <c r="O52" t="n">
-        <v>2.1681</v>
+        <v>0.8968</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C129319.html</t>
+          <t>https://www.lcsc.com/product-detail/C165143.html</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
+          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over Current Protection、Over-Temperature</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>U14 U15</t>
+          <t>USBC1 USBC2</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -4273,32 +4273,32 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>TPS61160DRVR</t>
+          <t>type-c-31-m-12</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C165143</t>
+          <t>C165948</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>TPS61160DRVR</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Korean Hroparts Elec</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>WSON-6-EP(2x2)</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>11619</v>
+        <v>218120</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
@@ -4316,62 +4316,62 @@
         <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>0.4484</v>
+        <v>0.1791</v>
       </c>
       <c r="O53" t="n">
-        <v>0.8968</v>
+        <v>0.3582</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165143.html</t>
+          <t>https://www.lcsc.com/product-detail/C165948.html</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over Current Protection、Over-Temperature</t>
+          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>USBC1 USBC2</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>type-c-31-m-12</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>C3035748</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>CH340X</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Korean Hroparts Elec</t>
+          <t>WCH(Jiangsu Qin Heng)</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>MSOP-10</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4380,35 +4380,35 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>219915</v>
+        <v>20176</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N54" t="n">
-        <v>0.1791</v>
+        <v>0.6632</v>
       </c>
       <c r="O54" t="n">
-        <v>0.3582</v>
+        <v>0.6632</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165948.html</t>
+          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
+          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -4419,32 +4419,32 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>msm381acb026</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>mems</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>C3035748</t>
+          <t>C51928208</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>CH340X</t>
+          <t>MSM381ACB026</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>WCH(Jiangsu Qin Heng)</t>
+          <t>MEMS</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>MSOP-10</t>
+          <t>LGA-3(1.9x2.8)</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>21712</v>
+        <v>6264</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4462,26 +4462,26 @@
         <v>1</v>
       </c>
       <c r="N55" t="n">
-        <v>0.6632</v>
+        <v>0.3026</v>
       </c>
       <c r="O55" t="n">
-        <v>0.6632</v>
+        <v>0.3026</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
+          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
+          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -4492,32 +4492,32 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>msm381acb026</t>
+          <t>w25n02kvzeir</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>mems</t>
+          <t>w25n02</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>C51928208</t>
+          <t>C17626844</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>MSM381ACB026</t>
+          <t>W25N02KVZEIR</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>MEMS</t>
+          <t>Winbond Elec</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>LGA-3(1.9x2.8)</t>
+          <t>WSON-8(6x8)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -4526,7 +4526,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>6264</v>
+        <v>7624</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
@@ -4535,26 +4535,26 @@
         <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>0.3026</v>
+        <v>11.1553</v>
       </c>
       <c r="O56" t="n">
-        <v>0.3026</v>
+        <v>11.1553</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
+          <t>https://www.lcsc.com/product-detail/C17626844.html</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
+          <t>-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 25ns 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>B1_N</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -4565,69 +4565,31 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>w25n02kvzeir</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>w25n02</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>C3010298</t>
-        </is>
-      </c>
+          <t>TESTP</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>W25N02KVZEIR</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>Winbond Elec</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>WSON-8-EP(6x8)</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="K57" t="n">
-        <v>6091</v>
-      </c>
-      <c r="L57" t="n">
-        <v>1</v>
-      </c>
-      <c r="M57" t="n">
-        <v>1</v>
-      </c>
-      <c r="N57" t="n">
-        <v>11.0628</v>
-      </c>
-      <c r="O57" t="n">
-        <v>11.0628</v>
-      </c>
-      <c r="P57" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lcsc.com/product-detail/C3010298.html</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function、ECC </t>
-        </is>
-      </c>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>B1_N</t>
+          <t>B1_P</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -4662,7 +4624,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>B1_P</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -4673,7 +4635,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>TESTP</t>
+          <t>Connector 2PIn</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -4697,7 +4659,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -4732,7 +4694,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>JB1</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -4767,7 +4729,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>JB1</t>
+          <t>JB2</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -4802,7 +4764,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>JB2</t>
+          <t>JT</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -4837,7 +4799,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>JT</t>
+          <t>ANT1</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -4848,7 +4810,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Connector 2PIn</t>
+          <t>MIFI</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -4872,7 +4834,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ANT1</t>
+          <t>PR1</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -4883,7 +4845,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>MIFI</t>
+          <t>CON5P</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -4904,49 +4866,14 @@
       <c r="P65" t="inlineStr"/>
       <c r="Q65" t="inlineStr"/>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>PR1</t>
-        </is>
-      </c>
-      <c r="B66" t="n">
-        <v>1</v>
-      </c>
-      <c r="C66" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>CON5P</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>NO PART</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
-      <c r="Q66" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
+    <row r="67">
+      <c r="A67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="O68" t="n">
-        <v>41.19</v>
+      <c r="O67" t="n">
+        <v>41.28</v>
       </c>
     </row>
   </sheetData>
@@ -5006,7 +4933,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fabrication and assembly package from the 18:54 export (FB4 on the 0603 land, inner ground extended to the antenna edge)
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>45329</v>
+        <v>42075</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -593,10 +593,10 @@
         <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>0.7665999999999999</v>
+        <v>0.7667</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7665999999999999</v>
+        <v>0.7667</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -666,10 +666,10 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>2.2026</v>
+        <v>2.2029</v>
       </c>
       <c r="O3" t="n">
-        <v>2.2026</v>
+        <v>2.2029</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>3148979</v>
+        <v>2789858</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>226657</v>
+        <v>176406</v>
       </c>
       <c r="L5" t="n">
         <v>1</v>
@@ -812,10 +812,10 @@
         <v>53</v>
       </c>
       <c r="N5" t="n">
-        <v>0.003</v>
+        <v>0.0021</v>
       </c>
       <c r="O5" t="n">
-        <v>0.159</v>
+        <v>0.1113</v>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>13659974</v>
+        <v>12969649</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -885,10 +885,10 @@
         <v>12</v>
       </c>
       <c r="N6" t="n">
-        <v>0.0097</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="O6" t="n">
-        <v>0.1164</v>
+        <v>0.1056</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3858379</v>
+        <v>3685337</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1518263</v>
+        <v>1303966</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1031,10 +1031,10 @@
         <v>2</v>
       </c>
       <c r="N8" t="n">
-        <v>0.0055</v>
+        <v>0.0054</v>
       </c>
       <c r="O8" t="n">
-        <v>0.011</v>
+        <v>0.0108</v>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>826630</v>
+        <v>764083</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2936052</v>
+        <v>2788449</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>841582</v>
+        <v>660890</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>615179</v>
+        <v>568081</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1415,33 +1415,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>L1 L2 L3 L4 L5</t>
+          <t>FB1 FB2 FB3 FB4</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>DFE201612E-R47M=P2</t>
+          <t>BLM18PG121SN1D</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FP-DFE201612C-IPC_C</t>
+          <t>FP-BLM18-0_15-t0_8-IPC_B</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>C668312</t>
+          <t>C14709</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>DFE201612E-R47M=P2</t>
+          <t>BLM18PG121SN1D</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1451,70 +1451,70 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>0806</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K14" t="n">
-        <v>8899</v>
+        <v>2350694</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N14" t="n">
-        <v>0.1716</v>
+        <v>0.0151</v>
       </c>
       <c r="O14" t="n">
-        <v>0.858</v>
+        <v>0.0604</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C668312.html</t>
+          <t>https://www.lcsc.com/product-detail/C14709.html</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>26mΩ 4.5A 470nH 5.5A ±20% 0806 Power Inductors ROHS</t>
+          <t>-55℃~+125℃ 1 120Ω@100MHz 2A 50mΩ ±25% 0603 Ferrite Beads ROHS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>L6 L7</t>
+          <t>L1 L2 L3 L4 L5</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>DFE252012F-100M=P2</t>
+          <t>DFE201612E-R47M=P2</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FP-DFE252012C-IPC_B</t>
+          <t>FP-DFE201612C-IPC_C</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>C703141</t>
+          <t>C668312</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>DFE252012F-100M=P2</t>
+          <t>DFE201612E-R47M=P2</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1008</t>
+          <t>0806</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1533,71 +1533,71 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>17841</v>
+        <v>8634</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N15" t="n">
-        <v>0.1541</v>
+        <v>0.1716</v>
       </c>
       <c r="O15" t="n">
-        <v>0.3082</v>
+        <v>0.858</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C703141.html</t>
+          <t>https://www.lcsc.com/product-detail/C668312.html</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.4A 10uH 400mΩ 950mA ±20% 1008 Power Inductors ROHS</t>
+          <t>26mΩ 4.5A 470nH 5.5A ±20% 0806 Power Inductors ROHS</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>U5 U8 U10</t>
+          <t>L6 L7</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>TPS63802DLAR</t>
+          <t>DFE252012F-100M=P2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FP-DLA0010A-MFG</t>
+          <t>FP-DFE252012C-IPC_B</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C2845237</t>
+          <t>C703141</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>TPS63802DLAR</t>
+          <t>DFE252012F-100M=P2</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Murata Electronics</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>VSON-10(2x3)</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1606,61 +1606,61 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>6818</v>
+        <v>16885</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N16" t="n">
-        <v>0.9814000000000001</v>
+        <v>0.1542</v>
       </c>
       <c r="O16" t="n">
-        <v>2.9442</v>
+        <v>0.3084</v>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2845237.html</t>
+          <t>https://www.lcsc.com/product-detail/C703141.html</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>-40℃~+125℃@(TJ) 1 1.3V~5.5V 1.4MHz、1.6MHz、2.1MHz 1.8V~5.2V 11uA 2A Adjustable Buck-Boost Buck-Boost Built-in Yes VSON-10</t>
+          <t>1.4A 10uH 400mΩ 950mA ±20% 1008 Power Inductors ROHS</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>U6 U7</t>
+          <t>U5 U8 U10</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TPS62823DLCR</t>
+          <t>TPS63802DLAR</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FP-DLC0008A-MFG</t>
+          <t>FP-DLA0010A-MFG</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>C2693497</t>
+          <t>C2845237</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>TPS62823DLCR</t>
+          <t>TPS63802DLAR</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>VSON-8(1.5x2)</t>
+          <t>VSON-10(2x3)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1679,119 +1679,119 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>8341</v>
+        <v>6884</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N17" t="n">
-        <v>1.0864</v>
+        <v>0.98</v>
       </c>
       <c r="O17" t="n">
-        <v>2.1728</v>
+        <v>2.94</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2693497.html</t>
+          <t>https://www.lcsc.com/product-detail/C2845237.html</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t xml:space="preserve">-40℃~+125℃@(TJ) 1 2.2MHz 2.4V~5.5V 3A 4uA 600mV~4V Adjustable Buck Built-in Overcurrent Protection、Light load efficient </t>
+          <t>-40℃~+125℃@(TJ) 1 1.3V~5.5V 1.4MHz、1.6MHz、2.1MHz 1.8V~5.2V 11uA 2A Adjustable Buck-Boost Buck-Boost Built-in Yes VSON-10</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C2 C3 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106</t>
+          <t>U6 U7</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10uF GRM188R61A106ME69D</t>
+          <t>TPS62823DLCR</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FP-GRM188-0_15-MFG</t>
+          <t>FP-DLC0008A-MFG</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>C19702</t>
+          <t>C2693497</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>CL10A106KP8NNNC</t>
+          <t>TPS62823DLCR</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Samsung Electro-Mechanics</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>VSON-8(1.5x2)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K18" t="n">
-        <v>12898031</v>
+        <v>8272</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="N18" t="n">
-        <v>0.0308</v>
+        <v>1.0866</v>
       </c>
       <c r="O18" t="n">
-        <v>0.4004</v>
+        <v>2.1732</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C19702.html</t>
+          <t>https://www.lcsc.com/product-detail/C2693497.html</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>10V 10uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t xml:space="preserve">-40℃~+125℃@(TJ) 1 2.2MHz 2.4V~5.5V 3A 4uA 600mV~4V Adjustable Buck Built-in Overcurrent Protection、Light load efficient </t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C86</t>
+          <t>C2 C3 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1uF 0603</t>
+          <t>10uF GRM188R61A106ME69D</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1801,17 +1801,17 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>C696901</t>
+          <t>C19702</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>TCC0603X5R105K160CT</t>
+          <t>CL10A106KP8NNNC</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>CCTC</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1821,70 +1821,70 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K19" t="n">
-        <v>594601</v>
+        <v>11625980</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="N19" t="n">
-        <v>0.0086</v>
+        <v>0.0308</v>
       </c>
       <c r="O19" t="n">
-        <v>0.0086</v>
+        <v>0.4004</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C696901.html</t>
+          <t>https://www.lcsc.com/product-detail/C19702.html</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>16V 1uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>10V 10uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C14 C17 C18 C20 C87 C89</t>
+          <t>C86</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>22uF GRM188R60J226MEA0J</t>
+          <t>1uF 0603</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FP-GRM188-0_2-IPC_C</t>
+          <t>FP-GRM188-0_15-MFG</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>C59461</t>
+          <t>C696901</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>CL10A226MQ8NRNC</t>
+          <t>TCC0603X5R105K160CT</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Samsung Electro-Mechanics</t>
+          <t>CCTC</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1894,70 +1894,70 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K20" t="n">
-        <v>9747290</v>
+        <v>425221</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N20" t="n">
-        <v>0.03</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="O20" t="n">
-        <v>0.18</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C59461.html</t>
+          <t>https://www.lcsc.com/product-detail/C696901.html</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>22uF 6.3V X5R ±20% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>16V 1uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FB1 FB2 FB3 FB4</t>
+          <t>C14 C17 C18 C20 C87 C89</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>BLM18PG121SN1D</t>
+          <t>22uF GRM188R60J226MEA0J</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FP-MMZ0603-MFG</t>
+          <t>FP-GRM188-0_2-IPC_C</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>C14709</t>
+          <t>C59461</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>BLM18PG121SN1D</t>
+          <t>CL10A226MQ8NRNC</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Murata Electronics</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1971,28 +1971,28 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>2571527</v>
+        <v>8791042</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N21" t="n">
-        <v>0.0151</v>
+        <v>0.03</v>
       </c>
       <c r="O21" t="n">
-        <v>0.0604</v>
+        <v>0.18</v>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C14709.html</t>
+          <t>https://www.lcsc.com/product-detail/C59461.html</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 1 120Ω@100MHz 2A 50mΩ ±25% 0603 Ferrite Beads ROHS</t>
+          <t>22uF 6.3V X5R ±20% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>2683178</v>
+        <v>2682008</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>3451946</v>
+        <v>2943361</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>444384</v>
+        <v>829838</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>853002</v>
+        <v>819062</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>60081</v>
+        <v>59416</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2345,10 +2345,10 @@
         <v>3</v>
       </c>
       <c r="N26" t="n">
-        <v>0.103</v>
+        <v>0.09370000000000001</v>
       </c>
       <c r="O26" t="n">
-        <v>0.309</v>
+        <v>0.2811</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>8607876</v>
+        <v>8816690</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -2418,10 +2418,10 @@
         <v>1</v>
       </c>
       <c r="N27" t="n">
-        <v>0.0036</v>
+        <v>0.0031</v>
       </c>
       <c r="O27" t="n">
-        <v>0.0036</v>
+        <v>0.0031</v>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>829211</v>
+        <v>763608</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2491,10 +2491,10 @@
         <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>0.0027</v>
+        <v>0.0025</v>
       </c>
       <c r="O28" t="n">
-        <v>0.0027</v>
+        <v>0.0025</v>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>24168</v>
+        <v>31564</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2628,7 +2628,7 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>15696</v>
+        <v>15627</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
@@ -2637,10 +2637,10 @@
         <v>3</v>
       </c>
       <c r="N30" t="n">
-        <v>0.2126</v>
+        <v>0.2127</v>
       </c>
       <c r="O30" t="n">
-        <v>0.6378</v>
+        <v>0.6381</v>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>361</v>
+        <v>351</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
@@ -2710,10 +2710,10 @@
         <v>1</v>
       </c>
       <c r="N31" t="n">
-        <v>13.3061</v>
+        <v>13.3081</v>
       </c>
       <c r="O31" t="n">
-        <v>13.3061</v>
+        <v>13.3081</v>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
@@ -2774,7 +2774,7 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>2433127</v>
+        <v>2285268</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>11106200</v>
+        <v>9640522</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>27241761</v>
+        <v>25360732</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2929,10 +2929,10 @@
         <v>18</v>
       </c>
       <c r="N34" t="n">
-        <v>0.003</v>
+        <v>0.0033</v>
       </c>
       <c r="O34" t="n">
-        <v>0.054</v>
+        <v>0.0594</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>794946</v>
+        <v>732376</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3002,10 +3002,10 @@
         <v>1</v>
       </c>
       <c r="N35" t="n">
-        <v>0.0012</v>
+        <v>0.0011</v>
       </c>
       <c r="O35" t="n">
-        <v>0.0012</v>
+        <v>0.0011</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>2669920</v>
+        <v>2810004</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3075,10 +3075,10 @@
         <v>2</v>
       </c>
       <c r="N36" t="n">
-        <v>0.0023</v>
+        <v>0.0025</v>
       </c>
       <c r="O36" t="n">
-        <v>0.0046</v>
+        <v>0.005</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>11498424</v>
+        <v>10288780</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2961683</v>
+        <v>2771586</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2201352</v>
+        <v>2667840</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3294,10 +3294,10 @@
         <v>1</v>
       </c>
       <c r="N39" t="n">
-        <v>0.0019</v>
+        <v>0.0017</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0019</v>
+        <v>0.0017</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1685692</v>
+        <v>1454309</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>6229772</v>
+        <v>3963119</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>343298</v>
+        <v>335656</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>9900</v>
+        <v>9140</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3650,7 +3650,7 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>1394466</v>
+        <v>1355483</v>
       </c>
       <c r="L44" t="n">
         <v>1</v>
@@ -3659,10 +3659,10 @@
         <v>1</v>
       </c>
       <c r="N44" t="n">
-        <v>0.0089</v>
+        <v>0.0056</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0089</v>
+        <v>0.0056</v>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>17710758</v>
+        <v>16736633</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3732,10 +3732,10 @@
         <v>6</v>
       </c>
       <c r="N45" t="n">
-        <v>0.0028</v>
+        <v>0.0026</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0168</v>
+        <v>0.0156</v>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>5930253</v>
+        <v>5939945</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3805,10 +3805,10 @@
         <v>1</v>
       </c>
       <c r="N46" t="n">
-        <v>0.0026</v>
+        <v>0.0025</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0026</v>
+        <v>0.0025</v>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>7233955</v>
+        <v>6739622</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -3878,10 +3878,10 @@
         <v>4</v>
       </c>
       <c r="N47" t="n">
-        <v>0.0024</v>
+        <v>0.0023</v>
       </c>
       <c r="O47" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0092</v>
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>7820</v>
+        <v>7800</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>2216812</v>
+        <v>2064635</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>132302</v>
+        <v>131182</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>382</v>
+        <v>367</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
@@ -4170,10 +4170,10 @@
         <v>1</v>
       </c>
       <c r="N51" t="n">
-        <v>2.1681</v>
+        <v>2.1684</v>
       </c>
       <c r="O51" t="n">
-        <v>2.1681</v>
+        <v>2.1684</v>
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
@@ -4234,7 +4234,7 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>11619</v>
+        <v>11609</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
@@ -4243,10 +4243,10 @@
         <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>0.4484</v>
+        <v>0.4485</v>
       </c>
       <c r="O52" t="n">
-        <v>0.8968</v>
+        <v>0.897</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>218120</v>
+        <v>108762</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>20176</v>
+        <v>17645</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4389,10 +4389,10 @@
         <v>1</v>
       </c>
       <c r="N54" t="n">
-        <v>0.6632</v>
+        <v>0.6633</v>
       </c>
       <c r="O54" t="n">
-        <v>0.6632</v>
+        <v>0.6633</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>6264</v>
+        <v>6244</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4535,10 +4535,10 @@
         <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>11.1553</v>
+        <v>11.157</v>
       </c>
       <c r="O56" t="n">
-        <v>11.1553</v>
+        <v>11.157</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
@@ -4873,7 +4873,7 @@
         </is>
       </c>
       <c r="O67" t="n">
-        <v>41.28</v>
+        <v>41.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fabrication and assembly package from the 22 Sep 16:04 export (antenna redesigned for the inner ground reference)
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>42075</v>
+        <v>41887</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -593,10 +593,10 @@
         <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>0.7667</v>
+        <v>0.767</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7667</v>
+        <v>0.767</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -666,10 +666,10 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>2.2029</v>
+        <v>2.2035</v>
       </c>
       <c r="O3" t="n">
-        <v>2.2029</v>
+        <v>2.2035</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2789858</v>
+        <v>2705630</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>12969649</v>
+        <v>12567866</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -885,10 +885,10 @@
         <v>12</v>
       </c>
       <c r="N6" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="O6" t="n">
-        <v>0.1056</v>
+        <v>0.1008</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3685337</v>
+        <v>3637569</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1303966</v>
+        <v>1276796</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>764083</v>
+        <v>749847</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2788449</v>
+        <v>2489223</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>660890</v>
+        <v>646720</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>568081</v>
+        <v>563798</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1396,10 +1396,10 @@
         <v>2</v>
       </c>
       <c r="N13" t="n">
-        <v>0.1656</v>
+        <v>0.1657</v>
       </c>
       <c r="O13" t="n">
-        <v>0.3312</v>
+        <v>0.3314</v>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2350694</v>
+        <v>2259510</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1469,10 +1469,10 @@
         <v>4</v>
       </c>
       <c r="N14" t="n">
-        <v>0.0151</v>
+        <v>0.0152</v>
       </c>
       <c r="O14" t="n">
-        <v>0.0604</v>
+        <v>0.0608</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>8634</v>
+        <v>8190</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1542,10 +1542,10 @@
         <v>5</v>
       </c>
       <c r="N15" t="n">
-        <v>0.1716</v>
+        <v>0.1717</v>
       </c>
       <c r="O15" t="n">
-        <v>0.858</v>
+        <v>0.8585</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>16885</v>
+        <v>16359</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>6884</v>
+        <v>18536</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
@@ -1688,10 +1688,10 @@
         <v>3</v>
       </c>
       <c r="N17" t="n">
-        <v>0.98</v>
+        <v>0.9802</v>
       </c>
       <c r="O17" t="n">
-        <v>2.94</v>
+        <v>2.9406</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>8272</v>
+        <v>8274</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -1761,10 +1761,10 @@
         <v>2</v>
       </c>
       <c r="N18" t="n">
-        <v>1.0866</v>
+        <v>1.0869</v>
       </c>
       <c r="O18" t="n">
-        <v>2.1732</v>
+        <v>2.1738</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>11625980</v>
+        <v>11371140</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>8791042</v>
+        <v>8659730</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>2682008</v>
+        <v>2663348</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>2943361</v>
+        <v>2844395</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>829838</v>
+        <v>807684</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2199,10 +2199,10 @@
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="O24" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>819062</v>
+        <v>809002</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>59416</v>
+        <v>58836</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>8816690</v>
+        <v>8720168</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>763608</v>
+        <v>758260</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>31564</v>
+        <v>30408</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2564,10 +2564,10 @@
         <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>0.0784</v>
+        <v>0.0785</v>
       </c>
       <c r="O29" t="n">
-        <v>0.0784</v>
+        <v>0.0785</v>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
@@ -2628,7 +2628,7 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>15627</v>
+        <v>15506</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
@@ -2710,10 +2710,10 @@
         <v>1</v>
       </c>
       <c r="N31" t="n">
-        <v>13.3081</v>
+        <v>13.3119</v>
       </c>
       <c r="O31" t="n">
-        <v>13.3081</v>
+        <v>13.3119</v>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
@@ -2774,7 +2774,7 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>2285268</v>
+        <v>2243481</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>9640522</v>
+        <v>9382870</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>25360732</v>
+        <v>24975907</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>732376</v>
+        <v>724600</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>2810004</v>
+        <v>2764269</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>10288780</v>
+        <v>9855951</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2771586</v>
+        <v>2753252</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2667840</v>
+        <v>2636190</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1454309</v>
+        <v>1404852</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>3963119</v>
+        <v>3782977</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>335656</v>
+        <v>322406</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>9140</v>
+        <v>8260</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3650,7 +3650,7 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>1355483</v>
+        <v>1347534</v>
       </c>
       <c r="L44" t="n">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>16736633</v>
+        <v>16540594</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>5939945</v>
+        <v>5871007</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>6739622</v>
+        <v>6679905</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>2064635</v>
+        <v>2035272</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>131182</v>
+        <v>130662</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>367</v>
+        <v>356</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
@@ -4170,10 +4170,10 @@
         <v>1</v>
       </c>
       <c r="N51" t="n">
-        <v>2.1684</v>
+        <v>2.169</v>
       </c>
       <c r="O51" t="n">
-        <v>2.1684</v>
+        <v>2.169</v>
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
@@ -4243,10 +4243,10 @@
         <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>0.4485</v>
+        <v>0.4486</v>
       </c>
       <c r="O52" t="n">
-        <v>0.897</v>
+        <v>0.8972</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>108762</v>
+        <v>105811</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
@@ -4316,10 +4316,10 @@
         <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>0.1791</v>
+        <v>0.1792</v>
       </c>
       <c r="O53" t="n">
-        <v>0.3582</v>
+        <v>0.3584</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>17645</v>
+        <v>16618</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4389,10 +4389,10 @@
         <v>1</v>
       </c>
       <c r="N54" t="n">
-        <v>0.6633</v>
+        <v>0.6634</v>
       </c>
       <c r="O54" t="n">
-        <v>0.6633</v>
+        <v>0.6634</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
@@ -4462,10 +4462,10 @@
         <v>1</v>
       </c>
       <c r="N55" t="n">
-        <v>0.3026</v>
+        <v>0.3027</v>
       </c>
       <c r="O55" t="n">
-        <v>0.3026</v>
+        <v>0.3027</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
@@ -4535,10 +4535,10 @@
         <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>11.157</v>
+        <v>11.1602</v>
       </c>
       <c r="O56" t="n">
-        <v>11.157</v>
+        <v>11.1602</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fabrication and assembly package from the 22 Sep 16:43 export (SOD-123FL land for the Schottky diodes)
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>41887</v>
+        <v>41885</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2705630</v>
+        <v>2704080</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>12567866</v>
+        <v>12551905</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3637569</v>
+        <v>3637497</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1276796</v>
+        <v>1274216</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>749847</v>
+        <v>749597</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1196,80 +1196,80 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>J4 J5</t>
+          <t>D2 D7 D8</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>05b20l22p</t>
+          <t>DSK24</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>FLEX_CON_22P</t>
+          <t>DSK24</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>C22459552</t>
+          <t>C22466352</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>05B20L22P</t>
+          <t>DSK24</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>HanElectricity</t>
+          <t>hongjiacheng</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>SMD,P=0.5mm,Surface Mount，Right Angle</t>
+          <t>SOD-123FL</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Promo</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>2004</v>
+        <v>2663348</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N11" t="n">
-        <v>0.0698</v>
+        <v>0.0247</v>
       </c>
       <c r="O11" t="n">
-        <v>0.1396</v>
+        <v>0.0741</v>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22459552.html</t>
+          <t>https://www.lcsc.com/product-detail/C22466352.html</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 0.3mm 0.5mm 22P 2mm 400mA 50V Bottom Contact Phosphor bronze Slide Lock Surface Mount, Right Angle Tin SMD,P=0</t>
+          <t>-55℃~+125℃ 2A 40V 500uA@40V 50A 550mV@2A Standalone SOD-123FL Schottky Diodes ROHS</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C1 C104</t>
+          <t>J4 J5</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1280,41 +1280,41 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1uF 50V 1206</t>
+          <t>05b20l22p</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>FP-1206-L_3_2_0_2-W_1_6_0-IPC_B</t>
+          <t>FLEX_CON_22P</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>C1848</t>
+          <t>C22459552</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>CL31B105KBHNNNE</t>
+          <t>05B20L22P</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Samsung Electro-Mechanics</t>
+          <t>HanElectricity</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>SMD,P=0.5mm,Surface Mount，Right Angle</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K12" t="n">
-        <v>646720</v>
+        <v>2004</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1323,26 +1323,26 @@
         <v>2</v>
       </c>
       <c r="N12" t="n">
-        <v>0.0493</v>
+        <v>0.0698</v>
       </c>
       <c r="O12" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.1396</v>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C1848.html</t>
+          <t>https://www.lcsc.com/product-detail/C22459552.html</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1uF 50V X7R ±10% 1206 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>-25℃~+85℃ 0.3mm 0.5mm 22P 2mm 400mA 50V Bottom Contact Phosphor bronze Slide Lock Surface Mount, Right Angle Tin SMD,P=0</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Y1 Y3</t>
+          <t>C1 C104</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1353,32 +1353,32 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Q13FC13500004</t>
+          <t>1uF 50V 1206</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FP-ABS07-MFG</t>
+          <t>FP-1206-L_3_2_0_2-W_1_6_0-IPC_B</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>C32346</t>
+          <t>C1848</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Q13FC13500004</t>
+          <t>CL31B105KBHNNNE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Seiko Epson</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>SMD3215-2P</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>563798</v>
+        <v>646685</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1396,62 +1396,62 @@
         <v>2</v>
       </c>
       <c r="N13" t="n">
-        <v>0.1657</v>
+        <v>0.0493</v>
       </c>
       <c r="O13" t="n">
-        <v>0.3314</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C32346.html</t>
+          <t>https://www.lcsc.com/product-detail/C1848.html</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 12.5pF 32.768kHz 70kΩ Crystal Oscillator ±20ppm SMD3215-2P Crystals ROHS</t>
+          <t>1uF 50V X7R ±10% 1206 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FB1 FB2 FB3 FB4</t>
+          <t>Y1 Y3</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>BLM18PG121SN1D</t>
+          <t>Q13FC13500004</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>FP-BLM18-0_15-t0_8-IPC_B</t>
+          <t>FP-ABS07-MFG</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>C14709</t>
+          <t>C32346</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>BLM18PG121SN1D</t>
+          <t>Q13FC13500004</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Murata Electronics</t>
+          <t>Seiko Epson</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SMD3215-2P</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1460,61 +1460,61 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>2259510</v>
+        <v>563906</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N14" t="n">
-        <v>0.0152</v>
+        <v>0.1657</v>
       </c>
       <c r="O14" t="n">
-        <v>0.0608</v>
+        <v>0.3314</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C14709.html</t>
+          <t>https://www.lcsc.com/product-detail/C32346.html</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 1 120Ω@100MHz 2A 50mΩ ±25% 0603 Ferrite Beads ROHS</t>
+          <t>-40℃~+85℃ 12.5pF 32.768kHz 70kΩ Crystal Oscillator ±20ppm SMD3215-2P Crystals ROHS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>L1 L2 L3 L4 L5</t>
+          <t>FB1 FB2 FB3 FB4</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>DFE201612E-R47M=P2</t>
+          <t>BLM18PG121SN1D</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FP-DFE201612C-IPC_C</t>
+          <t>FP-BLM18-0_15-t0_8-IPC_B</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>C668312</t>
+          <t>C14709</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>DFE201612E-R47M=P2</t>
+          <t>BLM18PG121SN1D</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1524,70 +1524,70 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>0806</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K15" t="n">
-        <v>8190</v>
+        <v>2258939</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N15" t="n">
-        <v>0.1717</v>
+        <v>0.0152</v>
       </c>
       <c r="O15" t="n">
-        <v>0.8585</v>
+        <v>0.0608</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C668312.html</t>
+          <t>https://www.lcsc.com/product-detail/C14709.html</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>26mΩ 4.5A 470nH 5.5A ±20% 0806 Power Inductors ROHS</t>
+          <t>-55℃~+125℃ 1 120Ω@100MHz 2A 50mΩ ±25% 0603 Ferrite Beads ROHS</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>L6 L7</t>
+          <t>L1 L2 L3 L4 L5</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>DFE252012F-100M=P2</t>
+          <t>DFE201612E-R47M=P2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FP-DFE252012C-IPC_B</t>
+          <t>FP-DFE201612C-IPC_C</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C703141</t>
+          <t>C668312</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>DFE252012F-100M=P2</t>
+          <t>DFE201612E-R47M=P2</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1008</t>
+          <t>0806</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1606,71 +1606,71 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>16359</v>
+        <v>8190</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N16" t="n">
-        <v>0.1542</v>
+        <v>0.1717</v>
       </c>
       <c r="O16" t="n">
-        <v>0.3084</v>
+        <v>0.8585</v>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C703141.html</t>
+          <t>https://www.lcsc.com/product-detail/C668312.html</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>1.4A 10uH 400mΩ 950mA ±20% 1008 Power Inductors ROHS</t>
+          <t>26mΩ 4.5A 470nH 5.5A ±20% 0806 Power Inductors ROHS</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>U5 U8 U10</t>
+          <t>L6 L7</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TPS63802DLAR</t>
+          <t>DFE252012F-100M=P2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>FP-DLA0010A-MFG</t>
+          <t>FP-DFE252012C-IPC_B</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>C2845237</t>
+          <t>C703141</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>TPS63802DLAR</t>
+          <t>DFE252012F-100M=P2</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Murata Electronics</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>VSON-10(2x3)</t>
+          <t>1008</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1679,61 +1679,61 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>18536</v>
+        <v>16359</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N17" t="n">
-        <v>0.9802</v>
+        <v>0.1542</v>
       </c>
       <c r="O17" t="n">
-        <v>2.9406</v>
+        <v>0.3084</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2845237.html</t>
+          <t>https://www.lcsc.com/product-detail/C703141.html</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>-40℃~+125℃@(TJ) 1 1.3V~5.5V 1.4MHz、1.6MHz、2.1MHz 1.8V~5.2V 11uA 2A Adjustable Buck-Boost Buck-Boost Built-in Yes VSON-10</t>
+          <t>1.4A 10uH 400mΩ 950mA ±20% 1008 Power Inductors ROHS</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>U6 U7</t>
+          <t>U5 U8 U10</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>TPS62823DLCR</t>
+          <t>TPS63802DLAR</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>FP-DLC0008A-MFG</t>
+          <t>FP-DLA0010A-MFG</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>C2693497</t>
+          <t>C2845237</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>TPS62823DLCR</t>
+          <t>TPS63802DLAR</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>VSON-8(1.5x2)</t>
+          <t>VSON-10(2x3)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1752,119 +1752,119 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>8274</v>
+        <v>18516</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N18" t="n">
-        <v>1.0869</v>
+        <v>0.9802</v>
       </c>
       <c r="O18" t="n">
-        <v>2.1738</v>
+        <v>2.9406</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2693497.html</t>
+          <t>https://www.lcsc.com/product-detail/C2845237.html</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t xml:space="preserve">-40℃~+125℃@(TJ) 1 2.2MHz 2.4V~5.5V 3A 4uA 600mV~4V Adjustable Buck Built-in Overcurrent Protection、Light load efficient </t>
+          <t>-40℃~+125℃@(TJ) 1 1.3V~5.5V 1.4MHz、1.6MHz、2.1MHz 1.8V~5.2V 11uA 2A Adjustable Buck-Boost Buck-Boost Built-in Yes VSON-10</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C2 C3 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106</t>
+          <t>U6 U7</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10uF GRM188R61A106ME69D</t>
+          <t>TPS62823DLCR</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>FP-GRM188-0_15-MFG</t>
+          <t>FP-DLC0008A-MFG</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>C19702</t>
+          <t>C2693497</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>CL10A106KP8NNNC</t>
+          <t>TPS62823DLCR</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Samsung Electro-Mechanics</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>VSON-8(1.5x2)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K19" t="n">
-        <v>11371140</v>
+        <v>8274</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="N19" t="n">
-        <v>0.0308</v>
+        <v>1.0869</v>
       </c>
       <c r="O19" t="n">
-        <v>0.4004</v>
+        <v>2.1738</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C19702.html</t>
+          <t>https://www.lcsc.com/product-detail/C2693497.html</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>10V 10uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t xml:space="preserve">-40℃~+125℃@(TJ) 1 2.2MHz 2.4V~5.5V 3A 4uA 600mV~4V Adjustable Buck Built-in Overcurrent Protection、Light load efficient </t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C86</t>
+          <t>C2 C3 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1uF 0603</t>
+          <t>10uF GRM188R61A106ME69D</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1874,17 +1874,17 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>C696901</t>
+          <t>C19702</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>TCC0603X5R105K160CT</t>
+          <t>CL10A106KP8NNNC</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CCTC</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1894,70 +1894,70 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K20" t="n">
-        <v>425221</v>
+        <v>11367820</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="N20" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0308</v>
       </c>
       <c r="O20" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.4004</v>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C696901.html</t>
+          <t>https://www.lcsc.com/product-detail/C19702.html</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>16V 1uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>10V 10uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>C14 C17 C18 C20 C87 C89</t>
+          <t>C86</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>22uF GRM188R60J226MEA0J</t>
+          <t>1uF 0603</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FP-GRM188-0_2-IPC_C</t>
+          <t>FP-GRM188-0_15-MFG</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>C59461</t>
+          <t>C696901</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>CL10A226MQ8NRNC</t>
+          <t>TCC0603X5R105K160CT</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Samsung Electro-Mechanics</t>
+          <t>CCTC</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1967,105 +1967,105 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K21" t="n">
-        <v>8659730</v>
+        <v>425221</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N21" t="n">
-        <v>0.03</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="O21" t="n">
-        <v>0.18</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C59461.html</t>
+          <t>https://www.lcsc.com/product-detail/C696901.html</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>22uF 6.3V X5R ±20% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>16V 1uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>D2 D7 D8</t>
+          <t>C14 C17 C18 C20 C87 C89</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DSK24</t>
+          <t>22uF GRM188R60J226MEA0J</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FP-S8-V-3910_01-001-MFG</t>
+          <t>FP-GRM188-0_2-IPC_C</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>C22466352</t>
+          <t>C59461</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>DSK24</t>
+          <t>CL10A226MQ8NRNC</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>hongjiacheng</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>SOD-123FL</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Promo</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K22" t="n">
-        <v>2663348</v>
+        <v>8659613</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N22" t="n">
-        <v>0.0247</v>
+        <v>0.03</v>
       </c>
       <c r="O22" t="n">
-        <v>0.0741</v>
+        <v>0.18</v>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22466352.html</t>
+          <t>https://www.lcsc.com/product-detail/C59461.html</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 2A 40V 500uA@40V 50A 550mV@2A Standalone SOD-123FL Schottky Diodes ROHS</t>
+          <t>22uF 6.3V X5R ±20% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>2844395</v>
+        <v>2838252</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>807684</v>
+        <v>807053</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>809002</v>
+        <v>808908</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>8720168</v>
+        <v>8719592</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>758260</v>
+        <v>758135</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2555,19 +2555,19 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>30408</v>
+        <v>428</v>
       </c>
       <c r="L29" t="n">
-        <v>1</v>
+        <v>139</v>
       </c>
       <c r="M29" t="n">
-        <v>1</v>
+        <v>139</v>
       </c>
       <c r="N29" t="n">
-        <v>0.0785</v>
+        <v>0.06279999999999999</v>
       </c>
       <c r="O29" t="n">
-        <v>0.0785</v>
+        <v>8.729200000000001</v>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
@@ -2774,7 +2774,7 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>2243481</v>
+        <v>2243457</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>9382870</v>
+        <v>9380266</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>24975907</v>
+        <v>24991895</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>724600</v>
+        <v>724620</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>2764269</v>
+        <v>2770004</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>9855951</v>
+        <v>9846534</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2753252</v>
+        <v>2753292</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2636190</v>
+        <v>2636200</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1404852</v>
+        <v>1413882</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>3782977</v>
+        <v>3796591</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3650,7 +3650,7 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>1347534</v>
+        <v>1347584</v>
       </c>
       <c r="L44" t="n">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>16540594</v>
+        <v>16543099</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>5871007</v>
+        <v>5870576</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>6679905</v>
+        <v>6685820</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>2035272</v>
+        <v>2035017</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>105811</v>
+        <v>105237</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
@@ -4873,7 +4873,7 @@
         </is>
       </c>
       <c r="O67" t="n">
-        <v>41.2</v>
+        <v>49.85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
LED drive for 4 white + 4 IR per side: R66/R68 5.6 ohm (C322191, same 0603 footprint)
One series string of 8 LEDs per camera side: 35.7 mA, 18.2 V typ / 21.0 V max, switch peak
0.48 A at a 3.0 V battery (TPS61160 limit 0.56 A min, OVP 37 V min). R66 was 4.7 ohm, which
would hit the current limit on a low battery; R68 was 10 ohm, half the light on that side.
LED_RING.md: ring board parts (C385305 white, C385305/C53191414 in SMD2835), counts, mounting.
Buy list includes both rings.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q67"/>
+  <dimension ref="A1:Q66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>41885</v>
+        <v>41631</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -593,10 +593,10 @@
         <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>0.767</v>
+        <v>0.7664</v>
       </c>
       <c r="O2" t="n">
-        <v>0.767</v>
+        <v>0.7664</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -666,10 +666,10 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>2.2035</v>
+        <v>2.2379</v>
       </c>
       <c r="O3" t="n">
-        <v>2.2035</v>
+        <v>2.2379</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2704080</v>
+        <v>2647489</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -739,10 +739,10 @@
         <v>2</v>
       </c>
       <c r="N4" t="n">
-        <v>0.0385</v>
+        <v>0.0384</v>
       </c>
       <c r="O4" t="n">
-        <v>0.077</v>
+        <v>0.07679999999999999</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>176406</v>
+        <v>175178</v>
       </c>
       <c r="L5" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>12551905</v>
+        <v>12041675</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3637497</v>
+        <v>3576151</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1274216</v>
+        <v>1159094</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>749597</v>
+        <v>728539</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2489223</v>
+        <v>2469635</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>2663348</v>
+        <v>2663156</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>646685</v>
+        <v>640040</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1396,10 +1396,10 @@
         <v>2</v>
       </c>
       <c r="N13" t="n">
-        <v>0.0493</v>
+        <v>0.0469</v>
       </c>
       <c r="O13" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.09379999999999999</v>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>563906</v>
+        <v>549087</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1469,10 +1469,10 @@
         <v>2</v>
       </c>
       <c r="N14" t="n">
-        <v>0.1657</v>
+        <v>0.1655</v>
       </c>
       <c r="O14" t="n">
-        <v>0.3314</v>
+        <v>0.331</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>2258939</v>
+        <v>2190108</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1542,10 +1542,10 @@
         <v>4</v>
       </c>
       <c r="N15" t="n">
-        <v>0.0152</v>
+        <v>0.0151</v>
       </c>
       <c r="O15" t="n">
-        <v>0.0608</v>
+        <v>0.0604</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>8190</v>
+        <v>8148</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -1615,10 +1615,10 @@
         <v>5</v>
       </c>
       <c r="N16" t="n">
-        <v>0.1717</v>
+        <v>0.1715</v>
       </c>
       <c r="O16" t="n">
-        <v>0.8585</v>
+        <v>0.8575</v>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>16359</v>
+        <v>16381</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
@@ -1688,10 +1688,10 @@
         <v>2</v>
       </c>
       <c r="N17" t="n">
-        <v>0.1542</v>
+        <v>0.1541</v>
       </c>
       <c r="O17" t="n">
-        <v>0.3084</v>
+        <v>0.3082</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>18516</v>
+        <v>18173</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -1761,10 +1761,10 @@
         <v>3</v>
       </c>
       <c r="N18" t="n">
-        <v>0.9802</v>
+        <v>0.9795</v>
       </c>
       <c r="O18" t="n">
-        <v>2.9406</v>
+        <v>2.9385</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>8274</v>
+        <v>8269</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1834,10 +1834,10 @@
         <v>2</v>
       </c>
       <c r="N19" t="n">
-        <v>1.0869</v>
+        <v>1.086</v>
       </c>
       <c r="O19" t="n">
-        <v>2.1738</v>
+        <v>2.172</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>11367820</v>
+        <v>11382311</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>425221</v>
+        <v>425016</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>8659613</v>
+        <v>8607360</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>2838252</v>
+        <v>4117194</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2126,10 +2126,10 @@
         <v>1</v>
       </c>
       <c r="N23" t="n">
-        <v>0.0072</v>
+        <v>0.0073</v>
       </c>
       <c r="O23" t="n">
-        <v>0.0072</v>
+        <v>0.0073</v>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>807053</v>
+        <v>803210</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2199,10 +2199,10 @@
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="O24" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>808908</v>
+        <v>808966</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2272,10 +2272,10 @@
         <v>2</v>
       </c>
       <c r="N25" t="n">
-        <v>0.08160000000000001</v>
+        <v>0.0815</v>
       </c>
       <c r="O25" t="n">
-        <v>0.1632</v>
+        <v>0.163</v>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>58836</v>
+        <v>2530</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2345,10 +2345,10 @@
         <v>3</v>
       </c>
       <c r="N26" t="n">
-        <v>0.09370000000000001</v>
+        <v>0.4028</v>
       </c>
       <c r="O26" t="n">
-        <v>0.2811</v>
+        <v>1.2084</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
@@ -2364,18 +2364,18 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>R68</t>
+          <t>R66 R68</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10R</t>
+          <t>5.6R</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2385,17 +2385,17 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C22859</t>
+          <t>C322191</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0603WAF100JT5E</t>
+          <t>RS-03L5R60FT</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2405,39 +2405,39 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K27" t="n">
-        <v>8719592</v>
+        <v>15400</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N27" t="n">
-        <v>0.0031</v>
+        <v>0.0032</v>
       </c>
       <c r="O27" t="n">
-        <v>0.0031</v>
+        <v>0.0064</v>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C22859.html</t>
+          <t>https://www.lcsc.com/product-detail/C322191.html</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 10Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100mW 5.6Ω 50V Thick Film Resistor ±1% ±250ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>R66</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2448,41 +2448,41 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>4.7R</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FP-SR0603-MFG</t>
+          <t>FP-XRCGB_F_N-MFG</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C23164</t>
+          <t>C2965580</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0603WAF470KT5E</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>YXC Crystal Oscillators</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SMD2016-4P</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K28" t="n">
-        <v>758135</v>
+        <v>4388</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2491,62 +2491,62 @@
         <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>0.0025</v>
+        <v>0.0784</v>
       </c>
       <c r="O28" t="n">
-        <v>0.0025</v>
+        <v>0.0784</v>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C23164.html</t>
+          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 4.7Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Y2</t>
+          <t>S1 S2 S3</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>S2B-PH-K-S(LF)(SN)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>FP-XRCGB_F_N-MFG</t>
+          <t>JST-S2B-PH-K-S_V</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C2965580</t>
+          <t>C157932</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>S2B-PH-K-S-GW</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>YXC Crystal Oscillators</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>SMD2016-4P</t>
+          <t>Push-Pull,P=2mm</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2555,71 +2555,71 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>428</v>
+        <v>14990</v>
       </c>
       <c r="L29" t="n">
-        <v>139</v>
+        <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>139</v>
+        <v>3</v>
       </c>
       <c r="N29" t="n">
-        <v>0.06279999999999999</v>
+        <v>0.2125</v>
       </c>
       <c r="O29" t="n">
-        <v>8.729200000000001</v>
+        <v>0.6375</v>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
+          <t>https://www.lcsc.com/product-detail/C157932.html</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
+          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>S1 S2 S3</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S(LF)(SN)</t>
+          <t>k230d</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>JST-S2B-PH-K-S_V</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C157932</t>
+          <t>C42414902</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S-GW</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Canaan</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Push-Pull,P=2mm</t>
+          <t>BGA-256</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2628,119 +2628,119 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>15506</v>
+        <v>351</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N30" t="n">
-        <v>0.2127</v>
+        <v>13.3015</v>
       </c>
       <c r="O30" t="n">
-        <v>0.6381</v>
+        <v>13.3015</v>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C157932.html</t>
+          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
+          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>R5 R12</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>k230d</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>RES_0402</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C42414902</t>
+          <t>C25867</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>0402WGF1501TCE</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Canaan</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BGA-256</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K31" t="n">
-        <v>351</v>
+        <v>2203451</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N31" t="n">
-        <v>13.3119</v>
+        <v>0.0028</v>
       </c>
       <c r="O31" t="n">
-        <v>13.3119</v>
+        <v>0.0056</v>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
+          <t>https://www.lcsc.com/product-detail/C25867.html</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
+          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>R5 R12</t>
+          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2750,12 +2750,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C25867</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0402WGF1501TCE</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2774,46 +2774,46 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>2243457</v>
+        <v>9249331</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="N32" t="n">
-        <v>0.0028</v>
+        <v>0.0024</v>
       </c>
       <c r="O32" t="n">
-        <v>0.0056</v>
+        <v>0.048</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25867.html</t>
+          <t>https://www.lcsc.com/product-detail/C25741.html</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
+          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C33" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2823,12 +2823,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C25744</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0402WGF1003TCE</t>
+          <t>0402WGF1002TCE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2847,46 +2847,46 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>9380266</v>
+        <v>24445606</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N33" t="n">
-        <v>0.0024</v>
+        <v>0.0033</v>
       </c>
       <c r="O33" t="n">
-        <v>0.048</v>
+        <v>0.0594</v>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25741.html</t>
+          <t>https://www.lcsc.com/product-detail/C25744.html</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>120k</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2896,12 +2896,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C25744</t>
+          <t>C25750</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>0402WGF1002TCE</t>
+          <t>0402WGF1203TCE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2916,50 +2916,50 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Promo</t>
         </is>
       </c>
       <c r="K34" t="n">
-        <v>24991895</v>
+        <v>709720</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="N34" t="n">
-        <v>0.0033</v>
+        <v>0.0011</v>
       </c>
       <c r="O34" t="n">
-        <v>0.0594</v>
+        <v>0.0011</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25744.html</t>
+          <t>https://www.lcsc.com/product-detail/C25750.html</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R71 R72</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>120k</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2969,12 +2969,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C25750</t>
+          <t>C26083</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0402WGF1203TCE</t>
+          <t>0402WGF1004TCE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2989,50 +2989,50 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Promo</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K35" t="n">
-        <v>724620</v>
+        <v>2735258</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N35" t="n">
-        <v>0.0011</v>
+        <v>0.0025</v>
       </c>
       <c r="O35" t="n">
-        <v>0.0011</v>
+        <v>0.005</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25750.html</t>
+          <t>https://www.lcsc.com/product-detail/C26083.html</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R71 R72</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C26083</t>
+          <t>C11702</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>0402WGF1004TCE</t>
+          <t>0402WGF1001TCE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3066,46 +3066,46 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>2770004</v>
+        <v>9047392</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N36" t="n">
-        <v>0.0025</v>
+        <v>0.0018</v>
       </c>
       <c r="O36" t="n">
-        <v>0.005</v>
+        <v>0.0018</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C26083.html</t>
+          <t>https://www.lcsc.com/product-detail/C11702.html</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R37 R62</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>200R</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3115,12 +3115,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C11702</t>
+          <t>C25087</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>0402WGF1001TCE</t>
+          <t>0402WGF2000TCE</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3139,46 +3139,46 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>9846534</v>
+        <v>2708225</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N37" t="n">
-        <v>0.0021</v>
+        <v>0.0028</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0021</v>
+        <v>0.0056</v>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C11702.html</t>
+          <t>https://www.lcsc.com/product-detail/C25087.html</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R37 R62</t>
+          <t>R59</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>200R</t>
+          <t>200k</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3188,12 +3188,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C25087</t>
+          <t>C25764</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0402WGF2000TCE</t>
+          <t>0402WGF2003TCE</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3212,35 +3212,35 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2753292</v>
+        <v>2569868</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N38" t="n">
-        <v>0.0028</v>
+        <v>0.0017</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0056</v>
+        <v>0.0017</v>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25087.html</t>
+          <t>https://www.lcsc.com/product-detail/C25764.html</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R59</t>
+          <t>R69</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>200k</t>
+          <t>20k</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C25764</t>
+          <t>C25765</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0402WGF2003TCE</t>
+          <t>0402WGF2002TCE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2636200</v>
+        <v>1347758</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3294,26 +3294,26 @@
         <v>1</v>
       </c>
       <c r="N39" t="n">
-        <v>0.0017</v>
+        <v>0.0022</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0017</v>
+        <v>0.0022</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25764.html</t>
+          <t>https://www.lcsc.com/product-detail/C25765.html</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 20kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>R69</t>
+          <t>R42</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>20k</t>
+          <t>22R</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3334,12 +3334,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>C25765</t>
+          <t>C25092</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>0402WGF2002TCE</t>
+          <t>0402WGF220JTCE</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1413882</v>
+        <v>3574900</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3367,37 +3367,37 @@
         <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>0.0022</v>
+        <v>0.0027</v>
       </c>
       <c r="O40" t="n">
-        <v>0.0022</v>
+        <v>0.0027</v>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25765.html</t>
+          <t>https://www.lcsc.com/product-detail/C25092.html</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 20kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>R42</t>
+          <t>R33 R46 R47 R48</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>22R</t>
+          <t>240R</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3407,17 +3407,17 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>C25092</t>
+          <t>C324768</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>0402WGF220JTCE</t>
+          <t>RC-02K2400FT</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3427,50 +3427,50 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K41" t="n">
-        <v>3796591</v>
+        <v>298336</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N41" t="n">
-        <v>0.0028</v>
+        <v>0.0013</v>
       </c>
       <c r="O41" t="n">
-        <v>0.0028</v>
+        <v>0.0052</v>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25092.html</t>
+          <t>https://www.lcsc.com/product-detail/C324768.html</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>R33 R46 R47 R48</t>
+          <t>R63</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>240R</t>
+          <t>30k</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3480,17 +3480,17 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>C324768</t>
+          <t>C49653548</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>RC-02K2400FT</t>
+          <t>GR0402F30KTAG00</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>FH (Guangdong Fenghua Advanced Tech)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3504,35 +3504,35 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>322406</v>
+        <v>7960</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N42" t="n">
-        <v>0.0013</v>
+        <v>0.0008</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0052</v>
+        <v>0.0008</v>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C324768.html</t>
+          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>R63</t>
+          <t>R25</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>30k</t>
+          <t>33k</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3553,17 +3553,17 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>C49653548</t>
+          <t>C25779</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>GR0402F30KTAG00</t>
+          <t>0402WGF3302TCE</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3573,11 +3573,11 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K43" t="n">
-        <v>8260</v>
+        <v>1337901</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3586,37 +3586,37 @@
         <v>1</v>
       </c>
       <c r="N43" t="n">
-        <v>0.0008</v>
+        <v>0.0056</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0008</v>
+        <v>0.0056</v>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
+          <t>https://www.lcsc.com/product-detail/C25779.html</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>R14 R15 R17 R18 R73 R74</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>33k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3626,12 +3626,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>C25779</t>
+          <t>C25900</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>0402WGF3302TCE</t>
+          <t>0402WGF4701TCE</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3650,46 +3650,46 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>1347584</v>
+        <v>16340863</v>
       </c>
       <c r="L44" t="n">
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N44" t="n">
-        <v>0.0056</v>
+        <v>0.0026</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0056</v>
+        <v>0.0156</v>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25779.html</t>
+          <t>https://www.lcsc.com/product-detail/C25900.html</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>R14 R15 R17 R18 R73 R74</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>47k</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3699,12 +3699,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>C25900</t>
+          <t>C25792</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>0402WGF4701TCE</t>
+          <t>0402WGF4702TCE</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3723,46 +3723,46 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>16543099</v>
+        <v>5836672</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N45" t="n">
-        <v>0.0026</v>
+        <v>0.0025</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0156</v>
+        <v>0.0025</v>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25900.html</t>
+          <t>https://www.lcsc.com/product-detail/C25792.html</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R1 R4 R9 R11</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>47k</t>
+          <t>5.1k</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3772,12 +3772,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>C25792</t>
+          <t>C25905</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>0402WGF4702TCE</t>
+          <t>0402WGF5101TCE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3796,46 +3796,46 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>5870576</v>
+        <v>6575807</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N46" t="n">
-        <v>0.0025</v>
+        <v>0.0023</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0025</v>
+        <v>0.0092</v>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25792.html</t>
+          <t>https://www.lcsc.com/product-detail/C25905.html</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>R1 R4 R9 R11</t>
+          <t>R22 R50</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>5.1k</t>
+          <t>511k</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3845,17 +3845,17 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>C25905</t>
+          <t>C49655223</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>0402WGF5101TCE</t>
+          <t>GR0402F511KTAG00</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3865,50 +3865,50 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K47" t="n">
-        <v>6685820</v>
+        <v>7680</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N47" t="n">
-        <v>0.0023</v>
+        <v>0.0008</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0092</v>
+        <v>0.0016</v>
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25905.html</t>
+          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>R22 R50</t>
+          <t>R56</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>511k</t>
+          <t>51k</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3918,17 +3918,17 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>C49655223</t>
+          <t>C25794</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>GR0402F511KTAG00</t>
+          <t>0402WGF5102TCE</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3938,50 +3938,50 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K48" t="n">
-        <v>7800</v>
+        <v>2013455</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N48" t="n">
-        <v>0.0008</v>
+        <v>0.0018</v>
       </c>
       <c r="O48" t="n">
-        <v>0.0016</v>
+        <v>0.0018</v>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
+          <t>https://www.lcsc.com/product-detail/C25794.html</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 51kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>R56</t>
+          <t>R24 R55</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>51k</t>
+          <t>91k</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3991,17 +3991,17 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>C25794</t>
+          <t>C54920709</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>0402WGF5102TCE</t>
+          <t>HRC0402F9102DNTO</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4011,75 +4011,75 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K49" t="n">
-        <v>2035017</v>
+        <v>130638</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N49" t="n">
-        <v>0.0018</v>
+        <v>0.0007</v>
       </c>
       <c r="O49" t="n">
-        <v>0.0018</v>
+        <v>0.0014</v>
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25794.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 51kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>R24 R55</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>91k</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>RES_0402</t>
+          <t>RGT0016C_V</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C54920709</t>
+          <t>C129319</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>HRC0402F9102DNTO</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>QFN-16-EP(3x3)</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -4088,61 +4088,61 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>130662</v>
+        <v>356</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N50" t="n">
-        <v>0.0007</v>
+        <v>2.1673</v>
       </c>
       <c r="O50" t="n">
-        <v>0.0014</v>
+        <v>2.1673</v>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
+          <t>https://www.lcsc.com/product-detail/C129319.html</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>U14 U15</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>TPS61160DRVR</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>RGT0016C_V</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>C129319</t>
+          <t>C165143</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>TPS61160DRVR</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>QFN-16-EP(3x3)</t>
+          <t>WSON-6-EP(2x2)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -4161,35 +4161,35 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>356</v>
+        <v>9909</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N51" t="n">
-        <v>2.169</v>
+        <v>0.4482</v>
       </c>
       <c r="O51" t="n">
-        <v>2.169</v>
+        <v>0.8964</v>
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C129319.html</t>
+          <t>https://www.lcsc.com/product-detail/C165143.html</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
+          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over Current Protection、Over-Temperature</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>U14 U15</t>
+          <t>USBC1 USBC2</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -4200,32 +4200,32 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>TPS61160DRVR</t>
+          <t>type-c-31-m-12</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C165143</t>
+          <t>C165948</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>TPS61160DRVR</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Korean Hroparts Elec</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>WSON-6-EP(2x2)</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -4234,7 +4234,7 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>11609</v>
+        <v>99053</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
@@ -4243,62 +4243,62 @@
         <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>0.4486</v>
+        <v>0.179</v>
       </c>
       <c r="O52" t="n">
-        <v>0.8972</v>
+        <v>0.358</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165143.html</t>
+          <t>https://www.lcsc.com/product-detail/C165948.html</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over Current Protection、Over-Temperature</t>
+          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>USBC1 USBC2</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>type-c-31-m-12</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>C3035748</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>CH340X</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Korean Hroparts Elec</t>
+          <t>WCH(Jiangsu Qin Heng)</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>MSOP-10</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4307,35 +4307,35 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>105237</v>
+        <v>16103</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N53" t="n">
-        <v>0.1792</v>
+        <v>0.6629</v>
       </c>
       <c r="O53" t="n">
-        <v>0.3584</v>
+        <v>0.6629</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165948.html</t>
+          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
+          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -4346,32 +4346,32 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>msm381acb026</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>mems</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>C3035748</t>
+          <t>C51928208</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>CH340X</t>
+          <t>MSM381ACB026</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>WCH(Jiangsu Qin Heng)</t>
+          <t>MEMS</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>MSOP-10</t>
+          <t>LGA-3(1.9x2.8)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>16618</v>
+        <v>6244</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4389,26 +4389,26 @@
         <v>1</v>
       </c>
       <c r="N54" t="n">
-        <v>0.6634</v>
+        <v>0.3025</v>
       </c>
       <c r="O54" t="n">
-        <v>0.6634</v>
+        <v>0.3025</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
+          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
+          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -4419,32 +4419,32 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>msm381acb026</t>
+          <t>w25n02kvzeir</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>mems</t>
+          <t>w25n02</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>C51928208</t>
+          <t>C17626844</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>MSM381ACB026</t>
+          <t>W25N02KVZEIR</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>MEMS</t>
+          <t>Winbond Elec</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>LGA-3(1.9x2.8)</t>
+          <t>WSON-8(6x8)</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>6244</v>
+        <v>7624</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4462,26 +4462,26 @@
         <v>1</v>
       </c>
       <c r="N55" t="n">
-        <v>0.3027</v>
+        <v>11.1515</v>
       </c>
       <c r="O55" t="n">
-        <v>0.3027</v>
+        <v>11.1515</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
+          <t>https://www.lcsc.com/product-detail/C17626844.html</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
+          <t>-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 25ns 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>B1_N</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -4492,69 +4492,31 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>w25n02kvzeir</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>w25n02</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>C17626844</t>
-        </is>
-      </c>
+          <t>TESTP</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>W25N02KVZEIR</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>Winbond Elec</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>WSON-8(6x8)</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>Extended</t>
-        </is>
-      </c>
-      <c r="K56" t="n">
-        <v>7624</v>
-      </c>
-      <c r="L56" t="n">
-        <v>1</v>
-      </c>
-      <c r="M56" t="n">
-        <v>1</v>
-      </c>
-      <c r="N56" t="n">
-        <v>11.1602</v>
-      </c>
-      <c r="O56" t="n">
-        <v>11.1602</v>
-      </c>
-      <c r="P56" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lcsc.com/product-detail/C17626844.html</t>
-        </is>
-      </c>
-      <c r="Q56" t="inlineStr">
-        <is>
-          <t>-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 25ns 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function</t>
-        </is>
-      </c>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>B1_N</t>
+          <t>B1_P</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -4589,7 +4551,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>B1_P</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -4600,7 +4562,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>TESTP</t>
+          <t>Connector 2PIn</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -4624,7 +4586,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -4659,7 +4621,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>JB1</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -4694,7 +4656,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>JB1</t>
+          <t>JB2</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -4729,7 +4691,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>JB2</t>
+          <t>JT</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -4764,7 +4726,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>JT</t>
+          <t>ANT1</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -4775,7 +4737,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Connector 2PIn</t>
+          <t>MIFI</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -4799,7 +4761,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ANT1</t>
+          <t>PR1</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -4810,7 +4772,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>MIFI</t>
+          <t>CON5P</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -4831,49 +4793,14 @@
       <c r="P64" t="inlineStr"/>
       <c r="Q64" t="inlineStr"/>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>PR1</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>1</v>
-      </c>
-      <c r="C65" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>CON5P</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>NO PART</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="O67" t="n">
-        <v>49.85</v>
+      <c r="O66" t="n">
+        <v>42.13</v>
       </c>
     </row>
   </sheetData>
@@ -4932,7 +4859,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
LED strips: separate white and IR chains, domed 3535 LEDs, R66 6.8 ohm
Four 36 x 6 mm strips (2 white + 2 IR each), panelled with the main board and cut by hand.
White chain on U14/J1, IR chain on U15/J2, so they switch and dim independently.
R66 6.8 ohm (C23214, same 0603 footprint): 29.4 mA keeps eight white LEDs inside the TPS61160
switch current limit on a low battery. R68 stays 5.6 ohm (IR 35.7 mA).
LEDs: Xinglight XL-HD3535UWC-A2 (C3646951, 2.00 mm) and JNJ JNJ-LTJI0112W120 850 nm
(C19185834, 2.10 mm), domed so the lens stands out through the printed cover; one shared
3-pad footprint.
LED_STRIPS.txt replaces LED_RING.md: topology, electrical limits, parts and alternatives,
footprint, mechanics, glare, RF, brightness estimate, open items.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q66"/>
+  <dimension ref="A1:Q67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>41631</v>
+        <v>40409</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2647489</v>
+        <v>2644508</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>12041675</v>
+        <v>12026309</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3576151</v>
+        <v>3575007</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1159094</v>
+        <v>1158086</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>728539</v>
+        <v>728419</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2469635</v>
+        <v>2468340</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>2663156</v>
+        <v>2662984</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>640040</v>
+        <v>645612</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>549087</v>
+        <v>548307</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>2190108</v>
+        <v>2184531</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>8148</v>
+        <v>8141</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>18173</v>
+        <v>18178</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>11382311</v>
+        <v>11363079</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>8607360</v>
+        <v>8607373</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>4117194</v>
+        <v>4108093</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>803210</v>
+        <v>802715</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>808966</v>
+        <v>806312</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2364,14 +2364,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>R66 R68</t>
+          <t>R68</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2415,13 +2415,13 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N27" t="n">
         <v>0.0032</v>
       </c>
       <c r="O27" t="n">
-        <v>0.0064</v>
+        <v>0.0032</v>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
@@ -2437,7 +2437,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Y2</t>
+          <t>R66</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2448,32 +2448,32 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>6.8R</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FP-XRCGB_F_N-MFG</t>
+          <t>FP-SR0603-MFG</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C2965580</t>
+          <t>C23214</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>XL7EL89CKI-111YLC-24M</t>
+          <t>0603WAF680KT5E</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>YXC Crystal Oscillators</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>SMD2016-4P</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>4388</v>
+        <v>307509</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2491,62 +2491,62 @@
         <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>0.0784</v>
+        <v>0.0044</v>
       </c>
       <c r="O28" t="n">
-        <v>0.0784</v>
+        <v>0.0044</v>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
+          <t>https://www.lcsc.com/product-detail/C23214.html</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
+          <t>-55℃~+155℃ 100mW 6.8Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>S1 S2 S3</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S(LF)(SN)</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>JST-S2B-PH-K-S_V</t>
+          <t>FP-XRCGB_F_N-MFG</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C157932</t>
+          <t>C2965580</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S-GW</t>
+          <t>XL7EL89CKI-111YLC-24M</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>YXC Crystal Oscillators</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Push-Pull,P=2mm</t>
+          <t>SMD2016-4P</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2555,71 +2555,71 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>14990</v>
+        <v>4358</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>0.2125</v>
+        <v>0.0784</v>
       </c>
       <c r="O29" t="n">
-        <v>0.6375</v>
+        <v>0.0784</v>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C157932.html</t>
+          <t>https://www.lcsc.com/product-detail/C2965580.html</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
+          <t>-40℃~+85℃ 100Ω 24MHz 8pF Crystal Oscillator ±10ppm ±20ppm SMD2016-4P Crystals ROHS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>S1 S2 S3</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>k230d</t>
+          <t>S2B-PH-K-S(LF)(SN)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>JST-S2B-PH-K-S_V</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C42414902</t>
+          <t>C157932</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>S2B-PH-K-S-GW</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Canaan</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>BGA-256</t>
+          <t>Push-Pull,P=2mm</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2628,119 +2628,119 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>351</v>
+        <v>14990</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N30" t="n">
-        <v>13.3015</v>
+        <v>0.2125</v>
       </c>
       <c r="O30" t="n">
-        <v>13.3015</v>
+        <v>0.6375</v>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
+          <t>https://www.lcsc.com/product-detail/C157932.html</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
+          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>R5 R12</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>k230d</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>RES_0402</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C25867</t>
+          <t>C42414902</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>0402WGF1501TCE</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>Canaan</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>BGA-256</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K31" t="n">
-        <v>2203451</v>
+        <v>351</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N31" t="n">
-        <v>0.0028</v>
+        <v>13.3015</v>
       </c>
       <c r="O31" t="n">
-        <v>0.0056</v>
+        <v>13.3015</v>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25867.html</t>
+          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
+          <t>R5 R12</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2750,12 +2750,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C25867</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0402WGF1003TCE</t>
+          <t>0402WGF1501TCE</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2774,46 +2774,46 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>9249331</v>
+        <v>2202841</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="N32" t="n">
-        <v>0.0024</v>
+        <v>0.0028</v>
       </c>
       <c r="O32" t="n">
-        <v>0.048</v>
+        <v>0.0056</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25741.html</t>
+          <t>https://www.lcsc.com/product-detail/C25867.html</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
+          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C33" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2823,12 +2823,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C25744</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0402WGF1002TCE</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2847,46 +2847,46 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>24445606</v>
+        <v>9254736</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="N33" t="n">
-        <v>0.0033</v>
+        <v>0.0024</v>
       </c>
       <c r="O33" t="n">
-        <v>0.0594</v>
+        <v>0.048</v>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25744.html</t>
+          <t>https://www.lcsc.com/product-detail/C25741.html</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>120k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2896,12 +2896,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C25750</t>
+          <t>C25744</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>0402WGF1203TCE</t>
+          <t>0402WGF1002TCE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2916,50 +2916,50 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Promo</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K34" t="n">
-        <v>709720</v>
+        <v>24437585</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="N34" t="n">
-        <v>0.0011</v>
+        <v>0.0033</v>
       </c>
       <c r="O34" t="n">
-        <v>0.0011</v>
+        <v>0.0594</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25750.html</t>
+          <t>https://www.lcsc.com/product-detail/C25744.html</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>R71 R72</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>120k</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2969,12 +2969,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C26083</t>
+          <t>C25750</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0402WGF1004TCE</t>
+          <t>0402WGF1203TCE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2989,50 +2989,50 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Promo</t>
         </is>
       </c>
       <c r="K35" t="n">
-        <v>2735258</v>
+        <v>710710</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
-        <v>0.0025</v>
+        <v>0.0011</v>
       </c>
       <c r="O35" t="n">
-        <v>0.005</v>
+        <v>0.0011</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C26083.html</t>
+          <t>https://www.lcsc.com/product-detail/C25750.html</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R71 R72</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C11702</t>
+          <t>C26083</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>0402WGF1001TCE</t>
+          <t>0402WGF1004TCE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3066,46 +3066,46 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>9047392</v>
+        <v>2736244</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N36" t="n">
-        <v>0.0018</v>
+        <v>0.0025</v>
       </c>
       <c r="O36" t="n">
-        <v>0.0018</v>
+        <v>0.005</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C11702.html</t>
+          <t>https://www.lcsc.com/product-detail/C26083.html</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R37 R62</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>200R</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3115,12 +3115,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C25087</t>
+          <t>C11702</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>0402WGF2000TCE</t>
+          <t>0402WGF1001TCE</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3139,46 +3139,46 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>2708225</v>
+        <v>9048991</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N37" t="n">
-        <v>0.0028</v>
+        <v>0.0018</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0056</v>
+        <v>0.0018</v>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25087.html</t>
+          <t>https://www.lcsc.com/product-detail/C11702.html</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R59</t>
+          <t>R37 R62</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>200k</t>
+          <t>200R</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3188,12 +3188,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C25764</t>
+          <t>C25087</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0402WGF2003TCE</t>
+          <t>0402WGF2000TCE</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3212,35 +3212,35 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2569868</v>
+        <v>2707591</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N38" t="n">
-        <v>0.0017</v>
+        <v>0.0028</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0017</v>
+        <v>0.0056</v>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25764.html</t>
+          <t>https://www.lcsc.com/product-detail/C25087.html</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R69</t>
+          <t>R59</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>20k</t>
+          <t>200k</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C25765</t>
+          <t>C25764</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0402WGF2002TCE</t>
+          <t>0402WGF2003TCE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>1347758</v>
+        <v>2573703</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3294,26 +3294,26 @@
         <v>1</v>
       </c>
       <c r="N39" t="n">
-        <v>0.0022</v>
+        <v>0.0017</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0022</v>
+        <v>0.0017</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25765.html</t>
+          <t>https://www.lcsc.com/product-detail/C25764.html</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 20kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>R42</t>
+          <t>R69</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>22R</t>
+          <t>20k</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3334,12 +3334,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>C25092</t>
+          <t>C25765</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>0402WGF220JTCE</t>
+          <t>0402WGF2002TCE</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>3574900</v>
+        <v>1350277</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3367,37 +3367,37 @@
         <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>0.0027</v>
+        <v>0.0022</v>
       </c>
       <c r="O40" t="n">
-        <v>0.0027</v>
+        <v>0.0022</v>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25092.html</t>
+          <t>https://www.lcsc.com/product-detail/C25765.html</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 20kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>R33 R46 R47 R48</t>
+          <t>R42</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>240R</t>
+          <t>22R</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3407,17 +3407,17 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>C324768</t>
+          <t>C25092</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>RC-02K2400FT</t>
+          <t>0402WGF220JTCE</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>FH (Guangdong Fenghua Advanced Tech)</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3427,50 +3427,50 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K41" t="n">
-        <v>298336</v>
+        <v>3572614</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N41" t="n">
-        <v>0.0013</v>
+        <v>0.0027</v>
       </c>
       <c r="O41" t="n">
-        <v>0.0052</v>
+        <v>0.0027</v>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C324768.html</t>
+          <t>https://www.lcsc.com/product-detail/C25092.html</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>R63</t>
+          <t>R33 R46 R47 R48</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>30k</t>
+          <t>240R</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3480,17 +3480,17 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>C49653548</t>
+          <t>C324768</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>GR0402F30KTAG00</t>
+          <t>RC-02K2400FT</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3504,35 +3504,35 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>7960</v>
+        <v>298336</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N42" t="n">
-        <v>0.0008</v>
+        <v>0.0013</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0008</v>
+        <v>0.0052</v>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
+          <t>https://www.lcsc.com/product-detail/C324768.html</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>R63</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>33k</t>
+          <t>30k</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3553,17 +3553,17 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>C25779</t>
+          <t>C49653548</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>0402WGF3302TCE</t>
+          <t>GR0402F30KTAG00</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3573,11 +3573,11 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K43" t="n">
-        <v>1337901</v>
+        <v>7960</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3586,37 +3586,37 @@
         <v>1</v>
       </c>
       <c r="N43" t="n">
-        <v>0.0056</v>
+        <v>0.0008</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0056</v>
+        <v>0.0008</v>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25779.html</t>
+          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>R14 R15 R17 R18 R73 R74</t>
+          <t>R25</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>33k</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3626,12 +3626,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>C25900</t>
+          <t>C25779</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>0402WGF4701TCE</t>
+          <t>0402WGF3302TCE</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3650,46 +3650,46 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>16340863</v>
+        <v>1337621</v>
       </c>
       <c r="L44" t="n">
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N44" t="n">
-        <v>0.0026</v>
+        <v>0.0056</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0156</v>
+        <v>0.0056</v>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25900.html</t>
+          <t>https://www.lcsc.com/product-detail/C25779.html</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R14 R15 R17 R18 R73 R74</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>47k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3699,12 +3699,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>C25792</t>
+          <t>C25900</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>0402WGF4702TCE</t>
+          <t>0402WGF4701TCE</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3723,46 +3723,46 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>5836672</v>
+        <v>16346429</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N45" t="n">
-        <v>0.0025</v>
+        <v>0.0026</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0025</v>
+        <v>0.0156</v>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25792.html</t>
+          <t>https://www.lcsc.com/product-detail/C25900.html</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R1 R4 R9 R11</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>5.1k</t>
+          <t>47k</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3772,12 +3772,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>C25905</t>
+          <t>C25792</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>0402WGF5101TCE</t>
+          <t>0402WGF4702TCE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3796,46 +3796,46 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>6575807</v>
+        <v>5835918</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N46" t="n">
-        <v>0.0023</v>
+        <v>0.0025</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0092</v>
+        <v>0.0025</v>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25905.html</t>
+          <t>https://www.lcsc.com/product-detail/C25792.html</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>R22 R50</t>
+          <t>R1 R4 R9 R11</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>511k</t>
+          <t>5.1k</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3845,17 +3845,17 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>C49655223</t>
+          <t>C25905</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>GR0402F511KTAG00</t>
+          <t>0402WGF5101TCE</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3865,50 +3865,50 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K47" t="n">
-        <v>7680</v>
+        <v>6575334</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N47" t="n">
-        <v>0.0008</v>
+        <v>0.0023</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0016</v>
+        <v>0.0092</v>
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
+          <t>https://www.lcsc.com/product-detail/C25905.html</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>R56</t>
+          <t>R22 R50</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>51k</t>
+          <t>511k</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3918,17 +3918,17 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>C25794</t>
+          <t>C49655223</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>0402WGF5102TCE</t>
+          <t>GR0402F511KTAG00</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3938,50 +3938,50 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K48" t="n">
-        <v>2013455</v>
+        <v>7480</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N48" t="n">
-        <v>0.0018</v>
+        <v>0.0008</v>
       </c>
       <c r="O48" t="n">
-        <v>0.0018</v>
+        <v>0.0016</v>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25794.html</t>
+          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 51kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>R24 R55</t>
+          <t>R56</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>91k</t>
+          <t>51k</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3991,17 +3991,17 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>C54920709</t>
+          <t>C25794</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>HRC0402F9102DNTO</t>
+          <t>0402WGF5102TCE</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4011,75 +4011,75 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K49" t="n">
-        <v>130638</v>
+        <v>2020150</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N49" t="n">
-        <v>0.0007</v>
+        <v>0.0018</v>
       </c>
       <c r="O49" t="n">
-        <v>0.0014</v>
+        <v>0.0018</v>
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
+          <t>https://www.lcsc.com/product-detail/C25794.html</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 51kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>R24 R55</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>91k</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>RGT0016C_V</t>
+          <t>RES_0402</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C129319</t>
+          <t>C54920709</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>HRC0402F9102DNTO</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>QFN-16-EP(3x3)</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -4088,61 +4088,61 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>356</v>
+        <v>130638</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N50" t="n">
-        <v>2.1673</v>
+        <v>0.0007</v>
       </c>
       <c r="O50" t="n">
-        <v>2.1673</v>
+        <v>0.0014</v>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C129319.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
+          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>U14 U15</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>TPS61160DRVR</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>RGT0016C_V</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>C165143</t>
+          <t>C129319</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>TPS61160DRVR</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>WSON-6-EP(2x2)</t>
+          <t>QFN-16-EP(3x3)</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -4161,35 +4161,35 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>9909</v>
+        <v>356</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N51" t="n">
-        <v>0.4482</v>
+        <v>2.1673</v>
       </c>
       <c r="O51" t="n">
-        <v>0.8964</v>
+        <v>2.1673</v>
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165143.html</t>
+          <t>https://www.lcsc.com/product-detail/C129319.html</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over Current Protection、Over-Temperature</t>
+          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>USBC1 USBC2</t>
+          <t>U14 U15</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -4200,32 +4200,32 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>type-c-31-m-12</t>
+          <t>TPS61160DRVR</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>C165143</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>TPS61160DRVR</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Korean Hroparts Elec</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>WSON-6-EP(2x2)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -4234,7 +4234,7 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>99053</v>
+        <v>9909</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
@@ -4243,62 +4243,62 @@
         <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>0.179</v>
+        <v>0.4482</v>
       </c>
       <c r="O52" t="n">
-        <v>0.358</v>
+        <v>0.8964</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165948.html</t>
+          <t>https://www.lcsc.com/product-detail/C165143.html</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
+          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over Current Protection、Over-Temperature</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>USBC1 USBC2</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>type-c-31-m-12</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C3035748</t>
+          <t>C165948</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>CH340X</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>WCH(Jiangsu Qin Heng)</t>
+          <t>Korean Hroparts Elec</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>MSOP-10</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4307,35 +4307,35 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>16103</v>
+        <v>98944</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>0.6629</v>
+        <v>0.179</v>
       </c>
       <c r="O53" t="n">
-        <v>0.6629</v>
+        <v>0.358</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
+          <t>https://www.lcsc.com/product-detail/C165948.html</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
+          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -4346,32 +4346,32 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>msm381acb026</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>mems</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>C51928208</t>
+          <t>C3035748</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>MSM381ACB026</t>
+          <t>CH340X</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>MEMS</t>
+          <t>WCH(Jiangsu Qin Heng)</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>LGA-3(1.9x2.8)</t>
+          <t>MSOP-10</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>6244</v>
+        <v>16003</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4389,26 +4389,26 @@
         <v>1</v>
       </c>
       <c r="N54" t="n">
-        <v>0.3025</v>
+        <v>0.6629</v>
       </c>
       <c r="O54" t="n">
-        <v>0.3025</v>
+        <v>0.6629</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
+          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
+          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -4419,32 +4419,32 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>w25n02kvzeir</t>
+          <t>msm381acb026</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>w25n02</t>
+          <t>mems</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>C17626844</t>
+          <t>C51928208</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>W25N02KVZEIR</t>
+          <t>MSM381ACB026</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Winbond Elec</t>
+          <t>MEMS</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>WSON-8(6x8)</t>
+          <t>LGA-3(1.9x2.8)</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>7624</v>
+        <v>6244</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4462,26 +4462,26 @@
         <v>1</v>
       </c>
       <c r="N55" t="n">
-        <v>11.1515</v>
+        <v>0.3025</v>
       </c>
       <c r="O55" t="n">
-        <v>11.1515</v>
+        <v>0.3025</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17626844.html</t>
+          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 25ns 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function</t>
+          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>B1_N</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -4492,31 +4492,69 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>TESTP</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
+          <t>w25n02kvzeir</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>w25n02</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>C17626844</t>
+        </is>
+      </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>NO PART</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
+          <t>W25N02KVZEIR</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Winbond Elec</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>WSON-8(6x8)</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="K56" t="n">
+        <v>7624</v>
+      </c>
+      <c r="L56" t="n">
+        <v>1</v>
+      </c>
+      <c r="M56" t="n">
+        <v>1</v>
+      </c>
+      <c r="N56" t="n">
+        <v>11.1515</v>
+      </c>
+      <c r="O56" t="n">
+        <v>11.1515</v>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lcsc.com/product-detail/C17626844.html</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 25ns 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>B1_P</t>
+          <t>B1_N</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -4551,7 +4589,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>B1_P</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -4562,7 +4600,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Connector 2PIn</t>
+          <t>TESTP</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -4586,7 +4624,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -4621,7 +4659,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>JB1</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -4656,7 +4694,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>JB2</t>
+          <t>JB1</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -4691,7 +4729,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>JT</t>
+          <t>JB2</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -4726,7 +4764,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ANT1</t>
+          <t>JT</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -4737,7 +4775,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>MIFI</t>
+          <t>Connector 2PIn</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -4761,7 +4799,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>PR1</t>
+          <t>ANT1</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -4772,7 +4810,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>CON5P</t>
+          <t>MIFI</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -4793,13 +4831,48 @@
       <c r="P64" t="inlineStr"/>
       <c r="Q64" t="inlineStr"/>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>PR1</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>CON5P</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="O66" t="n">
+      <c r="O67" t="n">
         <v>42.13</v>
       </c>
     </row>
@@ -4859,6 +4932,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
LED drive at maximum current: R66 3.0 ohm (white 66.7 mA), R68 1.5 ohm (IR 133 mA)
Targets sit at the TPS61160 switch current limit on a typical unit with a nominal battery
(datasheet Eq. 3/4: white 60-69 mA, IR 127-156 mA over 3.3-4.2 V); above that the driver runs
in cycle-by-cycle current limit, far below OVP. PWM duty backs the current off where needed.
C23157 / C22769, UNI-ROYAL 0603 1 %, same FP-SR0603-MFG footprint.
LED_STRIPS.txt: electrical limits per corner, component stress, battery load, brightness at 2 m.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2644508</v>
+        <v>2644148</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>12026309</v>
+        <v>12027069</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3575007</v>
+        <v>3574812</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>728419</v>
+        <v>728399</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>645612</v>
+        <v>643193</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>548307</v>
+        <v>548310</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>2184531</v>
+        <v>2184529</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>11363079</v>
+        <v>11361998</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>8607373</v>
+        <v>8607295</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>4108093</v>
+        <v>4108025</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>806312</v>
+        <v>806292</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>5.6R</t>
+          <t>1.5R</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2385,17 +2385,17 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C322191</t>
+          <t>C22769</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>RS-03L5R60FT</t>
+          <t>0603WAF150KT5E</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>FH (Guangdong Fenghua Advanced Tech)</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>15400</v>
+        <v>112785</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -2418,19 +2418,19 @@
         <v>1</v>
       </c>
       <c r="N27" t="n">
-        <v>0.0032</v>
+        <v>0.0043</v>
       </c>
       <c r="O27" t="n">
-        <v>0.0032</v>
+        <v>0.0043</v>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C322191.html</t>
+          <t>https://www.lcsc.com/product-detail/C22769.html</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 5.6Ω 50V Thick Film Resistor ±1% ±250ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1.5Ω 100mW 75V Thick Film Resistor ±1% ±200ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>6.8R</t>
+          <t>3R</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2458,12 +2458,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C23214</t>
+          <t>C23157</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0603WAF680KT5E</t>
+          <t>0603WAF300KT5E</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>307509</v>
+        <v>43669</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2491,19 +2491,19 @@
         <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>0.0044</v>
+        <v>0.0039</v>
       </c>
       <c r="O28" t="n">
-        <v>0.0044</v>
+        <v>0.0039</v>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C23214.html</t>
+          <t>https://www.lcsc.com/product-detail/C23157.html</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100mW 6.8Ω 75V Thick Film Resistor ±1% ±400ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100mW 3Ω 75V Thick Film Resistor ±1% ±200ppm/℃ 0603 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
@@ -2774,7 +2774,7 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>2202841</v>
+        <v>2202741</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>9254736</v>
+        <v>9254451</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>24437585</v>
+        <v>24432200</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>2736244</v>
+        <v>2736284</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>9048991</v>
+        <v>9038526</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2573703</v>
+        <v>2573723</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1350277</v>
+        <v>1350237</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>3572614</v>
+        <v>3572664</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>298336</v>
+        <v>298316</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>16346429</v>
+        <v>16338974</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>6575334</v>
+        <v>6575124</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
LED drivers U14/U15: TPS61161DRVR (C324075, 38 V OVP) instead of TPS61160DRVR
The TPS61160 trips open-LED protection at 25-27 V; the eight-white chain runs at 22-26 V.
TPS61161 is the same WSON-6 2x2 part with 38 V OVP: same pinout and footprint, netlist unchanged.
Order lists regenerated from the schematic (new LED strip parts, probe and filter resistors);
LCSC cart covers RB1-RB6 47k and RD1/RD2 1.5k. LED_STRIPS.txt corrected.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q67"/>
+  <dimension ref="A1:Q77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>40409</v>
+        <v>40399</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2644148</v>
+        <v>2638347</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>175178</v>
+        <v>175546</v>
       </c>
       <c r="L5" t="n">
         <v>1</v>
@@ -831,14 +831,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C5 C6 C7 C8 C23 C24 C32 C88 C92 C95 C109 C110</t>
+          <t>C5 C6 C7 C8 C9 C23 C24 C32 C88 C92 C95 C109 CT1</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -876,19 +876,19 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>12027069</v>
+        <v>12029136</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N6" t="n">
         <v>0.008399999999999999</v>
       </c>
       <c r="O6" t="n">
-        <v>0.1008</v>
+        <v>0.1092</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3574812</v>
+        <v>3575761</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1158086</v>
+        <v>1158226</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>728399</v>
+        <v>728243</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2468340</v>
+        <v>2467602</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>2662984</v>
+        <v>2663141</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>643193</v>
+        <v>643077</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>548310</v>
+        <v>548117</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>2184529</v>
+        <v>2183317</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>8141</v>
+        <v>8124</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>18178</v>
+        <v>18163</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -1853,14 +1853,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C2 C3 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106</t>
+          <t>C2 C3 C4 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1898,19 +1898,19 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>11361998</v>
+        <v>11365002</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="N20" t="n">
         <v>0.0308</v>
       </c>
       <c r="O20" t="n">
-        <v>0.4004</v>
+        <v>0.4312</v>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>425016</v>
+        <v>185016</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>8607295</v>
+        <v>8606300</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>4108025</v>
+        <v>4108412</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>802715</v>
+        <v>802102</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>806292</v>
+        <v>802887</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>2530</v>
+        <v>2525</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>4358</v>
+        <v>37072</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2729,14 +2729,14 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>R5 R12</t>
+          <t>R5 R12 RD1 RD2</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2774,19 +2774,19 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>2202741</v>
+        <v>2202449</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N32" t="n">
         <v>0.0028</v>
       </c>
       <c r="O32" t="n">
-        <v>0.0056</v>
+        <v>0.0112</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>9254451</v>
+        <v>9251477</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2875,14 +2875,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70</t>
+          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70 RBT1</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C34" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2920,19 +2920,19 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>24432200</v>
+        <v>24434115</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N34" t="n">
         <v>0.0033</v>
       </c>
       <c r="O34" t="n">
-        <v>0.0594</v>
+        <v>0.06270000000000001</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>710710</v>
+        <v>710920</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>2736284</v>
+        <v>2735892</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>9038526</v>
+        <v>9043248</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2707591</v>
+        <v>2707515</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2573723</v>
+        <v>2573903</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1350237</v>
+        <v>1349677</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>3572664</v>
+        <v>3571844</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3459,14 +3459,14 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>R33 R46 R47 R48</t>
+          <t>R33 R46 R47 R48 R52</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C42" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N42" t="n">
         <v>0.0013</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0052</v>
+        <v>0.0065</v>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
@@ -3650,7 +3650,7 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>1337621</v>
+        <v>1337444</v>
       </c>
       <c r="L44" t="n">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>16338974</v>
+        <v>16342107</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3751,14 +3751,14 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R21 RB1 RB2 RB3 RB4 RB5 RB6</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -3796,19 +3796,19 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>5835918</v>
+        <v>5835600</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N46" t="n">
         <v>0.0025</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0025</v>
+        <v>0.0175</v>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>6575124</v>
+        <v>6573651</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>2020150</v>
+        <v>2017249</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>TPS61160DRVR</t>
+          <t>TPS61161DRVR</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4210,12 +4210,12 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C165143</t>
+          <t>C324075</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>TPS61160DRVR</t>
+          <t>TPS61161DRVR</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4234,7 +4234,7 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>9909</v>
+        <v>2574</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
@@ -4243,19 +4243,19 @@
         <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>0.4482</v>
+        <v>0.4106</v>
       </c>
       <c r="O52" t="n">
-        <v>0.8964</v>
+        <v>0.8212</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165143.html</t>
+          <t>https://www.lcsc.com/product-detail/C324075.html</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 2% 2.7V~18V 26V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over Current Protection、Over-Temperature</t>
+          <t>-40℃~+85℃ 1 2% 2.7V~18V 38V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
         </is>
       </c>
     </row>
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>98944</v>
+        <v>98803</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>16003</v>
+        <v>16113</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4408,43 +4408,43 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>LED3 LED6 LED7 LED10 LED11 LED14 LED15 LED16</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>msm381acb026</t>
+          <t>jnj-ltji0112w120/35mil/845-860nm</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>mems</t>
+          <t>jnj-ltji0112w120/35mil/845-860nm</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>C51928208</t>
+          <t>C19185834</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>MSM381ACB026</t>
+          <t>JNJ-LTJI0112W120/35mil/845-860nm</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>MEMS</t>
+          <t>JNJ OPTOELECTRONICS</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>LGA-3(1.9x2.8)</t>
+          <t>SMD3535-3P</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -4453,35 +4453,35 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>6244</v>
+        <v>438</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N55" t="n">
-        <v>0.3025</v>
+        <v>0.3385</v>
       </c>
       <c r="O55" t="n">
-        <v>0.3025</v>
+        <v>3.385</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
+          <t>https://www.lcsc.com/product-detail/C19185834.html</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
+          <t>-40℃~+100℃ 1.4V~2.1V、1.5V~2.3V 120° 1A 50nm 5V 75mW/sr@IF=350mA、140mW/sr@IF=1000mA 850nm SMD3535-3P Infrared LED Emitter</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -4492,32 +4492,32 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>w25n02kvzeir</t>
+          <t>msm381acb026</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>w25n02</t>
+          <t>mems</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>C17626844</t>
+          <t>C51928208</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>W25N02KVZEIR</t>
+          <t>MSM381ACB026</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Winbond Elec</t>
+          <t>MEMS</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>WSON-8(6x8)</t>
+          <t>LGA-3(1.9x2.8)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -4526,7 +4526,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>7624</v>
+        <v>6244</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
@@ -4535,26 +4535,26 @@
         <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>11.1515</v>
+        <v>0.3025</v>
       </c>
       <c r="O56" t="n">
-        <v>11.1515</v>
+        <v>0.3025</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17626844.html</t>
+          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 25ns 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function</t>
+          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>B1_N</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -4565,66 +4565,142 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>TESTP</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
+          <t>w25n02kvzeir</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>w25n02</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>C17626844</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>NO PART</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
+          <t>W25N02KVZEIR</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Winbond Elec</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>WSON-8(6x8)</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="K57" t="n">
+        <v>7624</v>
+      </c>
+      <c r="L57" t="n">
+        <v>1</v>
+      </c>
+      <c r="M57" t="n">
+        <v>1</v>
+      </c>
+      <c r="N57" t="n">
+        <v>11.1515</v>
+      </c>
+      <c r="O57" t="n">
+        <v>11.1515</v>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lcsc.com/product-detail/C17626844.html</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 25ns 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>B1_P</t>
+          <t>LED1 LED2 LED4 LED5 LED8 LED9 LED12 LED13</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>TESTP</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
+          <t>xl-hd3535uwc-a2</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>xl-hd3535uwc-a2</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>C3646951</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>NO PART</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
+          <t>XL-HD3535UWC-A2</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>XINGLIGHT</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>SMD3535-3P</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Extended</t>
+        </is>
+      </c>
+      <c r="K58" t="n">
+        <v>19724</v>
+      </c>
+      <c r="L58" t="n">
+        <v>1</v>
+      </c>
+      <c r="M58" t="n">
+        <v>8</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0.3078</v>
+      </c>
+      <c r="O58" t="n">
+        <v>2.4624</v>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lcsc.com/product-detail/C3646951.html</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>-40℃~+85℃ 130° 1W 2.8V~3.6V 350mA 5500K~7000K Discrete Diode Top-mount Water Clear White SMD3535-3P LED Indication - Dis</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>B1_N</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -4635,7 +4711,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Connector 2PIn</t>
+          <t>TESTP</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -4659,7 +4735,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>B1_P</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -4670,7 +4746,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Connector 2PIn</t>
+          <t>TESTP</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -4694,7 +4770,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>JB1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -4729,7 +4805,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>JB2</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -4764,7 +4840,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>JT</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -4799,7 +4875,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ANT1</t>
+          <t>J7</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -4810,7 +4886,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>MIFI</t>
+          <t>Connector 2PIn</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -4834,7 +4910,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PR1</t>
+          <t>J9</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -4845,7 +4921,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>CON5P</t>
+          <t>Connector 2PIn</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -4866,14 +4942,364 @@
       <c r="P65" t="inlineStr"/>
       <c r="Q65" t="inlineStr"/>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>J11</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Connector 2PIn</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+    </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
+          <t>J6</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Connector 2PIn</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>J8</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>1</v>
+      </c>
+      <c r="C68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Connector 2PIn</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>J10</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Connector 2PIn</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>J12</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Connector 2PIn</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>JB1</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Connector 2PIn</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>JB2</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Connector 2PIn</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>JT</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>1</v>
+      </c>
+      <c r="C73" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Connector 2PIn</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ANT1</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>1</v>
+      </c>
+      <c r="C74" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>MIFI</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>PR1</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>CON5P</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="O67" t="n">
-        <v>42.13</v>
+      <c r="O77" t="n">
+        <v>47.97</v>
       </c>
     </row>
   </sheetData>
@@ -4933,6 +5359,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P58" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
CT1 not fitted; fab zip for the 61 x 65 mm panel; assembly BOM and CPL from the schematic
CT1 (antenna feed shunt pad): comment NF, no part number, left out of BOM and CPL.
LEAKCAM_gerber.zip rebuilt from the 2026-09-24 outputs, outline 61.00 x 65.00 mm from the
ODB++ profile, no small cutouts on the outline layer.
BOM_ASSEMBLY.csv built from the schematic (U14/U15 TPS61161DRVR C324075, not the stale
PCB export); its 242 designators match PickPlace_MIFA.csv one to one. Order lists regenerated.
LCSC hand-build cart: 100 nF 0402 50 V X7R as C131394 (C307331 has 100 pcs left at LCSC).
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q77"/>
+  <dimension ref="A1:Q78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>40399</v>
+        <v>40084</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -593,10 +593,10 @@
         <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>0.7664</v>
+        <v>0.7652</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7664</v>
+        <v>0.7652</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -666,10 +666,10 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>2.2379</v>
+        <v>2.2345</v>
       </c>
       <c r="O3" t="n">
-        <v>2.2379</v>
+        <v>2.2345</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2638347</v>
+        <v>2559768</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -831,14 +831,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C5 C6 C7 C8 C9 C23 C24 C32 C88 C92 C95 C109 CT1</t>
+          <t>C5 C6 C7 C8 C9 C23 C24 C32 C88 C92 C95 C109</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -876,19 +876,19 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>12029136</v>
+        <v>11871497</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N6" t="n">
         <v>0.008399999999999999</v>
       </c>
       <c r="O6" t="n">
-        <v>0.1092</v>
+        <v>0.1008</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3575761</v>
+        <v>3507965</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1158226</v>
+        <v>1146422</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>728243</v>
+        <v>719780</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2467602</v>
+        <v>2454283</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>2663141</v>
+        <v>2663217</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -1250,10 +1250,10 @@
         <v>3</v>
       </c>
       <c r="N11" t="n">
-        <v>0.0247</v>
+        <v>0.0246</v>
       </c>
       <c r="O11" t="n">
-        <v>0.0741</v>
+        <v>0.0738</v>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
@@ -1323,10 +1323,10 @@
         <v>2</v>
       </c>
       <c r="N12" t="n">
-        <v>0.0698</v>
+        <v>0.0697</v>
       </c>
       <c r="O12" t="n">
-        <v>0.1396</v>
+        <v>0.1394</v>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>643077</v>
+        <v>639782</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1396,10 +1396,10 @@
         <v>2</v>
       </c>
       <c r="N13" t="n">
-        <v>0.0469</v>
+        <v>0.0468</v>
       </c>
       <c r="O13" t="n">
-        <v>0.09379999999999999</v>
+        <v>0.0936</v>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>548117</v>
+        <v>531383</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1469,10 +1469,10 @@
         <v>2</v>
       </c>
       <c r="N14" t="n">
-        <v>0.1655</v>
+        <v>0.1653</v>
       </c>
       <c r="O14" t="n">
-        <v>0.331</v>
+        <v>0.3306</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>2183317</v>
+        <v>2145796</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>8124</v>
+        <v>8072</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -1615,10 +1615,10 @@
         <v>5</v>
       </c>
       <c r="N16" t="n">
-        <v>0.1715</v>
+        <v>0.1713</v>
       </c>
       <c r="O16" t="n">
-        <v>0.8575</v>
+        <v>0.8565</v>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>16381</v>
+        <v>16359</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
@@ -1688,10 +1688,10 @@
         <v>2</v>
       </c>
       <c r="N17" t="n">
-        <v>0.1541</v>
+        <v>0.1539</v>
       </c>
       <c r="O17" t="n">
-        <v>0.3082</v>
+        <v>0.3078</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>18163</v>
+        <v>18117</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -1761,10 +1761,10 @@
         <v>3</v>
       </c>
       <c r="N18" t="n">
-        <v>0.9795</v>
+        <v>0.978</v>
       </c>
       <c r="O18" t="n">
-        <v>2.9385</v>
+        <v>2.934</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
@@ -1834,10 +1834,10 @@
         <v>2</v>
       </c>
       <c r="N19" t="n">
-        <v>1.086</v>
+        <v>1.0844</v>
       </c>
       <c r="O19" t="n">
-        <v>2.172</v>
+        <v>2.1688</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>11365002</v>
+        <v>11255089</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1907,10 +1907,10 @@
         <v>14</v>
       </c>
       <c r="N20" t="n">
-        <v>0.0308</v>
+        <v>0.0307</v>
       </c>
       <c r="O20" t="n">
-        <v>0.4312</v>
+        <v>0.4298</v>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>185016</v>
+        <v>180566</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>8606300</v>
+        <v>8419104</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2053,10 +2053,10 @@
         <v>6</v>
       </c>
       <c r="N22" t="n">
-        <v>0.03</v>
+        <v>0.0299</v>
       </c>
       <c r="O22" t="n">
-        <v>0.18</v>
+        <v>0.1794</v>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>4108412</v>
+        <v>4072836</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>802102</v>
+        <v>792900</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2199,10 +2199,10 @@
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.0906</v>
       </c>
       <c r="O24" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.0906</v>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>802887</v>
+        <v>792933</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2272,10 +2272,10 @@
         <v>2</v>
       </c>
       <c r="N25" t="n">
-        <v>0.0815</v>
+        <v>0.0814</v>
       </c>
       <c r="O25" t="n">
-        <v>0.163</v>
+        <v>0.1628</v>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
@@ -2345,10 +2345,10 @@
         <v>3</v>
       </c>
       <c r="N26" t="n">
-        <v>0.4028</v>
+        <v>0.4022</v>
       </c>
       <c r="O26" t="n">
-        <v>1.2084</v>
+        <v>1.2066</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>112785</v>
+        <v>112535</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>37072</v>
+        <v>36929</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2564,10 +2564,10 @@
         <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>0.0784</v>
+        <v>0.07829999999999999</v>
       </c>
       <c r="O29" t="n">
-        <v>0.0784</v>
+        <v>0.07829999999999999</v>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
@@ -2583,43 +2583,43 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>S1 S2 S3</t>
+          <t>LED3 LED6 LED7 LED10 LED11 LED14 LED15 LED16</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S(LF)(SN)</t>
+          <t>jnj-ltji0112w120/35mil/845-860nm</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>JST-S2B-PH-K-S_V</t>
+          <t>JNJ-LTJI0112W120</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C157932</t>
+          <t>C19185834</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>S2B-PH-K-S-GW</t>
+          <t>JNJ-LTJI0112W120/35mil/845-860nm</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>JNJ OPTOELECTRONICS</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Push-Pull,P=2mm</t>
+          <t>SMD3535-3P</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2628,71 +2628,71 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>14990</v>
+        <v>438</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="N30" t="n">
-        <v>0.2125</v>
+        <v>0.338</v>
       </c>
       <c r="O30" t="n">
-        <v>0.6375</v>
+        <v>3.38</v>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C157932.html</t>
+          <t>https://www.lcsc.com/product-detail/C19185834.html</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
+          <t>-40℃~+100℃ 1.4V~2.1V、1.5V~2.3V 120° 1A 50nm 5V 75mW/sr@IF=350mA、140mW/sr@IF=1000mA 850nm SMD3535-3P Infrared LED Emitter</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>S1 S2 S3</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>k230d</t>
+          <t>S2B-PH-K-S(LF)(SN)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>JST-S2B-PH-K-S_V</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C42414902</t>
+          <t>C157932</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>K230D</t>
+          <t>S2B-PH-K-S-GW</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Canaan</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>BGA-256</t>
+          <t>Push-Pull,P=2mm</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2701,119 +2701,119 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>351</v>
+        <v>14970</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N31" t="n">
-        <v>13.3015</v>
+        <v>0.2122</v>
       </c>
       <c r="O31" t="n">
-        <v>13.3015</v>
+        <v>0.6366000000000001</v>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
+          <t>https://www.lcsc.com/product-detail/C157932.html</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
+          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 4.8mm 5.9mm 7.6mm Brass K Pin PA66 PH Right Angle Tin UL94V-0 White 弯插,P=2mm Wire To B</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>R5 R12 RD1 RD2</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>k230d</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>RES_0402</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C25867</t>
+          <t>C42414902</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0402WGF1501TCE</t>
+          <t>K230D</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>Canaan</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>BGA-256</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K32" t="n">
-        <v>2202449</v>
+        <v>340</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N32" t="n">
-        <v>0.0028</v>
+        <v>13.2813</v>
       </c>
       <c r="O32" t="n">
-        <v>0.0112</v>
+        <v>13.2813</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25867.html</t>
+          <t>https://www.lcsc.com/product-detail/C42414902.html</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>BGA-256 Microcontrollers (MCU/MPU/SOC) ROHS</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
+          <t>R5 R12 RD1 RD2</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="C33" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>1.5k</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2823,12 +2823,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C25741</t>
+          <t>C25867</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0402WGF1003TCE</t>
+          <t>0402WGF1501TCE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2847,46 +2847,46 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>9251477</v>
+        <v>2196154</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="N33" t="n">
-        <v>0.0024</v>
+        <v>0.0028</v>
       </c>
       <c r="O33" t="n">
-        <v>0.048</v>
+        <v>0.0112</v>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25741.html</t>
+          <t>https://www.lcsc.com/product-detail/C25867.html</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1.5kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70 RBT1</t>
+          <t>R6 R8 R19 R20 R23 R26 R27 R28 R30 R32 R35 R38 R45 R49 R51 R53 R58 R60 R61 R76</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C34" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2896,12 +2896,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C25744</t>
+          <t>C25741</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>0402WGF1002TCE</t>
+          <t>0402WGF1003TCE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2920,46 +2920,46 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>24434115</v>
+        <v>9086474</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N34" t="n">
-        <v>0.0033</v>
+        <v>0.0024</v>
       </c>
       <c r="O34" t="n">
-        <v>0.06270000000000001</v>
+        <v>0.048</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25744.html</t>
+          <t>https://www.lcsc.com/product-detail/C25741.html</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R2 R3 R10 R13 R16 R31 R34 R36 R39 R40 R41 R43 R44 R57 R64 R65 R67 R70 RBT1</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>120k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2969,12 +2969,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>C25750</t>
+          <t>C25744</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0402WGF1203TCE</t>
+          <t>0402WGF1002TCE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2989,50 +2989,50 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Promo</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K35" t="n">
-        <v>710920</v>
+        <v>24047452</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="N35" t="n">
-        <v>0.0011</v>
+        <v>0.0033</v>
       </c>
       <c r="O35" t="n">
-        <v>0.0011</v>
+        <v>0.06270000000000001</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25750.html</t>
+          <t>https://www.lcsc.com/product-detail/C25744.html</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R71 R72</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>120k</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C26083</t>
+          <t>C25750</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>0402WGF1004TCE</t>
+          <t>0402WGF1203TCE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3062,50 +3062,50 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Promo</t>
         </is>
       </c>
       <c r="K36" t="n">
-        <v>2735892</v>
+        <v>709925</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N36" t="n">
-        <v>0.0025</v>
+        <v>0.0011</v>
       </c>
       <c r="O36" t="n">
-        <v>0.005</v>
+        <v>0.0011</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C26083.html</t>
+          <t>https://www.lcsc.com/product-detail/C25750.html</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 120kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R71 R72</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3115,12 +3115,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>C11702</t>
+          <t>C26083</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>0402WGF1001TCE</t>
+          <t>0402WGF1004TCE</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3139,46 +3139,46 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>9043248</v>
+        <v>2709452</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N37" t="n">
-        <v>0.0018</v>
+        <v>0.0025</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0018</v>
+        <v>0.005</v>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C11702.html</t>
+          <t>https://www.lcsc.com/product-detail/C26083.html</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1MΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R37 R62</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>200R</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3188,12 +3188,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>C25087</t>
+          <t>C11702</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0402WGF2000TCE</t>
+          <t>0402WGF1001TCE</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3212,46 +3212,46 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>2707515</v>
+        <v>8811831</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N38" t="n">
-        <v>0.0028</v>
+        <v>0.0018</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0056</v>
+        <v>0.0018</v>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25087.html</t>
+          <t>https://www.lcsc.com/product-detail/C11702.html</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R59</t>
+          <t>R37 R62</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>200k</t>
+          <t>200R</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C25764</t>
+          <t>C25087</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0402WGF2003TCE</t>
+          <t>0402WGF2000TCE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3285,35 +3285,35 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2573903</v>
+        <v>2686228</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N39" t="n">
-        <v>0.0017</v>
+        <v>0.0028</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0017</v>
+        <v>0.0056</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25764.html</t>
+          <t>https://www.lcsc.com/product-detail/C25087.html</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>R69</t>
+          <t>R59</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>20k</t>
+          <t>200k</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3334,12 +3334,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>C25765</t>
+          <t>C25764</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>0402WGF2002TCE</t>
+          <t>0402WGF2003TCE</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>1349677</v>
+        <v>2495780</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3367,26 +3367,26 @@
         <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>0.0022</v>
+        <v>0.0017</v>
       </c>
       <c r="O40" t="n">
-        <v>0.0022</v>
+        <v>0.0017</v>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25765.html</t>
+          <t>https://www.lcsc.com/product-detail/C25764.html</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 20kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>R42</t>
+          <t>R69</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>22R</t>
+          <t>20k</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3407,12 +3407,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>C25092</t>
+          <t>C25765</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>0402WGF220JTCE</t>
+          <t>0402WGF2002TCE</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>3571844</v>
+        <v>1297912</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3440,37 +3440,37 @@
         <v>1</v>
       </c>
       <c r="N41" t="n">
-        <v>0.0027</v>
+        <v>0.0022</v>
       </c>
       <c r="O41" t="n">
-        <v>0.0027</v>
+        <v>0.0022</v>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25092.html</t>
+          <t>https://www.lcsc.com/product-detail/C25765.html</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 20kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>R33 R46 R47 R48 R52</t>
+          <t>R42</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>240R</t>
+          <t>22R</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3480,17 +3480,17 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>C324768</t>
+          <t>C25092</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>RC-02K2400FT</t>
+          <t>0402WGF220JTCE</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>FH (Guangdong Fenghua Advanced Tech)</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3500,50 +3500,50 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K42" t="n">
-        <v>298316</v>
+        <v>4161612</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N42" t="n">
-        <v>0.0013</v>
+        <v>0.0026</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0065</v>
+        <v>0.0026</v>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C324768.html</t>
+          <t>https://www.lcsc.com/product-detail/C25092.html</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>R63</t>
+          <t>R33 R46 R47 R48 R52</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>30k</t>
+          <t>240R</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3553,17 +3553,17 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>C49653548</t>
+          <t>C324768</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>GR0402F30KTAG00</t>
+          <t>RC-02K2400FT</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>FH (Guangdong Fenghua Advanced Tech)</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3577,35 +3577,35 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>7960</v>
+        <v>297406</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N43" t="n">
-        <v>0.0008</v>
+        <v>0.0013</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0008</v>
+        <v>0.0065</v>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
+          <t>https://www.lcsc.com/product-detail/C324768.html</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 240Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>R63</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -3616,7 +3616,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>33k</t>
+          <t>30k</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3626,17 +3626,17 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>C25779</t>
+          <t>C49653548</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>0402WGF3302TCE</t>
+          <t>GR0402F30KTAG00</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3646,11 +3646,11 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K44" t="n">
-        <v>1337444</v>
+        <v>7960</v>
       </c>
       <c r="L44" t="n">
         <v>1</v>
@@ -3659,37 +3659,37 @@
         <v>1</v>
       </c>
       <c r="N44" t="n">
-        <v>0.0056</v>
+        <v>0.0008</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0056</v>
+        <v>0.0008</v>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25779.html</t>
+          <t>https://www.lcsc.com/product-detail/C49653548.html</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 30kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>R14 R15 R17 R18 R73 R74</t>
+          <t>R25</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>33k</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3699,12 +3699,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>C25900</t>
+          <t>C25779</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>0402WGF4701TCE</t>
+          <t>0402WGF3302TCE</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3723,46 +3723,46 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>16342107</v>
+        <v>1324136</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N45" t="n">
-        <v>0.0026</v>
+        <v>0.0056</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0156</v>
+        <v>0.0056</v>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25900.html</t>
+          <t>https://www.lcsc.com/product-detail/C25779.html</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 33kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R21 RB1 RB2 RB3 RB4 RB5 RB6</t>
+          <t>R14 R15 R17 R18 R73 R74</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>47k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3772,12 +3772,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>C25792</t>
+          <t>C25900</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>0402WGF4702TCE</t>
+          <t>0402WGF4701TCE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3796,46 +3796,46 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>5835600</v>
+        <v>16266118</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N46" t="n">
-        <v>0.0025</v>
+        <v>0.0026</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0175</v>
+        <v>0.0156</v>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25792.html</t>
+          <t>https://www.lcsc.com/product-detail/C25900.html</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>R1 R4 R9 R11</t>
+          <t>R21 RB1 RB2 RB3 RB4 RB5 RB6</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C47" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>5.1k</t>
+          <t>47k</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3845,12 +3845,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>C25905</t>
+          <t>C25792</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>0402WGF5101TCE</t>
+          <t>0402WGF4702TCE</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3869,46 +3869,46 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>6573651</v>
+        <v>5815081</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N47" t="n">
-        <v>0.0023</v>
+        <v>0.0025</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0092</v>
+        <v>0.0175</v>
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25905.html</t>
+          <t>https://www.lcsc.com/product-detail/C25792.html</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>R22 R50</t>
+          <t>R1 R4 R9 R11</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C48" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>511k</t>
+          <t>5.1k</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3918,17 +3918,17 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>C49655223</t>
+          <t>C25905</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>GR0402F511KTAG00</t>
+          <t>0402WGF5101TCE</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>GiantOhm</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3938,50 +3938,50 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K48" t="n">
-        <v>7480</v>
+        <v>6529013</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N48" t="n">
-        <v>0.0008</v>
+        <v>0.0023</v>
       </c>
       <c r="O48" t="n">
-        <v>0.0016</v>
+        <v>0.0092</v>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
+          <t>https://www.lcsc.com/product-detail/C25905.html</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>R56</t>
+          <t>R22 R50</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>51k</t>
+          <t>511k</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3991,17 +3991,17 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>C25794</t>
+          <t>C49655223</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>0402WGF5102TCE</t>
+          <t>GR0402F511KTAG00</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>UNI-ROYAL(Uniroyal Elec)</t>
+          <t>GiantOhm</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4011,50 +4011,50 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="K49" t="n">
-        <v>2017249</v>
+        <v>7480</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N49" t="n">
-        <v>0.0018</v>
+        <v>0.0008</v>
       </c>
       <c r="O49" t="n">
-        <v>0.0018</v>
+        <v>0.0016</v>
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C25794.html</t>
+          <t>https://www.lcsc.com/product-detail/C49655223.html</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 51kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 511kΩ 62.5mW Thick Film Resistor ±1% 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>R24 R55</t>
+          <t>R56</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>91k</t>
+          <t>51k</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -4064,17 +4064,17 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C54920709</t>
+          <t>C25794</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>HRC0402F9102DNTO</t>
+          <t>0402WGF5102TCE</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>HWA CHN</t>
+          <t>UNI-ROYAL(Uniroyal Elec)</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4084,75 +4084,75 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K50" t="n">
-        <v>130638</v>
+        <v>2009174</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N50" t="n">
-        <v>0.0007</v>
+        <v>0.0018</v>
       </c>
       <c r="O50" t="n">
-        <v>0.0014</v>
+        <v>0.0018</v>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
+          <t>https://www.lcsc.com/product-detail/C25794.html</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 50V 51kΩ 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>R24 R55</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>91k</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>RGT0016C_V</t>
+          <t>RES_0402</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>C129319</t>
+          <t>C54920709</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>BQ24072TRGTR</t>
+          <t>HRC0402F9102DNTO</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>HWA CHN</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>QFN-16-EP(3x3)</t>
+          <t>0402</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -4161,61 +4161,61 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>356</v>
+        <v>130638</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N51" t="n">
-        <v>2.1673</v>
+        <v>0.0007</v>
       </c>
       <c r="O51" t="n">
-        <v>2.1673</v>
+        <v>0.0014</v>
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C129319.html</t>
+          <t>https://www.lcsc.com/product-detail/C54920709.html</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
+          <t>-55℃~+155℃ 50V 62.5mW 91kΩ Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>U14 U15</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>TPS61161DRVR</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>TPS61160ADRVT</t>
+          <t>RGT0016C_V</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C324075</t>
+          <t>C129319</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>TPS61161DRVR</t>
+          <t>BQ24072TRGTR</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>WSON-6-EP(2x2)</t>
+          <t>QFN-16-EP(3x3)</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -4234,35 +4234,35 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>2574</v>
+        <v>361</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>0.4106</v>
+        <v>2.164</v>
       </c>
       <c r="O52" t="n">
-        <v>0.8212</v>
+        <v>2.164</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C324075.html</t>
+          <t>https://www.lcsc.com/product-detail/C129319.html</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 2% 2.7V~18V 38V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
+          <t>0℃~+125℃ 1.5A 1.5mA 4.2V 4.35V~6.4V Charging IC Lithium Battery Support QFN-16-EP(3x3) Battery Management ROHS</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>USBC1 USBC2</t>
+          <t>U14 U15</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -4273,32 +4273,32 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>type-c-31-m-12</t>
+          <t>TPS61161DRVR</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>TPS61160ADRVT</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>C324075</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>TPS61161DRVR</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Korean Hroparts Elec</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>SMD</t>
+          <t>WSON-6-EP(2x2)</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>98803</v>
+        <v>2574</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
@@ -4316,62 +4316,62 @@
         <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>0.179</v>
+        <v>0.41</v>
       </c>
       <c r="O53" t="n">
-        <v>0.358</v>
+        <v>0.82</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C165948.html</t>
+          <t>https://www.lcsc.com/product-detail/C324075.html</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
+          <t>-40℃~+85℃ 1 2% 2.7V~18V 38V 600kHz Boost Built-in DC-DC Over Voltage Protection、Over-Temperature Protection (OTP) PWM WS</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>USBC1 USBC2</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>type-c-31-m-12</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ch340x</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>C3035748</t>
+          <t>C165948</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>CH340X</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>WCH(Jiangsu Qin Heng)</t>
+          <t>Korean Hroparts Elec</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>MSOP-10</t>
+          <t>SMD</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4380,35 +4380,35 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>16113</v>
+        <v>94752</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N54" t="n">
-        <v>0.6629</v>
+        <v>0.1787</v>
       </c>
       <c r="O54" t="n">
-        <v>0.6629</v>
+        <v>0.3574</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
+          <t>https://www.lcsc.com/product-detail/C165948.html</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
+          <t>-30℃~+80℃ 1 10,000 cycles 16P 20V 5A 7.35mm Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LED3 LED6 LED7 LED10 LED11 LED14 LED15 LED16</t>
+          <t>LED1 LED2 LED4 LED5 LED8 LED9 LED12 LED13</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -4419,27 +4419,27 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>jnj-ltji0112w120/35mil/845-860nm</t>
+          <t>xl-hd3535uwc-a2</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>jnj-ltji0112w120/35mil/845-860nm</t>
+          <t>XL-HD3535UWC-A2</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>C19185834</t>
+          <t>C3646951</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>JNJ-LTJI0112W120/35mil/845-860nm</t>
+          <t>XL-HD3535UWC-A2</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>JNJ OPTOELECTRONICS</t>
+          <t>XINGLIGHT</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -4453,35 +4453,35 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>438</v>
+        <v>19724</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="N55" t="n">
-        <v>0.3385</v>
+        <v>0.3074</v>
       </c>
       <c r="O55" t="n">
-        <v>3.385</v>
+        <v>2.4592</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C19185834.html</t>
+          <t>https://www.lcsc.com/product-detail/C3646951.html</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>-40℃~+100℃ 1.4V~2.1V、1.5V~2.3V 120° 1A 50nm 5V 75mW/sr@IF=350mA、140mW/sr@IF=1000mA 850nm SMD3535-3P Infrared LED Emitter</t>
+          <t>-40℃~+85℃ 130° 1W 2.8V~3.6V 350mA 5500K~7000K Discrete Diode Top-mount Water Clear White SMD3535-3P LED Indication - Dis</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>U13</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -4492,32 +4492,32 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>msm381acb026</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>mems</t>
+          <t>ch340x</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>C51928208</t>
+          <t>C3035748</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>MSM381ACB026</t>
+          <t>CH340X</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>MEMS</t>
+          <t>WCH(Jiangsu Qin Heng)</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>LGA-3(1.9x2.8)</t>
+          <t>MSOP-10</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -4526,7 +4526,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>6244</v>
+        <v>15712</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
@@ -4535,26 +4535,26 @@
         <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>0.3025</v>
+        <v>0.6619</v>
       </c>
       <c r="O56" t="n">
-        <v>0.3025</v>
+        <v>0.6619</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
+          <t>https://www.lcsc.com/product-detail/C3035748.html</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
+          <t>-20℃~+70℃ 2Mbps 3.3V、5V USB 2.0 USB to serial、USB to Parallel MSOP-10 USB Converters ROHS</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>U16</t>
+          <t>U13</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -4565,32 +4565,32 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>w25n02kvzeir</t>
+          <t>msm381acb026</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>w25n02</t>
+          <t>mems</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>C17626844</t>
+          <t>C51928208</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>W25N02KVZEIR</t>
+          <t>MSM381ACB026</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Winbond Elec</t>
+          <t>MEMS</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>WSON-8(6x8)</t>
+          <t>LGA-3(1.9x2.8)</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="K57" t="n">
-        <v>7624</v>
+        <v>6244</v>
       </c>
       <c r="L57" t="n">
         <v>1</v>
@@ -4608,62 +4608,62 @@
         <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>11.1515</v>
+        <v>0.302</v>
       </c>
       <c r="O57" t="n">
-        <v>11.1515</v>
+        <v>0.302</v>
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17626844.html</t>
+          <t>https://www.lcsc.com/product-detail/C51928208.html</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 25ns 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function</t>
+          <t xml:space="preserve">-38dB 0.9mm 1.85mm 170Ω 175uA 2.75mm 3.6V 64dB Analog output Omnidirectional Omnidirectional pickup LGA-3(1.9x2.8) MEMS </t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>LED1 LED2 LED4 LED5 LED8 LED9 LED12 LED13</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C58" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>xl-hd3535uwc-a2</t>
+          <t>w25n02kvzeir</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>xl-hd3535uwc-a2</t>
+          <t>w25n02</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>C3646951</t>
+          <t>C17626844</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>XL-HD3535UWC-A2</t>
+          <t>W25N02KVZEIR</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>XINGLIGHT</t>
+          <t>Winbond Elec</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>SMD3535-3P</t>
+          <t>WSON-8(6x8)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -4672,28 +4672,28 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>19724</v>
+        <v>7614</v>
       </c>
       <c r="L58" t="n">
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="N58" t="n">
-        <v>0.3078</v>
+        <v>11.1345</v>
       </c>
       <c r="O58" t="n">
-        <v>2.4624</v>
+        <v>11.1345</v>
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C3646951.html</t>
+          <t>https://www.lcsc.com/product-detail/C17626844.html</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 130° 1W 2.8V~3.6V 350mA 5500K~7000K Discrete Diode Top-mount Water Clear White SMD3535-3P LED Indication - Dis</t>
+          <t>-40℃~+85℃ 10 years 104MHz 10uA 2.7V~3.6V 25ns 2Gbit 2ms 60,000 Cycles 700us Read buffer function、Software reset function</t>
         </is>
       </c>
     </row>
@@ -5292,14 +5292,49 @@
       <c r="P75" t="inlineStr"/>
       <c r="Q75" t="inlineStr"/>
     </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>CT1</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>NF</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>NO PART</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="O77" t="n">
-        <v>47.97</v>
+      <c r="O78" t="n">
+        <v>47.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fab package from the 2026-09-24 22:48 outputs: gerbers, JLCPCB BOM and CPL
LEAKCAM_gerber.zip: all copper, mask, silk, paste and both drill files byte-identical to the
Altium export; outline 61.00 x 65.00 mm from the ODB++ profile, no cutouts on it.
BOM_ASSEMBLY.csv / PickPlace_MIFA.csv: 244 placements, 56 part numbers, 0 mismatches against the
schematic and the ODB++ board; S1-S3 hand-soldered. New: CB1 10 uF, CB2 100 nF on MIC_BIAS.
Order lists regenerated from the schematic with JLCPCB stock (lowest: U11 216, U3 340, U1 356,
IR LEDs 438; all cover a board).
FAB_NOTES: the mic acoustic port moved with U13, now X57.566 Y2.563.
DESIGN.md: MIC_BIAS caps and PR1 pad 6 done; C97/C101 move stays optional.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>40084</v>
+        <v>39775</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2559768</v>
+        <v>2573418</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -758,14 +758,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C10 C12 C13 C25 C26 C27 C28 C29 C30 C31 C37 C39 C40 C42 C43 C44 C45 C46 C47 C48 C49 C51 C52 C53 C54 C55 C56 C57 C58 C63 C65 C66 C67 C68 C69 C70 C71 C72 C73 C74 C75 C76 C77 C78 C79 C80 C81 C82 C84 C85 C93 C94 C100</t>
+          <t>C10 C12 C13 C25 C26 C27 C28 C29 C30 C31 C37 C39 C40 C42 C43 C44 C45 C46 C47 C48 C49 C51 C52 C53 C54 C55 C56 C57 C58 C63 C65 C66 C67 C68 C69 C70 C71 C72 C73 C74 C75 C76 C77 C78 C79 C80 C81 C82 C84 C85 C93 C94 C100 CB2</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C5" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -809,13 +809,13 @@
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N5" t="n">
         <v>0.0021</v>
       </c>
       <c r="O5" t="n">
-        <v>0.1113</v>
+        <v>0.1134</v>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>11871497</v>
+        <v>11747101</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -885,10 +885,10 @@
         <v>12</v>
       </c>
       <c r="N6" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="O6" t="n">
-        <v>0.1008</v>
+        <v>0.1044</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3507965</v>
+        <v>3487438</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>1146422</v>
+        <v>2088873</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>719780</v>
+        <v>715398</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2454283</v>
+        <v>2418673</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>2663217</v>
+        <v>2663114</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>639782</v>
+        <v>630235</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>531383</v>
+        <v>502470</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>2145796</v>
+        <v>2123653</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1542,10 +1542,10 @@
         <v>4</v>
       </c>
       <c r="N15" t="n">
-        <v>0.0151</v>
+        <v>0.014</v>
       </c>
       <c r="O15" t="n">
-        <v>0.0604</v>
+        <v>0.056</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>8072</v>
+        <v>8073</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>16359</v>
+        <v>16347</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>18117</v>
+        <v>18161</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>8269</v>
+        <v>8249</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1853,14 +1853,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C2 C3 C4 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106</t>
+          <t>C2 C3 C4 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106 CB1</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C20" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1898,19 +1898,19 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>11255089</v>
+        <v>11157124</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="N20" t="n">
         <v>0.0307</v>
       </c>
       <c r="O20" t="n">
-        <v>0.4298</v>
+        <v>0.4605</v>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>180566</v>
+        <v>177596</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>8419104</v>
+        <v>8380462</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>4072836</v>
+        <v>4032884</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>792900</v>
+        <v>784767</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>792933</v>
+        <v>1079991</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>2525</v>
+        <v>2425</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>112535</v>
+        <v>112055</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>36929</v>
+        <v>33690</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>14970</v>
+        <v>14960</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2196154</v>
+        <v>2189608</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>9086474</v>
+        <v>8993673</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>24047452</v>
+        <v>23760892</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>709925</v>
+        <v>708282</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>2709452</v>
+        <v>2687913</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>8811831</v>
+        <v>8698876</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2686228</v>
+        <v>2674322</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2495780</v>
+        <v>2475159</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1297912</v>
+        <v>1292693</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>4161612</v>
+        <v>4126691</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>297406</v>
+        <v>296106</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>1324136</v>
+        <v>1317264</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>16266118</v>
+        <v>16179485</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>5815081</v>
+        <v>5801606</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>6529013</v>
+        <v>6495106</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>7480</v>
+        <v>7460</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>2009174</v>
+        <v>1989838</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>130638</v>
+        <v>130618</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
@@ -4234,7 +4234,7 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>2574</v>
+        <v>2074</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>94752</v>
+        <v>92055</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>19724</v>
+        <v>19504</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4526,7 +4526,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>15712</v>
+        <v>16877</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
@@ -5260,7 +5260,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>PR1</t>
+          <t>CT1</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>CON5P</t>
+          <t>NF</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -5295,7 +5295,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CT1</t>
+          <t>PR1</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>NF</t>
+          <t>CON6P</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -5334,7 +5334,7 @@
         </is>
       </c>
       <c r="O78" t="n">
-        <v>47.89</v>
+        <v>47.92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
C86 1 uF 0603: C696901 (Extended) -> C15849 (Basic), saves a loading fee
Same 0603 package (FP-GRM188: 1.6 x 0.8 mm; CL10A105KB8NNNC 1.6 x 0.8 x 0.8 mm), 50 V X5R
instead of 16 V, on 3V3. Description set in FLASH.SchDoc; the pick-and-place CSV's Comment/
Description re-synced from the sheets (coordinates untouched) until the next PCB update;
BOM_ASSEMBLY, CPL and order lists regenerated, 0 mismatches against sheets and board.
R22/R50 511k stay: the only fee-free 510k (C11616) has a JLCPCB minimum order of 2006 pcs,
which costs more than the fee it saves.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2573418</v>
+        <v>2573413</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>11747101</v>
+        <v>11747051</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>502470</v>
+        <v>502460</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>8249</v>
+        <v>8244</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>11157124</v>
+        <v>11157194</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1947,17 +1947,17 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>C696901</t>
+          <t>C15849</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>TCC0603X5R105K160CT</t>
+          <t>CL10A105KB8NNNC</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CCTC</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1967,11 +1967,11 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="K21" t="n">
-        <v>177596</v>
+        <v>6222545</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -1980,19 +1980,19 @@
         <v>1</v>
       </c>
       <c r="N21" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0147</v>
       </c>
       <c r="O21" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0147</v>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C696901.html</t>
+          <t>https://www.lcsc.com/product-detail/C15849.html</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>16V 1uF X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>1uF 50V X5R ±10% 0603 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>8380462</v>
+        <v>8380482</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>4032884</v>
+        <v>4032496</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>784767</v>
+        <v>784743</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>1079991</v>
+        <v>1079967</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>8993673</v>
+        <v>8993380</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>23760892</v>
+        <v>23760830</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>2687913</v>
+        <v>2687563</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1292693</v>
+        <v>1292673</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>4126691</v>
+        <v>4126411</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>1317264</v>
+        <v>1317244</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>16179485</v>
+        <v>16179440</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>6495106</v>
+        <v>6495076</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>92055</v>
+        <v>92009</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -5334,7 +5334,7 @@
         </is>
       </c>
       <c r="O78" t="n">
-        <v>47.92</v>
+        <v>47.93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fab package from the 07:06 export: R54 at the K230 end, ground returns fixed
Gerber zip: all 14 Altium files byte-identical, outline 61.00 x 65.00 mm from the ODB++ profile.
BOM_ASSEMBLY / CPL: 245 placements, 56 part numbers (R54 22R shares C25092 with R42), 0 mismatches
against sheets and board. Order lists regenerated with JLCPCB stock.
Layout review (ODB++): no reference gaps on the SDIO clock or SPI_IO0/USB, every SDIO via within
1 mm of a GND via except D1/D2 at the K230 (1.8 mm), 403 GND vias, no plane point more than 5 mm
from one; worst estimated reflection 0.7 % (SDIO) / 3 % (MIPI), crosstalk 38 mV.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>39775</v>
+        <v>39770</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -593,10 +593,10 @@
         <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>0.7652</v>
+        <v>0.765</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7652</v>
+        <v>0.765</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -666,10 +666,10 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>2.2345</v>
+        <v>2.2339</v>
       </c>
       <c r="O3" t="n">
-        <v>2.2345</v>
+        <v>2.2339</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2573413</v>
+        <v>2573977</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>11747051</v>
+        <v>11725148</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3487438</v>
+        <v>3485378</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>2088873</v>
+        <v>2088014</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>715398</v>
+        <v>714817</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2418673</v>
+        <v>2417993</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>630235</v>
+        <v>629963</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>502460</v>
+        <v>502309</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1469,10 +1469,10 @@
         <v>2</v>
       </c>
       <c r="N14" t="n">
-        <v>0.1653</v>
+        <v>0.1652</v>
       </c>
       <c r="O14" t="n">
-        <v>0.3306</v>
+        <v>0.3304</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>2123653</v>
+        <v>2122375</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>8073</v>
+        <v>8066</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -1615,10 +1615,10 @@
         <v>5</v>
       </c>
       <c r="N16" t="n">
-        <v>0.1713</v>
+        <v>0.1712</v>
       </c>
       <c r="O16" t="n">
-        <v>0.8565</v>
+        <v>0.856</v>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
@@ -1688,10 +1688,10 @@
         <v>2</v>
       </c>
       <c r="N17" t="n">
-        <v>0.1539</v>
+        <v>0.1538</v>
       </c>
       <c r="O17" t="n">
-        <v>0.3078</v>
+        <v>0.3076</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>18161</v>
+        <v>18150</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -1761,10 +1761,10 @@
         <v>3</v>
       </c>
       <c r="N18" t="n">
-        <v>0.978</v>
+        <v>0.9778</v>
       </c>
       <c r="O18" t="n">
-        <v>2.934</v>
+        <v>2.9334</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
@@ -1834,10 +1834,10 @@
         <v>2</v>
       </c>
       <c r="N19" t="n">
-        <v>1.0844</v>
+        <v>1.0841</v>
       </c>
       <c r="O19" t="n">
-        <v>2.1688</v>
+        <v>2.1682</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>11157194</v>
+        <v>11165420</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>6222545</v>
+        <v>6242395</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>8380482</v>
+        <v>8380118</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>4032496</v>
+        <v>4031889</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>784743</v>
+        <v>783615</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>1079967</v>
+        <v>1078056</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2345,10 +2345,10 @@
         <v>3</v>
       </c>
       <c r="N26" t="n">
-        <v>0.4022</v>
+        <v>0.4021</v>
       </c>
       <c r="O26" t="n">
-        <v>1.2066</v>
+        <v>1.2063</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
@@ -2637,10 +2637,10 @@
         <v>10</v>
       </c>
       <c r="N30" t="n">
-        <v>0.338</v>
+        <v>0.3379</v>
       </c>
       <c r="O30" t="n">
-        <v>3.38</v>
+        <v>3.379</v>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
@@ -2783,10 +2783,10 @@
         <v>1</v>
       </c>
       <c r="N32" t="n">
-        <v>13.2813</v>
+        <v>13.2782</v>
       </c>
       <c r="O32" t="n">
-        <v>13.2813</v>
+        <v>13.2782</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2189608</v>
+        <v>2187929</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>8993380</v>
+        <v>8990856</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>23760830</v>
+        <v>23783214</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>2687563</v>
+        <v>2684788</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>8698876</v>
+        <v>8701757</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2674322</v>
+        <v>2674127</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2475159</v>
+        <v>2474160</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1292673</v>
+        <v>1295185</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3459,14 +3459,14 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>R42</t>
+          <t>R42 R54</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -3504,19 +3504,19 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>4126411</v>
+        <v>4120724</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N42" t="n">
         <v>0.0026</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0026</v>
+        <v>0.0052</v>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>296106</v>
+        <v>296076</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>1317244</v>
+        <v>1315820</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>16179440</v>
+        <v>16178720</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>5801606</v>
+        <v>5812591</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>6495076</v>
+        <v>6493121</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>7460</v>
+        <v>7360</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>1989838</v>
+        <v>2002350</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>130618</v>
+        <v>130518</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
@@ -4243,10 +4243,10 @@
         <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>2.164</v>
+        <v>2.1635</v>
       </c>
       <c r="O52" t="n">
-        <v>2.164</v>
+        <v>2.1635</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
@@ -4316,10 +4316,10 @@
         <v>2</v>
       </c>
       <c r="N53" t="n">
-        <v>0.41</v>
+        <v>0.4099</v>
       </c>
       <c r="O53" t="n">
-        <v>0.82</v>
+        <v>0.8198</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>92009</v>
+        <v>91756</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4462,10 +4462,10 @@
         <v>8</v>
       </c>
       <c r="N55" t="n">
-        <v>0.3074</v>
+        <v>0.3073</v>
       </c>
       <c r="O55" t="n">
-        <v>2.4592</v>
+        <v>2.4584</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
@@ -4526,7 +4526,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>16877</v>
+        <v>16866</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
@@ -4535,10 +4535,10 @@
         <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>0.6619</v>
+        <v>0.6618000000000001</v>
       </c>
       <c r="O56" t="n">
-        <v>0.6619</v>
+        <v>0.6618000000000001</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
@@ -4681,10 +4681,10 @@
         <v>1</v>
       </c>
       <c r="N58" t="n">
-        <v>11.1345</v>
+        <v>11.1319</v>
       </c>
       <c r="O58" t="n">
-        <v>11.1345</v>
+        <v>11.1319</v>
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
@@ -5334,7 +5334,7 @@
         </is>
       </c>
       <c r="O78" t="n">
-        <v>47.93</v>
+        <v>47.92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fab package from the 2026-09-25 20:15 export: stitching vias tented
LEAKCAM_gerber.zip rebuilt: all 14 Altium files byte-identical, outline 61.00 x 65.00 mm.
The 153 GND stitching vias are now tented on both sides; the only via openings left are vias
inside pads (U3 BGA balls and SMD pads), which need epoxy filled & capped vias (FAB_NOTES).
BOM_ASSEMBLY and PickPlace_MIFA unchanged (placements identical, rotation corrections applied,
0 mismatches against sheets and board; every non-passive part lands pad for pad). Order lists
for 2 boards.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Needed (1 boards)</t>
+          <t>Needed (2 boards)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -546,7 +546,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -584,19 +584,19 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>39770</v>
+        <v>39761</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N2" t="n">
         <v>0.765</v>
       </c>
       <c r="O2" t="n">
-        <v>0.765</v>
+        <v>1.53</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -619,7 +619,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -663,13 +663,13 @@
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N3" t="n">
         <v>2.2339</v>
       </c>
       <c r="O3" t="n">
-        <v>2.2339</v>
+        <v>4.4678</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -692,7 +692,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -730,19 +730,19 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2573977</v>
+        <v>2506628</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N4" t="n">
         <v>0.0384</v>
       </c>
       <c r="O4" t="n">
-        <v>0.07679999999999999</v>
+        <v>0.1536</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
         <v>54</v>
       </c>
       <c r="C5" t="n">
-        <v>54</v>
+        <v>108</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -809,13 +809,13 @@
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>54</v>
+        <v>108</v>
       </c>
       <c r="N5" t="n">
         <v>0.0021</v>
       </c>
       <c r="O5" t="n">
-        <v>0.1134</v>
+        <v>0.2268</v>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
@@ -838,7 +838,7 @@
         <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -876,19 +876,19 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>11725148</v>
+        <v>11684241</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="N6" t="n">
         <v>0.008699999999999999</v>
       </c>
       <c r="O6" t="n">
-        <v>0.1044</v>
+        <v>0.2088</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -949,19 +949,19 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3485378</v>
+        <v>3484695</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N7" t="n">
         <v>0.004</v>
       </c>
       <c r="O7" t="n">
-        <v>0.008</v>
+        <v>0.016</v>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
@@ -984,7 +984,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1022,19 +1022,19 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>2088014</v>
+        <v>2087450</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N8" t="n">
         <v>0.0054</v>
       </c>
       <c r="O8" t="n">
-        <v>0.0108</v>
+        <v>0.0216</v>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
@@ -1057,7 +1057,7 @@
         <v>5</v>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1095,19 +1095,19 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>714817</v>
+        <v>715431</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N9" t="n">
         <v>0.007</v>
       </c>
       <c r="O9" t="n">
-        <v>0.035</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
@@ -1130,7 +1130,7 @@
         <v>2</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1168,19 +1168,19 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2417993</v>
+        <v>2407623</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N10" t="n">
         <v>0.0049</v>
       </c>
       <c r="O10" t="n">
-        <v>0.0098</v>
+        <v>0.0196</v>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
         <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1241,19 +1241,19 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>2663114</v>
+        <v>2663079</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N11" t="n">
         <v>0.0246</v>
       </c>
       <c r="O11" t="n">
-        <v>0.0738</v>
+        <v>0.1476</v>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
         <v>2</v>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1320,13 +1320,13 @@
         <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N12" t="n">
         <v>0.0697</v>
       </c>
       <c r="O12" t="n">
-        <v>0.1394</v>
+        <v>0.2788</v>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
         <v>2</v>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1387,19 +1387,19 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>629963</v>
+        <v>636429</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N13" t="n">
         <v>0.0468</v>
       </c>
       <c r="O13" t="n">
-        <v>0.0936</v>
+        <v>0.1872</v>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
@@ -1422,7 +1422,7 @@
         <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1460,19 +1460,19 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>502309</v>
+        <v>500802</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N14" t="n">
         <v>0.1652</v>
       </c>
       <c r="O14" t="n">
-        <v>0.3304</v>
+        <v>0.6608000000000001</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1533,19 +1533,19 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>2122375</v>
+        <v>2119409</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N15" t="n">
         <v>0.014</v>
       </c>
       <c r="O15" t="n">
-        <v>0.056</v>
+        <v>0.112</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
@@ -1568,7 +1568,7 @@
         <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1606,19 +1606,19 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>8066</v>
+        <v>8059</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N16" t="n">
         <v>0.1712</v>
       </c>
       <c r="O16" t="n">
-        <v>0.856</v>
+        <v>1.712</v>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
@@ -1641,7 +1641,7 @@
         <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1679,19 +1679,19 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>16347</v>
+        <v>16344</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N17" t="n">
         <v>0.1538</v>
       </c>
       <c r="O17" t="n">
-        <v>0.3076</v>
+        <v>0.6152</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
@@ -1714,7 +1714,7 @@
         <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1752,19 +1752,19 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>18150</v>
+        <v>18115</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N18" t="n">
         <v>0.9778</v>
       </c>
       <c r="O18" t="n">
-        <v>2.9334</v>
+        <v>5.8668</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
@@ -1787,7 +1787,7 @@
         <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1831,13 +1831,13 @@
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N19" t="n">
         <v>1.0841</v>
       </c>
       <c r="O19" t="n">
-        <v>2.1682</v>
+        <v>4.3364</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
@@ -1860,7 +1860,7 @@
         <v>15</v>
       </c>
       <c r="C20" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1898,19 +1898,19 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>11165420</v>
+        <v>11251848</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="N20" t="n">
         <v>0.0307</v>
       </c>
       <c r="O20" t="n">
-        <v>0.4605</v>
+        <v>0.921</v>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
@@ -1933,7 +1933,7 @@
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1971,19 +1971,19 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>6242395</v>
+        <v>6248852</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N21" t="n">
         <v>0.0147</v>
       </c>
       <c r="O21" t="n">
-        <v>0.0147</v>
+        <v>0.0294</v>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
@@ -2006,7 +2006,7 @@
         <v>6</v>
       </c>
       <c r="C22" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2044,19 +2044,19 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>8380118</v>
+        <v>8373464</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="N22" t="n">
         <v>0.0299</v>
       </c>
       <c r="O22" t="n">
-        <v>0.1794</v>
+        <v>0.3588</v>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2117,19 +2117,19 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>4031889</v>
+        <v>4013302</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N23" t="n">
         <v>0.0073</v>
       </c>
       <c r="O23" t="n">
-        <v>0.0073</v>
+        <v>0.0146</v>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
@@ -2152,7 +2152,7 @@
         <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2190,19 +2190,19 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>783615</v>
+        <v>783049</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N24" t="n">
         <v>0.0906</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0906</v>
+        <v>0.1812</v>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
@@ -2225,7 +2225,7 @@
         <v>2</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2263,19 +2263,19 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>1078056</v>
+        <v>1073957</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N25" t="n">
         <v>0.0814</v>
       </c>
       <c r="O25" t="n">
-        <v>0.1628</v>
+        <v>0.3256</v>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2342,13 +2342,13 @@
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N26" t="n">
         <v>0.4021</v>
       </c>
       <c r="O26" t="n">
-        <v>1.2063</v>
+        <v>2.4126</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
@@ -2371,7 +2371,7 @@
         <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2415,13 +2415,13 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N27" t="n">
         <v>0.0043</v>
       </c>
       <c r="O27" t="n">
-        <v>0.0043</v>
+        <v>0.0086</v>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
@@ -2444,7 +2444,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2482,19 +2482,19 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>43669</v>
+        <v>43619</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N28" t="n">
         <v>0.0039</v>
       </c>
       <c r="O28" t="n">
-        <v>0.0039</v>
+        <v>0.0078</v>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         <v>1</v>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2561,13 +2561,13 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N29" t="n">
         <v>0.07829999999999999</v>
       </c>
       <c r="O29" t="n">
-        <v>0.07829999999999999</v>
+        <v>0.1566</v>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
@@ -2590,7 +2590,7 @@
         <v>8</v>
       </c>
       <c r="C30" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2634,13 +2634,13 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="N30" t="n">
         <v>0.3379</v>
       </c>
       <c r="O30" t="n">
-        <v>3.379</v>
+        <v>5.4064</v>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
@@ -2663,7 +2663,7 @@
         <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2707,13 +2707,13 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N31" t="n">
         <v>0.2122</v>
       </c>
       <c r="O31" t="n">
-        <v>0.6366000000000001</v>
+        <v>1.2732</v>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
@@ -2736,7 +2736,7 @@
         <v>1</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2780,13 +2780,13 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N32" t="n">
         <v>13.2782</v>
       </c>
       <c r="O32" t="n">
-        <v>13.2782</v>
+        <v>26.5564</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
@@ -2809,7 +2809,7 @@
         <v>4</v>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2847,19 +2847,19 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2187929</v>
+        <v>2186424</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N33" t="n">
         <v>0.0028</v>
       </c>
       <c r="O33" t="n">
-        <v>0.0112</v>
+        <v>0.0224</v>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
@@ -2882,7 +2882,7 @@
         <v>20</v>
       </c>
       <c r="C34" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2920,19 +2920,19 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>8990856</v>
+        <v>8980361</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="N34" t="n">
         <v>0.0024</v>
       </c>
       <c r="O34" t="n">
-        <v>0.048</v>
+        <v>0.096</v>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
@@ -2955,7 +2955,7 @@
         <v>19</v>
       </c>
       <c r="C35" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2993,19 +2993,19 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>23783214</v>
+        <v>23769742</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="N35" t="n">
         <v>0.0033</v>
       </c>
       <c r="O35" t="n">
-        <v>0.06270000000000001</v>
+        <v>0.1254</v>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
@@ -3028,7 +3028,7 @@
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -3066,19 +3066,19 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>708282</v>
+        <v>708170</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N36" t="n">
         <v>0.0011</v>
       </c>
       <c r="O36" t="n">
-        <v>0.0011</v>
+        <v>0.0022</v>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
@@ -3101,7 +3101,7 @@
         <v>2</v>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -3139,19 +3139,19 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>2684788</v>
+        <v>2682285</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N37" t="n">
         <v>0.0025</v>
       </c>
       <c r="O37" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
@@ -3174,7 +3174,7 @@
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -3212,19 +3212,19 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>8701757</v>
+        <v>8695277</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N38" t="n">
         <v>0.0018</v>
       </c>
       <c r="O38" t="n">
-        <v>0.0018</v>
+        <v>0.0036</v>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
@@ -3247,7 +3247,7 @@
         <v>2</v>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -3285,19 +3285,19 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2674127</v>
+        <v>2672337</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N39" t="n">
         <v>0.0028</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0056</v>
+        <v>0.0112</v>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
@@ -3320,7 +3320,7 @@
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -3358,19 +3358,19 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2474160</v>
+        <v>2454057</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N40" t="n">
         <v>0.0017</v>
       </c>
       <c r="O40" t="n">
-        <v>0.0017</v>
+        <v>0.0034</v>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
@@ -3393,7 +3393,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3431,19 +3431,19 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1295185</v>
+        <v>1295158</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N41" t="n">
         <v>0.0022</v>
       </c>
       <c r="O41" t="n">
-        <v>0.0022</v>
+        <v>0.0044</v>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
@@ -3466,7 +3466,7 @@
         <v>2</v>
       </c>
       <c r="C42" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -3504,19 +3504,19 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>4120724</v>
+        <v>4130780</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N42" t="n">
         <v>0.0026</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0052</v>
+        <v>0.0104</v>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
@@ -3539,7 +3539,7 @@
         <v>5</v>
       </c>
       <c r="C43" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -3583,13 +3583,13 @@
         <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N43" t="n">
         <v>0.0013</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0065</v>
+        <v>0.013</v>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -3656,13 +3656,13 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N44" t="n">
         <v>0.0008</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0008</v>
+        <v>0.0016</v>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
@@ -3685,7 +3685,7 @@
         <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -3723,19 +3723,19 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>1315820</v>
+        <v>1315050</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N45" t="n">
         <v>0.0056</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0056</v>
+        <v>0.0112</v>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
@@ -3758,7 +3758,7 @@
         <v>6</v>
       </c>
       <c r="C46" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -3796,19 +3796,19 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>16178720</v>
+        <v>16169345</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
       </c>
       <c r="M46" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="N46" t="n">
         <v>0.0026</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0156</v>
+        <v>0.0312</v>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
@@ -3831,7 +3831,7 @@
         <v>7</v>
       </c>
       <c r="C47" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3869,19 +3869,19 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>5812591</v>
+        <v>5812552</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="N47" t="n">
         <v>0.0025</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0175</v>
+        <v>0.035</v>
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
@@ -3904,7 +3904,7 @@
         <v>4</v>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3942,19 +3942,19 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>6493121</v>
+        <v>6490134</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
       </c>
       <c r="M48" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N48" t="n">
         <v>0.0023</v>
       </c>
       <c r="O48" t="n">
-        <v>0.0092</v>
+        <v>0.0184</v>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
@@ -3977,7 +3977,7 @@
         <v>2</v>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -4021,13 +4021,13 @@
         <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N49" t="n">
         <v>0.0008</v>
       </c>
       <c r="O49" t="n">
-        <v>0.0016</v>
+        <v>0.0032</v>
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
@@ -4050,7 +4050,7 @@
         <v>1</v>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -4088,19 +4088,19 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>2002350</v>
+        <v>2002312</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N50" t="n">
         <v>0.0018</v>
       </c>
       <c r="O50" t="n">
-        <v>0.0018</v>
+        <v>0.0036</v>
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
         <v>2</v>
       </c>
       <c r="C51" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -4167,13 +4167,13 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N51" t="n">
         <v>0.0007</v>
       </c>
       <c r="O51" t="n">
-        <v>0.0014</v>
+        <v>0.0028</v>
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
@@ -4196,7 +4196,7 @@
         <v>1</v>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -4240,13 +4240,13 @@
         <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N52" t="n">
         <v>2.1635</v>
       </c>
       <c r="O52" t="n">
-        <v>2.1635</v>
+        <v>4.327</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
@@ -4269,7 +4269,7 @@
         <v>2</v>
       </c>
       <c r="C53" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -4313,13 +4313,13 @@
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N53" t="n">
         <v>0.4099</v>
       </c>
       <c r="O53" t="n">
-        <v>0.8198</v>
+        <v>1.6396</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
@@ -4342,7 +4342,7 @@
         <v>2</v>
       </c>
       <c r="C54" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -4380,19 +4380,19 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>91756</v>
+        <v>89623</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N54" t="n">
         <v>0.1787</v>
       </c>
       <c r="O54" t="n">
-        <v>0.3574</v>
+        <v>0.7148</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
@@ -4415,7 +4415,7 @@
         <v>8</v>
       </c>
       <c r="C55" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -4459,13 +4459,13 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="N55" t="n">
         <v>0.3073</v>
       </c>
       <c r="O55" t="n">
-        <v>2.4584</v>
+        <v>4.9168</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
@@ -4488,7 +4488,7 @@
         <v>1</v>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -4526,19 +4526,19 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>16866</v>
+        <v>16766</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
       </c>
       <c r="M56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N56" t="n">
         <v>0.6618000000000001</v>
       </c>
       <c r="O56" t="n">
-        <v>0.6618000000000001</v>
+        <v>1.3236</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
@@ -4561,7 +4561,7 @@
         <v>1</v>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -4605,13 +4605,13 @@
         <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N57" t="n">
         <v>0.302</v>
       </c>
       <c r="O57" t="n">
-        <v>0.302</v>
+        <v>0.604</v>
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
@@ -4634,7 +4634,7 @@
         <v>1</v>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -4678,13 +4678,13 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N58" t="n">
         <v>11.1319</v>
       </c>
       <c r="O58" t="n">
-        <v>11.1319</v>
+        <v>22.2638</v>
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
@@ -4707,7 +4707,7 @@
         <v>1</v>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -4742,7 +4742,7 @@
         <v>1</v>
       </c>
       <c r="C60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -4777,7 +4777,7 @@
         <v>1</v>
       </c>
       <c r="C61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -4812,7 +4812,7 @@
         <v>1</v>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -4847,7 +4847,7 @@
         <v>1</v>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -4882,7 +4882,7 @@
         <v>1</v>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -4917,7 +4917,7 @@
         <v>1</v>
       </c>
       <c r="C65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -4952,7 +4952,7 @@
         <v>1</v>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -4987,7 +4987,7 @@
         <v>1</v>
       </c>
       <c r="C67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -5022,7 +5022,7 @@
         <v>1</v>
       </c>
       <c r="C68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -5057,7 +5057,7 @@
         <v>1</v>
       </c>
       <c r="C69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -5092,7 +5092,7 @@
         <v>1</v>
       </c>
       <c r="C70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -5127,7 +5127,7 @@
         <v>1</v>
       </c>
       <c r="C71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -5162,7 +5162,7 @@
         <v>1</v>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -5197,7 +5197,7 @@
         <v>1</v>
       </c>
       <c r="C73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -5232,7 +5232,7 @@
         <v>1</v>
       </c>
       <c r="C74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -5267,7 +5267,7 @@
         <v>1</v>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -5302,7 +5302,7 @@
         <v>1</v>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -5334,7 +5334,7 @@
         </is>
       </c>
       <c r="O78" t="n">
-        <v>47.92</v>
+        <v>94.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fab package from the 2026-09-29 05:19 export: 0.2 mm vias, C38/C41/C59 placed
LEAKCAM_gerber.zip rebuilt: all 14 Altium files byte-identical, outline 61.00 x 65.00 mm.
Plated holes are 0.2 mm (917, 0.35 mm pads), 0.6 mm (26) and 0.7 mm (6); no 0.3 mm left.
BOM_ASSEMBLY / CPL: 248 placements, 56 part numbers, now including the bulk caps C38, C41,
C59 (C19702); 0 mismatches against sheets and board, all 191 footprinted parts land pad for
pad with the rotation corrections. Order lists for 2 boards.
</commit_message>
<xml_diff>
--- a/BOM_LCSC.xlsx
+++ b/BOM_LCSC.xlsx
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>39761</v>
+        <v>39411</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
@@ -593,10 +593,10 @@
         <v>2</v>
       </c>
       <c r="N2" t="n">
-        <v>0.765</v>
+        <v>0.7652</v>
       </c>
       <c r="O2" t="n">
-        <v>1.53</v>
+        <v>1.5304</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="L3" t="n">
         <v>1</v>
@@ -666,10 +666,10 @@
         <v>2</v>
       </c>
       <c r="N3" t="n">
-        <v>2.2339</v>
+        <v>2.2346</v>
       </c>
       <c r="O3" t="n">
-        <v>4.4678</v>
+        <v>4.4692</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2506628</v>
+        <v>2389284</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -739,10 +739,10 @@
         <v>4</v>
       </c>
       <c r="N4" t="n">
-        <v>0.0384</v>
+        <v>0.0382</v>
       </c>
       <c r="O4" t="n">
-        <v>0.1536</v>
+        <v>0.1528</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>175546</v>
+        <v>445428</v>
       </c>
       <c r="L5" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>11684241</v>
+        <v>13393314</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
@@ -885,10 +885,10 @@
         <v>24</v>
       </c>
       <c r="N6" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0086</v>
       </c>
       <c r="O6" t="n">
-        <v>0.2088</v>
+        <v>0.2064</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>3484695</v>
+        <v>3401082</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>2087450</v>
+        <v>2026152</v>
       </c>
       <c r="L8" t="n">
         <v>1</v>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>715431</v>
+        <v>675259</v>
       </c>
       <c r="L9" t="n">
         <v>1</v>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>2407623</v>
+        <v>2373107</v>
       </c>
       <c r="L10" t="n">
         <v>1</v>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>2663079</v>
+        <v>2654366</v>
       </c>
       <c r="L11" t="n">
         <v>1</v>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>2004</v>
+        <v>2000</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>636429</v>
+        <v>528492</v>
       </c>
       <c r="L13" t="n">
         <v>1</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>500802</v>
+        <v>478482</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
@@ -1469,10 +1469,10 @@
         <v>4</v>
       </c>
       <c r="N14" t="n">
-        <v>0.1652</v>
+        <v>0.1653</v>
       </c>
       <c r="O14" t="n">
-        <v>0.6608000000000001</v>
+        <v>0.6612</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>2119409</v>
+        <v>2039603</v>
       </c>
       <c r="L15" t="n">
         <v>1</v>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>8059</v>
+        <v>7978</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
@@ -1615,10 +1615,10 @@
         <v>10</v>
       </c>
       <c r="N16" t="n">
-        <v>0.1712</v>
+        <v>0.1713</v>
       </c>
       <c r="O16" t="n">
-        <v>1.712</v>
+        <v>1.713</v>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>16344</v>
+        <v>13040</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
@@ -1688,10 +1688,10 @@
         <v>4</v>
       </c>
       <c r="N17" t="n">
-        <v>0.1538</v>
+        <v>0.1539</v>
       </c>
       <c r="O17" t="n">
-        <v>0.6152</v>
+        <v>0.6156</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>18115</v>
+        <v>17701</v>
       </c>
       <c r="L18" t="n">
         <v>1</v>
@@ -1761,10 +1761,10 @@
         <v>6</v>
       </c>
       <c r="N18" t="n">
-        <v>0.9778</v>
+        <v>0.9624</v>
       </c>
       <c r="O18" t="n">
-        <v>5.8668</v>
+        <v>5.7744</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>8244</v>
+        <v>7714</v>
       </c>
       <c r="L19" t="n">
         <v>1</v>
@@ -1834,10 +1834,10 @@
         <v>4</v>
       </c>
       <c r="N19" t="n">
-        <v>1.0841</v>
+        <v>1.0845</v>
       </c>
       <c r="O19" t="n">
-        <v>4.3364</v>
+        <v>4.338</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
@@ -1853,14 +1853,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C2 C3 C4 C11 C15 C16 C19 C50 C90 C96 C99 C102 C105 C106 CB1</t>
+          <t>C2 C3 C4 C11 C15 C16 C19 C38 C41 C50 C59 C90 C96 C99 C102 C105 C106 CB1</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C20" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1898,19 +1898,19 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>11251848</v>
+        <v>10811881</v>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="N20" t="n">
         <v>0.0307</v>
       </c>
       <c r="O20" t="n">
-        <v>0.921</v>
+        <v>1.1052</v>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>6248852</v>
+        <v>6528534</v>
       </c>
       <c r="L21" t="n">
         <v>1</v>
@@ -1980,10 +1980,10 @@
         <v>2</v>
       </c>
       <c r="N21" t="n">
-        <v>0.0147</v>
+        <v>0.016</v>
       </c>
       <c r="O21" t="n">
-        <v>0.0294</v>
+        <v>0.032</v>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>8373464</v>
+        <v>8138278</v>
       </c>
       <c r="L22" t="n">
         <v>1</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>4013302</v>
+        <v>3826305</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>783049</v>
+        <v>829216</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -2199,10 +2199,10 @@
         <v>2</v>
       </c>
       <c r="N24" t="n">
-        <v>0.0906</v>
+        <v>0.0907</v>
       </c>
       <c r="O24" t="n">
-        <v>0.1812</v>
+        <v>0.1814</v>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>1073957</v>
+        <v>1024590</v>
       </c>
       <c r="L25" t="n">
         <v>1</v>
@@ -2336,7 +2336,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>2425</v>
+        <v>107395</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -2345,10 +2345,10 @@
         <v>6</v>
       </c>
       <c r="N26" t="n">
-        <v>0.4021</v>
+        <v>0.1301</v>
       </c>
       <c r="O26" t="n">
-        <v>2.4126</v>
+        <v>0.7806</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>112055</v>
+        <v>111195</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>43619</v>
+        <v>42969</v>
       </c>
       <c r="L28" t="n">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>33690</v>
+        <v>33638</v>
       </c>
       <c r="L29" t="n">
         <v>1</v>
@@ -2628,7 +2628,7 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>438</v>
+        <v>422</v>
       </c>
       <c r="L30" t="n">
         <v>1</v>
@@ -2637,10 +2637,10 @@
         <v>16</v>
       </c>
       <c r="N30" t="n">
-        <v>0.3379</v>
+        <v>0.338</v>
       </c>
       <c r="O30" t="n">
-        <v>5.4064</v>
+        <v>5.408</v>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>14960</v>
+        <v>14917</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
@@ -2774,7 +2774,7 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="L32" t="n">
         <v>1</v>
@@ -2783,10 +2783,10 @@
         <v>2</v>
       </c>
       <c r="N32" t="n">
-        <v>13.2782</v>
+        <v>13.2821</v>
       </c>
       <c r="O32" t="n">
-        <v>26.5564</v>
+        <v>26.5642</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2186424</v>
+        <v>2195093</v>
       </c>
       <c r="L33" t="n">
         <v>1</v>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>8980361</v>
+        <v>9302722</v>
       </c>
       <c r="L34" t="n">
         <v>1</v>
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>23769742</v>
+        <v>22565709</v>
       </c>
       <c r="L35" t="n">
         <v>1</v>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>708170</v>
+        <v>635440</v>
       </c>
       <c r="L36" t="n">
         <v>1</v>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>2682285</v>
+        <v>2558402</v>
       </c>
       <c r="L37" t="n">
         <v>1</v>
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>8695277</v>
+        <v>8193723</v>
       </c>
       <c r="L38" t="n">
         <v>1</v>
@@ -3285,7 +3285,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>2672337</v>
+        <v>2647584</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>2454057</v>
+        <v>2398772</v>
       </c>
       <c r="L40" t="n">
         <v>1</v>
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>1295158</v>
+        <v>3249061</v>
       </c>
       <c r="L41" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>4130780</v>
+        <v>4845613</v>
       </c>
       <c r="L42" t="n">
         <v>1</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>296076</v>
+        <v>226576</v>
       </c>
       <c r="L43" t="n">
         <v>1</v>
@@ -3650,7 +3650,7 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>7960</v>
+        <v>4940</v>
       </c>
       <c r="L44" t="n">
         <v>1</v>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>1315050</v>
+        <v>1246785</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>16169345</v>
+        <v>15797686</v>
       </c>
       <c r="L46" t="n">
         <v>1</v>
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>5812552</v>
+        <v>5635923</v>
       </c>
       <c r="L47" t="n">
         <v>1</v>
@@ -3942,7 +3942,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>6490134</v>
+        <v>6422447</v>
       </c>
       <c r="L48" t="n">
         <v>1</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>7360</v>
+        <v>7320</v>
       </c>
       <c r="L49" t="n">
         <v>1</v>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>2002312</v>
+        <v>1956469</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>130518</v>
+        <v>130458</v>
       </c>
       <c r="L51" t="n">
         <v>1</v>
@@ -4234,7 +4234,7 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>356</v>
+        <v>324</v>
       </c>
       <c r="L52" t="n">
         <v>1</v>
@@ -4243,10 +4243,10 @@
         <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>2.1635</v>
+        <v>2.1642</v>
       </c>
       <c r="O52" t="n">
-        <v>4.327</v>
+        <v>4.3284</v>
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>2074</v>
+        <v>2029</v>
       </c>
       <c r="L53" t="n">
         <v>1</v>
@@ -4316,10 +4316,10 @@
         <v>4</v>
       </c>
       <c r="N53" t="n">
-        <v>0.4099</v>
+        <v>0.41</v>
       </c>
       <c r="O53" t="n">
-        <v>1.6396</v>
+        <v>1.64</v>
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>89623</v>
+        <v>444029</v>
       </c>
       <c r="L54" t="n">
         <v>1</v>
@@ -4389,10 +4389,10 @@
         <v>4</v>
       </c>
       <c r="N54" t="n">
-        <v>0.1787</v>
+        <v>0.1788</v>
       </c>
       <c r="O54" t="n">
-        <v>0.7148</v>
+        <v>0.7151999999999999</v>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
@@ -4453,7 +4453,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>19504</v>
+        <v>19388</v>
       </c>
       <c r="L55" t="n">
         <v>1</v>
@@ -4462,10 +4462,10 @@
         <v>16</v>
       </c>
       <c r="N55" t="n">
-        <v>0.3073</v>
+        <v>0.3074</v>
       </c>
       <c r="O55" t="n">
-        <v>4.9168</v>
+        <v>4.9184</v>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
@@ -4526,7 +4526,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>16766</v>
+        <v>15627</v>
       </c>
       <c r="L56" t="n">
         <v>1</v>
@@ -4535,10 +4535,10 @@
         <v>2</v>
       </c>
       <c r="N56" t="n">
-        <v>0.6618000000000001</v>
+        <v>0.662</v>
       </c>
       <c r="O56" t="n">
-        <v>1.3236</v>
+        <v>1.324</v>
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="K57" t="n">
-        <v>6244</v>
+        <v>6189</v>
       </c>
       <c r="L57" t="n">
         <v>1</v>
@@ -4608,10 +4608,10 @@
         <v>2</v>
       </c>
       <c r="N57" t="n">
-        <v>0.302</v>
+        <v>0.3021</v>
       </c>
       <c r="O57" t="n">
-        <v>0.604</v>
+        <v>0.6042</v>
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>7614</v>
+        <v>7602</v>
       </c>
       <c r="L58" t="n">
         <v>1</v>
@@ -4681,10 +4681,10 @@
         <v>2</v>
       </c>
       <c r="N58" t="n">
-        <v>11.1319</v>
+        <v>11.1352</v>
       </c>
       <c r="O58" t="n">
-        <v>22.2638</v>
+        <v>22.2704</v>
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
@@ -5334,7 +5334,7 @@
         </is>
       </c>
       <c r="O78" t="n">
-        <v>94.48</v>
+        <v>92.97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>